<commit_message>
Show all user list with Search filter and pagination
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re245fdc2573040f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R8cd2ddd66bcc41a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R18608a34070b4562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R862cd5550efa4eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R4397aa53f95242b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R1b9794baca4246a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -654,7 +654,7 @@
       </x:c>
       <x:c r="B7" s="15" t="n">
         <x:f>COUNTIF(Stories!H4:H73,"In progress")</x:f>
-        <x:v>10</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C7" s="15" t="n"/>
     </x:row>
@@ -694,7 +694,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>FB-009</x:v>
+        <x:v>FB-021</x:v>
       </x:c>
       <x:c r="C10" s="15" t="n"/>
       <x:c r="D10" s="18" t="inlineStr">
@@ -709,15 +709,17 @@
           <x:t xml:space="preserve">Verified progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="29" t="str">
-        <x:v>2026-10-28: non-password creation checks/review evidence retained; phone cleanup remains failed but repair/review/retest explicitly deferred to project end by developer. Password and username-concurrency deferrals preserved. Developer requested user-list lessons now; no new item marked Complete.</x:v>
+      <x:c r="B11" s="29" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-28: non-password creation checks/review evidence retained; phone cleanup remains failed but repair/review/retest explicitly deferred to project end by developer. Password and username-concurrency deferrals preserved. Developer requested user-list lessons now; no new item marked Complete.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C11" s="15" t="n"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="15" t="n"/>
       <x:c r="B12" s="15" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Index.vue with only template, main class p-4 and h1 Users. This shell is not yet routed and displays no records. Next connect UserController::index Inertia response and GET /users in small lessons using existing inspected response conventions; local fictional-only scaffold until viewAny authorization and actor-specific query are enforced. Teach props/v-for/stable keys, then layout and each filter/pagination separately. Review whole list feature at checkpoint; developer-first tests unless explicitly delegated. Preserve all deferred phone/password/concurrency work and prior evidence; no creation/list completion inferred.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n"/>
       <x:c r="D12" s="15" t="n"/>
@@ -733,7 +735,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>FB-009</x:v>
+        <x:v>FB-021</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="100" customHeight="1">
@@ -743,7 +745,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>Start user-list page shell: developer creates users/Index.vue with a Users heading and existing p-4 spacing. Route and data follow in separate lessons.</x:v>
+        <x:v>2026-10-29 developer replied done to UserPolicy::update actor+target rule lesson. Recorded as application confirmation only; no inspection or behaviour test performed. Next small lesson supplied: create minimal users/Edit.vue using existing shared card layout and heading. Page not yet connected to controller/route; no new browser check requested.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -753,7 +755,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Index.vue with only template, main class p-4 and h1 Users. This shell is not yet routed and displays no records. Next connect UserController::index Inertia response and GET /users in small lessons using existing inspected response conventions; local fictional-only scaffold until viewAny authorization and actor-specific query are enforced. Teach props/v-for/stable keys, then layout and each filter/pagination separately. Review whole list feature at checkpoint; developer-first tests unless explicitly delegated. Preserve all deferred phone/password/concurrency work and prior evidence; no creation/list completion inferred.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -763,7 +765,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Waiting for developer to create the minimal users/Index.vue page file. No browser test requested for the unrouted shell.</x:v>
+        <x:v>Waiting for developer to create minimal users/Edit.vue; no application tests requested or delegated.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -772,8 +774,10 @@
           <x:t xml:space="preserve">Last reviewed revision</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" s="22" t="str">
-        <x:v>2026-10-28 review at HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus working Create.vue/settings route changes. SHA256 and reviewed paths in Stories. Browser evidence /tmp/foodbank-browser-checks/. Phone finding prevents passed creation review.</x:v>
+      <x:c r="B17" s="22" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -1689,15 +1693,19 @@
       <x:c r="P8" s="30" t="n">
         <x:v>46321</x:v>
       </x:c>
-      <x:c r="Q8" s="10" t="str">
-        <x:v>2026-10-26: Developer delegated all tests. Assistant ran existing suite against SQLite :memory: (34 passed, 2 registration tests skipped, 103 assertions) at dbb7dce585b629b40bf4514412abd0119c239d4f. Brave checks passed: logout, direct dashboard URL redirects to login, blank login, missing password and invalid password errors. Asked developer to sign in for Remember me; developer replied no need, checks are done. Stopped browser testing as requested; no assistant verification of remembered-session persistence or inactive-session denial. Source review confirms missing active-session restriction. Keep access work open.
+      <x:c r="Q8" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-26: Developer delegated all tests. Assistant ran existing suite against SQLite :memory: (34 passed, 2 registration tests skipped, 103 assertions) at dbb7dce585b629b40bf4514412abd0119c239d4f. Brave checks passed: logout, direct dashboard URL redirects to login, blank login, missing password and invalid password errors. Asked developer to sign in for Remember me; developer replied no need, checks are done. Stopped browser testing as requested; no assistant verification of remembered-session persistence or inactive-session denial. Source review confirms missing active-session restriction. Keep access work open.
 2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.
 2026-10-26 explicit developer decision: keep existing self-service password-reset feature/routes enabled for now. Withdraw the proposed removal of Features::resetPasswords(). This is an accepted temporary configuration exception, not approval to expand the recovery feature or mark it verified. Do not repeatedly ask to disable it. Full self-service recovery remains FUTURE.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
-      </x:c>
-      <x:c r="R8" s="10" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. Resume remaining access/foundation checkpoint review and evidence reconciliation without re-requesting stopped browser checks. Inactive existing-session enforcement is deferred to FB-022; existing password-reset routes are intentionally retained for now per 2026-10-26 developer instruction. Do not teach their removal. Preserve original test/review evidence and do not infer missing checks passed. Existing Super Admin password and must_change_password=0 stay unchanged; new-account setup verification remains deferred to FB-019.
-Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R8" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. Resume remaining access/foundation checkpoint review and evidence reconciliation without re-requesting stopped browser checks. Inactive existing-session enforcement is deferred to FB-022; existing password-reset routes are intentionally retained for now per 2026-10-26 developer instruction. Do not teach their removal. Preserve original test/review evidence and do not infer missing checks passed. Existing Super Admin password and must_change_password=0 stay unchanged; new-account setup verification remains deferred to FB-019.
+Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S8" s="10" t="n"/>
     </x:row>
@@ -1743,25 +1751,34 @@
           <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="J9" s="11" t="str">
-        <x:v>Changes needed</x:v>
-      </x:c>
-      <x:c r="K9" s="11" t="str">
-        <x:v>
+      <x:c r="J9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Changes needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-26 partial connected-save source review, working tree based on f5ab5c17f023f0ff30b422a8fa66d2746f2d5cb1: UserController, UserPolicy, routes/web.php, StoreUserRequest, User and Role models, GenerateUsername, GetAssignableRoles, users/Create.vue, create_users_table migration, config/auth.php and app.ts inspected. GET/POST create policy, permitted target roles, fields, hash cast, save, flash and temporary dashboard redirect connected. Original-name checks now precede normalization. Finding: UserPolicy update currently permits managers against any target; restrict to volunteer targets before enabling edits. Username concurrent collision handling and complete access tests remain open. No assistant application edits or runtime tests; not full feature review.
-2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:v>
-      </x:c>
-      <x:c r="L9" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M9" s="11" t="str">
-        <x:v>Assistant (explicitly delegated; prior developer evidence retained)</x:v>
-      </x:c>
-      <x:c r="N9" s="11" t="str">
-        <x:v>Failed</x:v>
-      </x:c>
-      <x:c r="O9" s="11" t="str">
-        <x:v>2026-10-26 developer-reported PASS: confirms database-backed role dropdown is working following explicit Super Admin choice/selection check. No assistant runtime test; other account/role permissions and full creation remain untested.
+2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L9" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="M9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Assistant (explicitly delegated; prior developer evidence retained)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Failed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-26 developer-reported PASS: confirms database-backed role dropdown is working following explicit Super Admin choice/selection check. No assistant runtime test; other account/role permissions and full creation remain untested.
 2026-10-26 developer-reported PASS: migration applied successfully and users-table check shows Super, Admin and +1 506-555-0100 in the three added columns. No assistant runtime test or completed-feature review.
 2026-10-26 assistant-executed php artisan test, explicitly delegated by developer: 35 tests, 33 passed, 2 failed, 112 assertions, exit 1. Failures: ProfileUpdateTest.php:25 and UserSeedingTest.php:40 compare pre-reload model attributes with database-loaded attributes; defaults, boolean representation and key order differ. Proposed correction: take original snapshot using $user-&gt;fresh()-&gt;getAttributes() in both tests. No source changes made. Suite requires rerun; browser checks and full creation review remain pending.
 2026-10-26 explicit developer authorization: do the changes. Assistant changed original snapshots to fresh()-&gt;getAttributes() in tests/Feature/Settings/ProfileUpdateTest.php and tests/Feature/UserSeedingTest.php. Delegated php artisan test rerun passed: 35 tests, 115 assertions, exit 0. git diff --check passed. These two failures are resolved. Browser name/initials, settings navigation and unavailable profile checks remain pending; full account-creation review/testing incomplete.
@@ -1769,13 +1786,15 @@
 2026-10-26 developer-reported PASS: after explicit fictional-account browser save and database inspection instructions, developer confirmed everything worked, account created, and invalid-input checks behaved as expected. This confirms the requested dashboard/success and stored-field checks, including role/status/setup flag/password hash, as developer reports only. Additional invalid-input cases were not enumerated; do not claim exhaustive validation, denied-access, concurrency or first-login testing.
 2026-10-28 assistant-executed checks, explicitly delegated by developer, using ChatGPT in-app browser (not Brave), local http://foodbank.test, existing Super Admin session signed in by developer. PASS: Manager/Volunteer choices; required first/last/email/phone and missing-role errors; processing button disabled then reenabled; incomplete-phone rejection and retained input; Bad@Name and --- rejected; first/last 101-character rejection; 255-character email rejected as invalid (max-specific error not independently exercised); uppercase duplicate email rejected; accented/curly-apostrophe/hyphenated/internal-space names preserved and outer spaces trimmed; normalized sequential usernames emilie.oconnor, .01 and .02 across roles; default Active, explicit Inactive, shared phone; details redirect, success toast, formatted saved phone and reload persistence. PASS responsive Create form at 375x850 (no horizontal overflow, one column) and 1100x850 (two columns). Phone normal typing, extra-digit limit, selecting/replacing final four digits, clear and actual clipboard formatted paste passed. FAIL: type 506 then x into empty Phone; +1 506x remains visible. Screenshot /tmp/foodbank-browser-checks/phone-nondigit-failure.png. Shared Input passive local value and unchanged parent sanitized value explain display mismatch. No application code changed. Evidence JSON and screenshots in /tmp/foodbank-browser-checks/.
 2026-10-28 assistant-executed isolated HTTP permission checks, SQLite :memory: with explicit isolation guard, no development users altered: Manager GET create 200; forged Manager-to-Manager POST role_id validation error and unchanged user count; Super Admin forbidden Super Admin target role rejected without saving; Volunteer GET and POST 403 with unchanged count; Manager-to-Volunteer POST saved correct role. Five grouped checks passed. Initial one-off harness completed assertions but failed in PHPUnit teardown without runner configuration; corrected ephemeral harness rerun closed the in-memory connection directly and exited 0. No application/test source files written. These are isolated HTTP checks, not Manager browser sign-in evidence. No password checks run.
-2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:v>
-      </x:c>
-      <x:c r="P9" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q9" s="11" t="str">
-        <x:v>2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes.
+2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P9" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="Q9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes.
 Create-user lesson 1 issued: developer creates resources/js/pages/users/Create.vue containing template, main and Create user heading only. No route, persistence or behaviour check yet; await developer confirmation.
 Poker inspected 2026-10-26: routes/web.php uses -&gt;can(create, Player::class) on GET create and POST store. app/Http/Controllers/PlayerController.php create returns Inertia::render(players/Create); store validates with StorePlayerRequest and directly creates the simple record. app/Policies/PlayerPolicy.php owns permission; app/Http/Requests/Players/StorePlayerRequest.php authorize returns true because routes enforce policy. FoodBank target-role restrictions and details redirect follow approved requirements, not Poker domain rules.
 2026-10-26: Developer confirmed minimal users/Create.vue creation. No intermediate review or behaviour test. Lesson 2: explain controller responsibility and ask developer to run php artisan make:controller UserController. Await command confirmation.
@@ -1826,10 +1845,13 @@
 2026-10-26 developer asked how to confirm case-insensitive database email uniqueness. Assistant read-only live MySQL inspection via Laravel: users.email COLLATION_NAME=utf8mb4_unicode_ci; unique index users_email_unique, Non_unique=0, Seq_in_index=1, full email column (Sub_part null). Read-only comparison of Amina@example.com and amina@example.com under this collation returned same_email=1. No records changed or duplicate inserts attempted. Built-in unique:users,email recommended for this MySQL configuration; replacing custom callback has not been approved/applied. SQLite-memory test configuration differs and must not be claimed to provide identical case-insensitive behavior. No whole-feature completion.
 2026-10-26 developer confirms replacing custom email callback with unique:users,email and asks next. Treat built-in rule as approved/applied by developer, not reviewed/tested. Prior MySQL case-insensitive full unique index evidence retained; SQLite caveat remains. Next small lesson: change generated StoreUserRequest authorize() to return true, matching inspected Poker StorePlayerRequest where routes own resource policy checks. Explain false rejects request before rules; true does not itself grant application permission or save anything. Approved local fictional save-before-policy teaching exception retained. Required UserPolicy create must guard GET /users/create and POST /users via route can middleware before real use/feature completion; Rule::in permitted target IDs stays separate. Await developer application, no unsolicited source review or assistant edits/tests.
 2026-10-26 developer confirms authorize return true step; ordinary coding confirmation, no review/test. Next small le
-2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:v>
-      </x:c>
-      <x:c r="R9" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:v>
+2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R9" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S9" s="11" t="n"/>
     </x:row>
@@ -1875,33 +1897,44 @@
           <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="J10" s="10" t="str">
-        <x:v>Changes needed</x:v>
-      </x:c>
-      <x:c r="K10" s="10" t="str">
-        <x:v>
-2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:v>
-      </x:c>
-      <x:c r="L10" s="30" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M10" s="10" t="str">
-        <x:v>Assistant (explicitly delegated; prior developer evidence retained)</x:v>
-      </x:c>
-      <x:c r="N10" s="10" t="str">
-        <x:v>Failed</x:v>
-      </x:c>
-      <x:c r="O10" s="10" t="str">
-        <x:v>
+      <x:c r="J10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Changes needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L10" s="30" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="M10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Assistant (explicitly delegated; prior developer evidence retained)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Failed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-28 assistant-executed checks, explicitly delegated by developer, using ChatGPT in-app browser (not Brave), local http://foodbank.test, existing Super Admin session signed in by developer. PASS: Manager/Volunteer choices; required first/last/email/phone and missing-role errors; processing button disabled then reenabled; incomplete-phone rejection and retained input; Bad@Name and --- rejected; first/last 101-character rejection; 255-character email rejected as invalid (max-specific error not independently exercised); uppercase duplicate email rejected; accented/curly-apostrophe/hyphenated/internal-space names preserved and outer spaces trimmed; normalized sequential usernames emilie.oconnor, .01 and .02 across roles; default Active, explicit Inactive, shared phone; details redirect, success toast, formatted saved phone and reload persistence. PASS responsive Create form at 375x850 (no horizontal overflow, one column) and 1100x850 (two columns). Phone normal typing, extra-digit limit, selecting/replacing final four digits, clear and actual clipboard formatted paste passed. FAIL: type 506 then x into empty Phone; +1 506x remains visible. Screenshot /tmp/foodbank-browser-checks/phone-nondigit-failure.png. Shared Input passive local value and unchanged parent sanitized value explain display mismatch. No application code changed. Evidence JSON and screenshots in /tmp/foodbank-browser-checks/.
 2026-10-28 assistant-executed isolated HTTP permission checks, SQLite :memory: with explicit isolation guard, no development users altered: Manager GET create 200; forged Manager-to-Manager POST role_id validation error and unchanged user count; Super Admin forbidden Super Admin target role rejected without saving; Volunteer GET and POST 403 with unchanged count; Manager-to-Volunteer POST saved correct role. Five grouped checks passed. Initial one-off harness completed assertions but failed in PHPUnit teardown without runner configuration; corrected ephemeral harness rerun closed the in-memory connection directly and exited 0. No application/test source files written. These are isolated HTTP checks, not Manager browser sign-in evidence. No password checks run.
-2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:v>
-      </x:c>
-      <x:c r="P10" s="30" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q10" s="10" t="str">
-        <x:v>2026-10-27 static audit at 8ac5a6a: Create.vue has a one-column mobile/two-column wider layout and phone field, but no automatic Canadian phone formatting while typing. Source inspection only; review and behaviour test remain open.
+2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P10" s="30" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="Q10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-27 static audit at 8ac5a6a: Create.vue has a one-column mobile/two-column wider layout and phone field, but no automatic Canadian phone formatting while typing. Source inspection only; review and behaviour test remain open.
 2026-10-28 resumed after account-creation checkpoint inspection at HEAD fca09f784ede715423dc167d1a6ab966c7431451 confirmed missing automatic phone formatting. Current small lesson: add updatePhone(value: string | number) to Create.vue, strip non-digits using String(value).replace(/\D/g, empty string), replace phone v-model with :model-value and @update:model-value. Temporary digits-only step, not finished phone formatting and not ready for saving. Next add country prefix/grouping separately. Shared Input emits update:modelValue with string|number. No assistant application edits/tests; developer applies code.
 2026-10-28 developer replied done after the digits-only phone lesson and paste experiment. Accepted as developer confirmation of this intermediate lesson only, not feature-wide review/test completion. No source inspection after done. Next lesson: updatePhone converts incoming value to text, removes an existing leading +1 before digit cleanup, and adds one +1 plus a space when digits exist; empty input stays empty. Keep existing explicit model-value/event binding. Grouping and full behaviour checks follow separately.
 2026-10-28 developer replied done after the +1 prefix lesson and typing experiment. Accepted as confirmation of that intermediate lesson only; no source review or feature-wide completion. Next lesson replaces only final assignment in updatePhone with progressive hyphen grouping: first 3 digits, next 3 once present, remaining digits after 6; add country prefix when digits exist. Explain let, slice start/end and if. Ten-digit limiting and complete paste/deletion behaviour remain later lessons/checks.
@@ -1913,10 +1946,13 @@
 2026-10-28 learning checkpoint passed: developer explained that removing the existing +1 prevents adding it again each time they type. Next small behaviour check: with +1 506-555-0123 displayed, select only final 0123 and replace with 9876; expect +1 506-555-9876. This checks correction within an already full-length formatted input. No source review or application tests executed by assistant.
 2026-10-28 developer clarified displayed example was placeholder, not selectable entered text, and explicitly asked to move forward because satisfied with current phone behaviour. Final-four-digits correction check was NOT performed and is not a pass. Stop further phone exercises now; preserve earlier specific reported evidence and keep FB-017 open pending review/remaining evidence. No broader project-end deferral inferred for phone checks.
 2026-10-28 delegated checks completed: formatting/length/replacement/clear/paste/layout PASS, but typing a letter after 506 leaves +1 506x visible. Failed non-digit cleanup is recorded; no fix applied.
-2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:v>
-      </x:c>
-      <x:c r="R10" s="10" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:v>
+2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R10" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S10" s="10" t="n"/>
     </x:row>
@@ -1962,39 +1998,51 @@
           <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="J11" s="11" t="str">
-        <x:v>Changes needed</x:v>
-      </x:c>
-      <x:c r="K11" s="11" t="str">
-        <x:v>
-2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:v>
-      </x:c>
-      <x:c r="L11" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M11" s="11" t="str">
-        <x:v>Assistant (delegated browser checks)</x:v>
+      <x:c r="J11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Changes needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L11" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="M11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Assistant (delegated browser checks)</x:t>
+        </x:is>
       </x:c>
       <x:c r="N11" s="11" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Not tested</x:t>
         </x:is>
       </x:c>
-      <x:c r="O11" s="11" t="str">
-        <x:v>
-2026-10-28 delegated browser PASS for serial normalization/collisions: Émilie O’Connor -&gt; emilie.oconnor; Emilie O'Connor -&gt; .01; Émi-lie O Connor -&gt; .02, across Volunteer/Manager roles; names preserved and trimmed, invalid symbols/unusable/overlong names rejected. Simultaneous-save fix/test explicitly deferred and not passed.</x:v>
-      </x:c>
-      <x:c r="P11" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q11" s="11" t="str">
-        <x:v>2026-10-27 static audit at 8ac5a6a: GenerateUsername.php implements first.last, accent conversion, name-part validation and numbered suffix lookup. Concurrent collision handling and full behaviour checks remain open. Source inspection only; not a completed-feature review.
+      <x:c r="O11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-28 delegated browser PASS for serial normalization/collisions: Émilie O’Connor -&gt; emilie.oconnor; Emilie O'Connor -&gt; .01; Émi-lie O Connor -&gt; .02, across Volunteer/Manager roles; names preserved and trimmed, invalid symbols/unusable/overlong names rejected. Simultaneous-save fix/test explicitly deferred and not passed.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P11" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="Q11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-27 static audit at 8ac5a6a: GenerateUsername.php implements first.last, accent conversion, name-part validation and numbered suffix lookup. Concurrent collision handling and full behaviour checks remain open. Source inspection only; not a completed-feature review.
 2026-10-28 correction to earlier source finding: curly apostrophe issue retracted. Read-only inspection of vendor/laravel/framework/src/Illuminate/Support/Str.php and vendor/voku/portable-ascii/src/voku/helper/ASCII.php plus data/ascii_by_languages.php shows existing Str::ascii conversion handles non-ASCII punctuation before the later ASCII-only check (curly apostrophe mapping exists); no application fix justified by the previous claim. No runtime test run. Concurrent username selection/save handling remains an actual open concern. Next explain two simultaneous same-name saves and request focused Poker save/duplicate-conflict reference lookup because inspected reference Security workflow does not cover it. Do not invent a Laravel action/transaction/retry convention.
 2026-10-28 developer declined further Poker lookup for this issue and asked whether a database lock can solve username-save concurrency. Read-only inspection reconfirms GenerateUsername exists-then-create gap and users.username unique index. Explain robust locking needs a shared existing lock target covering generation plus save; locking a candidate username lookup alone is not a sufficient general solution because username may not exist and gap locking depends on query/isolation. Simpler proposal: keep unique index and bounded retry only for confirmed username-constraint collision, regenerating candidate on retry. No approach chosen yet; no application edits/tests authorized or performed. Do not renew the declined Poker lookup request.
-2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now.</x:v>
-      </x:c>
-      <x:c r="R11" s="11" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. Username concurrency work deferred by developer until final project verification after FB-070 implementation/review/testing. Then choose locking or bounded username-conflict retry, teach developer-written fix, review actual code and verify concurrent saves plus existing username rules. Approach undecided; no resolution/pass claimed. Keep FB-018 open and preserve prior evidence. Continue eligible connected work meanwhile.</x:v>
+2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R11" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. Username concurrency work deferred by developer until final project verification after FB-070 implementation/review/testing. Then choose locking or bounded username-conflict retry, teach developer-written fix, review actual code and verify concurrent saves plus existing username rules. Approach undecided; no resolution/pass claimed. Keep FB-018 open and preserve prior evidence. Continue eligible connected work meanwhile.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S11" s="11" t="n"/>
     </x:row>
@@ -2142,39 +2190,50 @@
           <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
-      <x:c r="J13" s="11" t="str">
-        <x:v>Changes needed</x:v>
-      </x:c>
-      <x:c r="K13" s="11" t="str">
-        <x:v>
+      <x:c r="J13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Changes needed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-26 partial connected-save source review, working tree based on f5ab5c17f023f0ff30b422a8fa66d2746f2d5cb1: UserController, UserPolicy, routes/web.php, StoreUserRequest, User and Role models, GenerateUsername, GetAssignableRoles, users/Create.vue, create_users_table migration, config/auth.php and app.ts inspected. GET/POST create policy, permitted target roles, fields, hash cast, save, flash and temporary dashboard redirect connected. Original-name checks now precede normalization. Finding: UserPolicy update currently permits managers against any target; restrict to volunteer targets before enabling edits. Username concurrent collision handling and complete access tests remain open. No assistant application edits or runtime tests; not full feature review.
 2026-10-28 account-creation checkpoint source inspection, working tree HEAD fca09f784ede715423dc167d1a6ab966c7431451: inspected routes/web.php, UserController, UserPolicy, StoreUserRequest, GenerateUsername, GetAssignableRoles, User/Role models, RoleCode enum, users/Create.vue, shared Input component, SetupPasswordController and bootstrap/app.php. Not a passed full review. Findings: required automatic phone formatting absent in Create.vue (FB-017/REQ-038); GenerateUsername permits curly apostrophe before normalization but removes only straight apostrophe afterward, so supported-looking names can be rejected; username exists-then-create concurrency handling remains unresolved from prior review. Overbroad update ability remains FB-021 and is not exposed by a current edit route. No application tests or browser checks executed. Address creation findings before user lists; preserve explicit password/setup deferrals.
 2026-10-28 correction to earlier source finding: curly apostrophe issue retracted. Read-only inspection of vendor/laravel/framework/src/Illuminate/Support/Str.php and vendor/voku/portable-ascii/src/voku/helper/ASCII.php plus data/ascii_by_languages.php shows existing Str::ascii conversion handles non-ASCII punctuation before the later ASCII-only check (curly apostrophe mapping exists); no application fix justified by the previous claim. No runtime test run. Concurrent username selection/save handling remains an actual open concern.
 2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now.
-2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:v>
-      </x:c>
-      <x:c r="L13" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="M13" s="11" t="str">
-        <x:v>Assistant (explicitly delegated; prior developer evidence retained)</x:v>
-      </x:c>
-      <x:c r="N13" s="11" t="str">
-        <x:v>Failed</x:v>
-      </x:c>
-      <x:c r="O13" s="11" t="str">
-        <x:v>
+2026-10-28 completed account-creation checkpoint review of routes/web.php; UserController; StoreUserRequest; GenerateUsername; GetAssignableRoles; UserPolicy; User/Role models and RoleCode; create_users migration; users/Create.vue; users/Show.vue; shared ui/input/Input.vue; HandleInertiaRequests; flashToast and app.ts. Creation GET/POST create policy, target-role validation, field allowlist, name generation, persistence, named details redirect and global toast connected. Finding: phone cleanup is not consistently reflected in displayed shared Input when sanitized parent value does not change; confirmed by browser +1 506x. Keep affected items open. Concurrent username-save handling remains explicitly deferred, not fixed; overbroad update policy remains FB-021 and no edit route is exposed. Earlier apostrophe finding remains retracted. Create.vue SHA256 5942b63c5506f9f17a51a31e98f9dbab66dfcccc96fc92927a0a3a61d61f5d82; shared Input SHA256 7a55fe41c84a9addb5e8dbaa3b1c84d892062276a9a8d8fcd59a65e68e79c85c.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L13" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="M13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Assistant (explicitly delegated; prior developer evidence retained)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="N13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Failed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-26 developer-reported PASS: after explicit fictional-account browser save and database inspection instructions, developer confirmed everything worked, account created, and invalid-input checks behaved as expected. This confirms the requested dashboard/success and stored-field checks, including role/status/setup flag/password hash, as developer reports only. Additional invalid-input cases were not enumerated; do not claim exhaustive validation, denied-access, concurrency or first-login testing.\n2026-10-28 assistant-run local browser checks, Manager account: dropdown offered Volunteer only; blank required fields, invalid phone format, uppercase duplicate email, and 101-character first name were rejected. Names with outer spaces were saved trimmed. Created fictional QA Volunteer (user 16, qa.check, fb019-check-20261028@example.com); details page showed Volunteer, Active, and success toast. Initial-password login reached Set your password. Requesting /users/create while setup was required returned to Set your password. Source trace: POST route uses create policy; StoreUserRequest restricts role_id to GetAssignableRoles (Manager receives Volunteer only).
 2026-10-28 developer-reported PASS: replied done after explicit Super Admin Manager-creation check. Confirms Manager/Volunteer role choices, selecting Manager and Active, successful fictional account save, generated username, formatted phone +1 506-555-0142, details redirect and success message. Suggested fixture Casey Morgan with unique example.com email; no exact database id or actual email reported. This is creation evidence only, not new-account setup/login, concurrent-save evidence, full source-review pass or all feature completion.
 2026-10-28 assistant-executed checks, explicitly delegated by developer, using ChatGPT in-app browser (not Brave), local http://foodbank.test, existing Super Admin session signed in by developer. PASS: Manager/Volunteer choices; required first/last/email/phone and missing-role errors; processing button disabled then reenabled; incomplete-phone rejection and retained input; Bad@Name and --- rejected; first/last 101-character rejection; 255-character email rejected as invalid (max-specific error not independently exercised); uppercase duplicate email rejected; accented/curly-apostrophe/hyphenated/internal-space names preserved and outer spaces trimmed; normalized sequential usernames emilie.oconnor, .01 and .02 across roles; default Active, explicit Inactive, shared phone; details redirect, success toast, formatted saved phone and reload persistence. PASS responsive Create form at 375x850 (no horizontal overflow, one column) and 1100x850 (two columns). Phone normal typing, extra-digit limit, selecting/replacing final four digits, clear and actual clipboard formatted paste passed. FAIL: type 506 then x into empty Phone; +1 506x remains visible. Screenshot /tmp/foodbank-browser-checks/phone-nondigit-failure.png. Shared Input passive local value and unchanged parent sanitized value explain display mismatch. No application code changed. Evidence JSON and screenshots in /tmp/foodbank-browser-checks/.
 2026-10-28 assistant-executed isolated HTTP permission checks, SQLite :memory: with explicit isolation guard, no development users altered: Manager GET create 200; forged Manager-to-Manager POST role_id validation error and unchanged user count; Super Admin forbidden Super Admin target role rejected without saving; Volunteer GET and POST 403 with unchanged count; Manager-to-Volunteer POST saved correct role. Five grouped checks passed. Initial one-off harness completed assertions but failed in PHPUnit teardown without runner configuration; corrected ephemeral harness rerun closed the in-memory connection directly and exited 0. No application/test source files written. These are isolated HTTP checks, not Manager browser sign-in evidence. No password checks run.
-2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:v>
-      </x:c>
-      <x:c r="P13" s="31" t="d">
-        <x:v>2026-10-28T12:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="Q13" s="11" t="str">
-        <x:v>
+2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P13" s="31" t="n">
+        <x:v>46323.5</x:v>
+      </x:c>
+      <x:c r="Q13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Build saving and create the first local user, then teach FB-006/FB-007. Return to verify FB-016–FB-020 and deferred FB-004 evidence before starting FB-009. This is one connected feature; FB-019 need not be marked Complete before its setup lessons.
 2026-10-26 developer-approved design: use a roles database table plus a PHP role enum in Laravel; load permitted create-user dropdown options from the table through Inertia. Preserve Super Admin -&gt; manager/volunteer and manager -&gt; volunteer permissions; validate permitted roles on submission. Supersedes pending hardcoded controller role arrays. Plan enum/table population and user-role connection before form integration, preserving existing accounts. No implementation or testing claimed.
 2026-10-26: first frontend account save and database check passed (developer-reported). Status changed by developer request from toggle to Active/Inactive radio choices, default Active. useForm fields/errors, processing button, submit, create policy and GET/POST checks implemented; dashboard redirect temporary. Next: build read-only details page in small steps, starting users/Show.vue heading shell. Attach view policy before exposing account props. No list yet; full creation and password setup remain open.
@@ -2193,10 +2252,13 @@
 2026-10-28 assistant-executed isolated HTTP permission checks, SQLite :memory: with explicit isolation guard, no development users altered: Manager GET create 200; forged Manager-to-Manager POST role_id validation error and unchanged user count; Super Admin forbidden Super Admin target role rejected without saving; Volunteer GET and POST 403 with unchanged count; Manager-to-Volunteer POST saved correct role. Five grouped checks passed. Initial one-off harness completed assertions but failed in PHPUnit teardown without runner configuration; corrected ephemeral harness rerun closed the in-memory connection directly and exited 0. No application/test source files written. These are isolated HTTP checks, not Manager browser sign-in evidence. No password checks run.
 2026-10-28 delegated non-password existing tests: filtered UserSeedingTest/ProfileUpdateTest covering user-factory fields, settings redirect, and disabled self-service profile routes: 3 passed, 18 assertions, exit 0. npm run types:check passed (exit 0); php -l UserController/StoreUserRequest passed; git diff --check passed. Password suites excluded. Source snapshot HEAD fca09f784ede715423dc167d1a6ab966c7431451 plus pre-existing working changes in Create.vue and routes/settings.php; source unchanged by assistant.
 Three fictional local accounts created and left in place: /users/15 emilie.oconnor, Inactive Volunteer, fb-browser-20261028-a@example.com; /users/16 emilie.oconnor.01, Active Manager, fb-browser-20261028-b@example.com; /users/17 emilie.oconnor.02, Active Volunteer, fb-browser-20261028-c@example.com. Shared phone +1 506-555-0181. Historical tracker IDs 15/16 referred to different prior fixtures; do not assume those older IDs identify current QA accounts. At final verification reidentify any original QA Volunteer by its recorded email and actual current details, not old ID alone. No credentials were changed or setup tested.
-2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:v>
-      </x:c>
-      <x:c r="R13" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:v>
+2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R13" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Current non-password review/test evidence is retained. Phone-display cleanup repair and verification are explicitly deferred until final project verification after FB-070; preserve failure and keep affected items open. Developer directed user-list lessons FB-009 onward now. Preserve all password-related and username-concurrency final-checkpoint deferrals.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S13" s="11" t="n"/>
     </x:row>
@@ -2275,8 +2337,9 @@
       <x:c r="P14" s="30" t="n">
         <x:v>46322</x:v>
       </x:c>
-      <x:c r="Q14" s="10" t="str">
-        <x:v>2026-10-26: Continue same access feature with FB-006 small UI lesson. Developer to create resources/js/pages/auth/SetupPassword.vue with template/main/h1 heading only. Not yet routed, no behaviour test requested. Existing Super Admin bypass remains unchanged. FB-004/FB-005 stay open for final evidence reconciliation; no prerequisite completion inferred. New-account journey test remains deferred to FB-019, inactive sessions to FB-022, reset routes retained by decision.
+      <x:c r="Q14" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-26: Continue same access feature with FB-006 small UI lesson. Developer to create resources/js/pages/auth/SetupPassword.vue with template/main/h1 heading only. Not yet routed, no behaviour test requested. Existing Super Admin bypass remains unchanged. FB-004/FB-005 stay open for final evidence reconciliation; no prerequisite completion inferred. New-account journey test remains deferred to FB-019, inactive sessions to FB-022, reset routes retained by decision.
 2026-10-26 developer-approved deferral: postpone BUILDING as well as verifying personal-password setup (FB-006/FB-007) until a new user is created through the frontend at FB-019. Withdraw SetupPassword.vue creation instruction; no implementation confirmed. Build the setup screen, access restriction and save/logout/re-login flow in small connected lessons at that checkpoint, before treating account creation as complete. Current scope retained, not FUTURE or verified.
 2026-10-27: developer requested first-login password setup as the next teaching work, using must_change_password, a separate setup form, matching confirmation, password save, logout and fresh login. Existing Laravel settings/reset password module is to remain unchanged. FB-020 account details remains open. Password-rule decision pending because REQ-093 also specifies 12–128 characters and rejecting the initial/current password; no new scope or behaviour is verified.
 2026-10-27 developer decision: first-login setup password validation is minimum 8 characters plus matching confirmation only. No maximum, character-mixture or initial/current-password difference check for this setup. Existing Laravel settings/reset password module remains unchanged. REQ-079/REQ-092 updated to state the consequence if the user chooses the same text as the shared initial password. No lesson or code change started.
@@ -2300,14 +2363,17 @@
 2026-10-27 developer-reported PASS after requested npm run build and refresh: intermittent mint colour no longer appears. Visual fix evidence only; no application source edit or assistant browser test. FB-006/007 remain open for deferred long-password and connected journey evidence.
 2026-10-27 scheduling decision: bcrypt 72-byte long-password repair moved to FB-069 immediately before FB-070. No code fix or new test; existing failed evidence remains. Continue remaining first-login journey work without treating long-password correctness as verified.
 2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
-Three fictional local accounts created and left in place: /users/15 emilie.oconnor, Inactive Volunteer, fb-browser-20261028-a@example.com; /users/16 emilie.oconnor.01, Active Manager, fb-browser-20261028-b@example.com; /users/17 emilie.oconnor.02, Active Volunteer, fb-browser-20261028-c@example.com. Shared phone +1 506-555-0181. Historical tracker IDs 15/16 referred to different prior fixtures; do not assume those older IDs identify current QA accounts. At final verification reidentify any original QA Volunteer by its recorded email and actual current details, not old ID alone. No credentials were changed or setup tested.</x:v>
-      </x:c>
-      <x:c r="R14" s="10" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk. Redirect-loop fix is now reviewed and narrowly tested: web.php/settings.php auth-only groups, unverified pending account reaches setup, completed unverified account reaches dashboard/appearance and password-confirmation/security flow. Await next developer instruction; latest test scope is redirect loop only, do not rerun broader suites automatically. Long-password/bcrypt issue remains deferred and unverified, so FB-006/007 remain open. Earlier seed-test and date-type findings retained; old email-verification redirect test now contradicts approved auth-only policy and needs a later developer-written update before project-wide gates pass. FB-020 connected details still open; do not infer account-creation completion.
+Three fictional local accounts created and left in place: /users/15 emilie.oconnor, Inactive Volunteer, fb-browser-20261028-a@example.com; /users/16 emilie.oconnor.01, Active Manager, fb-browser-20261028-b@example.com; /users/17 emilie.oconnor.02, Active Volunteer, fb-browser-20261028-c@example.com. Shared phone +1 506-555-0181. Historical tracker IDs 15/16 referred to different prior fixtures; do not assume those older IDs identify current QA accounts. At final verification reidentify any original QA Volunteer by its recorded email and actual current details, not old ID alone. No credentials were changed or setup tested.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R14" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk. Redirect-loop fix is now reviewed and narrowly tested: web.php/settings.php auth-only groups, unverified pending account reaches setup, completed unverified account reaches dashboard/appearance and password-confirmation/security flow. Await next developer instruction; latest test scope is redirect loop only, do not rerun broader suites automatically. Long-password/bcrypt issue remains deferred and unverified, so FB-006/007 remain open. Earlier seed-test and date-type findings retained; old email-verification redirect test now contradicts approved auth-only policy and needs a later developer-written update before project-wide gates pass. FB-020 connected details still open; do not infer account-creation completion.
 Before starting this item or feature: reread AGENTS.md from disk. Mint-colour refresh issue resolved by developer report. Resume first-login setup/connected account creation in small lessons on developer instruction; preserve deferred long-password finding and open review/test status.
 Before starting this item or feature: reread AGENTS.md from disk. Resume remaining first-login and connected account-creation checks. The bcrypt repair is assigned to late FB-069, not current teaching steps; preserve failed evidence and current open status until applicable review/test gates pass.
 Developer-directed 2026-10-28 timing: the connected QA Volunteer password-setup and post-setup access/logout/re-login checks are deferred to final project verification after FB-070 implementation, review, and testing. Keep this item open until the required final checks and its review/test gates pass.
-Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:v>
+Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S14" s="10" t="n"/>
     </x:row>
@@ -2389,8 +2455,9 @@
       <x:c r="P15" s="31" t="n">
         <x:v>46322</x:v>
       </x:c>
-      <x:c r="Q15" s="11" t="str">
-        <x:v>
+      <x:c r="Q15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-26 developer-approved deferral: postpone BUILDING as well as verifying personal-password setup (FB-006/FB-007) until a new user is created through the frontend at FB-019. Withdraw SetupPassword.vue creation instruction; no implementation confirmed. Build the setup screen, access restriction and save/logout/re-login flow in small connected lessons at that checkpoint, before treating account creation as complete. Current scope retained, not FUTURE or verified.
 2026-10-27 developer decision: first-login setup password validation is minimum 8 characters plus matching confirmation only. No maximum, character-mixture or initial/current-password difference check for this setup. Existing Laravel settings/reset password module remains unchanged. REQ-079/REQ-092 updated to state the consequence if the user chooses the same text as the shared initial password. No lesson or code change started.
 2026-10-27 developer-approved placement: register the first-login setup guard once in the whole web middleware group in bootstrap/app.php. Its check passes guests and signed-in users with must_change_password=0; users with must_change_password=1 may reach setup display, setup submission and logout, and are redirected from other web routes to setup. Setup routes remain authenticated and outside verified. Resolve the existing email-verification routing for newly created users before claiming the final dashboard journey works.
@@ -2407,13 +2474,16 @@
 2026-10-27 redirect-loop fix verification: user confirmed settings change and explicitly requested checking/rerunning only redirect-loop tests after interrupting prior broader request. Read both current route files: verified removed from both, auth retained; User create can() permissions, Settings RequirePassword and throttle remain. Reviewed working tree at8ac5a6a: routes/web.php SHA2568e8a37664511db0e017ea69bc6e26d048be3178cf819cd097b6449affd14ee6f; routes/settings.php SHA25650b17a1ee63951836d1bfe4367fe65ebaac946dbf487dda6c14a68abf3679bb1. Narrow temporary isolated-SQLite HTTP harness PASS2/2: old null-verification pending account dashboard redirects to setup, setup returns200, email/verify redirects to setup which returns200 (loop terminated), appearance remains blocked until setup; completed null-verification account dashboard/appearance200, setup redirectsdashboard, security redirects to password-confirmation and that page200. No actual password changes required in these focused checks. Results:/tmp/foodbank-redirect-loop-results.json. No application source edits or repository tests added. Broad php artisan test had already started before user narrowed scope; attempted stop found it already finished:32pass,2fail,1error; additional old EmailVerificationTest expectation requires a redirect now deliberately removed, plus previously known2seed issues. No broader rerun after narrowing; no long-password retest. git diff --check passed during original interrupted check. Redirect-loop finding is resolved; preserve old failure as historical evidence and keep overall Changes needed/Failed for deferred long-password issue.
 2026-10-27 developer directed moving the bcrypt repair to the end. Assigned the repair and repeat test to FB-069, immediately before FB-070, preserving the existing failure and no-max requirement. No application edit or new test.
 2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
-Three fictional local accounts created and left in place: /users/15 emilie.oconnor, Inactive Volunteer, fb-browser-20261028-a@example.com; /users/16 emilie.oconnor.01, Active Manager, fb-browser-20261028-b@example.com; /users/17 emilie.oconnor.02, Active Volunteer, fb-browser-20261028-c@example.com. Shared phone +1 506-555-0181. Historical tracker IDs 15/16 referred to different prior fixtures; do not assume those older IDs identify current QA accounts. At final verification reidentify any original QA Volunteer by its recorded email and actual current details, not old ID alone. No credentials were changed or setup tested.</x:v>
-      </x:c>
-      <x:c r="R15" s="11" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk. Redirect-loop fix is now reviewed and narrowly tested: web.php/settings.php auth-only groups, unverified pending account reaches setup, completed unverified account reaches dashboard/appearance and password-confirmation/security flow. Await next developer instruction; latest test scope is redirect loop only, do not rerun broader suites automatically. Long-password/bcrypt issue remains deferred and unverified, so FB-006/007 remain open. Earlier seed-test and date-type findings retained; old email-verification redirect test now contradicts approved auth-only policy and needs a later developer-written update before project-wide gates pass. FB-020 connected details still open; do not infer account-creation completion.
+Three fictional local accounts created and left in place: /users/15 emilie.oconnor, Inactive Volunteer, fb-browser-20261028-a@example.com; /users/16 emilie.oconnor.01, Active Manager, fb-browser-20261028-b@example.com; /users/17 emilie.oconnor.02, Active Volunteer, fb-browser-20261028-c@example.com. Shared phone +1 506-555-0181. Historical tracker IDs 15/16 referred to different prior fixtures; do not assume those older IDs identify current QA accounts. At final verification reidentify any original QA Volunteer by its recorded email and actual current details, not old ID alone. No credentials were changed or setup tested.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R15" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk. Redirect-loop fix is now reviewed and narrowly tested: web.php/settings.php auth-only groups, unverified pending account reaches setup, completed unverified account reaches dashboard/appearance and password-confirmation/security flow. Await next developer instruction; latest test scope is redirect loop only, do not rerun broader suites automatically. Long-password/bcrypt issue remains deferred and unverified, so FB-006/007 remain open. Earlier seed-test and date-type findings retained; old email-verification redirect test now contradicts approved auth-only policy and needs a later developer-written update before project-wide gates pass. FB-020 connected details still open; do not infer account-creation completion.
 Before starting this item or feature: reread AGENTS.md from disk. Continue first-login setup and connected account-creation work in small steps. Do not repair bcrypt now; FB-069 owns that late repair and repeat test. Keep historical failed evidence and do not mark this item Complete without a scoped completed-feature review and passed applicable behaviour checks.
 Developer-directed 2026-10-28 timing: the connected QA Volunteer password-setup and post-setup access/logout/re-login checks are deferred to final project verification after FB-070 implementation, review, and testing. Keep this item open until the required final checks and its review/test gates pass.
-Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:v>
+Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S15" s="11" t="n"/>
     </x:row>
@@ -2436,9 +2506,11 @@
           <x:t xml:space="preserve">Change the signed-in user’s password</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" s="4" t="str">
-        <x:v>All roles supply correct current password plus matching new password. Enforce agreed rules; logout all sessions and require new login. No self-service name/email/phone editing.
-Signed-in users open Security directly without a separate confirmation prompt; current password is checked when saving.</x:v>
+      <x:c r="E16" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">All roles supply correct current password plus matching new password. Enforce agreed rules; logout all sessions and require new login. No self-service name/email/phone editing.
+Signed-in users open Security directly without a separate confirmation prompt; current password is checked when saving.</x:t>
+        </x:is>
       </x:c>
       <x:c r="F16" s="4" t="inlineStr">
         <x:is>
@@ -2453,8 +2525,10 @@
         <x:f>IF(I16="Not started","Not started",IF(I16="Blocked","Blocked",IF(I16="In progress","In progress",IF(J16&lt;&gt;"Passed","Awaiting code review",IF(OR(K16="",NOT(ISNUMBER(L16))),"Awaiting review evidence",IF(N16&lt;&gt;"Passed","Awaiting test",IF(OR(M16="",O16="",NOT(ISNUMBER(P16))),"Awaiting test evidence","Complete")))))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I16" s="10" t="str">
-        <x:v>In progress</x:v>
+      <x:c r="I16" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">In progress</x:t>
+        </x:is>
       </x:c>
       <x:c r="J16" s="10" t="inlineStr">
         <x:is>
@@ -2471,8 +2545,9 @@
       </x:c>
       <x:c r="O16" s="10" t="n"/>
       <x:c r="P16" s="30" t="n"/>
-      <x:c r="Q16" s="10" t="str">
-        <x:v>
+      <x:c r="Q16" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-27: Security/settings password confirmation failed in MySQL because Fortify treated the sign-in input name login as a users column. Developer explicitly authorized a focused assistant code fix. app/Providers/FortifyServiceProvider.php now registers Fortify::confirmPasswordsUsing; it checks the current signed-in user password hash, with a missing password returning false. PHP syntax and git diff check passed. Browser behaviour remains for developer to test. At FB-024, teach why the dual username/email login field differs from a stored database column and how the callback avoids the lookup.
 2026-10-27 developer-reported browser PASS: after the focused Fortify confirmation callback fix, entering the correct current password opens Settings &gt; Security. This confirms the formerly failing positive path. Incorrect-password rejection has not been reported tested; this is partial fix evidence, not completed FB-024 evidence.
 2026-10-27 pause: developer said “done for now” and will resume in a new chat. This is a pause request, not confirmation that the incorrect-password check was performed. Correct-password Security access remains developer-reported PASS; wrong-password rejection remains unverified. Keep the Fortify callback teaching note for FB-024.
@@ -2485,11 +2560,14 @@
 2026-10-28 developer-reported PASS: developer replied done to explicit test of incorrect current password plus matching new passwords of at least 8 characters; requested result was current-password error and no saved password change. This is partial behaviour evidence, not full feature completion. Next: explain confirmed rule and ask developer to submit correct current password with differing new entries, expecting mismatch error and no change.
 2026-10-28 developer-reported PASS: developer replied done after explicit test using correct current password and differing new-password entries, expecting confirmation error and no saved change. Next small behaviour check: correct current password, matching new entries of seven characters, expecting minimum-eight-character validation error and no saved change. FB-024 remains open pending completed-feature review, remaining tests, and deferred logout work.
 2026-10-28 developer explicitly deferred ALL remaining checks for FB-024 until project end, after FB-070 implementation, review and testing. This includes the pending minimum-eight-character rejection check, remaining validation/role/session/browser/automated checks and completed-feature source review. Preserve existing partial developer-reported successful-save, incorrect-current-password and mismatch evidence. No remaining check is claimed passed. The already deferred all-session/current-session logout implementation, focused Poker lookup and login redirect verification remain at that final checkpoint. FB-024 stays open and unverified.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
-      </x:c>
-      <x:c r="R16" s="10" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. All remaining FB-024 checks and full source review are deferred by developer to final project verification after FB-070 implementation/review/testing. Resume there: minimum-length and remaining validation/role/session checks; focused Poker logout lookup; implement required all-session/current-session logout and login redirect; review actual code and verify the full journey. Preserve prior partial evidence. Keep FB-024 open until BOTH review and behaviour testing pass. Continue eligible work meanwhile without bypassing other non-deferred prerequisites.
-Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R16" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. All remaining FB-024 checks and full source review are deferred by developer to final project verification after FB-070 implementation/review/testing. Resume there: minimum-length and remaining validation/role/session checks; focused Poker logout lookup; implement required all-session/current-session logout and login redirect; review actual code and verify the full journey. Preserve prior partial evidence. Keep FB-024 open until BOTH review and behaviour testing pass. Continue eligible work meanwhile without bypassing other non-deferred prerequisites.
+Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S16" s="10" t="n"/>
     </x:row>
@@ -2514,7 +2592,7 @@
       </x:c>
       <x:c r="E17" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Manager sees volunteers; Super Admin sees managers and volunteers. Render fictional records first and explain props/loops/stable keys. No volunteer access to others’ account records.</x:t>
+          <x:t xml:space="preserve">Shared directory available to every signed-in user; all three roles, active and inactive. SIX separate columns First name, Last name, Email, Phone, Role, Status. Fictional props/loops/stable keys first. Separate full-details/management permissions. No pictures now. REQ-041.</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="9" t="inlineStr">
@@ -2530,8 +2608,10 @@
         <x:f>IF(I17="Not started","Not started",IF(I17="Blocked","Blocked",IF(I17="In progress","In progress",IF(J17&lt;&gt;"Passed","Awaiting code review",IF(OR(K17="",NOT(ISNUMBER(L17))),"Awaiting review evidence",IF(N17&lt;&gt;"Passed","Awaiting test",IF(OR(M17="",O17="",NOT(ISNUMBER(P17))),"Awaiting test evidence","Complete")))))))</x:f>
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I17" s="11" t="str">
-        <x:v>In progress</x:v>
+      <x:c r="I17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">In progress</x:t>
+        </x:is>
       </x:c>
       <x:c r="J17" s="11" t="inlineStr">
         <x:is>
@@ -2539,21 +2619,81 @@
         </x:is>
       </x:c>
       <x:c r="K17" s="11" t="n"/>
-      <x:c r="L17" s="31" t="n"/>
-      <x:c r="M17" s="11" t="n"/>
+      <x:c r="L17" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N17" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O17" s="11" t="n"/>
-      <x:c r="P17" s="31" t="n"/>
-      <x:c r="Q17" s="11" t="str">
-        <x:v>
-2026-10-28 user explicitly requested starting user lists after deferring phone-display fix. AGENTS.md reread; full FB-009 row and related requirements read. Non-password account-creation source review and delegated behaviour evidence collected; remaining identified defects/checks explicitly deferred. Teaching progression: empty list-page shell, connect controller and authenticated GET route, local fictional props/loops/stable keys, then resource authorization and permitted query before real records, then layout and each filter/pagination in separate lessons. First small step: developer creates resources/js/pages/users/Index.vue with template/main p-4/h1 Users only. No application source written by assistant, no route/data/list behaviour claimed. Existing UserController Create/Show and previously inspected Poker Security response establish Inertia::render-to-Vue naming; no new uninspected Laravel query/action pattern introduced. Required list policy ability is UserPolicy::viewAny enforced on GET /users; query must scope Manager to Volunteers and Super Admin to Managers/Volunteers, Volunteer denied before live records.</x:v>
-      </x:c>
-      <x:c r="R17" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Index.vue with only template, main class p-4 and h1 Users. This shell is not yet routed and displays no records. Next connect UserController::index Inertia response and GET /users in small lessons using existing inspected response conventions; local fictional-only scaffold until viewAny authorization and actor-specific query are enforced. Teach props/v-for/stable keys, then layout and each filter/pagination separately. Review whole list feature at checkpoint; developer-first tests unless explicitly delegated. Preserve all deferred phone/password/concurrency work and prior evidence; no creation/list completion inferred.</x:v>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 developer reported after explicit refresh/rendering check: all six fictional user values showing under table headings. PASS for local scaffold rendering only; no real-record access/query/search/pagination verification or completed-feature review.
+2026-10-29 developer-reported PASS after explicit refresh: up to 10 real directory rows with six fields in correct headings; no full-directory acceptance or all-role/guest checks claimed.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P17" s="31" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-28 user explicitly requested starting user lists after deferring phone-display fix. AGENTS.md reread; full FB-009 row and related requirements read. Non-password account-creation source review and delegated behaviour evidence collected; remaining identified defects/checks explicitly deferred. Teaching progression: empty list-page shell, connect controller and authenticated GET route, local fictional props/loops/stable keys, then resource authorization and permitted query before real records, then layout and each filter/pagination in separate lessons. First small step: developer creates resources/js/pages/users/Index.vue with template/main p-4/h1 Users only. No application source written by assistant, no route/data/list behaviour claimed. Existing UserController Create/Show and previously inspected Poker Security response establish Inertia::render-to-Vue naming; no new uninspected Laravel query/action pattern introduced. Required list policy ability is UserPolicy::viewAny enforced on GET /users; query must scope Manager to Volunteers and Super Admin to Managers/Volunteers, Volunteer denied before live records.
+2026-10-28 developer replied done to creating the minimal users/Index.vue template/main p-4/h1 Users shell. Accepted as ordinary lesson confirmation only; no source inspection or browser verification, no item completion. Next small step: replace UserController::index(): void placeholder with index(): Response returning Inertia::render(users/Index); existing imports already supply Inertia and Inertia Response. Still no data or URL connection yet. Explain class method, return type and Vue page naming before route/authorization lesson.
+2026-10-28 developer replied done to index(): Response returning users/Index. Accepted as ordinary lesson confirmation; controller not inspected, no test/review claimed. Read existing routes/web.php and UserPolicy.php solely for upcoming route/authorization conventions. Poker routes/web.php uses authenticated GET controller routes, named routes and can(viewAny, Model::class) for list authorization. UserPolicy::viewAny currently denies all. Next tiny lesson: authenticated GET users named users.index opens empty local scaffold; no records. Policy and route can check follow before live data. Previously inspected Poker Settings/SecurityController.php confirms Inertia Response/render pattern.
+2026-10-28 developer explicitly requested assistant adding user-list sidebar button with only auth check for now. Authorized narrow exception to developer-written code. Read AppSidebar.vue, NavMain.vue and generated route helper to follow existing navigation pattern; routes/web.php already contains GET users -&gt; index named users.index inside auth with no can check. Assistant added Users icon/import, index helper import and Users nav entry in resources/js/components/AppSidebar.vue only. No route/policy changes. Read-only route helper confirms index export. Browser test requested from developer: click Users while signed in, expect Users heading. No assistant application tests or browser acceptance checks run; no feature completion/review claimed. Auth-only is temporary for empty local scaffold; real records still require policy and scoped query.
+2026-10-28 developer replied done after explicit instruction to click Users sidebar link while signed in and confirm Users heading. Record developer-reported PASS for that narrow local navigation/page check only. No assistant code inspection or application tests run; completed-feature code review and full-list tests remain pending. Next lesson sends one fictional user (id 1, first_name Amina, last_name Rahman) as users prop via second Inertia::render argument. Vue defineProps and rendering follow separately. Developer writes code; prior assistant-write exception was sidebar only.
+2026-10-28 developer replied done to adding fictional users prop in UserController::index. Ordinary lesson confirmation only; no source inspection or behaviour-test evidence claimed. Current small step: add script setup lang=ts with defineProps&lt;{ users: { id: number; first_name: string; last_name: string; }[]; }&gt;(); above existing users/Index.vue template. Explain script versus template, incoming props, TypeScript shape, number/string and list brackets. Receiving only; rendering follows next lesson. No application source changed by assistant.
+2026-10-28 developer replied done to typed defineProps in users/Index.vue. Ordinary lesson confirmation only; no inspection or behaviour evidence claimed. Next small lesson: below heading inside main, add ul/li v-for="user in users" :key="user.id" rendering first_name and last_name with double-brace interpolation. Explain list wrapper/item, per-user alias, stable key and dynamic binding. Developer-first check: refresh /users while signed in and confirm Amina Rahman appears below Users heading. No application source changed or tests run by assistant; feature review remains pending.
+2026-10-28 developer reported fictional list working after explicit refresh/name-display check. Developer-reported narrow scaffold rendering PASS; no completed-feature review or real-record authorization evidence. Developer then proposed hypothetically a table with first name, last name, email and phone, visible to every logged-in user and filterable by any column. Treat as scope discussion, not approval to replace canonical requirements or implement. Read related existing Requirements: Super Admin managers/volunteers combined list, Manager volunteer list, existing name/username/email search and role/status filters, 10-row pagination. First clarification: should Volunteers see other users contact details? Leave Requirements unchanged pending decisions.
+2026-10-28 developer confirmed directory access for all signed-in users, explicitly including volunteers finding managers phone numbers. Update REQ-041 and affected story acceptance: shared read-only contact directory showing first name, last name, email and phone, filterable by those columns. Directory visibility no longer restricted by viewer role. Existing edit/deactivate/full-details permissions remain separate. Clarify one global search versus separate column inputs next; prior role/status filter behavior and record inclusion details remain unresolved before their implementation. No application changes authorized or made this turn. AGENTS.md reread for revised scope.
+2026-10-28 developer chose ONE search box covering first name, last name, email and phone. REQ-041/FB-011 acceptance updated. Match across full directory before existing 10-row pagination. Next single scope clarification: active users only or inactive accounts too? No application-code changes or testing this turn.
+2026-10-28 developer confirmed inactive accounts must appear in directory as well as active accounts. Updated REQ-041 and FB-009/FB-015 acceptance. This concerns contact visibility only; inactive-account login/session restrictions unchanged. Next scope question: should Super Admin account also appear alongside Managers/Volunteers? No application changes or tests performed.
+2026-10-28 developer confirmed Super Admin accounts must also appear in directory. Approved record scope now all three existing roles (Super Admin, Manager, Volunteer), active and inactive, visible to all signed-in users. REQ-041 and FB-009/FB-015 acceptance updated. Remaining scope clarification: retain or remove earlier role/status dropdown filters alongside the approved single four-field search? No application-code changes or tests performed.
+2026-10-28 developer chose ONLY one search box, no separate role/status dropdowns, and added role-name search with partial matches (manager/mana/manag). Four displayed columns remain first name, last name, email, phone. User asked page size 10/15/20; instructor recommends existing approved 10 records/page for manageable layout, particularly narrow screens. No new page-size choice inferred. Updated REQ-041/REQ-060 and refined FB-012/013 lessons while preserving stable IDs, no completion evidence invented. Resume fictional table progression before incremental search/pagination. No application changes/tests performed.
+2026-10-28 developer explicitly approved 10 results per page and requires database-query pagination to handle growing users table. Search conditions must run in query before page limit; only current-page records returned to application/Vue, not full-table loading then slicing. Updated REQ-042 and FB-014 acceptance. No application changes, query inspection or performance tests performed; scope discussion only.
+2026-10-28 developer requested organized learning: first show table/data, add search box, implement search, then pagination. Instructor progression: fictional four-field sample -&gt; Vue prop shape -&gt; table structure/layout in small lessons -&gt; unfiltered database display with proper signed-in access/minimal fields -&gt; search input -&gt; binding -&gt; contact query -&gt; partial-role query -&gt; clear/empty -&gt; DB paginate(10)/controls -&gt; developer-first full checks and completed-feature code review. Any unpaginated learning scaffold remains local with fictional accounts; final list must paginate in DB. AGENTS.md reread. Focused upcoming-reference inspection: skander/app/Http/Controllers/PlayerController.php index uses IndexPlayersRequest safe filters, injected ListPlayers action and Inertia props; app/Http/Requests/Players/IndexPlayersRequest.php validates search/page, delegates authorization to route policy; app/Actions/Players/ListPlayers.php get builds grouped OR LIKE search, stable name/id ordering, paginate(20)-&gt;appends(filters), then through maps approved fields. FoodBank uses agreed 10, no poker balance/owing logic. No components/ui/table exists in FoodBank; teach plain semantic table rather than invent a shared table import. Current tiny lesson adds email amina@example.com and phone +1 506-555-0100 to existing fictional user in controller only. No source changes/tests by assistant.
+2026-10-28 developer asked which method; clarified UserController::index fictional user array. Then requested role and status as well. Suggest role Volunteer and status Active display strings beside email/phone in fictional sample. Clarify whether also visible columns before changing authoritative four-column table scope. No status-search/dropdown approval inferred. No assistant application-code changes, review or testing.
+2026-10-28 developer explicitly approved Role and Status as visible columns, bringing table to six columns. REQ-041 and FB-009/FB-010 acceptance updated. Current tiny lesson: add email:string, phone:string, role:string, status:string inside existing typed user object in users/Index.vue defineProps. Explain TypeScript describes incoming data, does not create values. No status search or dropdown inferred. No application-code changes, source review or tests by assistant.
+2026-10-29 developer supplied /Users/arafat/Desktop/Screenshot 2026-10-29 at 12.00.43 AM.png and requested matching name/role stacking without pictures. Latest approved layout supersedes six separate columns: User (first+last name above role), Email, Phone, Status. Pictures deferred explicitly as ##FUTURE, not current implementation. Screenshot Project/Team/Budget/Pending/Cancel are reference-only, not approved domain fields/statuses. Earlier typed prop additions not confirmed; do not infer done. Current tiny lesson replaces existing ul with plain table/thead/tr and four th scope=col headings; data rows and layout taught separately. No application-code changes, inspection of latest developer edits or tests by assistant.
+2026-10-29 developer corrected screenshot proposal: everything in separate columns, complex designs later. SIX columns First name, Last name, Email, Phone, Role, Status. Prior four-column header not confirmed applied. Current lesson: six-column plain header; data rows/styling later. No source edits/review/tests by assistant.
+2026-10-29 developer requested same card layout as other screens. Read existing users/Create.vue and users/Show.vue layout, plus ui/card Card/CardHeader/CardContent/CardTitle internals strictly for teaching conventions. Existing pattern main p-4 -&gt; Card w-full max-w-3xl -&gt; CardHeader/CardTitle -&gt; CardContent. Shared card supplies border/rounded corners, vertical spacing and padding. Current small lesson imports shared components and wraps existing table without duplicating standalone h1. No latest Index review, application changes or behaviour tests by assistant. Await developer application before proceeding.
+2026-10-29 developer replied done after receiving full Index.vue through typed props, shared card and six headings. Accepted as ordinary coding confirmation only; no unsolicited code inspection. Current lesson adds tbody/tr v-for with stable user.id key and six td interpolations in heading order. Developer-first check requested: refresh /users signed in and confirm Amina Rahman contact/role/status values under correct headings. No assistant source edits or tests; completed-feature review still pending.
+2026-10-29 developer confirmed all six values showing and requested spacing. Continue layout lessons in FB-010 without marking FB-009 complete; completed-feature review and live-directory verification remain outstanding.
+2026-10-29 resume database baseline after basic card spacing. AGENTS.md reread and full FB-009 row read; Requirements cached current scope used. Focused FoodBank convention reads for upcoming lesson: User has role()-&gt;belongsTo(Role), is_active boolean cast; Role casts code to RoleCode; RoleCode::label returns human readable Super Admin/Manager/Volunteer. GetAssignableRoles action uses get method, Collection return and query/map to UI-friendly data. Reuse already-inspected Poker ListPlayers action/controller/request pattern, no repeat Poker analysis. Current tiny lesson: developer runs php artisan make:class Actions/Users/ListUsers to create skeleton; explain action centralizes list query/search/pagination and controller chooses page. No assistant source edits/generation/tests.
+2026-10-29 developer confirmed ListUsers generator step and requested adding code gradually. Current tiny lesson: import App\Models\User, add public get() method with $query = User::query();. Explain public access, method, variable assignment, model and query builder; no DB read until later execution, no return value/controller connection yet. Temporary method intentionally unfinished; final return type taught when result introduced. No application source inspection/changes/tests by assistant.
+2026-10-29 developer confirmed User::query() start and requested next query part. Current lesson adds select for id, first_name, last_name, email, phone, role_id, is_active. Explain columns vs rows, stable key, role relationship identifier and boolean status mapping; excludes unrelated account data. No DB execution/return/controller wiring yet. No assistant source inspection/changes/tests; await ordinary done then continue without inspection.
+2026-10-29 developer confirmed select fields and requested loading role. Current tiny lesson: -&gt;with('role') immediately after User::query(), retaining selected role_id. Explain existing User role() belongsTo, batching related-role retrieval on execution, still separate relationship rather than role label string; labels mapped later. No source inspection/edits/tests or DB query execution by assistant.
+2026-10-29 developer said done check next, authorizing intermediate check. Read only app/Actions/Users/ListUsers.php. Current code selects required seven fields then with(role); valid for unfinished query. No findings; with after select works. Snapshot SHA256 61283ccb0b11ff445e53ee9fa3d1be132f8f47a61effa3987c351f4a1dbe081c. This is narrow intermediate review, not completed-feature Passed review; no DB execution/tests. Next tiny lesson adds orderBy first_name, last_name, id to establish stable alphabetical order and unique tie-break for later pagination. No assistant source changes.
+2026-10-29 developer confirmed ordering and requested fetching users. Current small lesson: after query definition add $users = $query-&gt;limit(10)-&gt;get();. Temporary local first-10 preview, not finished page navigation; limit in DB avoids loading full users table while preserving requested search-then-pagination lesson order. Later pagination lesson replaces limit/get with paginate(10). get executes SQL and eager-loads roles when action is invoked; action not wired yet, no actual DB execution claimed. Next map minimal fields and readable role/status, then controller. No source inspection/edits/tests by assistant.
+2026-10-29: Developer questioned temporary limit/get; agreed to use paginate(10) immediately and confirmed done. Ordinary coding confirmation, no inspection or test evidence. Next small lesson prepares five identity/contact fields with paginator through and User::only; role/status mapping next. Pagination controls remain a later lesson.
+2026-10-29 developer requested intermediate check and next lesson; inspected ListUsers.php: selected seven fields, eager-loaded role, stable first/last/id ordering, paginate(10), through callback allowing five outgoing fields. No issue in current unfinished step; still direct return, not proposed userData variable. No role/status mapping, return type or controller connection yet. Source HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6; ListUsers SHA256 d9ad48e5e20d83c8bd9ee0623acd22850d74b4d20a4a95a918d0417890bbc4c0. No runtime tests or application source changes. Role.php/RoleCode.php read for upcoming label lesson: code cast to RoleCode; label() supplies Super Admin/Manager/Volunteer. Developer preference for Laravel built-ins (e.g. paginate) saved to AGENTS.md; outgoing intermediate variable preference retained. Current lesson introduces userData variable and readable role only, status separately.
+2026-10-29 requested intermediate check: ListUsers.php now correctly builds userData with five allowed identity/contact fields, role via role-&gt;code-&gt;label(), status via is_active conditional, then returns it inside paginator through. No finding for this unfinished step; no runtime tests or application changes. Read UserPolicy.php, routes/web.php, UserController.php solely to plan upcoming connection: viewAny currently false; users GET auth-only; controller still fictional. Must enforce approved all-signed-in directory permission before live records. Next lesson adds concrete LengthAwarePaginator return type. No completed-feature review or completion claimed.
+2026-10-29 developer requested splitting complex get method. Explained Poker inline approach vs three methods get/buildQuery/prepareUser and private helper responsibility; developer explicitly approved and asked to start prepareUser one step at a time. This is scoped approval of structural alternative, not assistant source editing. Current lesson creates unused private prepareUser(User $user): array returning temporary empty array; extraction/callback connection follow separately. No application inspection, edits or runtime tests this turn; no completion claimed.
+2026-10-29 developer confirmed helper skeleton then explicitly authorized current replacements. Assistant read ListUsers.php to apply scoped edit: get has LengthAwarePaginator return type and helper existed with empty array; populated only prepareUser body with existing only fields, role label, status and return. Original through callback deliberately retained per current lesson. Helper not yet called; no behaviour change intended. No application tests run and no completed-feature verification claimed. Next connect through to helper in separate small lesson.
+2026-10-29 developer requested intermediate check then buildQuery lesson one step at a time. Read ListUsers.php only: through callback correctly returns $this-&gt;prepareUser($user), helper returns approved contact fields and readable role/status, paginate(10) and return type retained. No issue found for current unfinished step; no runtime tests or completed-feature review. Current lesson adds unused buildQuery(): Builder returning User::query() with Eloquent Builder import; remaining query clauses and connection follow in separate small lessons. No application source changes by assistant.
+2026-10-29 developer explicitly asked assistant to create buildQuery, move query code from get, and call helper from get. Assistant changed only app/Actions/Users/ListUsers.php: Eloquent Builder import, private buildQuery(): Builder containing unchanged select/with/orderBy chain, and $query = $this-&gt;buildQuery() in get. paginate(10) and through/prepareUser retained. Read back confirms requested structure. No application runtime tests or browser acceptance run; current controller still fictional and feature remains open.
+2026-10-29 developer confirmed viewAny change and requested intermediate check and route lesson. Read only relevant UserPolicy.php and routes/web.php sections: viewAny(User $user): bool returns true as approved all-signed-in directory scope; users GET remains auth-only with users.index name; User class already imported. No findings for current step. Current lesson attaches can(viewAny, User::class) to directory GET following inspected Poker route pattern. No assistant application edits or runtime tests; full list authorization/behaviour review remains open.
+2026-10-29 developer replied done after explicit signed-in /users refresh check; accept developer-reported PASS for fictional list still accessible with route policy attached, not all-role/guest/full-directory verification. Requested intermediate check: inspected relevant routes/web.php and UserController.php; users GET correctly chains can(viewAny, User::class), controller still fictional index(): Response with no ListUsers import. No finding for current step. Current lesson adds ListUsers import and injected index parameter only. No application source changes or runtime tests by assistant; no completed-feature review or item completion.
+2026-10-29 developer continued controller lessons and confirmed ordinary done for $users = $action-&gt;get() and replacing fictional render prop with users =&gt; $users. No unsolicited controller review or runtime test; not behaviour evidence. Read resources/js/pages/users/Index.vue only to establish upcoming prop/loop changes: currently typed users array and user in users loop. Current lesson updates prop to users object containing data array and loop to users.data; Laravel paginator carries metadata preserved for later controls. No assistant application edits/tests or completed-feature review.
+2026-10-29 developer replied done after explicit signed-in real-directory refresh check (users.data loop). Developer-reported narrow PASS: up to 10 real user rows with six fields under correct headings. No assistant runtime tests and no all-role/guest/page navigation/search verification. Do not complete FB-009 until full-feature review. Proceed to search lessons within same directory feature, under completed-feature review timing. AGENTS reread in full, full FB-011 row and REQ-041/042/060 read. First search lesson establishes labelled Input only, no filtering. Existing Create.vue shared Input/Label import conventions inspected; no developer latest-source review.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R17" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S17" s="11" t="n"/>
     </x:row>
@@ -2578,7 +2718,7 @@
       </x:c>
       <x:c r="E18" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Teach list/table overflow and parent layout. Toolbar and rows remain usable at narrow and wide widths; reuse colours and typography.</x:t>
+          <x:t xml:space="preserve">Shared Card layout with six separate columns, main p-4, max-w-6xl; separate rounded search/table borders and footer groups. Teach padding/spacing progressively. REQ-041. ##FUTURE Phone layout, column hiding, breakpoints and narrow-layout checks explicitly deferred until AFTER project end by developer on2026-10-29; excluded from current completion requirements and unverified.</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="4" t="inlineStr">
@@ -2588,15 +2728,15 @@
       </x:c>
       <x:c r="G18" s="4" t="str">
         <x:f>IF(H18="Complete","Complete",IF(I18="Blocked","Blocked",IF(I18="In progress","Ready",IF(F18="","Ready",IF(COUNTIFS($B$4:$B$73,F18,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H18" s="4" t="str">
         <x:f>IF(I18="Not started","Not started",IF(I18="Blocked","Blocked",IF(I18="In progress","In progress",IF(J18&lt;&gt;"Passed","Awaiting code review",IF(OR(K18="",NOT(ISNUMBER(L18))),"Awaiting review evidence",IF(N18&lt;&gt;"Passed","Awaiting test",IF(OR(M18="",O18="",NOT(ISNUMBER(P18))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J18" s="10" t="inlineStr">
@@ -2605,20 +2745,41 @@
         </x:is>
       </x:c>
       <x:c r="K18" s="10" t="n"/>
-      <x:c r="L18" s="30" t="n"/>
-      <x:c r="M18" s="10" t="n"/>
+      <x:c r="L18" s="30" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M18" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N18" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O18" s="10" t="n"/>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O18" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 developer replied done after explicit refresh/check of applied px-4 py-3 cell padding. Developer-reported PASS for narrow padding visual check only; responsive layout/full feature review not yet verified.
+2026-10-29 developer replied done after explicit wider-browser card/table width check following max-w-6xl change. Developer-reported narrow width check PASS; responsive behavior not verified.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P18" s="30" t="n"/>
-      <x:c r="Q18" s="10" t="n"/>
+      <x:c r="Q18" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29 AGENTS.md reread in full; full FB-010 row and REQ-041/042 read before item start. Developer confirms fictional rows display and asks spacing. First small layout lesson: table class w-full only, explain parent CardContent width and card max-width. Subsequent steps: cell padding, heading alignment, overflow. No latest application source inspection, edits or tests by assistant; full review deferred to completed feature.
+2026-10-29 developer replied done after trying table w-full and requested cell padding. Record developer-reported narrow width experiment confirmation only. Current tiny lesson: class px-4 py-3 on all six th and six td, preserving scope/interpolation/loop. Explain inside-cell padding vs external margin, x left/right and y top/bottom. No assistant source inspection/edits/tests. Next alignment and overflow separately.
+2026-10-29 developer asked assistant to do current padding step and asked what scope means. Explicit narrow source-write exception: read resources/js/pages/users/Index.vue solely to apply requested change, then added class px-4 py-3 to six th and six td. No formatting/refactor or other source changes. scope=col retained; explained header-to-column association for screen readers and no visual effect. Asked developer to refresh/observe increased padding. No assistant application/browser tests or completed-feature review claimed.
+2026-10-29 padding visual check confirmed by developer. Next small layout lesson changes Card max-w-3xl to max-w-6xl while retaining w-full; six padded columns need more room. Explain max width is upper limit, not fixed size. Then teach horizontal overflow on narrow screens separately. No assistant application source inspection/edits/tests this turn.
+2026-10-29 developer confirmed wider card and explicitly deferred deciding/hiding columns on smaller screens until AFTER search and pagination. Keep responsive acceptance open; do not choose hidden columns or implement hiding now. Resume database baseline FB-009, then staged search/pagination, then return to responsive design.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R18" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S18" s="10" t="n"/>
@@ -2644,7 +2805,7 @@
       </x:c>
       <x:c r="E19" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Search by name, username or email across the full permitted dataset. Explain one input-to-request-to-results cycle and empty results.</x:t>
+          <x:t xml:space="preserve">ONE search box finds matching first name, last name, email OR phone across the full shared directory before pagination. Explain input-to-request-to-results cycle, clearing search and empty results. Related rule: REQ-041. Automatic search after a 300ms pause in typing; cancel/restart pending delay on subsequent changes and retain input/focus during results updates.</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="9" t="inlineStr">
@@ -2654,15 +2815,15 @@
       </x:c>
       <x:c r="G19" s="9" t="str">
         <x:f>IF(H19="Complete","Complete",IF(I19="Blocked","Blocked",IF(I19="In progress","Ready",IF(F19="","Ready",IF(COUNTIFS($B$4:$B$73,F19,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H19" s="9" t="str">
         <x:f>IF(I19="Not started","Not started",IF(I19="Blocked","Blocked",IF(I19="In progress","In progress",IF(J19&lt;&gt;"Passed","Awaiting code review",IF(OR(K19="",NOT(ISNUMBER(L19))),"Awaiting review evidence",IF(N19&lt;&gt;"Passed","Awaiting test",IF(OR(M19="",O19="",NOT(ISNUMBER(P19))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I19" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J19" s="11" t="inlineStr">
@@ -2671,20 +2832,67 @@
         </x:is>
       </x:c>
       <x:c r="K19" s="11" t="n"/>
-      <x:c r="L19" s="31" t="n"/>
-      <x:c r="M19" s="11" t="n"/>
+      <x:c r="L19" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N19" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O19" s="11" t="n"/>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 developer-reported PASS after explicit check: pause after typing updates URL search parameter, typed value retained, additional typing works without clicking/refocusing. Earlier search-ref preview followed typing. Backend filtering, full search cases and final review remain unverified.
+2026-10-29 developer-reported narrow PASS: after explicit normal users-page check following IndexUsersRequest controller connection, developer confirmed page loads. Invalid-input rejection and actual filtering not verified.
+2026-10-29 developer-reported narrow PASS: users page still loads after controller passes filters into ListUsers get(array $filters). Actual filtering not yet implemented/tested.
+2026-10-29 developer-reported narrow PASS: users page loads after passing filters from get into buildQuery(array $filters). Filtering remains pending.
+2026-10-29 developer-reported narrow PASS: replied done/search works to requested first-name fragment, zzzznomatch empty rows, and clearing search restores unfiltered first page checks. This covers first-name search only; other fields/full-feature verification remain pending.
+2026-10-29 developer-reported PASS: replied done/all searches work after explicit first/last/email/phone fragments, mana/volun/Super Admin, nonmatch and clearing checks. Covers requested search cases only; pagination/refresh/lifecycle/permissions/responsive and completed-feature review remain open.
+2026-10-29 developer-reported PASS after explicit refresh/clear-refresh instructions: done, refresh keeps search text and results. Search prop/ref initialization confirmed by requested source check. No assistant browser test.
+2026-10-29 developer-reported PASS: only one request after instructed Network Fetch/XHR check typing one character and immediately pressing Enter; source check confirms cancellation before router.get.
+2026-10-29 developer-reported narrow PASS: search still works after onUnmounted timer cleanup. Cleanup navigation behavior not runtime-tested.
+2026-10-29 developer-reported PASS: only100 characters allowed after long-paste instruction and normal search still works.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P19" s="31" t="n"/>
-      <x:c r="Q19" s="11" t="n"/>
+      <x:c r="Q19" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29 developer replied done after explicit signed-in real-directory refresh check (users.data loop). Developer-reported narrow PASS: up to 10 real user rows with six fields under correct headings. No assistant runtime tests and no all-role/guest/page navigation/search verification. Do not complete FB-009 until full-feature review. Proceed to search lessons within same directory feature, under completed-feature review timing. AGENTS reread in full, full FB-011 row and REQ-041/042/060 read. First search lesson establishes labelled Input only, no filtering. Existing Create.vue shared Input/Label import conventions inspected; no developer latest-source review.
+2026-10-29 search lessons progressed: developer reported temporary {{ search }} display followed typing correctly (narrow developer-reported Vue binding PASS). Developer confirmed left alignment intentionally, not right. Declined further Poker Vue lookup and asked simplest beginner approach; instructor recommended manual submission using Inertia router.get, route index helper, ref value. Current requested intermediate check read Index.vue: search ref, v-model, searchUsers() router.get(index.url(), {search: search.value}) correctly present, search wrapper still div, temporary preview removed. No source findings for current unfinished step. Create.vue read only for upcoming shared Button convention. Current lesson connects form event; backend search absent, no functional search verification or completion claimed. No assistant application edits or runtime tests.
+2026-10-29 developer asked about searching every keypress, then explicitly approved automatic search with 300ms delay and one-step lessons. Supersedes manual Search-button plan; debounce waits until typing pauses, previous pending timer cancelled, retain search value/focus during updates. Current small lesson introduces watch(search, callback) scaffold only; delayed request added next. No application source inspection, edits or runtime tests by assistant. Prior form/Enter URL check not confirmed and no test pass inferred.
+2026-10-29 requested intermediate checks: Index.vue watcher scaffold and let searchTimer: number | undefined correctly present. Confirmed source still has router.get without preserveState, so continuous typing test deferred until input-preservation lesson. Earlier read confirmed manual form @submit.prevent=searchUsers remains; address when finishing automatic search. Current lesson adds clearTimeout and setTimeout(300) callback calling searchUsers, no source editing or runtime tests by assistant; no full search functionality claimed.
+2026-10-29 requested intermediate check: Index.vue watcher correctly clears pending numeric timer and schedules searchUsers after 300ms. No functional issue found in current timer step. router.get currently lacks preserveState; manual form submit remains. Read installed Inertia router/types and Vue adapter: preserveState option keeps component key, supporting retained local input/state. Current small lesson adds preserveState only; no assistant source changes or runtime tests, no debounce/focus behaviour pass claimed yet.
+2026-10-29 developer reported automatic URL update, retained input and continued typing without refocusing all working after explicit check; developer-reported narrow PASS, not actual filtering. Requested intermediate check read Index.vue, UserController index and ListUsers: preserveState true present, timer matches 300ms, controller supplies paginated action output; backend no search yet. Manual form remains and timeout cleanup pending. Focused Poker IndexPlayersRequest read confirms authorize true for route policy, nullable string max255 search and integer positive bounded page rules. Current lesson generates FoodBank IndexUsersRequest scaffold only. No assistant application source changes/runtime tests or full-feature completion.
+2026-10-29 discussed simpler inline Request::validate alternative; developer declined and reaffirmed custom request/Poker convention. Kept IndexUsersRequest name matching index/list including pagination. Developer created file and requested intermediate check: inspected IndexUsersRequest.php, correct namespace/FormRequest scaffold, authorize false and rules empty as generated. Current lesson adds search nullable/string/max255 rule only; authorization change must precede controller connection. No application source edits or runtime tests by assistant; no completion claimed.
+2026-10-29 requested intermediate check: IndexUsersRequest search rule is nullable/string/max:100, with matching 100-character comment. Valid rule syntax; differs from suggested Poker 255-character bound. authorize remains false and request is not connected. No runtime tests or whole-feature review. Next tiny lesson adds page rule.
+2026-10-29 requested intermediate check: IndexUsersRequest page nullable/integer/min:1/max:2147483647 is correct; search max100 retained. authorize false remains. Read routes/web.php users.index auth group plus can(viewAny, User::class), and UserPolicy viewAny true, matching agreed shared signed-in directory. Next lesson changes request authorize to true following inspected Poker pattern. No application edits/runtime tests or full-feature completion.
+2026-10-29 requested intermediate check: IndexUsersRequest authorize true with route-policy comment is correct. Read UserController index: ListUsers-only signature and get() without filters. Poker PlayerController index inspected: IndexPlayersRequest parameter, safe()-&gt;only filter extraction, action filters and returned search prop. Current lesson imports/types IndexUsersRequest only; no assistant application edits/runtime tests or completion.
+2026-10-29 requested intermediate check: UserController imports IndexUsersRequest and index signature correctly accepts request before ListUsers. Developer explicitly confirmed normal users page loads after connection: narrow developer-reported PASS. Read ListUsers for upcoming lesson: get/buildQuery have no arguments, query paginates 10 with stable ordering and display preparation. Current lesson extracts validated search only. No assistant runtime tests/application edits or full-feature completion.
+2026-10-29 requested intermediate check: UserController index correctly extracts $request-&gt;safe()-&gt;only([search]) with quoted search. No finding in this step. Focused Poker ListPlayers inspection confirms get(array $filters), fallback search and grouped OR search before paginate/appends. Current lesson connects required filters argument between controller and ListUsers get; query changes remain subsequent. No application edits/runtime tests/full-feature completion.
+2026-10-29 requested intermediate check: UserController correctly passes filters to action and ListUsers get accepts array filters. Developer confirmed normal page still loads after explicit refresh check (narrow developer-reported PASS). buildQuery still takes no arguments; next lesson connects filters to that existing helper before query changes. No assistant application edits/runtime tests or full-feature completion.
+2026-10-29 requested intermediate check: ListUsers get correctly calls buildQuery($filters), helper accepts array filters. Developer confirms page loads after explicit refresh check (narrow developer-reported PASS). Query still unfiltered. Current lesson extracts search with empty fallback inside helper. No assistant application edits/runtime tests or full-feature completion.
+2026-10-29 requested intermediate check: ListUsers buildQuery correctly extracts search with null-coalescing empty-string fallback. Current lesson introduces conditional grouped first_name LIKE search after with(role) before ordering/pagination, consistent with inspected Poker pattern; remaining fields taught subsequently. Developer-first narrow first-name/nonmatch/clear checks requested. No assistant application edits/runtime tests or full-feature completion.
+2026-10-29 requested intermediate check: conditional grouped first_name LIKE condition correctly implemented before stable ordering and query pagination. Developer replied done/search works after explicit known-fragment, no-match and clearing instructions: developer-reported narrow PASS for those requested checks. Current lesson adds last_name OR condition within same group. No assistant runtime tests/application edits or completed-feature review.
+2026-10-29 developer chose existing where/orWhere syntax over discussed whereLike alternative and explicitly requested all conditions now (pacing exception). Read actual User role belongsTo, Role code cast, RoleCode values super_admin/manager/volunteer and display labels. Focused Poker relationship-query reference: CashoutController index whereHas(gameSession/latestVisit) uses callbacks to constrain related rows. Existing contact-group pattern from ListPlayers retained; use OR relationship variant for role. Current lesson includes all agreed search fields, with spaces normalized to underscore for role code. No assistant source edits/runtime tests/completion.
+2026-10-29 requested intermediate check: ListUsers has correct grouped first/last/email/phone LIKE alternatives plus related role-code search with spaces converted to underscore, before stable ordering and paginate(10). Developer confirms all requested contact/partial-role/full Super Admin/nonmatch/clear checks work (developer-reported PASS). Read current Vue/controller for next lesson: Vue initializes ref(empty string), defineProps users only, controller returns users only. Refresh would leave search input empty despite URL filtering; next lesson first returns search prop. Existing form submit and timer lifecycle fixes remain open. No assistant application edits/runtime tests or whole-feature completion.
+2026-10-29 requested intermediate check: UserController index correctly returns search prop from validated filters with empty fallback. Current Vue still has users-only defineProps at bottom of script and ref(empty string) near top. Next lesson moves/assigns existing props declaration, adds search:string and initializes local ref from props.search, without replacing full page. No assistant application edits/runtime tests or completion.
+2026-10-29 requested intermediate check: Index.vue now has const props defineProps including search:string above ref(props.search), correct initialization. Developer confirms refreshed search text/results retained after explicit refresh/clear check; developer-reported evidence only. Existing form Enter calls searchUsers directly while watcher timer can remain pending; current lesson clears pending timeout inside searchUsers before router.get. No assistant application edits/runtime tests or feature completion.
+2026-10-29 requested intermediate check: searchUsers correctly clears searchTimer before router.get; watcher still clears previous timer as required. Developer confirms one request after explicit Network Fetch/XHR immediate Enter check (developer-reported PASS). Current lesson adds Vue onUnmounted cleanup for pending timer. No assistant application edits/runtime tests/full-feature completion.
+2026-10-29 requested intermediate check: Vue import includes onUnmounted; callback correctly clears pending timer after watcher. Developer reports ordinary search still works after requested check. Lifecycle cleanup source checked only; no navigation-race runtime check. Next directory lesson FB-013 empty-results display; search remains unverified pending completed-feature review.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 requested correction check: search Input has maxlength100, matching IndexUsersRequest max100. Developer confirms &gt;100 paste capped and normal search works (developer-reported PASS). This resolves ordinary overlong-input path from checkpoint finding; server-side malformed URL validation/feedback not runtime-tested. Index.vue SHA256 04701bb1e9afa8b5ad322605a102057ac6bd1b8746e3ebade958a7057331ed5a
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R19" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S19" s="11" t="n"/>
@@ -2705,12 +2913,12 @@
       </x:c>
       <x:c r="D20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Add the account status filter</x:t>
+          <x:t xml:space="preserve">Extend directory search to partial role names</x:t>
         </x:is>
       </x:c>
       <x:c r="E20" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">All/Active/Inactive works alone and with search on the full dataset. Add only this filter in this lesson.</x:t>
+          <x:t xml:space="preserve">Same single search box matches role labels as well as first name, last name, email or phone. manager, mana and manag find Managers. Search applies before pagination; no separate status or role dropdown. Related rule: REQ-041.</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="4" t="inlineStr">
@@ -2720,15 +2928,15 @@
       </x:c>
       <x:c r="G20" s="4" t="str">
         <x:f>IF(H20="Complete","Complete",IF(I20="Blocked","Blocked",IF(I20="In progress","Ready",IF(F20="","Ready",IF(COUNTIFS($B$4:$B$73,F20,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H20" s="4" t="str">
         <x:f>IF(I20="Not started","Not started",IF(I20="Blocked","Blocked",IF(I20="In progress","In progress",IF(J20&lt;&gt;"Passed","Awaiting code review",IF(OR(K20="",NOT(ISNUMBER(L20))),"Awaiting review evidence",IF(N20&lt;&gt;"Passed","Awaiting test",IF(OR(M20="",O20="",NOT(ISNUMBER(P20))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I20" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J20" s="10" t="inlineStr">
@@ -2737,20 +2945,36 @@
         </x:is>
       </x:c>
       <x:c r="K20" s="10" t="n"/>
-      <x:c r="L20" s="30" t="n"/>
-      <x:c r="M20" s="10" t="n"/>
+      <x:c r="L20" s="30" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M20" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N20" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O20" s="10" t="n"/>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O20" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29 developer-reported partial role checks PASS: mana, volun, Super Admin within all-searches confirmation. manag-specific and full-feature verification pending.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P20" s="30" t="n"/>
-      <x:c r="Q20" s="10" t="n"/>
+      <x:c r="Q20" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-28 scope refinement: former account-status dropdown removed by developer search-only choice. Stable FB-012 retained for next incremental search behavior: partial role-name matching. No implementation/review/test evidence yet.
+2026-10-29 role search implemented together with contacts at developer explicit pacing request (see FB-011). Requested source checks saw grouped orWhereHas role/code LIKE with space-to-underscore normalization. Developer reported mana/volun/Super Admin searches pass after explicit checks. No completed-feature review or manag-specific check; keep item open.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R20" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S20" s="10" t="n"/>
@@ -2771,12 +2995,12 @@
       </x:c>
       <x:c r="D21" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Add the Super Admin role filter</x:t>
+          <x:t xml:space="preserve">Handle cleared searches and no matching users</x:t>
         </x:is>
       </x:c>
       <x:c r="E21" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">All/Managers/Volunteers works with search and status. Managers remain restricted to volunteers.</x:t>
+          <x:t xml:space="preserve">Clearing the single search restores the full permitted directory; a search with no matches displays an understandable empty result. Include contact and partial-role searches. No separate role/status dropdowns. Related rule: REQ-041.</x:t>
         </x:is>
       </x:c>
       <x:c r="F21" s="9" t="inlineStr">
@@ -2786,15 +3010,15 @@
       </x:c>
       <x:c r="G21" s="9" t="str">
         <x:f>IF(H21="Complete","Complete",IF(I21="Blocked","Blocked",IF(I21="In progress","Ready",IF(F21="","Ready",IF(COUNTIFS($B$4:$B$73,F21,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H21" s="9" t="str">
         <x:f>IF(I21="Not started","Not started",IF(I21="Blocked","Blocked",IF(I21="In progress","In progress",IF(J21&lt;&gt;"Passed","Awaiting code review",IF(OR(K21="",NOT(ISNUMBER(L21))),"Awaiting review evidence",IF(N21&lt;&gt;"Passed","Awaiting test",IF(OR(M21="",O21="",NOT(ISNUMBER(P21))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J21" s="11" t="inlineStr">
@@ -2803,20 +3027,42 @@
         </x:is>
       </x:c>
       <x:c r="K21" s="11" t="n"/>
-      <x:c r="L21" s="31" t="n"/>
-      <x:c r="M21" s="11" t="n"/>
+      <x:c r="L21" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N21" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O21" s="11" t="n"/>
-      <x:c r="P21" s="31" t="n"/>
-      <x:c r="Q21" s="11" t="n"/>
+          <x:t xml:space="preserve">Passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-29 developer-reported clearing/nonmatch backend behavior passes within FB-011 explicit search checks; empty-results message pending.
+2026-10-29 developer-reported PASS after explicit zzzznomatch/clear instructions: No users found shows, clearing returns users and removes message. No assistant runtime tests. Completed-feature review still pending.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P21" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="Q21" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-28 scope refinement: former Super Admin role dropdown removed by developer search-only choice. Stable FB-013 retained for search clear/empty-result behavior already included in search acceptance, now taught as its own small lesson. No implementation/review/test evidence yet.
+2026-10-29 AGENTS reread in full before beginning item. Prior FB-011 developer-reported checks cover clearing search restoring rows and nonmatches returning empty rows. Current Vue tbody has no empty-state message. Current lesson adds conditional six-column No users found row. No completed-feature review/test pass.
+2026-10-29 developer clarified requested borders belong to two separate groups inside this page CardContent (search form and table), not global Card/CardContent changes. Requested intermediate check: search form border border-border p-4 correct; no mb-4 or other gap currently. CardContent has no border. Existing No users found conditional row correctly present with colspan6, but developer has not explicitly confirmed empty-message checks. Current requested lesson adds table border and mt-4 gap. No assistant application edits/runtime tests/completion.
+2026-10-29 developer requests reducing space between inner div borders and outer Card. Read shared CardContent default px-6 and Card py-6/gap-6 plus current page rounded wrappers. Teach page-level px-4 horizontal override as one small change; not a global shared-component edit. Layout preferences do not verify functional empty-result checks.
+2026-10-29 developer says bottom spacing looks good and requests check/next. Read saved Index.vue and shared Card/CardContent: rounded bordered wrappers present; suggested page px-4/pb-4 overrides absent, shared defaults unchanged (no git diff). Appearance satisfaction is developer-reported; do not claim missing overrides applied. Existing conditional empty row correct by requested inspection; next explicitly request empty-message and clearing browser checks, still no full-feature completion.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R21" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S21" s="11" t="n"/>
@@ -2842,7 +3088,7 @@
       </x:c>
       <x:c r="E22" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">10 records per page with Previous/Next. Apply search and filters before pagination; preserve selections across pages.</x:t>
+          <x:t xml:space="preserve">DATABASE-QUERY pagination returns 10 users per page with Previous/Next. Apply single contact/partial-role search in database before limiting current page, preserve search across page requests and use stable ordering. Do not load entire users table then paginate in PHP/Vue. Verify page boundaries and search across full matching dataset. Related REQ-041/REQ-042.</x:t>
         </x:is>
       </x:c>
       <x:c r="F22" s="4" t="inlineStr">
@@ -2852,15 +3098,15 @@
       </x:c>
       <x:c r="G22" s="4" t="str">
         <x:f>IF(H22="Complete","Complete",IF(I22="Blocked","Blocked",IF(I22="In progress","Ready",IF(F22="","Ready",IF(COUNTIFS($B$4:$B$73,F22,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H22" s="4" t="str">
         <x:f>IF(I22="Not started","Not started",IF(I22="Blocked","Blocked",IF(I22="In progress","In progress",IF(J22&lt;&gt;"Passed","Awaiting code review",IF(OR(K22="",NOT(ISNUMBER(L22))),"Awaiting review evidence",IF(N22&lt;&gt;"Passed","Awaiting test",IF(OR(M22="",O22="",NOT(ISNUMBER(P22))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J22" s="10" t="inlineStr">
@@ -2869,20 +3115,51 @@
         </x:is>
       </x:c>
       <x:c r="K22" s="10" t="n"/>
-      <x:c r="L22" s="30" t="n"/>
-      <x:c r="M22" s="10" t="n"/>
+      <x:c r="L22" s="30" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M22" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N22" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O22" s="10" t="n"/>
-      <x:c r="P22" s="30" t="n"/>
-      <x:c r="Q22" s="10" t="n"/>
+          <x:t xml:space="preserve">Passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O22" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 developer-reported narrow layout PASS: Next button is on right after parent flex justify-end.
+2026-10-29 developer-reported PASS: seeded additional users and Next/Previous navigation works. Exact DB count independently unverified; filtered navigation/search reset/boundaries remain pending.
+2026-10-29 developer-reported PASS: all requested final pagination checks work: volunteer search10/page, Next retains filter/results and increments page, last page numbers match/Next absent, Previous decrements, changing search from page2 resets page1. No assistant runtime tests.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="P22" s="30" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="Q22" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2026-10-28 developer explicitly confirmed 10 records/page and database-query pagination for scalability. Required architecture recorded only; no implementation/review/test evidence yet.
+2026-10-29 AGENTS reread in full before item; full FB-014 row and REQ-042 read, related REQ-041 scope already inspected this chat. Existing ListUsers paginate(10) and buildQuery stable order already established; inspected Poker ListPlayers uses appends(filters) after paginate. Chosen lesson order: retain validated search in generated page links, then expose link metadata to Vue, then visible Previous/Next and behavior checks. Current lesson adds appends only, no assistant code edits or runtime checks.
+2026-10-29 requested intermediate check: ListUsers paginate(10)-&gt;appends($filters) correctly present and through preparation retains paginator. Current Vue users type has data only. Next lesson adds paginator previous/next nullable URL types; no source changes/runtime tests by assistant, no behavior or feature completion inferred.
+2026-10-29 requested intermediate check: Vue users type correctly includes nullable prev_page_url and next_page_url. Read shared Button.vue: Reka Primitive supports asChild, variants; existing Create.vue imports shared Button. Current lesson uses Button as-child around Inertia Link for conditional Next URL; no assistant application edits/runtime tests or completion.
+2026-10-29 requested intermediate check: Button/Link imports correct and conditional Button as-child Next Link correctly bound to users.next_page_url. Developer added wrapper mt-4 overflow-hidden and requested right alignment. Teach wrapper mt-4 flex justify-end; no assistant source edits/runtime tests. Developer done follows prior conditional navigation instructions; preserve as developer report without asserting record counts or exhaustive pagination.
+2026-10-29 requested intermediate check: Next parent has mt-4 flex justify-end correctly; developer explicitly confirms right alignment. Current requested lesson adds conditional Previous and parent gap-2. No assistant application edits/runtime tests or full-feature completion.
+2026-10-29 developer requested50 more random users (10 manager40 volunteer), steering pagination lesson. Read UserFactory, DemoUserSeeder, Role/RoleCode, GenerateUsername and users schema. Existing factory supplies random fictional contact values and verified timestamp but defaults password=password and random username, so upcoming Tinker recipe overrides password from config and uses GenerateUsername with factory names, sets active/setup flags explicitly. Developer performs creation; no assistant DB writes, source edits or runtime checks. Previous control still awaits requested source/behavior confirmation.
+2026-10-29 developer rejects Tinker approach; no Tinker execution or user creation reported. Switch to developer-written separate RandomUserSeeder, matching existing seeder/factory setup. First lesson generates scaffold only; no assistant source writes or DB changes.
+2026-10-29 requested intermediate check: RandomUserSeeder correct generated Database\Seeders namespace, extends Seeder, empty run method. Unused WithoutModelEvents import is generated boilerplate. Next tiny lesson adds existing app helpers/models/enum/DB imports and removes unused import; no assistant source edits, DB writes or runtime tests.
+2026-10-29 developer confirms seeder ran and Next/Previous work. Requested intermediate check read RandomUserSeeder, ListUsers, IndexUsersRequest, UserController index and full users Index.vue: seeder matches10/40 transaction/factory/username plan; pagination appends validated filters before through; Vue conditional Previous/Next with gap2/right alignment and nullable URLs correct. No findings for current pagination wiring. No assistant runtime tests/DB writes or completed-feature review; current next step checks filtered page navigation and reset-to-first-page on new search.
+2026-10-29 developer requested Page:1 of X display then left info/right buttons with justify-between. Requested intermediate check: current_page/last_page number types and text correctly present; footer currently flex justify-end items-center gap2 with paragraph and buttons all direct siblings. Teach grouping buttons in nested flex gap2 div so outer justify-between separates exactly two groups. No assistant application edits/runtime checks/completion.
+2026-10-29 requested intermediate check: footer outer flex items-center justify-between, inner flex gap2 grouping both links correct; developer chose pl-1 (4px) for page paragraph and reports appearance looks good. Outer overflow-hidden also present; defer keyboard clipping consideration to responsive/checkpoint. Next request filtered pagination/boundary/page-reset checks; prior requests not explicitly confirmed due layout steering. No assistant application edits/runtime tests/full-feature review.
+2026-10-29 completed-directory checkpoint source review: query filters/grouping, relation match, stable ordering before paginate10/appends, controller validated filters/props, nullable links/page metadata, empty row, Vue ref/watch/timer cleanup and routes/policy examined together; also sidebar, setup middleware/bootstrap, shared Input and seeder. Finding: UI accepts &gt;100 search characters but request max100 rejects and page displays no validation feedback. First small correction maxlength100; backend validation retained. No assistant tests; full completion pending correction and role/guest checks. Footer overflow-hidden unnecessary; desktop keyboard focus check pending. Snapshot: 2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R22" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S22" s="10" t="n"/>
@@ -2903,12 +3180,12 @@
       </x:c>
       <x:c r="D23" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Verify list access on the server</x:t>
+          <x:t xml:space="preserve">Verify shared directory access on the server</x:t>
         </x:is>
       </x:c>
       <x:c r="E23" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Super Admin lists managers/volunteers; managers list all volunteers regardless of creator; volunteers cannot access user lists by direct URL. Attach real data only after checks are enforced.</x:t>
+          <x:t xml:space="preserve">Signed-in Volunteers, Managers and Super Admin can access directory; guests cannot access it directly. Records include all three roles, active and inactive; inactive-account login restrictions stay enforced. Only approved contact fields are exposed; directory access does not expand full account-details/edit/deactivate permissions. Exact auth/policy implementation to settle before live records. Related rule: REQ-041.</x:t>
         </x:is>
       </x:c>
       <x:c r="F23" s="9" t="inlineStr">
@@ -2918,15 +3195,15 @@
       </x:c>
       <x:c r="G23" s="9" t="str">
         <x:f>IF(H23="Complete","Complete",IF(I23="Blocked","Blocked",IF(I23="In progress","Ready",IF(F23="","Ready",IF(COUNTIFS($B$4:$B$73,F23,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H23" s="9" t="str">
         <x:f>IF(I23="Not started","Not started",IF(I23="Blocked","Blocked",IF(I23="In progress","In progress",IF(J23&lt;&gt;"Passed","Awaiting code review",IF(OR(K23="",NOT(ISNUMBER(L23))),"Awaiting review evidence",IF(N23&lt;&gt;"Passed","Awaiting test",IF(OR(M23="",O23="",NOT(ISNUMBER(P23))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I23" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
+          <x:t xml:space="preserve">In progress</x:t>
         </x:is>
       </x:c>
       <x:c r="J23" s="11" t="inlineStr">
@@ -2936,19 +3213,34 @@
       </x:c>
       <x:c r="K23" s="11" t="n"/>
       <x:c r="L23" s="31" t="n"/>
-      <x:c r="M23" s="11" t="n"/>
+      <x:c r="M23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
       <x:c r="N23" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O23" s="11" t="n"/>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="O23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 developer-reported PASS: replied done after explicit private/incognito direct Users URL check: guest redirected to login, no contacts displayed. Signed-in role checks pending.
+2026-10-29 developer-reported PASS: Volunteer can see directory and search managers after explicit already-setup Volunteer instructions. Manager/Super Admin and separate-details checks pending.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="P23" s="31" t="n"/>
-      <x:c r="Q23" s="11" t="n"/>
+      <x:c r="Q23" s="11" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
+2026-10-29 before starting item AGENTS reread in full and full FB-015 row read; REQ-041 shared directory all signed-in roles and all records already inspected and phone deferral synchronized. Existing routes/web.php users.index under auth with can(viewAny, User::class), UserPolicy viewAny true verified in completed-feature source review; display is GET only, no directory mutation submission. Other account-detail permissions remain separate. First developer-first check guest direct URL via private window; no assistant browser tests or source edits.
+2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="R23" s="11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
+          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Resume implementation from next agreed item FB-008 after reading its full row/requirements; do not resume pending directory checks until end-of-project verification. Do not mark directory items Complete or recommend a verified-feature commit until required evidence passes.</x:t>
         </x:is>
       </x:c>
       <x:c r="S23" s="11" t="n"/>
@@ -3050,16 +3342,14 @@
       </x:c>
       <x:c r="G25" s="9" t="str">
         <x:f>IF(H25="Complete","Complete",IF(I25="Blocked","Blocked",IF(I25="In progress","Ready",IF(F25="","Ready",IF(COUNTIFS($B$4:$B$73,F25,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H25" s="9" t="str">
         <x:f>IF(I25="Not started","Not started",IF(I25="Blocked","Blocked",IF(I25="In progress","In progress",IF(J25&lt;&gt;"Passed","Awaiting code review",IF(OR(K25="",NOT(ISNUMBER(L25))),"Awaiting review evidence",IF(N25&lt;&gt;"Passed","Awaiting test",IF(OR(M25="",O25="",NOT(ISNUMBER(P25))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I25" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J25" s="11" t="inlineStr">
         <x:is>
@@ -3076,12 +3366,13 @@
       </x:c>
       <x:c r="O25" s="11" t="n"/>
       <x:c r="P25" s="31" t="n"/>
-      <x:c r="Q25" s="11" t="n"/>
-      <x:c r="R25" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="Q25" s="11" t="str">
+        <x:v>2026-10-29 developer explicitly requested FB-021 before FB-008. First small lesson supplied: replace UserPolicy::update actor-only permission with actor+target checks: Super Admin edits managers/volunteers; managers edit volunteers; no self-service contact editing. No source edits, application tests, or completed-feature review by assistant.
+Preparation at HEAD f3513bc plus working tree (2026-10-29): FoodBank UserPolicy update currently actor-only; UserController edit/update stubs, users Show/Create and StoreUserRequest inspected for upcoming lesson. Poker reference /Users/arafat/Projects/Herd/skander/routes/web.php uses GET edit and PATCH update with can(update,target); app/Policies/PlayerPolicy.php supplies update ability; app/Http/Controllers/PlayerController.php edit sends selected fields through Inertia, update saves validated data, flashes toast and redirects to details; app/Http/Requests/Players/UpdatePlayerRequest.php checks update ability and unique email ignoring target; resources/js/pages/players/Edit.vue prefills fields with default-value. Preparation evidence only, not passed FB-021 review. FoodBank existing useForm learning approach retained for now; discuss any actual pattern alternative before selecting it.
+2026-10-29 developer replied done to UserPolicy::update actor+target rule lesson. Recorded as application confirmation only; no inspection or behaviour test performed. Next small lesson supplied: create minimal users/Edit.vue using existing shared card layout and heading. Page not yet connected to controller/route; no new browser check requested.</x:v>
+      </x:c>
+      <x:c r="R25" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
       </x:c>
       <x:c r="S25" s="11" t="n"/>
     </x:row>
@@ -6191,16 +6482,22 @@
       </x:c>
       <x:c r="O72" s="10" t="n"/>
       <x:c r="P72" s="30" t="n"/>
-      <x:c r="Q72" s="10" t="str">
-        <x:v>
+      <x:c r="Q72" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">
 2026-10-27 developer decision: this late checkpoint, immediately before final FB-070, owns the previously failed bcrypt long-password distinction repair and repeat test. No fix or repeat test has been performed. Teach and verify it in small steps when reached.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
-      </x:c>
-      <x:c r="R72" s="10" t="str">
-        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
+End-of-project verification queue addition: 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R72" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.
 Before starting this item or feature: reread AGENTS.md from disk. After FB-068, first teach and implement the deferred bcrypt 72-byte distinction repair without a password maximum; ask developer to test first or accept explicit delegation, then review affected code and repeat the wrong-suffix login check. Only then complete the broader first-version verification. FB-070 remains last.
-Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.</x:v>
+Before starting/resuming this item: reread AGENTS.md from disk. Latest 2026-10-28 scheduling supersedes earlier pending password-test timing: all current pending password-related checks move to final project verification after FB-070 implementation/review/testing. Keep non-password work and already assigned implementation checkpoints in place; preserve evidence and do not mark these tests passed.
+Before starting/resuming this item or feature: reread AGENTS.md from disk. At final verification revisit deferred shared-directory FB-009–FB-015 remaining checks; preserve earlier passes, test only actual remaining/invalidated evidence. Phone layout implementation remains after project end, separately deferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="S72" s="10" t="n"/>
     </x:row>
@@ -6297,7 +6594,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd32c600a867d40af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0135941f6924467d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7578,9 +7875,11 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D41" s="28" t="str">
-        <x:v>Automatically format the phone field while typing, adding the +1 prefix, space, and hyphens so managers only need to enter the digits.
-2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:v>
+      <x:c r="D41" s="28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Automatically format the phone field while typing, adding the +1 prefix, space, and hyphens so managers only need to enter the digits.
+2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E41" s="28" t="inlineStr">
         <x:is>
@@ -7643,7 +7942,8 @@
       </x:c>
       <x:c r="D43" s="28" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">The Super Admin can list, view, edit, activate, and deactivate both managers and volunteers.</x:t>
+          <x:t xml:space="preserve">The Super Admin can list, view, edit, activate, and deactivate both managers and volunteers.
+2026-10-28 shared-directory decision: see REQ-041. Directory contact visibility is available to all signed-in roles; this supersedes earlier actor-role restrictions on that list only. Existing management/full-details permissions are not broadened. Search interface and retained role/status filters are to be clarified before implementation.</x:t>
         </x:is>
       </x:c>
       <x:c r="E43" s="28" t="inlineStr">
@@ -7675,7 +7975,20 @@
       </x:c>
       <x:c r="D44" s="4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">The Super Admin has a combined list of managers and volunteers, with an All / Managers / Volunteers role filter, search by name, username, or email, and an All / Active / Inactive status filter.</x:t>
+          <x:t xml:space="preserve">The Super Admin has a combined list of managers and volunteers, with an All / Managers / Volunteers role filter, search by name, username, or email, and an All / Active / Inactive status filter.
+2026-10-28 superseding developer-approved directory decision: the user list is a shared contact directory for every signed-in user, including Volunteers looking up Managers phone numbers. Display first name, last name, email and phone; support filtering by any of these columns. Previous actor-role restrictions on directory visibility are superseded. Existing account-management and full-details permissions remain separate. One global search versus separate per-column inputs is pending developer choice. Earlier role/status filter behavior and exact record inclusion (including inactive/Super Admin accounts) require clarification before dependent implementation; do not silently remove or broaden those details. Existing 10-row pagination and filtering before pagination remain agreed. This approves scope, not assistant application-code changes.
+2026-10-28 filter interface confirmed: ONE search box searches first name, last name, email OR phone. Separate per-column inputs are not required. Search applies to the full directory before existing 10-row pagination. Inactive-account inclusion and earlier role/status filters remain to clarify.
+2026-10-28 inactive-account inclusion confirmed: shared directory includes both ACTIVE and INACTIVE users and their four contact fields. This does not permit inactive users to sign in or change existing account-management permissions. Whether Super Admin accounts are included and retained role/status filter controls still need clarification.
+2026-10-28 Super Admin inclusion confirmed: directory contains Super Admin, Manager and Volunteer accounts, active and inactive, visible to every signed-in user. Exact role/status dropdown controls remain to clarify before teaching those items. Account-management and full-details permissions remain separate.
+2026-10-28 superseding search controls decision: ONLY one search box; remove earlier proposed role and status dropdown filters. Same box matches first name, last name, email, phone OR role name, including partial role labels such as manager, mana, manag matching Manager accounts. The table still displays four contact columns; no role column was requested. Search covers full directory before existing 10-record pagination. User asked 10/15/20; instructor recommends retaining existing 10, no change to agreed page size. Stable FB-012 now teaches partial-role search, FB-013 teaches cleared/empty searches.
+2026-10-28 superseding displayed-columns decision: developer explicitly approved Role and Status as visible columns too. Directory now displays SIX columns: first name, last name, email, phone, role, status. Single search still covers first/last name, email, phone and partial role labels; no status-search behavior or dropdown filters approved. Active and inactive accounts of all three roles remain included for all signed-in users.
+2026-10-29 superseding layout approved from developer screenshot: FOUR visible columns User, Email, Phone, Status. In User cell show first and last name together, with role on the line underneath. This supersedes six separate displayed columns; underlying data still includes both name fields and role/status. No pictures or avatar placeholders in current design. Preserve single search covering first/last name, email, phone and partial role labels, no dropdowns, all three roles active/inactive and DB-query pagination 10. Reference screenshot project/team/budget fields and Pending/Cancel statuses are not project scope. ##FUTURE Confirmed later direction: add user profile pictures, then integrate those pictures into this directory table. Timing, storage/upload and detailed rules remain undecided; excluded from current implementation totals.
+2026-10-29 latest developer correction supersedes preceding screenshot layout: SIX SEPARATE columns First name, Last name, Email, Phone, Role, Status. Keep design simple; complex designs/stacked name-role cell deferred until later discussion. Search/access/pagination requirements unchanged. Pictures and later directory integration remain ##FUTURE.
+2026-10-29 table presentation: developer explicitly requested the shared card layout already used on Create User and User Details. Reuse existing Card/CardHeader/CardTitle/CardContent components for users directory; keep simple six-column table inside card. Teach layout incrementally.
+2026-10-29 developer-directed lesson timing: on smaller screens some columns will be hidden, but WHICH columns and exact responsive behavior will be decided AFTER search and pagination are finished. Do not select/hide columns now. This responsive-design checkpoint remains part of current directory work; not verified by desktop layout checks.
+2026-10-29 developer-approved search interaction: automatic search after a 300ms pause in typing (debounce), replacing the planned manual Search button. Each subsequent keystroke cancels/restarts the pending delay. Preserve input value and focus while results update. Existing single-box contact/partial-role scope, database filtering before 10-record pagination and permissions unchanged.
+2026-10-29 superseding developer decision: ##FUTURE Defer this users-directory phone layout until AFTER the project ends. Includes phone-specific column hiding, breakpoints, narrow-table/footer layout and their checks. Exclude this deferred work from current feature completion requirements; not verified. This supersedes the earlier after-search/pagination timing, not other modules responsive requirements.
+##FUTURE 2026-10-29 latest developer instruction: defer ALL REMAINING checks for the current shared users-directory feature until end of project. Preserve passed developer-reported checks and source-review evidence; this is a verification-timing change, not proof of completion. Pending Manager/Super Admin access, separate full-details permission boundaries, inactive/all-role inclusion, server validation/malformed query checks, keyboard/focus/timer lifecycle and any remaining automated/regression checks move to final project verification. Do not ask for these checks during subsequent implementation lessons. Phone layout itself and its checks remain separately deferred until AFTER project end. No assistant tests delegated. Deferred verification is excluded from current lesson workload; feature scope/permissions remain unchanged and unverified items stay open.</x:t>
         </x:is>
       </x:c>
       <x:c r="E44" s="4" t="inlineStr">
@@ -7707,7 +8020,9 @@
       </x:c>
       <x:c r="D45" s="28" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">This combined list shows 10 records per page. Search and filters apply to the full list before pagination.</x:t>
+          <x:t xml:space="preserve">This combined list shows 10 records per page. Search and filters apply to the full list before pagination.
+2026-10-28 explicit developer confirmation: 10 users per page, pagination MUST be applied in the database query. Apply contact/partial-role search conditions to the query before limiting the page; retrieve only current-page records, never load the full users table into PHP or Vue and slice it there. Preserve search across pages. This is required for the shared directory in REQ-041, including active/inactive users of all three roles.
+2026-10-29 developer-approved pagination display: show Page: current_page of last_page below table, with page text on left and Previous/Next controls grouped on right using justify-between.</x:t>
         </x:is>
       </x:c>
       <x:c r="E45" s="28" t="inlineStr">
@@ -8157,9 +8472,11 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D59" s="28" t="str">
-        <x:v>Username format: lowercase first.last, with no number for the first available name (example: amina.rahman). Further matches receive numeric suffixes after a dot, starting at 01: amina.rahman.01, amina.rahman.02, and so on. Generated usernames must be unique across all users and roles, including when regenerated after a name change. An existing username held by any role requires the next available suffix.
-2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now.</x:v>
+      <x:c r="D59" s="28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Username format: lowercase first.last, with no number for the first available name (example: amina.rahman). Further matches receive numeric suffixes after a dot, starting at 01: amina.rahman.01, amina.rahman.02, and so on. Generated usernames must be unique across all users and roles, including when regenerated after a name change. An existing username held by any role requires the next available suffix.
+2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E59" s="28" t="inlineStr">
         <x:is>
@@ -8288,7 +8605,9 @@
       </x:c>
       <x:c r="D63" s="28" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">The volunteer list includes search by name, username, or email, and an All / Active / Inactive status filter in the current scope.</x:t>
+          <x:t xml:space="preserve">The volunteer list includes search by name, username, or email, and an All / Active / Inactive status filter in the current scope.
+2026-10-28 shared-directory decision: see REQ-041. Directory contact visibility is available to all signed-in roles; this supersedes earlier actor-role restrictions on that list only. Existing management/full-details permissions are not broadened. Search interface and retained role/status filters are to be clarified before implementation.
+2026-10-28 superseded directory controls: see REQ-041. Shared directory uses one search box across first name, last name, email, phone or partial role name; no separate role/status dropdown filters. Includes all three roles, active and inactive, for all signed-in viewers.</x:t>
         </x:is>
       </x:c>
       <x:c r="E63" s="28" t="inlineStr">
@@ -8831,10 +9150,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D80" s="4" t="str">
-        <x:v>Until setup is complete, accounts cannot access normal application features. Inactive accounts remain blocked from login. The setup guard is registered once in the whole web group: guests pass to authentication; setup-complete users continue, with setup display/submission redirected to dashboard; unfinished users can reach setup display, setup submission and logout, and other web routes redirect to setup. Latest 2026-10-27 developer-approved fix: remove verified from routes/web.php and routes/settings.php middleware groups, retain auth and all existing policy/throttle/password-confirmation checks. This supersedes earlier setup-inside-auth+verified choice and prevents setup/email-verification loops for older unverified accounts. Verification dates are not a current access prerequisite; no account-data rewrite or removal of verification endpoints required by this decision.
+      <x:c r="D80" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Until setup is complete, accounts cannot access normal application features. Inactive accounts remain blocked from login. The setup guard is registered once in the whole web group: guests pass to authentication; setup-complete users continue, with setup display/submission redirected to dashboard; unfinished users can reach setup display, setup submission and logout, and other web routes redirect to setup. Latest 2026-10-27 developer-approved fix: remove verified from routes/web.php and routes/settings.php middleware groups, retain auth and all existing policy/throttle/password-confirmation checks. This supersedes earlier setup-inside-auth+verified choice and prevents setup/email-verification loops for older unverified accounts. Verification dates are not a current access prerequisite; no account-data rewrite or removal of verification endpoints required by this decision.
 2026-10-28 superseding decision for Security display only: remove its RequirePassword middleware, retain auth, and check the current password on password-change submission (REQ-090).
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E80" s="4" t="inlineStr">
         <x:is>
@@ -8863,10 +9184,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D81" s="28" t="str">
-        <x:v>After successfully setting a personal password, the new user is logged out and redirected to the login screen. They must sign in again using their new password.
+      <x:c r="D81" s="28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">After successfully setting a personal password, the new user is logged out and redirected to the login screen. They must sign in again using their new password.
 2026-10-26 developer-approved deferral: postpone BUILDING as well as verifying personal-password setup (FB-006/FB-007) until a new user is created through the frontend at FB-019. Withdraw SetupPassword.vue creation instruction; no implementation confirmed. Build the setup screen, access restriction and save/logout/re-login flow in small connected lessons at that checkpoint, before treating account creation as complete. Current scope retained, not FUTURE or verified.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E81" s="28" t="inlineStr">
         <x:is>
@@ -9247,11 +9570,13 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D93" s="28" t="str">
-        <x:v>For password changes after initial setup, all users must enter their current password and enter the new password twice. The current password must be correct and both new entries must match.
+      <x:c r="D93" s="28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">For password changes after initial setup, all users must enter their current password and enter the new password twice. The current password must be correct and both new entries must match.
 2026-10-28 developer-approved exception to Poker pattern: signed-in users open Settings &gt; Security without a separate password-confirmation prompt. Remove RequirePassword from the Security GET route only; retain authentication and the server-side current-password check on password-change submission. Developer applies the code. This supersedes the Security-display confirmation retained in REQ-077; other confirmation flows remain unchanged.
 2026-10-28 developer explicitly deferred ALL remaining checks for FB-024 until project end, after FB-070 implementation, review and testing. This includes the pending minimum-eight-character rejection check, remaining validation/role/session/browser/automated checks and completed-feature source review. Preserve existing partial developer-reported successful-save, incorrect-current-password and mismatch evidence. No remaining check is claimed passed. The already deferred all-session/current-session logout implementation, focused Poker lookup and login redirect verification remain at that final checkpoint. FB-024 stays open and unverified.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E93" s="28" t="inlineStr">
         <x:is>
@@ -9280,10 +9605,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D94" s="4" t="str">
-        <x:v>After a successful password change, log the user out of all sessions, including the current session, and redirect to the login screen. They must sign in with their new password.
+      <x:c r="D94" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">After a successful password change, log the user out of all sessions, including the current session, and redirect to the login screen. They must sign in with their new password.
 2026-10-28 developer-approved scheduling: defer implementing and verifying logout of all sessions (including current) and redirect to login after personal password change until final project verification after FB-070 implementation, review and testing. Defer the focused Poker logout/session-cleanup lookup with that work. This remains required current scope, not FUTURE or passed. FB-024 remains open until these checks and other completion gates pass.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E94" s="4" t="inlineStr">
         <x:is>
@@ -9344,10 +9671,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D96" s="4" t="str">
-        <x:v>First-time personal-password setup requires at least 8 characters, matching confirmation, and two sequential rejection checks: (1) match to the account assigned initial password, using its existing stored credential before setup; (2) match to current config(auth.initial_password). Spaces allowed; no maximum or character-mixture rule. Latest 2026-10-27 decision supersedes earlier no-reuse exemption and single-check proposals. Later reset selection checks only current configuration per REQ-092; implement reset at its later lesson and clarify exact entry point before changing existing flows. No username-based or unique-random initial-password strategy approved.
+      <x:c r="D96" s="4" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">First-time personal-password setup requires at least 8 characters, matching confirmation, and two sequential rejection checks: (1) match to the account assigned initial password, using its existing stored credential before setup; (2) match to current config(auth.initial_password). Spaces allowed; no maximum or character-mixture rule. Latest 2026-10-27 decision supersedes earlier no-reuse exemption and single-check proposals. Later reset selection checks only current configuration per REQ-092; implement reset at its later lesson and clarify exact entry point before changing existing flows. No username-based or unique-random initial-password strategy approved.
 2026-10-27 scheduling decision: the known bcrypt 72-byte truncation defect is repaired and retested at FB-069, immediately before final FB-070. This remains current scope, with no password maximum. Existing failed long-password test is historical evidence, not a pass; no code change or repeat test was made by this decision.
-2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:v>
+2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E96" s="4" t="inlineStr">
         <x:is>
@@ -11873,15 +12202,17 @@
           <x:t xml:space="preserve">Project context</x:t>
         </x:is>
       </x:c>
-      <x:c r="D175" s="28" t="str">
-        <x:v>The current learning order is the # column on Stories in Docs/FoodBank_Developer_Story_Tracker.xlsx. FB-001 through FB-070 remain stable IDs, not sequence numbers. Revised 2026-10-25 against AGENTS.md: complete each module before dependants; introduce required storage/relationships before use; move catalogue verification before Receive and totals after Receive. Code review and passed behaviour testing are required for completion.
+      <x:c r="D175" s="28" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">The current learning order is the # column on Stories in Docs/FoodBank_Developer_Story_Tracker.xlsx. FB-001 through FB-070 remain stable IDs, not sequence numbers. Revised 2026-10-25 against AGENTS.md: complete each module before dependants; introduce required storage/relationships before use; move catalogue verification before Receive and totals after Receive. Code review and passed behaviour testing are required for completion.
 2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Account creation lessons FB-016–FB-020 precede FB-009–FB-015. FB-006/FB-007 connect after the first frontend-created user and before creation completion.
 2026-10-27 developer-directed late checkpoint: FB-069 now includes the bcrypt 72-byte long-password repair and repeat test before its combined verification. FB-070 remains the final implementation item. Earlier FB-007 failed evidence stays visible; rescheduling does not complete or validate it.
 2026-10-28 developer-directed timing change: defer final QA of the frontend-created QA Volunteer first-password setup, direct /users/create denial, logout, and personal-password re-login until final project verification after FB-070 implementation, review, and testing. These required checks remain open; this timing change does not verify FB-019 or FB-006/FB-007. Continue eligible work meanwhile and retain these checks as a final completion gate.
 2026-10-28 developer explicitly deferred ALL remaining checks for FB-024 until project end, after FB-070 implementation, review and testing. This includes the pending minimum-eight-character rejection check, remaining validation/role/session/browser/automated checks and completed-feature source review. Preserve existing partial developer-reported successful-save, incorrect-current-password and mismatch evidence. No remaining check is claimed passed. The already deferred all-session/current-session logout implementation, focused Poker lookup and login redirect verification remain at that final checkpoint. FB-024 stays open and unverified. Continue eligible lessons without treating this deferral as prerequisite completion; retain other account-creation non-deferred review/check prerequisites before user-list implementation.
 2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now. Continue eligible lessons while retaining other non-deferred account-creation prerequisites and all existing final-verification gates.
 2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
-2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:v>
+2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.</x:t>
+        </x:is>
       </x:c>
       <x:c r="E175" s="28" t="inlineStr">
         <x:is>
@@ -12165,7 +12496,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae31d309126f4f54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aef1d13cdba4b44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Edit user from index with proper permission
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R862cd5550efa4eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R4397aa53f95242b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R1b9794baca4246a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R48ba8a15605c48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R7c197e22cde64d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rcc1ccd24340c4cd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -654,7 +654,7 @@
       </x:c>
       <x:c r="B7" s="15" t="n">
         <x:f>COUNTIF(Stories!H4:H73,"In progress")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C7" s="15" t="n"/>
     </x:row>
@@ -719,7 +719,7 @@
     <x:row r="12">
       <x:c r="A12" s="15" t="n"/>
       <x:c r="B12" s="15" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer applying Index.vue canEdit:boolean and :disabled binding and reporting role-matrix check: manager volunteers only, volunteer none, Super Admin managers/volunteers only; own account always disabled under current rules. A done reply following these explicit checks records developer-reported testing only. Completed-feature review still required; navigation not yet connected. Preserve prior evidence and all pending/deferred checks.</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n"/>
       <x:c r="D12" s="15" t="n"/>
@@ -745,7 +745,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>2026-10-29 developer replied done to UserPolicy::update actor+target rule lesson. Recorded as application confirmation only; no inspection or behaviour test performed. Next small lesson supplied: create minimal users/Edit.vue using existing shared card layout and heading. Page not yet connected to controller/route; no new browser check requested.</x:v>
+        <x:v>2026-10-29 developer replied done to backend canEdit preparation lesson; application confirmation only, no review or behavior-test pass inferred. Next small Vue lesson supplied: users/Index.vue add canEdit:boolean to each data-row type and :disabled=!user.canEdit on existing Edit Button. Explain boolean, dynamic colon binding and negation. Ask developer to verify enabled/disabled buttons for manager, volunteer and Super Admin accounts using existing update permissions. No source edits, intermediate inspection, application tests or browser checks performed by assistant. Button navigation remains a later step.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -755,7 +755,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer applying Index.vue canEdit:boolean and :disabled binding and reporting role-matrix check: manager volunteers only, volunteer none, Super Admin managers/volunteers only; own account always disabled under current rules. A done reply following these explicit checks records developer-reported testing only. Completed-feature review still required; navigation not yet connected. Preserve prior evidence and all pending/deferred checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -765,7 +765,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Waiting for developer to create minimal users/Edit.vue; no application tests requested or delegated.</x:v>
+        <x:v>Awaiting developer applying Vue disabled binding and checking button states for each role; navigation remains unconnected.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -774,10 +774,8 @@
           <x:t xml:space="preserve">Last reviewed revision</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29 HEAD f3513bc325d12a35661e7c1cbfcb3aab2214ced6 plus working tree; SHA256 app/Actions/Users/ListUsers.php:f9f5b52d5054febdccd68d066bfd779d88c0e94b40bb1f3d28923ea6e087cd8e, app/Http/Requests/Users/IndexUsersRequest.php:6661ba40e65144b20ab1e026700f96122ff4a236f0a5c8438177413e10761287, app/Http/Controllers/UserController.php:58e8eda2baa2ddb3e92168ee9a2802c03ecc7e783ef93655f450cd3bd06e412c, resources/js/pages/users/Index.vue:3613d34a0908e4aca6332e67a3b59cf2f52b62a9d1dd7f6caf6bbe523a64eb60, routes/web.php:3c6d8af2b7b78e0d58ea2eddf38001066911830ecfbbe463b8c3d13b0eff73a4, app/Policies/UserPolicy.php:cbb943549c8cbb6a3208bba01b520bde6bcd86edb19a8385b4367f5fd0584973, resources/js/components/AppSidebar.vue:b17eb10bc7b74930d638d9649c3ecb39f67f43be934899b4d615e0a3632e5d8c, database/seeders/RandomUserSeeder.php:60853f2562d1eaccac810d352b9bbce4902b023fd58f4b416fe477854dca4003</x:t>
-        </x:is>
+      <x:c r="B17" s="22" t="str">
+        <x:v>2026-10-29 Edit.vue::submit confirmation-only change source-reviewed; actual function tested in18 focused scenarios. Backend unchanged since27-test role/status checkpoint.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -792,10 +790,9 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="15" t="n"/>
-      <x:c r="B19" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Working tree at 2d45afc; review evidence in Stories FB-020. Reviewed controller, details page, protected route/policy, role model/enum, and flash toast wiring on 2026-10-28.</x:t>
-        </x:is>
+      <x:c r="B19" s="15" t="str">
+        <x:v>Working tree at 2d45afc; review evidence in Stories FB-020. Reviewed controller, details page, protected route/policy, role model/enum, and flash toast wiring on 2026-10-28.
+2026-10-29 developer screenshot reported AppHeader.vue TS2322 optional BreadcrumbItem[] passed to required Breadcrumbs array at line282. Explicitly requested fix. Assistant changed ONLY child binding from breadcrumbs to props.breadcrumbs so it uses the withDefaults value (empty array when omitted), consistent with existing v-if. Source-reviewed one-line change. Vue type check, targeted header formatting and diff whitespace pass. No application feature/browser tests run. Current role/status lesson and all existing pending/deferred checks unchanged.</x:v>
       </x:c>
       <x:c r="C19" s="15" t="n"/>
       <x:c r="D19" s="15" t="n"/>
@@ -3330,10 +3327,8 @@
           <x:t xml:space="preserve">Build and save the separate edit page</x:t>
         </x:is>
       </x:c>
-      <x:c r="E25" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prefill permitted fields; roles stay fixed. Same validation and cross-role email uniqueness. Name change regenerates unique username and success message includes it. Redirect to details; reject unauthorized display and submit.</x:t>
-        </x:is>
+      <x:c r="E25" s="9" t="str">
+        <x:v>Prefill permitted fields; role/status controls prefill saved values and permitted changes persist; no Super Admin assignment; existing edit target permissions remain unchanged. Same validation and cross-role email uniqueness. Name change regenerates unique username and success message includes it. Redirect to the user list with success feedback; reject unauthorized display and submit.</x:v>
       </x:c>
       <x:c r="F25" s="9" t="inlineStr">
         <x:is>
@@ -3351,28 +3346,73 @@
       <x:c r="I25" s="11" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="J25" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not reviewed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K25" s="11" t="n"/>
-      <x:c r="L25" s="31" t="n"/>
-      <x:c r="M25" s="11" t="n"/>
-      <x:c r="N25" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O25" s="11" t="n"/>
-      <x:c r="P25" s="31" t="n"/>
+      <x:c r="J25" s="11" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K25" s="11" t="str">
+        <x:v>2026-10-29 FB-021 current-code review at HEAD 6a79da523dc0fd03487b76fc22311c2296f3d330 plus working tree. Reviewed routes/web.php (GET/PATCH update policy), UserPolicy.php actor/target rules, UserController.php selected edit props/validated conditional-name save/toast/details redirect, UpdateUserRequest.php authorization/unique email ignore/phone/name limits, GenerateUsername.php optional target exclusion, User model/fillable/casts/role enum and users schema, Edit.vue/Show.vue/shared inputs and button, setup middleware. Findings: Show has no permission-aware Edit navigation link; formatting checks fail Edit.vue, GenerateUsername.php, routes/web.php. New update rules/save behavior covered by delegated passing tests; retain final-project concurrency/phone/password deferrals. Source SHA256: GenerateUsername c20b8f7dab57e4147a2ec68e3c2cbfa4ad24fba195eeb768944a54d8355a4d13; UserController e6aeb7776d36900a8f05c0a65e5891f0aad5d4da9500fd1aef45d426eb80be4a; UpdateUserRequest 04b2575474147e97a6162e576ed78400dc560dc0f455d5c1c3e713d2d2bf94c5; UserPolicy 47650078c3a0f62fb693043c29e6d248338ebafd677b1b3840a890a09bc7afc5; routes 955f7e2629fed5ab77c254d63e19140351157306ad661e254998c01cae59fd95; Edit c5bd0ac37743c49448c1d12bc4e46ab2beb10280f1f7e746d48de3efc3604f8c; Show 143982ba4e04efe6fcf550092cae23cd47b5e7f6784d857efbe178ed3043e945.
+2026-10-29 follow-up review at same HEAD plus changed controller/Show: Show now receives id and canEdit from update policy; CardAction v-if canEdit wraps shared Button/Link to numeric selected account edit URL. Missing navigation finding resolved. Current SHA256 UserController c9490e86c6dd7632811a9e395dde8915cbb9e7ffaa709dbac594e75e4215c2e5; Show bdba2ae9b6313c16100461f178af459e45362541a71b844c3dfff2aff8d292cb. Formatting still fails in GenerateUsername/routes/Edit/Show; keep review Changes needed pending developer cleanup.
+2026-10-29 formatting follow-up review: previous new-code navigation and formatting findings resolved. Reviewed current generator exclusion, update/Show controller, rules/policy/routes, Edit/Show components. HEAD remains 6a79da523dc0fd03487b76fc22311c2296f3d330. Final hashes: GenerateUsername c5e715cab5841c9ffb099f5b5aeffae2db615a06e5a00b336da07f2e9f6a8040; UserController c9490e86c6dd7632811a9e395dde8915cbb9e7ffaa709dbac594e75e4215c2e5; UpdateUserRequest 04b2575474147e97a6162e576ed78400dc560dc0f455d5c1c3e713d2d2bf94c5; UserPolicy 47650078c3a0f62fb693043c29e6d248338ebafd677b1b3840a890a09bc7afc5; routes 468c9947ca36fa6ad0d2daebae208aac16e488973e108b22a26b59eadac63880; Edit 05aedd33d1631a1891feafd3f2d607e30cb852d4ad7224d8a30d36d30dea16ef; Show d579c0a50b0a562ec015faaac049d6bbd9c8359207a52a746b49efb9fb0dda99. Main edit-flow review passes; existing shared phone-input cleanup and simultaneous username-saving issues retain their project-end checkpoint, so do not interpret as complete application verification.
+2026-10-29 developer explicitly authorized only changing the successful edit redirect to the user list. Changed UserController::update final return to to_route(users.index) and its explanatory comment. Success toast and save logic retained. Source-reviewed this two-line change; PHP syntax check passed. Browser/behavior check pending developer; no application test suite run. All earlier role/status dropdown, validation, session and middleware changes were fully reverted at developer request before this change; do not treat role changes as implemented or approved for resumption.
+2026-10-29 developer requested only role dropdown and Active/Inactive checkboxes matching Create User layout with saved values selected. Assistant explicitly scoped this response to controls; persistence separate. Implemented Edit.vue Select bound to string saved role_id, linked boolean status checkboxes (one checked at a time), matching Create spacing/grid. UserController::edit sends role_id/is_active and database role choices via GetAssignableRoles::get(forEdit: true). Edit offers Manager/Volunteer; default Create behavior unchanged. Policies/routes/UpdateUserRequest/save logic and sessions untouched; role/status changes are NOT saved yet. Existing redirect to users.index retained. Source-reviewed display wiring; PHP syntax, targeted Pint, Vue type check and diff whitespace pass. No application behavior tests or browser checks performed; ask developer to verify controls first. Earlier broad attempted implementation remains reverted. No completion claimed.
+2026-10-29 explicit developer authorization: connect role/status changes to the existing Edit workflow and report files/methods. UpdateUserRequest::rules validates role_id using existing GetAssignableRoles::get(forEdit:true) and required boolean is_active. UserController::update now saves validated role/status and revokes target database sessions/Remember me token on active-to-inactive change inside DB transaction. Edit.vue::submit confirms loss of access/session termination before deactivation. New EnsureAccountIsActive::handle logs inactive users out and invalidates current session; registered before password-setup middleware in bootstrap/app.php. Existing UserPolicy and GET/PATCH can(update,target) checks unchanged; Super Admin edits managers/volunteers, manager edits volunteers and may promote to manager, then loses edit/view access to promoted account. Existing users.index success redirect retained. Current session driver confirmed database. Source reviewed these changes at HEAD 6a79da523dc0fd03487b76fc22311c2296f3d330 plus working tree; no new findings for this scoped change. No full feature completion claimed.
+2026-10-29 developer explicitly requested confirmation for promotion/demotion AND activation as well as deactivation, and testing only these current changes. Changed ONLY Edit.vue::submit application code: compare role/status against saved props, describe current-to-selected role and activation/deactivation consequences, combine all applicable details into one window.confirm before PATCH. Cancel returns without request and retains selections; unchanged role/status (including contact-only edit) does not prompt. Existing backend saving/permissions/session handling/list redirect untouched. Source-reviewed this confirmation change.</x:v>
+      </x:c>
+      <x:c r="L25" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="M25" s="11" t="str">
+        <x:v>Assistant (explicitly delegated); earlier developer page check retained</x:v>
+      </x:c>
+      <x:c r="N25" s="11" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="O25" s="11" t="str">
+        <x:v>
+2026-10-29 developer-reported PASS: replied page loads with the details after explicit fictional Volunteer edit-page check. Confirms page opening and saved details displayed only; no assistant browser/tests, no claim of readonly/typing/permission-negative/save verification.
+2026-10-29 assistant-delegated checks: temporary external PHPUnit harness /tmp/foodbank-fb021/EditUserTest.php, no repository test/source edits. PASS 31 scenarios/190 assertions on SQLite and again MySQL: all 3x3 actor/target GET/PATCH permissions, guest/self/missing/malformed targets, current-email/contact save, protected-field tampering ignored, name change/own-account and cross-role numbered collisions/accent preservation, 16 invalid-input cases with no persistence, cross-role duplicate email, shared phone, inactive target preservation, creation-generator compatibility, validation redirect/retained input and toast. Browser PASS on fictional fixture: phone save+refresh, same-base spelling keeps username, Maria Sharapova new username, required-name/duplicate-email errors, retained input, Cancel, denied self-edit, readonly fields, keyboard and phone/desktop layout. Evidence screenshot /tmp/foodbank-fb021/edit-browser-verified.png. Vue types PASS; diff whitespace PASS. npm check FAIL formatting Edit.vue; Pint FAIL formatting GenerateUsername.php and routes/web.php. Broader non-password regression 7 tests: 5 passed, 1 failed and 1 error in UserSeedingTest expecting one user while DatabaseSeeder also runs DemoUserSeeder. PHPStan with 512M reports 9 existing typing issues in ListUsers, create-user email_verified_at and Demo/SuperAdmin seeders; none in new update logic. No concurrent-save checks or deferred password/directory QA reopened. Missing Show Edit link means end-to-end navigation unverified/incomplete; loading timing only source-reviewed. Isolated MySQL DB and temporary server removed; live data untouched.
+2026-10-29 follow-up assistant-delegated PASS: 10 new details-page permission scenarios/78 assertions on isolated MySQL (temporary test harness filter test_details_page); checks numeric id and canEdit for allowed cross-role access, denied cross-role detail requests, and all 3 roles own-details canEdit false. Browser PASS manager volunteer Show -&gt; Edit -&gt; Cancel same account; My details no Edit link. Screenshot /tmp/foodbank-fb021/show-edit-button-verified.png. Vue type check PASS. npm check FAIL formatting Edit/Show; Pint FAIL formatting GenerateUsername/routes, diff whitespace PASS. Isolated DB/server cleaned up; live data and source unchanged by assistant.
+2026-10-29 after developer formatting, assistant-delegated PASS: all 41 focused EditUserTest scenarios/268 assertions on SQLite; npm types:check; npm check reports all64 formatted/no warnings or lint errors in55 files; targeted Pint passed; git diff check passed. Prior MySQL31/190 and navigation10/78, browser layout/navigation/save/error evidence retained for same behavior. No app source edits by assistant. Shared deferred phone/concurrency checks remain outstanding; N remains Partial to avoid claiming final shared-behavior verification. Main edit implementation is a useful stable commit milestone; suggested message Add protected user editing with username regeneration.
+2026-10-29 developer explicitly authorized only changing the successful edit redirect to the user list. Changed UserController::update final return to to_route(users.index) and its explanatory comment. Success toast and save logic retained. Source-reviewed this two-line change; PHP syntax check passed. Browser/behavior check pending developer; no application test suite run. All earlier role/status dropdown, validation, session and middleware changes were fully reverted at developer request before this change; do not treat role changes as implemented or approved for resumption.
+2026-10-29 assistant-executed under earlier narrow role/status test delegation: external /tmp/foodbank-fb021/EditRoleStatusTest.php PASS 27 tests/148 assertions on isolated in-memory SQLite. Covers role saves/promotion/demotion and unchanged values, both status transitions, combined role/status save, invalid role/status rejected, forbidden Super Admin assignment, existing-manager target denied, post-promotion edit denied, creation dropdown unchanged, prefilled edit props, target-only database session deletion/Remember me token rotation and reactivation preserving revocation, inactive signed-in sessions denied before setup. Targeted Pint/PHP syntax, Vue type check, Vue formatting and diff whitespace pass. No full workflow, password-login tests or browser confirmation/visual checks run. Earlier shared deferred phone/concurrency/password tests remain open; earlier 41-test evidence historical and not rerun for changed contracts.
+2026-10-29 scoped confirmation checks PASS: 18 scenarios in external /tmp/foodbank-fb021/confirmation-check.mjs execute actual submit() extracted from Edit.vue and transpiled with TypeScript, using stubbed confirm/patch. Includes both confirmation outcomes for promotion, demotion, activation, deactivation and all four combined role/status directions; only one prompt for combined changes, accurate details, Confirm submits once, Cancel sends no request and retains state, unchanged role/status skips prompt. Vue type check, targeted Vue formatting and diff whitespace pass. No browser/native-dialog rendering check, backend tests or full workflow rerun for this change. Earlier backend27/148 evidence retained, not repeated.</x:v>
+      </x:c>
+      <x:c r="P25" s="31" t="n">
+        <x:v>46324</x:v>
+      </x:c>
       <x:c r="Q25" s="11" t="str">
         <x:v>2026-10-29 developer explicitly requested FB-021 before FB-008. First small lesson supplied: replace UserPolicy::update actor-only permission with actor+target checks: Super Admin edits managers/volunteers; managers edit volunteers; no self-service contact editing. No source edits, application tests, or completed-feature review by assistant.
 Preparation at HEAD f3513bc plus working tree (2026-10-29): FoodBank UserPolicy update currently actor-only; UserController edit/update stubs, users Show/Create and StoreUserRequest inspected for upcoming lesson. Poker reference /Users/arafat/Projects/Herd/skander/routes/web.php uses GET edit and PATCH update with can(update,target); app/Policies/PlayerPolicy.php supplies update ability; app/Http/Controllers/PlayerController.php edit sends selected fields through Inertia, update saves validated data, flashes toast and redirects to details; app/Http/Requests/Players/UpdatePlayerRequest.php checks update ability and unique email ignoring target; resources/js/pages/players/Edit.vue prefills fields with default-value. Preparation evidence only, not passed FB-021 review. FoodBank existing useForm learning approach retained for now; discuss any actual pattern alternative before selecting it.
-2026-10-29 developer replied done to UserPolicy::update actor+target rule lesson. Recorded as application confirmation only; no inspection or behaviour test performed. Next small lesson supplied: create minimal users/Edit.vue using existing shared card layout and heading. Page not yet connected to controller/route; no new browser check requested.</x:v>
+2026-10-29 developer replied done to UserPolicy::update actor+target rule lesson. Recorded as application confirmation only; no inspection or behaviour test performed. Next small lesson supplied: create minimal users/Edit.vue using existing shared card layout and heading. Page not yet connected to controller/route; no new browser check requested.
+2026-10-29 developer explicitly reconfirmed original separate Edit page plan after discussing inline editing. Match Show layout AND borders, including shared outer Card border, inner rounded bordered section and shared Input field borders. First page-structure lesson supplied; await developer applying it. Earlier policy done remains application confirmation only, not code review/test. No application changes or tests performed by assistant.
+2026-10-29 developer explicitly requested the whole Vue page, overriding small-code-example pacing for this response only. Supplied full proposed Edit.vue in chat for developer to apply; no assistant source edits. Kept Show Card/CardContent inner rounded bordered container and username first-column row; added prefilled useForm/contact fields, readonly username/role/status, errors/processing, Save and Cancel. Preparation reads Show/Create and shared Button only, not review of developer edits. No applied code or behaviour check claimed. Backend routes/controller/save still to teach. Matching role/status data contract uses readable strings as in Show, plus numeric id.
+2026-10-29 developer said done check nxt, treated as explicit intermediate review request. Read resources/js/pages/users/Edit.vue and local Inertia useForm/FormDataErrors declarations, plus UserController and InputError. Page matches Show borders/layout, four editable contact fields and readonly username/role/status. Finding: form.errors.username references a key absent from four-field inferred form type; assistant supplied this mistake. Guided removal of that InputError only. No files changed by assistant; no type checker, application tests or browser checks run. Controller edit/update remain stubs. This partial review does not pass FB-021 completion gate.
+2026-10-29 developer replied done to removing invalid form.errors.username; application confirmation only, not re-inspected/tested. Next small lesson supplied: implement UserController edit response using selected saved fields plus readable role/status and numeric id, following inspected Poker edit selected-props pattern and existing FoodBank show data preparation. Existing Response/Inertia imports already present. No route added yet; no application code edited by assistant or tests run.
+2026-10-29 developer replied done to UserController::edit response lesson; application confirmation only, not re-inspected. Next lesson supplies protected GET users/{user}/edit route using same update ability as inspected Poker edit pattern. Explains numeric route binding then policy then controller/Inertia/Vue. Positive fictional Volunteer edit-page/prefill/readonly check requested of developer; no assistant tests or browser checks run. Save still unavailable until PATCH/controller/request taught.
+2026-10-29 developer explicitly confirmed edit page loads with details after protected GET-route lesson. Record positive page load and prefilled details as developer-reported PASS only; no claim of readonly/typing/denied-access/save checks. Next lesson asks developer to generate Users/UpdateUserRequest via artisan; explains FormRequest responsibility before save is connected. No assistant application source changes or tests.
+2026-10-29 developer replied done to generating Users/UpdateUserRequest; application confirmation only, no file inspection. Supplied first request lesson: import App Models User, retrieve selected route user, ensure bound User instance and authorize signed-in actor via update policy; explain instanceof, null-safe operator and false fallback. Follows already inspected Poker UpdatePlayerRequest. No application code edits or tests by assistant.
+2026-10-29 developer replied done to UpdateUserRequest authorize lesson; application confirmation only, not inspected/tested. Supplied small rules() lesson for first_name and last_name required/string/min1/max100; explain array field keys and rules and distinction from later username-supported-name validation. Existing Vue InputError will display field errors once submission is connected. Email and phone rules remain next; no assistant application edits or tests.
+2026-10-29 developer explicitly asked for all rules together, overriding splitting form-field rules for this response. Supplied full rules method matching existing StoreUserRequest limits plus edit-specific unique email ignoring route-bound target, following inspected Poker UpdatePlayerRequest guard/ignore pattern. Added Rule import. Explained basic field validation versus later supported-name/username checks and no Save connection yet. No application edits or tests by assistant; not confirmed applied.
+2026-10-29 developer explicitly requested check after full rules. Read UpdateUserRequest: authorize, target guard, four field rules and ignore(target) present; missing Illuminate Validation Rule import would resolve nonexistent request-namespace Rule at runtime. Guided import-only correction, no edits or tests by assistant. Also inspected existing GenerateUsername for upcoming save: signature only first/last, query includes edited account, optional target exclusion needed for same normalized name. Read controller/model/policy/routes: edit props and GET update policy present, update still stub, no PATCH route. Preparation/intermediate inspection only; FB-021 not complete.
+2026-10-29 developer replied done to missing Rule import fix; application confirmation only, no re-inspection/test. Next lesson supplies optional nullable User parameter on existing GenerateUsername::generate method as edit prerequisite. Existing App Models User import already present. Explain same normalized name (Mary Jane to Mary-Jane) should not cause suffix solely because account owns base username. Query exclusion will be taught next, creation behavior retained. No application edits/tests by assistant.
+2026-10-29 developer asked for clarification about own-account exclusion. Explained Mary Jane to Mary-Jane produces same base, while Maria Sharapova produces new base and checks all other accounts for suffix. Developer accepted explanation and requested changes shown; provided optional User signature plus conditional target-ID exclusion in existing while query. This is teaching code for developer, not authorization to edit source. No application edits/review/tests by assistant; query application not confirmed.
+2026-10-29 after generator line-by-line explanation, developer requested next step (no comprehension answer or explicit generator application/test confirmation claimed). Supplied controller saving lesson following inspected Poker controller validated-save/toast/details pattern, adding existing domain GenerateUsername only when first/last differs, passing target account for own-ID exclusion. Uses validated four contacts only; username server-generated; fixed role/status/password untouched by request data. No assistant source edits or tests. PATCH route remains next.
+2026-10-29 developer replied done to controller UpdateUserRequest import and update save method; application confirmation only, not re-inspected. Supplied protected PATCH users/{user} route matching Vue form.patch URL and inspected Poker route authorization pattern; explained PATCH, model binding, policy then request validation/authorization then controller save, redirect and props. Asked developer to test phone-only save/current unchanged email/username unchanged/details refresh and toast. No assistant application edits or tests; save not yet reported tested.
+2026-10-29 explicit delegation: you do all the tests please. Assistant executed 31 focused scenarios/190 assertions on SQLite and the same 31/190 on isolated MySQL, both PASS. Browser checks on isolated MySQL PASS: prefill/read-only contacts ownership, phone save/current email/username preservation, refresh persistence, Mary Jane to Mary-Jane self-exclusion, Maria Sharapova regenerated username/toast, required-field error/retained input, duplicate-email feedback, Cancel discards edits, manager self-edit 403, keyboard Tab and 390px single-column/1280px two-column layout without overflow. No source edits. Temp server/database removed. Missing Edit button leaves whole-user journey incomplete. Existing deferred phone cleanup not claimed fixed. Loading/duplicate prevention reviewed in source; no throttled-network timing test performed.
+2026-10-29 developer said ok go ahea after test findings and proposed Edit-button lesson. Continued developer-written teaching; no explicit exception to source-writing rule inferred. First small prerequisite supplied: Laravel Show props numeric user id plus canEdit from update policy, Request injected into show method. No visible page change expected yet. Previous delegated tests remain recorded for prior source snapshot; navigation not yet implemented or tested, formatting failures still open.
+2026-10-29 developer replied done to Show controller user id/canEdit prop changes; application confirmation only, not re-inspected or tested. Supplied Vue lesson importing Link/Button, extending props and adding conditional Edit link in shared CardAction next to title; explain CardHeader built-in grid and CardAction right-hand position. Shared CardHeader and CardAction read for upcoming layout convention, not review of developer changes. No application edits/tests by assistant.
+2026-10-29 developer applied Show.vue Edit button. Under retained explicit testing delegation, inspected Show/controller and executed 10 targeted MySQL tests (78 assertions), all PASS: cross-role details permissions and canEdit, all roles own-details canEdit false. Browser PASS: manager sees Edit for fictional volunteer, link opens correct edit URL, Cancel returns to same details, own My details has no Edit link. Vue types PASS; npm check FAIL formatting Edit and Show; Pint FAIL formatting GenerateUsername and routes; git diff check PASS. Temp test server/MySQL DB removed. Supplied developer-run targeted formatting commands. No application source edited by assistant.
+2026-10-29 developer ran targeted PHP/Vue formatters. Assistant inspected affected PHP/Vue and re-ran checks under retained explicit testing delegation. PASS Pint targeted PHP; npm types:check; npm check (64 formatted files, lint 55 files no warnings/errors); git diff check; complete focused external EditUserTest suite 41 tests/268 assertions on SQLite. Earlier main31 and navigation10 MySQL passes and browser evidence retained, formatting reviewed as non-behavioral. Main navigation/formatting review findings resolved; known shared phone-cleanup/concurrency deferrals still open and no full application green claim. No application source edited by assistant.
+2026-10-29 developer explicitly authorized only changing the successful edit redirect to the user list. Changed UserController::update final return to to_route(users.index) and its explanatory comment. Success toast and save logic retained. Source-reviewed this two-line change; PHP syntax check passed. Browser/behavior check pending developer; no application test suite run. All earlier role/status dropdown, validation, session and middleware changes were fully reverted at developer request before this change; do not treat role changes as implemented or approved for resumption.
+2026-10-29 developer requested only role dropdown and Active/Inactive checkboxes matching Create User layout with saved values selected. Assistant explicitly scoped this response to controls; persistence separate. Implemented Edit.vue Select bound to string saved role_id, linked boolean status checkboxes (one checked at a time), matching Create spacing/grid. UserController::edit sends role_id/is_active and database role choices via GetAssignableRoles::get(forEdit: true). Edit offers Manager/Volunteer; default Create behavior unchanged. Policies/routes/UpdateUserRequest/save logic and sessions untouched; role/status changes are NOT saved yet. Existing redirect to users.index retained. Source-reviewed display wiring; PHP syntax, targeted Pint, Vue type check and diff whitespace pass. No application behavior tests or browser checks performed; ask developer to verify controls first. Earlier broad attempted implementation remains reverted. No completion claimed.
+2026-10-29 explicit developer authorization: connect role/status changes to the existing Edit workflow and report files/methods. UpdateUserRequest::rules validates role_id using existing GetAssignableRoles::get(forEdit:true) and required boolean is_active. UserController::update now saves validated role/status and revokes target database sessions/Remember me token on active-to-inactive change inside DB transaction. Edit.vue::submit confirms loss of access/session termination before deactivation. New EnsureAccountIsActive::handle logs inactive users out and invalidates current session; registered before password-setup middleware in bootstrap/app.php. Existing UserPolicy and GET/PATCH can(update,target) checks unchanged; Super Admin edits managers/volunteers, manager edits volunteers and may promote to manager, then loses edit/view access to promoted account. Existing users.index success redirect retained. Current session driver confirmed database. Source reviewed these changes at HEAD 6a79da523dc0fd03487b76fc22311c2296f3d330 plus working tree; no new findings for this scoped change. No full feature completion claimed.
+2026-10-29 developer explicitly requested confirmation for promotion/demotion AND activation as well as deactivation, and testing only these current changes. Changed ONLY Edit.vue::submit application code: compare role/status against saved props, describe current-to-selected role and activation/deactivation consequences, combine all applicable details into one window.confirm before PATCH. Cancel returns without request and retains selections; unchanged role/status (including contact-only edit) does not prompt. Existing backend saving/permissions/session handling/list redirect untouched. Source-reviewed this confirmation change.
+2026-10-29 developer requested guidance only: add a user-list column with an Edit button for every listed user; do the rest later. Read current AGENTS.md in full and users/Index.vue to prepare lesson (not an unsolicited review). Proposed smallest visible scaffold: Actions heading after Status, one unlinked type=button shared Button in each v-for row, and empty-state colspan6-&gt;7. Button already imported. No application source edits or tests for this request. All-row button is a UI placeholder only, not broader editing permission; navigation and permission-aware visibility remain later work.
+2026-10-29 developer ordinary ok accepted as application confirmation of placeholder lesson only; no intermediate review/test inferred. Requested same UserPolicy update rules for list Edit-button availability: manager only volunteers, volunteers no buttons enabled, Super Admin managers/volunteers. Developer explicitly corrected earlier own-manager exception: cannot edit own account. Read full AGENTS.md and actual ListUsers, UserController index, UserPolicy and IndexUsersRequest for upcoming lesson; no Index.vue review or application source edits/tests. First backend lesson supplied: pass signed-in actor from UserController index to ListUsers get, through prepareUser, append canEdit using actor-&gt;can(update,target). Next separate Vue lesson types canEdit and binds disabled; actual button navigation remains separate.
+2026-10-29 developer replied done to backend canEdit preparation lesson; application confirmation only, no review or behavior-test pass inferred. Next small Vue lesson supplied: users/Index.vue add canEdit:boolean to each data-row type and :disabled=!user.canEdit on existing Edit Button. Explain boolean, dynamic colon binding and negation. Ask developer to verify enabled/disabled buttons for manager, volunteer and Super Admin accounts using existing update permissions. No source edits, intermediate inspection, application tests or browser checks performed by assistant. Button navigation remains a later step.</x:v>
       </x:c>
       <x:c r="R25" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer creating resources/js/pages/users/Edit.vue with shared Card/CardHeader/CardTitle and Edit User heading inside main p-4, Card w-full max-w-3xl. Ordinary done means continue without intermediate review. Next teach UserController edit response, then protected GET edit route using update ability before sending account data. Later prefill, layout/state, validation/save and protected PATCH route. Completed-feature review and developer-first testing still required. Preserve previous deferrals and FB-008 open status.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer applying Index.vue canEdit:boolean and :disabled binding and reporting role-matrix check: manager volunteers only, volunteer none, Super Admin managers/volunteers only; own account always disabled under current rules. A done reply following these explicit checks records developer-reported testing only. Completed-feature review still required; navigation not yet connected. Preserve prior evidence and all pending/deferred checks.</x:v>
       </x:c>
       <x:c r="S25" s="11" t="n"/>
     </x:row>
@@ -3408,42 +3448,48 @@
       </x:c>
       <x:c r="G26" s="4" t="str">
         <x:f>IF(H26="Complete","Complete",IF(I26="Blocked","Blocked",IF(I26="In progress","Ready",IF(F26="","Ready",IF(COUNTIFS($B$4:$B$73,F26,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H26" s="4" t="str">
         <x:f>IF(I26="Not started","Not started",IF(I26="Blocked","Blocked",IF(I26="In progress","In progress",IF(J26&lt;&gt;"Passed","Awaiting code review",IF(OR(K26="",NOT(ISNUMBER(L26))),"Awaiting review evidence",IF(N26&lt;&gt;"Passed","Awaiting test",IF(OR(M26="",O26="",NOT(ISNUMBER(P26))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I26" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I26" s="10" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J26" s="10" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Not reviewed</x:t>
         </x:is>
       </x:c>
-      <x:c r="K26" s="10" t="n"/>
+      <x:c r="K26" s="10" t="str">
+        <x:v>
+2026-10-29 explicit developer authorization: connect role/status changes to the existing Edit workflow and report files/methods. UpdateUserRequest::rules validates role_id using existing GetAssignableRoles::get(forEdit:true) and required boolean is_active. UserController::update now saves validated role/status and revokes target database sessions/Remember me token on active-to-inactive change inside DB transaction. Edit.vue::submit confirms loss of access/session termination before deactivation. New EnsureAccountIsActive::handle logs inactive users out and invalidates current session; registered before password-setup middleware in bootstrap/app.php. Existing UserPolicy and GET/PATCH can(update,target) checks unchanged; Super Admin edits managers/volunteers, manager edits volunteers and may promote to manager, then loses edit/view access to promoted account. Existing users.index success redirect retained. Current session driver confirmed database. Source reviewed these changes at HEAD 6a79da523dc0fd03487b76fc22311c2296f3d330 plus working tree; no new findings for this scoped change. No full feature completion claimed.
+2026-10-29 developer explicitly requested confirmation for promotion/demotion AND activation as well as deactivation, and testing only these current changes. Changed ONLY Edit.vue::submit application code: compare role/status against saved props, describe current-to-selected role and activation/deactivation consequences, combine all applicable details into one window.confirm before PATCH. Cancel returns without request and retains selections; unchanged role/status (including contact-only edit) does not prompt. Existing backend saving/permissions/session handling/list redirect untouched. Source-reviewed this confirmation change.</x:v>
+      </x:c>
       <x:c r="L26" s="30" t="n"/>
-      <x:c r="M26" s="10" t="n"/>
-      <x:c r="N26" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O26" s="10" t="n"/>
-      <x:c r="P26" s="30" t="n"/>
-      <x:c r="Q26" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">
-2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R26" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules. Build account deactivation/reactivation after prerequisites. Include deferred FB-005 session enforcement: Vue confirmation, authorized server operation, block existing and remembered sessions, reject new logins while inactive, and verify reactivation. Super Admin manages manager/volunteer accounts; managers retain agreed volunteer permissions. Developer writes code.</x:t>
-        </x:is>
+      <x:c r="M26" s="10" t="str">
+        <x:v>Assistant (explicit narrow test delegation)</x:v>
+      </x:c>
+      <x:c r="N26" s="10" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="O26" s="10" t="str">
+        <x:v>
+2026-10-29 assistant-executed under earlier narrow role/status test delegation: external /tmp/foodbank-fb021/EditRoleStatusTest.php PASS 27 tests/148 assertions on isolated in-memory SQLite. Covers role saves/promotion/demotion and unchanged values, both status transitions, combined role/status save, invalid role/status rejected, forbidden Super Admin assignment, existing-manager target denied, post-promotion edit denied, creation dropdown unchanged, prefilled edit props, target-only database session deletion/Remember me token rotation and reactivation preserving revocation, inactive signed-in sessions denied before setup. Targeted Pint/PHP syntax, Vue type check, Vue formatting and diff whitespace pass. No full workflow, password-login tests or browser confirmation/visual checks run. Earlier shared deferred phone/concurrency/password tests remain open; earlier 41-test evidence historical and not rerun for changed contracts.
+2026-10-29 scoped confirmation checks PASS: 18 scenarios in external /tmp/foodbank-fb021/confirmation-check.mjs execute actual submit() extracted from Edit.vue and transpiled with TypeScript, using stubbed confirm/patch. Includes both confirmation outcomes for promotion, demotion, activation, deactivation and all four combined role/status directions; only one prompt for combined changes, accurate details, Confirm submits once, Cancel sends no request and retains state, unchanged role/status skips prompt. Vue type check, targeted Vue formatting and diff whitespace pass. No browser/native-dialog rendering check, backend tests or full workflow rerun for this change. Earlier backend27/148 evidence retained, not repeated.</x:v>
+      </x:c>
+      <x:c r="P26" s="30" t="n">
+        <x:v>46324</x:v>
+      </x:c>
+      <x:c r="Q26" s="10" t="str">
+        <x:v>
+2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.
+2026-10-29 explicit developer authorization: connect role/status changes to the existing Edit workflow and report files/methods. UpdateUserRequest::rules validates role_id using existing GetAssignableRoles::get(forEdit:true) and required boolean is_active. UserController::update now saves validated role/status and revokes target database sessions/Remember me token on active-to-inactive change inside DB transaction. Edit.vue::submit confirms loss of access/session termination before deactivation. New EnsureAccountIsActive::handle logs inactive users out and invalidates current session; registered before password-setup middleware in bootstrap/app.php. Existing UserPolicy and GET/PATCH can(update,target) checks unchanged; Super Admin edits managers/volunteers, manager edits volunteers and may promote to manager, then loses edit/view access to promoted account. Existing users.index success redirect retained. Current session driver confirmed database. Source reviewed these changes at HEAD 6a79da523dc0fd03487b76fc22311c2296f3d330 plus working tree; no new findings for this scoped change. No full feature completion claimed.
+2026-10-29 developer explicitly requested confirmation for promotion/demotion AND activation as well as deactivation, and testing only these current changes. Changed ONLY Edit.vue::submit application code: compare role/status against saved props, describe current-to-selected role and activation/deactivation consequences, combine all applicable details into one window.confirm before PATCH. Cancel returns without request and retains selections; unchanged role/status (including contact-only edit) does not prompt. Existing backend saving/permissions/session handling/list redirect untouched. Source-reviewed this confirmation change.</x:v>
+      </x:c>
+      <x:c r="R26" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Role/status saving and confirmation implementation supplied. Current change has 18 focused submit-function checks passed; user may verify visible prompts on a fictional account. Preserve pending browser checks and existing shared deferred phone/concurrency/password checks; no whole-feature completion or full workflow rerun claimed. Continue according to developer direction.</x:v>
       </x:c>
       <x:c r="S26" s="10" t="n"/>
     </x:row>
@@ -6594,7 +6640,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0135941f6924467d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e328e8a7c13421b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7288,15 +7334,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D23" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Roles are fixed after account creation in the current version.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E23" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-004, FB-019</x:t>
-        </x:is>
+      <x:c r="D23" s="28" t="str">
+        <x:v>2026-10-29 superseding developer-approved current scope: existing account roles may change through Edit. Super Admin may edit existing manager/volunteer accounts and assign Manager or Volunteer (including demotion). Managers may edit existing volunteer accounts and assign Volunteer or Manager (including promotion). Existing target-account permissions remain unchanged; after promotion the original manager cannot view/edit the newly promoted manager. Super Admin assignment and self editing remain disallowed. Creation permissions remain unchanged. Latest explicit instruction authorizes persistence of role/status, superseding earlier UI-only checkpoint and fixed-role version-one rule.
+2026-10-29 approved: before saving a changed role, request confirmation describing the saved role and selected role (promotion or demotion). Cancel sends no save request. Combine with status confirmation when both change.</x:v>
+      </x:c>
+      <x:c r="E23" s="28" t="str">
+        <x:v>FB-004, FB-019, FB-021</x:v>
       </x:c>
       <x:c r="F23" s="28" t="inlineStr">
         <x:is>
@@ -7315,25 +7358,17 @@
           <x:t xml:space="preserve">1. Roles and account creation</x:t>
         </x:is>
       </x:c>
-      <x:c r="C24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">##FUTURE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">##FUTURE Changing an existing user's role, such as promoting a volunteer to manager.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deferred — no current item</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F24" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deferred</x:t>
-        </x:is>
+      <x:c r="C24" s="4" t="str">
+        <x:v>Current scope</x:v>
+      </x:c>
+      <x:c r="D24" s="4" t="str">
+        <x:v>2026-10-29 moved from deferred to approved current scope: role changes through Edit follow REQ-020. Super Admin assigns Manager/Volunteer to managed accounts; manager may promote an existing volunteer. No Super Admin assignment. Preserve current target-account authorization and creation limits.</x:v>
+      </x:c>
+      <x:c r="E24" s="4" t="str">
+        <x:v>FB-021</x:v>
+      </x:c>
+      <x:c r="F24" s="4" t="str">
+        <x:v>Stories!B25</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="52" customHeight="1">
@@ -7581,11 +7616,10 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D32" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Successful Create and Edit actions redirect to that user's details page and display a success message.
-2026-10-26 temporary learning sequence: developer requested saving and database inspection before building details, declined returning to create form. Dashboard redirect used for first successful save; final details redirect remains required. First frontend save now developer-confirmed; build details next, then complete setup and connected checks.</x:t>
-        </x:is>
+      <x:c r="D32" s="4" t="str">
+        <x:v>Successful Create and Edit actions redirect to that user's details page and display a success message.
+2026-10-26 temporary learning sequence: developer requested saving and database inspection before building details, declined returning to create form. Dashboard redirect used for first successful save; final details redirect remains required. First frontend save now developer-confirmed; build details next, then complete setup and connected checks.
+2026-10-29 superseding developer decision: successful Edit saves redirect to the user list (users.index, /users) with the existing success message. Create still redirects to the created user details page.</x:v>
       </x:c>
       <x:c r="E32" s="4" t="inlineStr">
         <x:is>
@@ -8052,11 +8086,10 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D46" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Inactive managers cannot log in or continue using an existing session. The Super Admin can reactivate them later.
-2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.</x:t>
-        </x:is>
+      <x:c r="D46" s="4" t="str">
+        <x:v>Inactive managers cannot log in or continue using an existing session. The Super Admin can reactivate them later.
+2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.
+2026-10-29 status saving now connected through Edit with confirmation, target database-session removal, Remember me revocation, and inactive-session middleware. Focused automated checks pass; browser confirmation/new-login checks remain unverified. Earlier sequencing deferral superseded for this implementation only.</x:v>
       </x:c>
       <x:c r="E46" s="4" t="inlineStr">
         <x:is>
@@ -8085,11 +8118,11 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D47" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deactivating a manager or volunteer requires confirmation explaining that the user will lose access and their existing sessions will end.
-2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.</x:t>
-        </x:is>
+      <x:c r="D47" s="28" t="str">
+        <x:v>Deactivating a manager or volunteer requires confirmation explaining that the user will lose access and their existing sessions will end.
+2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.
+2026-10-29 status saving now connected through Edit with confirmation, target database-session removal, Remember me revocation, and inactive-session middleware. Focused automated checks pass; browser confirmation/new-login checks remain unverified. Earlier sequencing deferral superseded for this implementation only.
+2026-10-29 approved extension: activation also requires confirmation, explaining that the account will be allowed to sign in again. If role and status both change, one combined confirmation describes both. Cancel prevents the entire edit save. Unchanged role/status needs no confirmation.</x:v>
       </x:c>
       <x:c r="E47" s="28" t="inlineStr">
         <x:is>
@@ -8343,11 +8376,10 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D55" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Inactive volunteers cannot log in or continue using an existing session. Their records remain available to managers, and any manager can reactivate them later.
-2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.</x:t>
-        </x:is>
+      <x:c r="D55" s="28" t="str">
+        <x:v>Inactive volunteers cannot log in or continue using an existing session. Their records remain available to managers, and any manager can reactivate them later.
+2026-10-26 developer-approved sequencing: defer implementation and verification of blocking existing/remembered sessions for inactive accounts to FB-022, when building the disable-account screen. Connect the Vue confirmation/action to Laravel enforcement then; a hidden button alone is insufficient. Preserve current password-login inactive check. This remains required current scope, not FUTURE and not verified.
+2026-10-29 status saving now connected through Edit with confirmation, target database-session removal, Remember me revocation, and inactive-session middleware. Focused automated checks pass; browser confirmation/new-login checks remain unverified. Earlier sequencing deferral superseded for this implementation only.</x:v>
       </x:c>
       <x:c r="E55" s="28" t="inlineStr">
         <x:is>
@@ -12000,30 +12032,20 @@
           <x:t xml:space="preserve">REQ-166</x:t>
         </x:is>
       </x:c>
-      <x:c r="B169" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">##FUTURE — Confirmed future direction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C169" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">##FUTURE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D169" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">##FUTURE Changes to existing users' roles; permissions and behaviour will be defined later.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E169" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deferred — no current item</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F169" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deferred</x:t>
-        </x:is>
+      <x:c r="B169" s="28" t="str">
+        <x:v>1. Roles and account creation</x:v>
+      </x:c>
+      <x:c r="C169" s="28" t="str">
+        <x:v>Current scope</x:v>
+      </x:c>
+      <x:c r="D169" s="28" t="str">
+        <x:v>2026-10-29 moved from deferred to approved current scope: role changes through Edit follow REQ-020. Super Admin assigns Manager/Volunteer to managed accounts; manager may promote an existing volunteer. No Super Admin assignment. Preserve current target-account authorization and creation limits.</x:v>
+      </x:c>
+      <x:c r="E169" s="28" t="str">
+        <x:v>FB-021</x:v>
+      </x:c>
+      <x:c r="F169" s="28" t="str">
+        <x:v>Stories!B25</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="76" customHeight="1">
@@ -12496,7 +12518,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aef1d13cdba4b44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3642f61181e46d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add authorized department creation and sample department seeder
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -696,7 +696,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>FB-021</t>
+          <t>FB-027</t>
         </is>
       </c>
       <c r="C10" s="15" t="n"/>
@@ -723,7 +723,7 @@
       <c r="A12" s="15" t="n"/>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Nine PHP type-description errors resolved and PHPStan now passes (scoped21tests288assertions/Pint/whitespace also pass). Remaining non-deferred user-module findings: long accepted names overflow username storage causing browser/MySQL500, and two existing test-fixture failures. Await developer direction to correct those; authorization for this turn covered only type descriptions. Preserve all existing final-project deferrals. Inventory not started; full completion still open.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -741,7 +741,7 @@
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>FB-021</t>
+          <t>FB-027</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>2026-10-29 developer explicitly authorized resolving the nine PHP type-description errors only. Assistant changed ListUsers method PHPDoc to describe optional search string/null, Builder&lt;User&gt;, paginator integer keys/prepared row values, and prepared row key/value types; User date import/properties now CarbonImmutable, matching AppServiceProvider Date::use and actual model datetime casts. No runtime behavior changes. Scoped diff/source review PASS. app/Actions/Users/ListUsers.php SHA256 2d6479cf5525d05cd23f6620749486a1ff479d242bb59c285800713e968c0d07; app/Models/User.php SHA256 6200c8c7f6c76054dd5a8e046d639d1a11a893d73360404f568946da383892e6. PHPStan512M PASS zero errors; targeted Pint PASS; whitespace PASS; external isolated SQLite ListEditPermissionTest21tests288assertions PASS. Read-only unsaved model check confirms email_verified_at/created_at/updated_at resolve CarbonImmutable; initial check incorrectly passed these guarded date fields to constructor, corrected harness to direct assignments, no source defect. No live DB writes/users created, no browser checks or unrelated/password tests. Earlier long-name MySQL500 and two existing test failures remain unresolved; all project-end deferrals retained. This supersedes only the nine-error finding, not full user-module review/test status.</t>
+          <t>FB-026 creation source review passed; developer reports all creation checks passed. Next FB-027 list: start shared Card Index page, then data and route, then rename.</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Nine PHP type-description errors resolved and PHPStan now passes (scoped21tests288assertions/Pint/whitespace also pass). Remaining non-deferred user-module findings: long accepted names overflow username storage causing browser/MySQL500, and two existing test-fixture failures. Await developer direction to correct those; authorization for this turn covered only type descriptions. Preserve all existing final-project deferrals. Inventory not started; full completion still open.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>Nine PHP type-description errors fixed; awaiting developer direction on remaining long-name save failure and two existing test-fixture failures.</t>
+          <t>Awaiting developer to create Department list page scaffold.</t>
         </is>
       </c>
     </row>
@@ -789,8 +789,7 @@
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>2026-10-29 HEAD91e157fb6d367016ef7181ce50ad81115e9648da plus existing Index.vue/routes working edits; completed-module review Changes needed.81focused/743assertions pass;2selected repo tests fail;9PHPStan errors;long-name MySQL/browser500.
-2026-10-29 type-description-only fix reviewed; PHPStan zero errors;21/288test PASS. app/Actions/Users/ListUsers.php SHA256 2d6479cf5525d05cd23f6620749486a1ff479d242bb59c285800713e968c0d07; app/Models/User.php SHA256 6200c8c7f6c76054dd5a8e046d639d1a11a893d73360404f568946da383892e6</t>
+          <t>2026-10-29 FB-026 creation review passed at befad9c working snapshot; hashes in Stories K29.</t>
         </is>
       </c>
     </row>
@@ -951,7 +950,8 @@
         <is>
           <t>2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Order: FB-016/017/018, prepare FB-020, FB-019, FB-006/007, FB-024, FB-009–015, FB-008, remaining accounts. Catalogue modules create before list; Product already does. Super Admin recovery stays last.
 2026-10-27 sequence decision: place the bcrypt 72-byte repair and repeat test within FB-069, immediately before final FB-070. Existing first-login review/test failures remain recorded; this timing change does not verify them.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</t>
+2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF17324D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3553,12 +3553,13 @@
 2026-10-29 developer explicitly delegated testing of list Edit-button permissions. Read full AGENTS.md and reviewed connected ListUsers get/prepareUser, UserController index, Index.vue row type/button/empty-state, shared Button attribute forwarding, UserPolicy update and protected GET/PATCH routes. Scoped review PASS, no findings. At HEAD6a79da523dc0fd03487b76fc22311c2296f3d330 plus developer-staged working tree. SHA256 ListUsers0291be9b73da0d27f7214a99b83984dbf38a8a48c81f1d587241778404eaba45; UserController6bc9daae2e6bf576c39d58284bc1acace5757c777ceba1f88e77098d298d8a00; Index8cbc5aa61958e64908ad248d7f479f63ac39db3a53d083456fbed70ae24c268d. No application source edits, commits or staging by assistant. Buttons remain unlinked, by current lesson scope.
 2026-10-29 developer requested guidance to connect list Edit buttons to existing Edit page. Preparation read Index.vue, generated users edit helper and protected GET/PATCH routes; Poker players Index and edit route confirm selected-ID navigation with update policy. Supplied small lesson: import edit alongside index and add @click="router.get(edit.url(user.id))" to existing disabled-aware button. Existing router import reused. No application edits or tests by assistant; developer application/navigation check pending. Existing completion evidence and deferrals preserved.
 2026-10-29 developer reported list Edit-button navigation is working fine after explicit navigation/disabled-button check instructions. Record as developer-reported PASS for that requested scoped check, not assistant-executed testing or full edit-feature completion. No source inspection performed on ordinary confirmation. Existing scoped permission review/test evidence retained; completed-feature review and remaining non-deferred edit acceptance checks still required. FB-008/FB-023 remain deferred to project end.
-2026-10-29 completed-module delegated review/test checkpoint recorded. Inventory not begun; findings need correction. All prior deferrals/evidence retained.</t>
+2026-10-29 completed-module delegated review/test checkpoint recorded. Inventory not begun; findings need correction. All prior deferrals/evidence retained.
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
       <c r="R25" s="11" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Nine PHP type-description errors resolved and PHPStan now passes (scoped21tests288assertions/Pint/whitespace also pass). Remaining non-deferred user-module findings: long accepted names overflow username storage causing browser/MySQL500, and two existing test-fixture failures. Await developer direction to correct those; authorization for this turn covered only type descriptions. Preserve all existing final-project deferrals. Inventory not started; full completion still open.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
       <c r="S25" s="11" t="n"/>
@@ -3812,14 +3813,13 @@
       <c r="Q28" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">
-2026-10-29 completed-module delegated review/test checkpoint recorded. Inventory not begun; findings need correction. All prior deferrals/evidence retained.</t>
+2026-10-29 completed-module delegated review/test checkpoint recorded. Inventory not begun; findings need correction. All prior deferrals/evidence retained.
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
       <c r="R28" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. 2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
       <c r="S28" s="10" t="n"/>
@@ -3863,30 +3863,49 @@
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Ready for review</t>
         </is>
       </c>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K29" s="11" t="n"/>
-      <c r="L29" s="31" t="n"/>
-      <c r="M29" s="11" t="n"/>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-29 requested intermediate scaffold review: Department model empty; migration id/timestamps only; seeder empty; controller methods empty; Store/Update requests authorize=false with empty rules; policy denies all. Namespaces/imports correctly placed. No Department routes or Vue UI. Not feature completion; no application tests run or edits made. Poker reference inspected: Models/Player.php protected $fillable; Requests/Players/StorePlayerRequest.php validation; Policies/PlayerPolicy.php abilities; PlayerController.php validated simple saves/Inertia feedback; routes/web.php -&gt;can on display/write. HEAD befad9c75df55a0608a1ee45f68792d80996232a Snapshot SHA256: app/Models/Department.php c0e27aa79fab4cc4c6f1fa3dc0d39bb7a0bebaaa92edd06185e2c65fa492f3e8; database/migrations/2026_10_29_121954_create_departments_table.php ca713f8069394dcd2bc21d6c8e9e1eaebb6eb9c6e76cb69766fc8530a181e28e; database/seeders/DepartmentSeeder.php af1151523a40742dfdb1bbd8008fe92d60d2634e241e71427843fd68da4b5eb4; app/Http/Controllers/DepartmentController.php 1156ecf4b4f75bb6ed06a8185e36256a313e75acd41d4ef3f0aeada1706c552b; app/Http/Requests/Departments/StoreDepartmentRequest.php f22e783ca2e5201002eef108468ebf022050c06301ed355fb280f7585f6202d5; app/Http/Requests/Departments/UpdateDepartmentRequest.php 3150a0f8c9bafb83180818233de0d9a6f000eebfba65f44a70bf5e3a80a95b6c; app/Policies/DepartmentPolicy.php 1cc1c746232f3149db409af77393d9f3e600de0e7748f5d341d867ff0815ba6e; routes/web.php 93ccbe0e562268518969445fb2e3f0906a8294a95e7ff37300c9fb891f3079c2
+2026-10-29 completed creation source review at HEAD befad9c75df55a0608a1ee45f68792d80996232a plus current working files: Passed, no blocking functional findings. GET/POST auth+create policy Manager/Super Admin; FormRequest validated required string max255 unique; Laravel standard trimming retained; migration unique name and model fillable; controller validated save/flash/back; Vue reactive binding, error display, processing disabled, success reset, responsive field/button; repeatable seeder. Unused policy Response import/import order/whitespace are cosmetic cleanup only. Index/edit/update remain unused scaffold and outside creation verification. No assistant application tests/browser checks. Snapshot SHA256: app/Models/Department.php 137bfc6b754c5fe00eb129777ea2a900242c495684a9225c1699ea9888118a7c; database/migrations/2026_10_29_121954_create_departments_table.php 8734f6600b1ec7fa25ff9cf1bf994f2ea23d58a1c72404cdfd1b0ac385d7eb70; database/seeders/DepartmentSeeder.php f41eb90ea8bd6350fc0dc6c61b2aff8b990f4e67bd4387efb57981beb64acdf9; app/Policies/DepartmentPolicy.php f2daa67a85b43b239152639f654d91171ed7dbf687f279fea36fc5fd3680db86; app/Http/Requests/Departments/StoreDepartmentRequest.php 6ce5d49bf67923ef0fbf45bef51c9473bf67ae456a453dfb32778bc263528aa8; app/Http/Controllers/DepartmentController.php 3ca3024e3b534ad236999bf1a2d6c63dd9990f92871f8d50c51cafebd8502381; resources/js/pages/departments/Create.vue 3718a428704dd69322e36f0146be784dbdaaca4be9a55a8c9aac52183f608b1e; routes/web.php 08b9ccec98fe21124a6f7fd98fc20a4a23d8519d2c34a9538693c7e971440f64</t>
+        </is>
+      </c>
+      <c r="L29" s="31">
+        <v>46324</v>
+      </c>
+      <c r="M29" s="11" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
       <c r="N29" s="11" t="inlineStr">
         <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O29" s="11" t="n"/>
-      <c r="P29" s="31" t="n"/>
-      <c r="Q29" s="11" t="n"/>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="O29" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-29 Developer-reported: migration successful; permitted create heading displayed; successful create stayed on page with success toast and cleared input; exact, lowercase and outer-space duplicates each showed name error; seeder ran successfully. Latest developer statement: "i have checked everything related to department creation." Recorded as overall developer-reported creation pass; remaining individual cases were not enumerated, so no assistant-executed or specific denied-request/overlength result is claimed.</t>
+        </is>
+      </c>
+      <c r="P29" s="31">
+        <v>46324</v>
+      </c>
+      <c r="Q29" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-29 creation complete based on passed source review and overall developer-reported creation testing. No assistant application testing. Seeder added under explicit permission and developer ran successfully.</t>
+        </is>
+      </c>
       <c r="R29" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Build Department model/storage, then complete and verify creation before its list at FB-027.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-026 complete; continue FB-027 Department list then rename.</t>
         </is>
       </c>
       <c r="S29" s="11" t="n"/>
@@ -3931,7 +3950,7 @@
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -3949,11 +3968,14 @@
       </c>
       <c r="O30" s="10" t="n"/>
       <c r="P30" s="30" t="n"/>
-      <c r="Q30" s="10" t="n"/>
+      <c r="Q30" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29 first lesson supplied: shared responsive Card scaffold in departments/Index.vue; no list implementation reviewed or tested yet.</t>
+        </is>
+      </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: After verified Department creation, display its list and then teach rename. Complete and verify the module before Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
         </is>
       </c>
       <c r="S30" s="10" t="n"/>
@@ -6836,7 +6858,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart ns1:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -12467,7 +12489,8 @@
 2026-10-28 developer explicitly deferred the simultaneous same-name username-selection/save conflict fix and its verification until project end, at the existing final project verification checkpoint after FB-070 implementation, review and testing. Locking versus bounded unique-constraint retry remains undecided; neither approach approved. Keep current unique index and serial username generation; do not claim concurrency resolved. FB-018 and affected FB-019 remain open. No further concurrency lesson or Poker lookup now. Continue eligible lessons while retaining other non-deferred account-creation prerequisites and all existing final-verification gates.
 2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
 2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</t>
+2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
         </is>
       </c>
       <c r="E175" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Department list with search implemented
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -723,7 +723,7 @@
       <c r="A12" s="15" t="n"/>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: ListDepartments action extraction lessons developer-confirmed applied; automatic search, clearing and filtered pagination developer-reported passed. Current small step: remove temporary You typed paragraph in departments/Index.vue and understanding checkpoint on action responsibility. Then resume rename edit display/protected GET, form/state/validation/save incrementally. No unsolicited intermediate source review; complete Department module review and developer-first rename checks before completion/Category.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -753,7 +753,7 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>FB-026 creation source review passed; developer reports all creation checks passed. Next FB-027 list: start shared Card Index page, then data and route, then rename.</t>
+          <t>FB-027: action extraction and search/pagination checks developer-reported passed; remove temporary learning text, then resume rename.</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: ListDepartments action extraction lessons developer-confirmed applied; automatic search, clearing and filtered pagination developer-reported passed. Current small step: remove temporary You typed paragraph in departments/Index.vue and understanding checkpoint on action responsibility. Then resume rename edit display/protected GET, form/state/validation/save incrementally. No unsolicited intermediate source review; complete Department module review and developer-first rename checks before completion/Category.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>Awaiting developer to create Department list page scaffold.</t>
+          <t>Awaiting developer cleanup and short explanation of ListDepartments responsibility.</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF17324D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3877,7 +3877,7 @@
 2026-10-29 completed creation source review at HEAD befad9c75df55a0608a1ee45f68792d80996232a plus current working files: Passed, no blocking functional findings. GET/POST auth+create policy Manager/Super Admin; FormRequest validated required string max255 unique; Laravel standard trimming retained; migration unique name and model fillable; controller validated save/flash/back; Vue reactive binding, error display, processing disabled, success reset, responsive field/button; repeatable seeder. Unused policy Response import/import order/whitespace are cosmetic cleanup only. Index/edit/update remain unused scaffold and outside creation verification. No assistant application tests/browser checks. Snapshot SHA256: app/Models/Department.php 137bfc6b754c5fe00eb129777ea2a900242c495684a9225c1699ea9888118a7c; database/migrations/2026_10_29_121954_create_departments_table.php 8734f6600b1ec7fa25ff9cf1bf994f2ea23d58a1c72404cdfd1b0ac385d7eb70; database/seeders/DepartmentSeeder.php f41eb90ea8bd6350fc0dc6c61b2aff8b990f4e67bd4387efb57981beb64acdf9; app/Policies/DepartmentPolicy.php f2daa67a85b43b239152639f654d91171ed7dbf687f279fea36fc5fd3680db86; app/Http/Requests/Departments/StoreDepartmentRequest.php 6ce5d49bf67923ef0fbf45bef51c9473bf67ae456a453dfb32778bc263528aa8; app/Http/Controllers/DepartmentController.php 3ca3024e3b534ad236999bf1a2d6c63dd9990f92871f8d50c51cafebd8502381; resources/js/pages/departments/Create.vue 3718a428704dd69322e36f0146be784dbdaaca4be9a55a8c9aac52183f608b1e; routes/web.php 08b9ccec98fe21124a6f7fd98fc20a4a23d8519d2c34a9538693c7e971440f64</t>
         </is>
       </c>
-      <c r="L29" s="31">
+      <c r="L29" s="31" t="n">
         <v>46324</v>
       </c>
       <c r="M29" s="11" t="inlineStr">
@@ -3895,7 +3895,7 @@
           <t>2026-10-29 Developer-reported: migration successful; permitted create heading displayed; successful create stayed on page with success toast and cleared input; exact, lowercase and outer-space duplicates each showed name error; seeder ran successfully. Latest developer statement: "i have checked everything related to department creation." Recorded as overall developer-reported creation pass; remaining individual cases were not enumerated, so no assistant-executed or specific denied-request/overlength result is claimed.</t>
         </is>
       </c>
-      <c r="P29" s="31">
+      <c r="P29" s="31" t="n">
         <v>46324</v>
       </c>
       <c r="Q29" s="11" t="inlineStr">
@@ -3932,7 +3932,8 @@
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Required catalogue-wide unique name ignoring case/outer spaces. Rename retains links; no moving/deleting hierarchy. Managers/Super Admin only on display and write routes; validate success and duplicate errors. Teach create and rename separately. Review and test the complete Department list/create/rename module before FB-028. Existing-child rename checks are repeated once Category exists; no speculative child relationships now.
-2026-10-26 sequence: use departments created and verified at FB-026 for the first list; teach props/loop/layout before rename. Creation is a prerequisite to listing.</t>
+2026-10-26 sequence: use departments created and verified at FB-026 for the first list; teach props/loop/layout before rename. Creation is a prerequisite to listing.
+REQ-181: Department-name partial search matching users; search full dataset before pagination, retain search in links and support clearing.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -3966,16 +3967,30 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O30" s="10" t="n"/>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+2026-10-29 Developer-reported PASS: replied done to explicit checks that Manager/Super Admin sees departments/Edit buttons at /departments and Volunteer receives403 at direct URL. No pagination, edit or rename behaviour verified yet; overall test status remains Not tested until feature checks complete.
+2026-10-29 Developer-reported PASS after explicit checks: missing Builder import corrected and direct URL partial-search/full-list checks passed; Vue input displays Laravel search prop; pressing Enter filters names and clearing plus Enter restores full list. These are developer reports, not assistant execution. Automatic search and pagination checks remain pending; whole feature not verified.
+2026-10-29 developer replied done after explicit automatic-search checks: partial search after typing pause, clearing restores list, immediate Enter. Developer-reported PASS only; pagination and final review remain pending.
+2026-10-29 Developer-reported PASS after action extraction: replied done to explicit checks for automatic partial-name filtering, clearing restores list, and Next retaining search with more than ten matching results. No assistant-run application tests or browser checks. Whole-module final review and rename remain pending.</t>
+        </is>
+      </c>
       <c r="P30" s="30" t="n"/>
       <c r="Q30" s="10" t="inlineStr">
         <is>
-          <t>2026-10-29 first lesson supplied: shared responsive Card scaffold in departments/Index.vue; no list implementation reviewed or tested yet.</t>
+          <t>2026-10-29 first lesson supplied: shared responsive Card scaffold in departments/Index.vue; no list implementation reviewed or tested yet.
+2026-10-29: Developer explicitly authorized assistant creation of departments/Index.vue matching Users layout (name/Actions/Edit, empty state and paginator), viewAny policy and direct index controller query. Developer approved direct controller query as a scoped Poker-pattern exception: alphabetical paginate(10) sent through Inertia departments/Index departments prop. PHP syntax checks passed for controller/policy; no assistant application/browser tests. Developer added protected GET route during lesson and replied done after explicit Manager/Super Admin list + Volunteer direct-URL403 checks. Full feature review remains pending; do not mark Complete. Next lesson: update permission before rename display/save. Reference: skander/app/Http/Controllers/PlayerController.php uses ListPlayers for filtered listing and Inertia response; Department simpler direct query approved by developer.
+2026-10-29 developer approved search before edit, same as users. Inspected users/Index.vue (ref/watch,300ms timer, immediate Enter, Inertia preserveState), Requests/Users/IndexUsersRequest.php (nullable string max100 and page validation). First lesson: visible search input only. No search implementation/review/tests completed. Resume context: DepartmentPolicy update already exists. Poker PlayerController edit uses only(id,name,...), route edit/update both can(update,player); no rename lesson confirmed applied.
+2026-10-29 lessons advanced: developer confirmed input/local ref, IndexDepartmentsRequest, validation and controller connection steps. Explicit intermediate review requested after database-search lesson. Read app/Http/Requests/Departments/IndexDepartmentsRequest.php, app/Http/Controllers/DepartmentController.php, resources/js/pages/departments/Index.vue, routes/web.php. Finding: query callback uses Builder without Illuminate\Database\Eloquent\Builder import; nonempty search will receive wrong namespaced type. Validation and protected viewAny route connected; where-like precedes paginate(10), withQueryString retains filters. Vue still intentionally local-only; prop/submission/timer lessons pending. No assistant application tests/browser checks, no behaviour pass inferred, no source changes. No completion claimed.
+Next small lesson supplied: watch local search, cancel prior timer, request after 300ms; cancel timer on Enter and component unmount. No automatic-search completion inferred.
+2026-10-29 developer requested ListDepartments action now query/search makes controller more complex. Approved move from earlier direct-query exception back to action pattern; no assistant application edits authorized. Inspected app/Actions/Users/ListUsers.php, UserController index and skander/app/Actions/Players/ListPlayers.php: controller takes validated filters, injected action get returns paginator; action owns filtering/order/pagination and appends validated filters. Next lesson only generate action class; move logic incrementally without copying unrelated user row preparation.
+2026-10-29 developer confirmed ListDepartments get(filters) and controller injection lessons applied. Suggested action uses Builder search closure, alphabetical order, paginate(10)-&gt;appends(validated filters); controller delegates and supplies search prop. These latest changes have not been source-reviewed; do not infer completion. Current cleanup lesson removes temporary You typed paragraph, with action responsibility understanding checkpoint.</t>
         </is>
       </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: build Department list using existing created records, first minimal departments/Index.vue with shared responsive card; then query/controller/props/rendering and authorized route in small connected steps. Manager/Super Admin list policy before exposing records. Rename separately after list; no deletion or speculative Category relationships. Completed-module review and developer-first testing required before Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-027: ListDepartments action extraction lessons developer-confirmed applied; automatic search, clearing and filtered pagination developer-reported passed. Current small step: remove temporary You typed paragraph in departments/Index.vue and understanding checkpoint on action responsibility. Then resume rename edit display/protected GET, form/state/validation/save incrementally. No unsolicited intermediate source review; complete Department module review and developer-first rename checks before completion/Category.</t>
         </is>
       </c>
       <c r="S30" s="10" t="n"/>
@@ -6858,7 +6873,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart ns1:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6870,7 +6885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F183"/>
+  <dimension ref="A1:F184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -12765,6 +12780,38 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>REQ-181</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Department list search</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Current scope</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>2026-10-29 developer approved a search bar above the Department list, matching existing user search: partial department-name matches across all departments before pagination; automatic request after 300ms typing pause, Enter submits immediately, clearing restores list, search retained in pagination links. Preserve Manager/Super Admin viewAny server authorization. Teach before rename within FB-027.</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>FB-027</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Stories!B30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
Category created with authorization
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -723,7 +723,7 @@
       <c r="A12" s="15" t="n"/>
       <c r="B12" t="inlineStr" s="15">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028: first lesson supplied: developer runs php artisan make:model Category -m to generate model and migration only. Await confirmation; then teach category name and department_id storage and required parent connection in small steps. Create/verify before list/rename. Manager/Super Admin viewAny/create/update checks on display/write routes. Repeat Department rename preserving Category links once Category exists. No assistant source-edit permission extends from Department edit to Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028 developer reported done after explicit creation checks; creation save/validation checks developer-reported passed. Assistant authorized CategorySeeder implementation: 3 realistic names for each of10 existing departments, parent categories()-&gt;firstOrCreate avoids duplicates. Read-only DB names confirmed match DepartmentSeeder. Developer runs php artisan db:seed --class=CategorySeeder, then reruns and verifies same examples without duplicates; assistant did not seed. After successful seed continue Category list in small lessons. Full module review, rename and parent rename-link verification still pending.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -753,7 +753,7 @@
       </c>
       <c r="B14" t="inlineStr" s="22">
         <is>
-          <t>Category storage first: developer generates Category model and migration; then name and Department connection.</t>
+          <t>Category creation checks developer-passed; CategorySeeder30 examples ready for developer execution.</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="B15" t="inlineStr" s="22">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028: first lesson supplied: developer runs php artisan make:model Category -m to generate model and migration only. Await confirmation; then teach category name and department_id storage and required parent connection in small steps. Create/verify before list/rename. Manager/Super Admin viewAny/create/update checks on display/write routes. Repeat Department rename preserving Category links once Category exists. No assistant source-edit permission extends from Department edit to Category.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028 developer reported done after explicit creation checks; creation save/validation checks developer-reported passed. Assistant authorized CategorySeeder implementation: 3 realistic names for each of10 existing departments, parent categories()-&gt;firstOrCreate avoids duplicates. Read-only DB names confirmed match DepartmentSeeder. Developer runs php artisan db:seed --class=CategorySeeder, then reruns and verifies same examples without duplicates; assistant did not seed. After successful seed continue Category list in small lessons. Full module review, rename and parent rename-link verification still pending.</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="B16" t="inlineStr" s="22">
         <is>
-          <t>Developer to run php artisan make:model Category -m and confirm generation.</t>
+          <t>Developer runs CategorySeeder and checks rerun avoids duplicates; Category list next.</t>
         </is>
       </c>
     </row>
@@ -787,9 +787,9 @@
           <t>Last reviewed revision</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
-        <is>
-          <t>2026-10-29 FB-027 source review passed; c1c0a96 + working changes, hashes in Stories K30.</t>
+      <c r="B17" t="inlineStr" s="22">
+        <is>
+          <t>2026-10-29 Category creation-only source review passed; working snapshot hashes in Stories Q31. Full module review pending.</t>
         </is>
       </c>
     </row>
@@ -4068,17 +4068,43 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O31" s="11" t="n"/>
+      <c r="O31" t="inlineStr" s="11">
+        <is>
+          <t>
+2026-10-29 Developer-reported: php artisan migrate completed successfully for Category migration. Storage command only; full feature behavior not yet tested.
+2026-10-29 Developer-reported PASS after requested creation display checks: page and department dropdown work; Volunteer direct URL returns403. These verify display only, not saving or full feature.
+2026-10-29 Developer-reported PASS: done after explicit checks for Manager/Super Admin creation, feedback/reset/stored parent, missing fields, duplicate same-department names including case/outer spaces, allowed same name across departments and phone layout. No assistant execution; no precise suite count or malformed-parent/denied POST result inferred.</t>
+        </is>
+      </c>
       <c r="P31" s="31" t="n"/>
       <c r="Q31" t="inlineStr" s="11">
         <is>
           <t>2026-10-29: Read current AGENTS.md, Category story and REQ-098–102/141. Category files absent. First small lesson: developer generates model and migration with php artisan make:model Category -m. Explain model vs storage instructions before adding fields. Upcoming parent connection follows inspected Poker protected fillable and Eloquent relationship conventions; no speculative Subcategory relation. No application edits or checks executed.
-2026-10-29 resumed Category after developer-reported Department layout pass. AGENTS.md reread fully, Category full row and related requirements read. No Category files found; generation step remains pending, no review of a newly applied step. Repeated first generation lesson; no source changes authorized or made.</t>
-        </is>
-      </c>
-      <c r="R31" s="11" t="inlineStr">
-        <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028: first lesson supplied: developer runs php artisan make:model Category -m to generate model and migration only. Await confirmation; then teach category name and department_id storage and required parent connection in small steps. Create/verify before list/rename. Manager/Super Admin viewAny/create/update checks on display/write routes. Repeat Department rename preserving Category links once Category exists. No assistant source-edit permission extends from Department edit to Category.</t>
+2026-10-29 resumed Category after developer-reported Department layout pass. AGENTS.md reread fully, Category full row and related requirements read. No Category files found; generation step remains pending, no review of a newly applied step. Repeated first generation lesson; no source changes authorized or made.
+2026-10-29 explicit intermediate scaffold review requested by developer: read app/Models/Category.php, database/migrations/2026_10_29_210437_create_categories_table.php, app/Http/Controllers/CategoryController.php, app/Http/Requests/StoreCategoryRequest.php, app/Http/Requests/UpdateCategoryRequest.php, app/Policies/CategoryPolicy.php, database/seeders/CategorySeeder.php. All are generated starter files: model empty, migration id/timestamps only, controller and seeder methods empty; requests and policy deny access with no validation rules. Request classes currently in Requests root with matching controller imports; later align with Departments/Users module folders before implementation. Unused generated policy/seeder imports cosmetic only. No feature implementation or behavior verification claimed; no application files modified or tests run. Snapshot: app/Models/Category.php e84cd2296cf7; database/migrations/2026_10_29_210437_create_categories_table.php f1e745a2e1be; app/Http/Controllers/CategoryController.php 90adf470daa5; app/Http/Requests/StoreCategoryRequest.php d3a4707c4324; app/Http/Requests/UpdateCategoryRequest.php e926ff1724ef; app/Policies/CategoryPolicy.php 06652cfa909f; database/seeders/CategorySeeder.php ea7d075e11e1
+2026-10-29 developer explicitly authorized Category request directory refactor. Moved StoreCategoryRequest.php and UpdateCategoryRequest.php into app/Http/Requests/Categories, changed namespaces to App\Http\Requests\Categories and updated CategoryController imports. No validation or authorization behavior changed. Source review and PHP syntax/whitespace checks passed; no application tests run. Earlier scaffold review paths in Requests root are historical; current paths use Categories subfolder.
+2026-10-29 migration lesson: explain name and required department_id together, IDs preserve links during Department rename. Existing Category migration still generated scaffold on lesson-context read. Poker migration examples found: database/migrations/2026_10_24_015321_create_player_game_visits_table.php uses foreignId()-&gt;constrained()-&gt;restrictOnDelete() and multi-column unique; create_payments_table.php uses same restricted foreign-key pattern. Selected same pattern for required Category parent; composite uniqueness taught next before execution. No behavior evidence or completion inferred.
+2026-10-29 developer confirmed migration name and department_id step applied. Supplied next small lesson: unique([department_id,name]) after timestamps. Same name allowed across departments; same department/name pair rejected. Configured MySQL collation handles case; trim via Laravel requests later. Not reviewed or tested; no completion claim.
+2026-10-29 developer confirmed composite uniqueness step applied and requested migration next. Explained developer-run php artisan migrate applies all pending migrations and creates categories table with parent constraint/unique pair. Await actual command result; no migration success inferred from coding-step done, no assistant source inspection or execution.
+2026-10-29 developer reported migration successful. Recorded as developer-reported migration execution pass only, not full Category behavior verification. Category model lesson supplied: protected $fillable with name and department_id; no assistant application edits or tests, no unsolicited inspection. Required Department relationship is next small step.
+2026-10-29 developer confirmed Category fillable applied and requested Department relationship. Focused Poker reference read: app/Models/PlayerGame.php player()/gameSession() use imported BelongsTo, generic @return BelongsTo&lt;Target,$this&gt; and belongsTo(Target::class); adapted same pattern for Category department(). Lesson includes import and one method only. No new Department inverse or Subcategory relationship taught. Developer implementation not inspected; no completion inferred.
+2026-10-29 developer approved keeping standard belongsTo approach after official Laravel13 documentation comparison, and confirmed department relationship added. No intermediate inspection. Next small creation prerequisite: CategoryPolicy create ability for Manager/Super Admin, matching previously inspected DepartmentPolicy role enum checks. Explain authentication vs permission and future GET/POST enforcement; policy alone not yet attached. No new scope or completion inferred.
+2026-10-29 developer asked to add inverse Department hasMany Categories before permissions. Explained independent directions, same department_id column/no migration; supplied HasMany import and categories() with generic return annotation following inspected Poker Player hasMany pattern. Developer confirmed added. Not source-reviewed or behavior-tested. Permission lesson paused; no evidence create ability has been applied. Next supportive understanding checkpoint before resuming.
+2026-10-29 developer correctly explained $department-&gt;categories because Department has many Categories. Understanding checkpoint passed (not runtime behavior evidence). Developer requested resume permissions; repeated small CategoryPolicy create method/import lesson. No permission implementation confirmation yet.
+2026-10-29 developer explicitly requested assistant apply CategoryPolicy create lesson. Added RoleCode import and role comparison only; source review, PHP syntax and whitespace checks passed. No application behavior tests or route enforcement yet. CategoryPolicy sha256 0277f642ef56. Read CategoryController existing scaffold to establish next lesson context; next controller/page code remains developer-written.
+2026-10-29 explicit scoped developer authorization: implemented CategoryController Inertia and Response imports and create method selecting categories/Create. Read existing create scaffold first; PHP syntax and whitespace checks passed. Page and route not yet created by assistant, no behavior completion claimed.
+2026-10-29 explicitly authorized assistant creation of resources/js/pages/categories/Create.vue following Department Create. Read Department Create and User Create shared Select pattern; adapted same card width, border, flex row at sm/stacked mobile, two flexible fields plus input-aligned submit button. Required departments array prop; backend data supply and routes/save still pending, not behavior-tested. Source-reviewed page and formatted. Page sha256 b47f65a7e2b2.
+2026-10-29 developer explicitly authorized controller dropdown data update. Added Department import; create method builds alphabetical id/name collection in intermediate variable and supplies departments Inertia prop matching Category Create.vue contract. Source reviewed; PHP syntax/Pint/whitespace checks requested. No migration or application behavior tests executed. Snapshot CategoryController sha256 c8a547811d71.
+2026-10-29 developer explicitly authorized protected creation display route. Added CategoryController/Category imports and GET categories/create -&gt;name(categories.create)-&gt;can(create,Category::class) inside existing auth group. PHP syntax, targeted Pint and whitespace checks passed. Display permission enforced before controller Department query. No POST route/save implementation. Requested developer display/dropdown/denied-access checks; no assistant execution.
+2026-10-29 developer reported page/dropdown working and Volunteer403 after requested display checks. Explicitly authorized saving route only: added POST categories -&gt;CategoryController store, named categories.store, with create policy inside auth group. Syntax/Pint/whitespace checks passed. Request authorization/validation and controller store remain pending; no assistant source edits beyond route or behavior tests.
+2026-10-29 explicitly authorized StoreCategoryRequest change. Added Category/Rule imports; authorize checks user can(create,Category::class) with guest false fallback. Validation: department_id bail|required|integer|exists departments.id; name bail|required|string|max255|unique scoped department_id. integer accessor gives safe scalar scope even if invalid department input; department rule separately rejects bad IDs. PHP syntax/targeted Pint/whitespace checks passed. No application tests or save claimed. Request sha256 5819301d79ab.
+2026-10-29 developer explicitly authorized store method following Department Create. Added RedirectResponse import/type; Category::create(validated), success toast and back(). PHP syntax/targeted Pint/whitespace pass. Connected CREATION checkpoint source review passed: protected GET/POST policy and request authorization, required existing parent/name scoped unique, fillable and inverse relations, migration FK restrict/composite uniqueness, Vue props/binding/errors/processing/reset and flash response. Minor preexisting blank-line formatting in models/unused generated policy import cosmetic only; not changed. No application tests/browser checks run by assistant. Whole Category module not reviewed or complete (list/rename pending). Working snapshot hashes: app/Http/Controllers/CategoryController.php 43117b4ffd44; app/Http/Requests/Categories/StoreCategoryRequest.php 5819301d79ab; app/Policies/CategoryPolicy.php 0277f642ef56; app/Models/Category.php c6b71ccfa049; app/Models/Department.php 02f8798b6af4; database/migrations/2026_10_29_210437_create_categories_table.php 50ae1cd2d815; routes/web.php 4977eeab000c; resources/js/pages/categories/Create.vue b47f65a7e2b2
+2026-10-29 developer replied done after explicit Category creation checks, then requested three real-life categories under each department using seeder. Implemented CategorySeeder map (30 examples), finds existing Department by name and uses categories()-&gt;firstOrCreate(name), preserving existing categories. Read-only tinker pluck confirmed10 exact DepartmentSeeder names; no database writes by assistant. PHP syntax/Pint/whitespace passed. Seeder execution delegated to developer; rerun/idempotence not yet verified. No extra category scope approved by example records.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr" s="11">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028 developer reported done after explicit creation checks; creation save/validation checks developer-reported passed. Assistant authorized CategorySeeder implementation: 3 realistic names for each of10 existing departments, parent categories()-&gt;firstOrCreate avoids duplicates. Read-only DB names confirmed match DepartmentSeeder. Developer runs php artisan db:seed --class=CategorySeeder, then reruns and verifies same examples without duplicates; assistant did not seed. After successful seed continue Category list in small lessons. Full module review, rename and parent rename-link verification still pending.</t>
         </is>
       </c>
       <c r="S31" s="11" t="n"/>

</xml_diff>

<commit_message>
Add subcategory creation with dependent department and category dropdowns
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -723,7 +723,7 @@
       <c r="A12" s="15" t="n"/>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-028 Category verified. Next ready item FB-029: introduce Subcategory storage and required Category relationship, then creation in small developer-written lessons; read its full story/requirements before teaching. Do not infer permission to implement next module from prior Category authorization.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-029 creation-only implementation reviewed and assistant-tested under explicit delegation; Department/dependent Category/name only. List remains pending, then FB-030 rename/full-module review. Do not mark row complete or implement list/search/edit without current scope authorization. Catalogue only; postpone stock design and size-dependent code decisions.</t>
         </is>
       </c>
       <c r="C12" s="15" t="n"/>
@@ -753,7 +753,7 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>Category module verified; Subcategory first lesson not yet supplied.</t>
+          <t>Subcategory creation verified with Department/Category dropdowns; list not implemented.</t>
         </is>
       </c>
     </row>
@@ -765,8 +765,7 @@
       </c>
       <c r="B15" s="22" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Build required storage/relationship and complete creation with review and developer-first checks; then display the subcategory list.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-029 creation-only implementation reviewed and assistant-tested under explicit delegation; Department/dependent Category/name only. List remains pending, then FB-030 rename/full-module review. Do not mark row complete or implement list/search/edit without current scope authorization. Catalogue only; postpone stock design and size-dependent code decisions.</t>
         </is>
       </c>
     </row>
@@ -778,7 +777,7 @@
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>Next lesson on developer request; no Subcategory implementation authorized.</t>
+          <t>Developer can try creation; list is next on request.</t>
         </is>
       </c>
     </row>
@@ -790,7 +789,7 @@
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>2026-10-29 revised Category department-change source review/tests passed; snapshots/evidence in Stories K31/O31.</t>
+          <t>2026-10-29 creation-only source review passed; snapshot in Stories K32. Full Subcategory module review pending.</t>
         </is>
       </c>
     </row>
@@ -802,7 +801,7 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -952,7 +951,9 @@
           <t>2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Order: FB-016/017/018, prepare FB-020, FB-019, FB-006/007, FB-024, FB-009–015, FB-008, remaining accounts. Catalogue modules create before list; Product already does. Super Admin recovery stays last.
 2026-10-27 sequence decision: place the bcrypt 72-byte repair and repeat test within FB-069, immediately before final FB-070. Existing first-login review/test failures remain recorded; this timing change does not verify them.
 2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
-2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</t>
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.
+2026-10-29 approved Product Catalogue/Stock Management separation recorded in revised Requirements. Catalogue excludes all size/unit/quantity/history data, including Subcategory summary units; deactivation server-checks Stock Management and blocks while ANY stock remains without displaying counts. Stable FB-034 repurposed/moved after catalogue checkpoint FB-067 and before FB-049 Receive; Product code FB-035 now depends on FB-033. Stock package-record structure/summary owner/classification locks remain open before stock implementation. Subcategory creation revert preserved; no code changes in design discussion.
+2026-10-29 planning approval: reusable package_sizes in Stock Management; stock_items connects product_id/package_size_id and owns separate movement/balance identity. See shared-package Requirement/FB-034. Current Subcategory still Category+name only and unstarted after revert. No application code/migrations or feature tests run for this planning change.</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3358,7 @@
     </row>
     <row r="24" ht="105" customHeight="1">
       <c r="A24" s="4" t="n">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -3429,7 +3430,7 @@
     </row>
     <row r="25" ht="105" customHeight="1">
       <c r="A25" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
@@ -3567,7 +3568,7 @@
     </row>
     <row r="26" ht="105" customHeight="1">
       <c r="A26" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -3663,7 +3664,7 @@
     </row>
     <row r="27" ht="105" customHeight="1">
       <c r="A27" s="9" t="n">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
@@ -3736,7 +3737,7 @@
     </row>
     <row r="28" ht="105" customHeight="1">
       <c r="A28" s="4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -3827,7 +3828,7 @@
     </row>
     <row r="29" ht="105" customHeight="1">
       <c r="A29" s="9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
@@ -3913,7 +3914,7 @@
     </row>
     <row r="30" ht="105" customHeight="1">
       <c r="A30" s="4" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
@@ -4016,7 +4017,7 @@
     </row>
     <row r="31" ht="105" customHeight="1">
       <c r="A31" s="9" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
@@ -4131,7 +4132,7 @@
     </row>
     <row r="32" ht="105" customHeight="1">
       <c r="A32" s="4" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
@@ -4150,7 +4151,7 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>After Category is verified, introduce Subcategory model/storage and Category relationship. Teach parent selection, summary-unit selection and authorized creation separately. Required names unique within category ignoring case/outer spaces. Summary units kg, litres or individual items; no skipped levels. Review and developer-test creation before displaying the list. Managers/Super Admin only on display/write. No speculative Product relationship.</t>
+          <t>Subcategory creation has Department and dependent Category dropdowns plus required name. Only selected Department categories appear; changing Department clears Category. Server validates matching parent selection; save category_id/name only. Names unique within Category ignoring case/outer spaces. Managers/Super Admin only. No sizes/units/quantities. Complete/verify creation before list; no speculative Product relationship.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -4168,7 +4169,7 @@
       </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
@@ -4176,7 +4177,11 @@
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K32" s="10" t="n"/>
+      <c r="K32" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29 explicit user authorization: implement Subcategory creation with Department/dependent Category/name and run all necessary tests. Creation-only source review PASS for app/Models/Subcategory.php, app/Models/Category.php, app/Http/Controllers/SubcategoryController.php, app/Http/Requests/Subcategories/StoreSubcategoryRequest.php, app/Policies/SubcategoryPolicy.php, database/migrations/2026_10_29_214439_create_subcategories_table.php, resources/js/pages/subcategories/Create.vue, routes/web.php, tests/Feature/SubcategoryCreateTest.php. Implemented Category hasMany Subcategory / Subcategory belongsTo Category; fillable only category_id/name. Migration FK restrict/composite category-name uniqueness, no department duplicate/stock fields. Controller alphabetical minimal dropdown data; Vue computed filters Categories by department, watch clears selected Category on department change; category disabled until usable choices, no-category placeholder; keyed Select clears display; Inertia useForm success reset/errors/processing. Server create policy at auth GET+POST and request recheck for Manager/Super Admin; validates existing Department and Category scoped to Department, required name max255 unique within category. Store safe only category_id/name; flash/back follows current Category/Poker pattern. Read all relevant files together; no blocking findings. Snapshot: app/Models/Subcategory.php 77fcceb49da0; app/Models/Category.php cd7247b2dfd2; app/Http/Controllers/SubcategoryController.php 6a2c07b38475; app/Http/Requests/Subcategories/StoreSubcategoryRequest.php f0e9809b77cd; app/Policies/SubcategoryPolicy.php b15f69c79371; database/migrations/2026_10_29_214439_create_subcategories_table.php 8ed44d2b7e96; resources/js/pages/subcategories/Create.vue 6dfc2aa48f55; routes/web.php 38c6bea83c4e; tests/Feature/SubcategoryCreateTest.php 6dcf08a984f1</t>
+        </is>
+      </c>
       <c r="L32" s="30" t="n"/>
       <c r="M32" s="10" t="n"/>
       <c r="N32" s="10" t="inlineStr">
@@ -4184,20 +4189,31 @@
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O32" s="10" t="n"/>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+2026-10-29 delegated tests: initial targeted suite failed7 page requests due stale Vite manifest (Subcategory and existing edit pages absent); npm run build PASS regenerated assets. Rerun php artisan test tests/Feature/SubcategoryCreateTest.php tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php PASS53 tests324 assertions (SQLite in-memory), covering both permitted roles, invalid fields, required name/parents, scoped duplicates, mismatched parent pair, stale Category moved after form load, guest redirects, Volunteer403 GET/POST, ignored stock/forged fields, relationship retention across Category rename/move; no full unrelated account suite run. npm run types:check PASS, targeted Pint/Vue formatter PASS, syntax and diff whitespace PASS. Applied only Subcategory migration successfully to local MySQL. Browser existing Super Admin /subcategories/create PASS: Category initially disabled; blank errors for all3 fields; Baby Care shows Baby Wipes/Diapers/Infant Formula only; selected Baby Wipes then switching to Bakery clears category; Bakery shows Bread/Pastries/Rolls and Buns. Created temporary QA Dropdown Creation 20261029 under Bakery/Bread, success toast and Department/Category/name reset with Category disabled. Database row relationship verified; MySQL case-insensitive duplicate validator PASS. Removed only that self-created fixture. Wide and390px screenshots passed; phone stacked controls/full-width button. DevTools/device preview restored/closed. No sizes/units/quantities anywhere in creation UI/model/table. List/edit not implemented or verified.</t>
+        </is>
+      </c>
       <c r="P32" s="30" t="n"/>
-      <c r="Q32" s="10" t="n"/>
+      <c r="Q32" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29 Subcategory creation implementation and applied migration were reverted at user request; original scaffolds restored and migration Pending. Approved redesign now removes summary-unit field from catalogue. No new application implementation authorized by this planning discussion. Earlier implementation tests do not verify the revised design.
+2026-10-29 planning approval: reusable package_sizes in Stock Management; stock_items connects product_id/package_size_id and owns separate movement/balance identity. See shared-package Requirement/FB-034. Current Subcategory still Category+name only and unstarted after revert. No application code/migrations or feature tests run for this planning change.
+2026-10-29 approved Subcategory creation UI: Department dropdown, Category dropdown and required Subcategory name only. Category choices belong to selected Department; changing Department clears Category. Server validates existing Department/Category and their matching relationship. Persist Category link (category_id); Department is derived through Category rather than duplicated on Subcategory. No units, sizes, package or quantity fields. Inventory/catalogue completion remains the focus; stock design and size-specific code discussion are deferred, not new approved implementation. Original Subcategory scaffold/migration remain reverted/unstarted.
+2026-10-29 explicit user authorization: implement Subcategory creation with Department/dependent Category/name and run all necessary tests. Creation-only source review PASS for app/Models/Subcategory.php, app/Models/Category.php, app/Http/Controllers/SubcategoryController.php, app/Http/Requests/Subcategories/StoreSubcategoryRequest.php, app/Policies/SubcategoryPolicy.php, database/migrations/2026_10_29_214439_create_subcategories_table.php, resources/js/pages/subcategories/Create.vue, routes/web.php, tests/Feature/SubcategoryCreateTest.php. Implemented Category hasMany Subcategory / Subcategory belongsTo Category; fillable only category_id/name. Migration FK restrict/composite category-name uniqueness, no department duplicate/stock fields. Controller alphabetical minimal dropdown data; Vue computed filters Categories by department, watch clears selected Category on department change; category disabled until usable choices, no-category placeholder; keyed Select clears display; Inertia useForm success reset/errors/processing. Server create policy at auth GET+POST and request recheck for Manager/Super Admin; validates existing Department and Category scoped to Department, required name max255 unique within category. Store safe only category_id/name; flash/back follows current Category/Poker pattern. Read all relevant files together; no blocking findings. Snapshot: app/Models/Subcategory.php 77fcceb49da0; app/Models/Category.php cd7247b2dfd2; app/Http/Controllers/SubcategoryController.php 6a2c07b38475; app/Http/Requests/Subcategories/StoreSubcategoryRequest.php f0e9809b77cd; app/Policies/SubcategoryPolicy.php b15f69c79371; database/migrations/2026_10_29_214439_create_subcategories_table.php 8ed44d2b7e96; resources/js/pages/subcategories/Create.vue 6dfc2aa48f55; routes/web.php 38c6bea83c4e; tests/Feature/SubcategoryCreateTest.php 6dcf08a984f1</t>
+        </is>
+      </c>
       <c r="R32" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Build required storage/relationship and complete creation with review and developer-first checks; then display the subcategory list.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-029 creation-only implementation reviewed and assistant-tested under explicit delegation; Department/dependent Category/name only. List remains pending, then FB-030 rename/full-module review. Do not mark row complete or implement list/search/edit without current scope authorization. Catalogue only; postpone stock design and size-dependent code decisions.</t>
         </is>
       </c>
       <c r="S32" s="10" t="n"/>
     </row>
     <row r="33" ht="105" customHeight="1">
       <c r="A33" s="9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
@@ -4216,7 +4232,7 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>Preserve links on renaming; existing paths show current names, even for past movements. No parent moves/deletion. Managers/Super Admin only; unit lock after movements is verified in later stock items. Complete list/create/rename review and developer-first checks before Product. Verify Category rename preserves the Subcategory link. Summary-unit editing before movements is checked now; the post-movement lock is explicitly deferred to FB-053.</t>
+          <t>Rename preserves links/current names; no moves/deletion. Managers/Super Admin. Verify list/create/rename and Category rename preserving Subcategory links. No summary-unit editing in catalogue.</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -4255,15 +4271,14 @@
       <c r="Q33" s="11" t="n"/>
       <c r="R33" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Teach rename separately, preserve the parent, and verify all existing Subcategory actions and permissions. Check editable summary units before stock movements. Record FB-053 as the later lock checkpoint; do not mark that later rule verified now.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
         </is>
       </c>
       <c r="S33" s="11" t="n"/>
     </row>
     <row r="34" ht="105" customHeight="1">
       <c r="A34" s="4" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
@@ -4330,7 +4345,7 @@
     </row>
     <row r="35" ht="105" customHeight="1">
       <c r="A35" s="9" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
@@ -4349,7 +4364,7 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>After Department, Category and Subcategory actions are verified, introduce Product model/storage and its required Subcategory relationship. Then display the form: required name, department/category/subcategory selection, counting unit, positive contents/unit and status; optional brand/tags, default Active and no balance input. Teach each dependent selection separately. Optional tag persistence/relationship is introduced at FB-037. Post-movement locks remain FB-053.</t>
+          <t>Product belongs to Subcategory. Required name/hierarchy/status; optional brand/tags; automatic code. No sizes, packaging, counting/contents units, balances or quantity fields. Introduce tag persistence at FB-037.</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
@@ -4388,15 +4403,14 @@
       <c r="Q35" s="11" t="n"/>
       <c r="R35" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Explain one Product belonging to one completed Subcategory. Start with only required Product storage and that relationship. Then display the plain form and teach the hierarchy selections one at a time; layout/state follow in FB-033. Do not create stock-movement relationships yet.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
         </is>
       </c>
       <c r="S35" s="11" t="n"/>
     </row>
     <row r="36" ht="105" customHeight="1">
       <c r="A36" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
@@ -4415,7 +4429,7 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Explain parent grid/flex, spacing, width and phone-to-desktop arrangement. Introduce local form state gradually; package preview reflects entered values before saving.</t>
+          <t>Teach responsive layout and temporary state for catalogue identity fields only. No package preview or stock values.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -4454,1071 +4468,1066 @@
       <c r="Q36" s="10" t="n"/>
       <c r="R36" s="10" t="inlineStr">
         <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S36" s="10" t="n"/>
+    </row>
+    <row r="37" ht="105" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>FB-035</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Generate permanent product codes</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Unique automatic PRD-000001 onward, at least six digits and growth beyond999999, never edited/reused or derived from categories. Codes identify catalogue products independently of package sizes.</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>FB-033</t>
+        </is>
+      </c>
+      <c r="G37" s="4">
+        <f>IF(H37="Complete","Complete",IF(I37="Blocked","Blocked",IF(I37="In progress","Ready",IF(F37="","Ready",IF(COUNTIFS($B$4:$B$73,F37,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H37" s="4">
+        <f>IF(I37="Not started","Not started",IF(I37="Blocked","Blocked",IF(I37="In progress","In progress",IF(J37&lt;&gt;"Passed","Awaiting code review",IF(OR(K37="",NOT(ISNUMBER(L37))),"Awaiting review evidence",IF(N37&lt;&gt;"Passed","Awaiting test",IF(OR(M37="",O37="",NOT(ISNUMBER(P37))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J37" s="10" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K37" s="10" t="n"/>
+      <c r="L37" s="30" t="n"/>
+      <c r="M37" s="10" t="n"/>
+      <c r="N37" s="10" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O37" s="10" t="n"/>
+      <c r="P37" s="30" t="n"/>
+      <c r="Q37" s="10" t="n"/>
+      <c r="R37" s="10" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S37" s="10" t="n"/>
+    </row>
+    <row r="38" ht="105" customHeight="1">
+      <c r="A38" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>FB-036</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Prevent duplicate catalogue products</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Compare name/brand/Subcategory, ignore case/outer spaces and include inactive products. No package contents, counting unit or size in catalogue duplicate identity.</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>FB-035</t>
+        </is>
+      </c>
+      <c r="G38" s="9">
+        <f>IF(H38="Complete","Complete",IF(I38="Blocked","Blocked",IF(I38="In progress","Ready",IF(F38="","Ready",IF(COUNTIFS($B$4:$B$73,F38,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H38" s="9">
+        <f>IF(I38="Not started","Not started",IF(I38="Blocked","Blocked",IF(I38="In progress","In progress",IF(J38&lt;&gt;"Passed","Awaiting code review",IF(OR(K38="",NOT(ISNUMBER(L38))),"Awaiting review evidence",IF(N38&lt;&gt;"Passed","Awaiting test",IF(OR(M38="",O38="",NOT(ISNUMBER(P38))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K38" s="11" t="n"/>
+      <c r="L38" s="31" t="n"/>
+      <c r="M38" s="11" t="n"/>
+      <c r="N38" s="11" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O38" s="11" t="n"/>
+      <c r="P38" s="31" t="n"/>
+      <c r="Q38" s="11" t="n"/>
+      <c r="R38" s="11" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S38" s="11" t="n"/>
+    </row>
+    <row r="39" ht="105" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>FB-037</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Save products and attach optional tags</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Managers/Super Admin create; Volunteers denied display/write. Save catalogue identity/classification/status only; no stock quantity/packaging. Optional shared tags; errors/retained input/processing and persisted fields.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>FB-036</t>
+        </is>
+      </c>
+      <c r="G39" s="4">
+        <f>IF(H39="Complete","Complete",IF(I39="Blocked","Blocked",IF(I39="In progress","Ready",IF(F39="","Ready",IF(COUNTIFS($B$4:$B$73,F39,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H39" s="4">
+        <f>IF(I39="Not started","Not started",IF(I39="Blocked","Blocked",IF(I39="In progress","In progress",IF(J39&lt;&gt;"Passed","Awaiting code review",IF(OR(K39="",NOT(ISNUMBER(L39))),"Awaiting review evidence",IF(N39&lt;&gt;"Passed","Awaiting test",IF(OR(M39="",O39="",NOT(ISNUMBER(P39))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J39" s="10" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K39" s="10" t="n"/>
+      <c r="L39" s="30" t="n"/>
+      <c r="M39" s="10" t="n"/>
+      <c r="N39" s="10" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O39" s="10" t="n"/>
+      <c r="P39" s="30" t="n"/>
+      <c r="Q39" s="10" t="n"/>
+      <c r="R39" s="10" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S39" s="10" t="n"/>
+    </row>
+    <row r="40" ht="105" customHeight="1">
+      <c r="A40" s="9" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>FB-038</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Display the unfiltered catalogue product list</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>All roles see product code/name/category path/brand/status. No size, measurement units, available quantity or totals. Verify server permissions.</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>FB-037</t>
+        </is>
+      </c>
+      <c r="G40" s="9">
+        <f>IF(H40="Complete","Complete",IF(I40="Blocked","Blocked",IF(I40="In progress","Ready",IF(F40="","Ready",IF(COUNTIFS($B$4:$B$73,F40,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H40" s="9">
+        <f>IF(I40="Not started","Not started",IF(I40="Blocked","Blocked",IF(I40="In progress","In progress",IF(J40&lt;&gt;"Passed","Awaiting code review",IF(OR(K40="",NOT(ISNUMBER(L40))),"Awaiting review evidence",IF(N40&lt;&gt;"Passed","Awaiting test",IF(OR(M40="",O40="",NOT(ISNUMBER(P40))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="n"/>
+      <c r="L40" s="31" t="n"/>
+      <c r="M40" s="11" t="n"/>
+      <c r="N40" s="11" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O40" s="11" t="n"/>
+      <c r="P40" s="31" t="n"/>
+      <c r="Q40" s="11" t="n"/>
+      <c r="R40" s="11" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S40" s="11" t="n"/>
+    </row>
+    <row r="41" ht="105" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>FB-039</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Arrange catalogue rows and filter toolbar</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Teach responsive widths, wrapping/table overflow/stacked toolbar for product identity/classification. No stock/size columns.</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>FB-038</t>
+        </is>
+      </c>
+      <c r="G41" s="4">
+        <f>IF(H41="Complete","Complete",IF(I41="Blocked","Blocked",IF(I41="In progress","Ready",IF(F41="","Ready",IF(COUNTIFS($B$4:$B$73,F41,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H41" s="4">
+        <f>IF(I41="Not started","Not started",IF(I41="Blocked","Blocked",IF(I41="In progress","In progress",IF(J41&lt;&gt;"Passed","Awaiting code review",IF(OR(K41="",NOT(ISNUMBER(L41))),"Awaiting review evidence",IF(N41&lt;&gt;"Passed","Awaiting test",IF(OR(M41="",O41="",NOT(ISNUMBER(P41))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I41" s="10" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J41" s="10" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K41" s="10" t="n"/>
+      <c r="L41" s="30" t="n"/>
+      <c r="M41" s="10" t="n"/>
+      <c r="N41" s="10" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O41" s="10" t="n"/>
+      <c r="P41" s="30" t="n"/>
+      <c r="Q41" s="10" t="n"/>
+      <c r="R41" s="10" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S41" s="10" t="n"/>
+    </row>
+    <row r="42" ht="105" customHeight="1">
+      <c r="A42" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>FB-040</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Products</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Add search by product code or name</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Search the full catalogue before pagination. Verify both code and name, clear search and no results.</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>FB-039</t>
+        </is>
+      </c>
+      <c r="G42" s="9">
+        <f>IF(H42="Complete","Complete",IF(I42="Blocked","Blocked",IF(I42="In progress","Ready",IF(F42="","Ready",IF(COUNTIFS($B$4:$B$73,F42,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>IF(I42="Not started","Not started",IF(I42="Blocked","Blocked",IF(I42="In progress","In progress",IF(J42&lt;&gt;"Passed","Awaiting code review",IF(OR(K42="",NOT(ISNUMBER(L42))),"Awaiting review evidence",IF(N42&lt;&gt;"Passed","Awaiting test",IF(OR(M42="",O42="",NOT(ISNUMBER(P42))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>Not reviewed</t>
+        </is>
+      </c>
+      <c r="K42" s="11" t="n"/>
+      <c r="L42" s="31" t="n"/>
+      <c r="M42" s="11" t="n"/>
+      <c r="N42" s="11" t="inlineStr">
+        <is>
+          <t>Not tested</t>
+        </is>
+      </c>
+      <c r="O42" s="11" t="n"/>
+      <c r="P42" s="31" t="n"/>
+      <c r="Q42" s="11" t="n"/>
+      <c r="R42" s="11" t="inlineStr">
+        <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S36" s="10" t="n"/>
-    </row>
-    <row r="37" ht="105" customHeight="1">
-      <c r="A37" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>FB-034</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="S42" s="11" t="n"/>
+    </row>
+    <row r="43" ht="105" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>FB-041</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Choose package units and validate contents</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>Counting units: bag, box, can, bottle, carton, jar, packet, individual item. Choose kg/g or litres/ml matching subcategory measure. Positive contents allow up to 3 decimals with fewer allowed; item counts are positive integers.</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>FB-033</t>
-        </is>
-      </c>
-      <c r="G37" s="9">
-        <f>IF(H37="Complete","Complete",IF(I37="Blocked","Blocked",IF(I37="In progress","Ready",IF(F37="","Ready",IF(COUNTIFS($B$4:$B$73,F37,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H37" s="9">
-        <f>IF(I37="Not started","Not started",IF(I37="Blocked","Blocked",IF(I37="In progress","In progress",IF(J37&lt;&gt;"Passed","Awaiting code review",IF(OR(K37="",NOT(ISNUMBER(L37))),"Awaiting review evidence",IF(N37&lt;&gt;"Passed","Awaiting test",IF(OR(M37="",O37="",NOT(ISNUMBER(P37))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I37" s="11" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Add the department filter</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Filter by department alone and with search. Explain selected state and request values; do not introduce remaining filters yet.</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>FB-040</t>
+        </is>
+      </c>
+      <c r="G43" s="4">
+        <f>IF(H43="Complete","Complete",IF(I43="Blocked","Blocked",IF(I43="In progress","Ready",IF(F43="","Ready",IF(COUNTIFS($B$4:$B$73,F43,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H43" s="4">
+        <f>IF(I43="Not started","Not started",IF(I43="Blocked","Blocked",IF(I43="In progress","In progress",IF(J43&lt;&gt;"Passed","Awaiting code review",IF(OR(K43="",NOT(ISNUMBER(L43))),"Awaiting review evidence",IF(N43&lt;&gt;"Passed","Awaiting test",IF(OR(M43="",O43="",NOT(ISNUMBER(P43))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I43" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J37" s="11" t="inlineStr">
+      <c r="J43" s="10" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K37" s="11" t="n"/>
-      <c r="L37" s="31" t="n"/>
-      <c r="M37" s="11" t="n"/>
-      <c r="N37" s="11" t="inlineStr">
+      <c r="K43" s="10" t="n"/>
+      <c r="L43" s="30" t="n"/>
+      <c r="M43" s="10" t="n"/>
+      <c r="N43" s="10" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O37" s="11" t="n"/>
-      <c r="P37" s="31" t="n"/>
-      <c r="Q37" s="11" t="n"/>
-      <c r="R37" s="11" t="inlineStr">
+      <c r="O43" s="10" t="n"/>
+      <c r="P43" s="30" t="n"/>
+      <c r="Q43" s="10" t="n"/>
+      <c r="R43" s="10" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S37" s="11" t="n"/>
-    </row>
-    <row r="38" ht="105" customHeight="1">
-      <c r="A38" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>FB-035</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="S43" s="10" t="n"/>
+    </row>
+    <row r="44" ht="105" customHeight="1">
+      <c r="A44" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>FB-042</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Generate permanent product codes</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>Automatically assign unique PRD-000001 onward, at least six digits with growth beyond 999999. Never edit/reuse codes or derive from categories. Each brand/size is a separate product; review collision handling.</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>FB-034</t>
-        </is>
-      </c>
-      <c r="G38" s="4">
-        <f>IF(H38="Complete","Complete",IF(I38="Blocked","Blocked",IF(I38="In progress","Ready",IF(F38="","Ready",IF(COUNTIFS($B$4:$B$73,F38,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H38" s="4">
-        <f>IF(I38="Not started","Not started",IF(I38="Blocked","Blocked",IF(I38="In progress","In progress",IF(J38&lt;&gt;"Passed","Awaiting code review",IF(OR(K38="",NOT(ISNUMBER(L38))),"Awaiting review evidence",IF(N38&lt;&gt;"Passed","Awaiting test",IF(OR(M38="",O38="",NOT(ISNUMBER(P38))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I38" s="10" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Add the category filter</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Filter by category and combine with department/search; changing parent must not leave incompatible selections.</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>FB-041</t>
+        </is>
+      </c>
+      <c r="G44" s="9">
+        <f>IF(H44="Complete","Complete",IF(I44="Blocked","Blocked",IF(I44="In progress","Ready",IF(F44="","Ready",IF(COUNTIFS($B$4:$B$73,F44,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H44" s="9">
+        <f>IF(I44="Not started","Not started",IF(I44="Blocked","Blocked",IF(I44="In progress","In progress",IF(J44&lt;&gt;"Passed","Awaiting code review",IF(OR(K44="",NOT(ISNUMBER(L44))),"Awaiting review evidence",IF(N44&lt;&gt;"Passed","Awaiting test",IF(OR(M44="",O44="",NOT(ISNUMBER(P44))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J38" s="10" t="inlineStr">
+      <c r="J44" s="11" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K38" s="10" t="n"/>
-      <c r="L38" s="30" t="n"/>
-      <c r="M38" s="10" t="n"/>
-      <c r="N38" s="10" t="inlineStr">
+      <c r="K44" s="11" t="n"/>
+      <c r="L44" s="31" t="n"/>
+      <c r="M44" s="11" t="n"/>
+      <c r="N44" s="11" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O38" s="10" t="n"/>
-      <c r="P38" s="30" t="n"/>
-      <c r="Q38" s="10" t="n"/>
-      <c r="R38" s="10" t="inlineStr">
+      <c r="O44" s="11" t="n"/>
+      <c r="P44" s="31" t="n"/>
+      <c r="Q44" s="11" t="n"/>
+      <c r="R44" s="11" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S38" s="10" t="n"/>
-    </row>
-    <row r="39" ht="105" customHeight="1">
-      <c r="A39" s="9" t="n">
-        <v>34</v>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>FB-036</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="S44" s="11" t="n"/>
+    </row>
+    <row r="45" ht="105" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>FB-043</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>Prevent duplicate products</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>Match name, brand, subcategory, counting unit and equivalent contents. Ignore case/outer spaces; 500g=0.5kg and 500ml=0.5litres. Include inactive products; retain name/brand distinctions and reject duplicates.</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>FB-035</t>
-        </is>
-      </c>
-      <c r="G39" s="9">
-        <f>IF(H39="Complete","Complete",IF(I39="Blocked","Blocked",IF(I39="In progress","Ready",IF(F39="","Ready",IF(COUNTIFS($B$4:$B$73,F39,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H39" s="9">
-        <f>IF(I39="Not started","Not started",IF(I39="Blocked","Blocked",IF(I39="In progress","In progress",IF(J39&lt;&gt;"Passed","Awaiting code review",IF(OR(K39="",NOT(ISNUMBER(L39))),"Awaiting review evidence",IF(N39&lt;&gt;"Passed","Awaiting test",IF(OR(M39="",O39="",NOT(ISNUMBER(P39))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I39" s="11" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Add the subcategory filter</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Filter by subcategory alongside existing selections; verify full path and no skipped/contradictory parent selection.</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>FB-042</t>
+        </is>
+      </c>
+      <c r="G45" s="4">
+        <f>IF(H45="Complete","Complete",IF(I45="Blocked","Blocked",IF(I45="In progress","Ready",IF(F45="","Ready",IF(COUNTIFS($B$4:$B$73,F45,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H45" s="4">
+        <f>IF(I45="Not started","Not started",IF(I45="Blocked","Blocked",IF(I45="In progress","In progress",IF(J45&lt;&gt;"Passed","Awaiting code review",IF(OR(K45="",NOT(ISNUMBER(L45))),"Awaiting review evidence",IF(N45&lt;&gt;"Passed","Awaiting test",IF(OR(M45="",O45="",NOT(ISNUMBER(P45))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I45" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J39" s="11" t="inlineStr">
+      <c r="J45" s="10" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K39" s="11" t="n"/>
-      <c r="L39" s="31" t="n"/>
-      <c r="M39" s="11" t="n"/>
-      <c r="N39" s="11" t="inlineStr">
+      <c r="K45" s="10" t="n"/>
+      <c r="L45" s="30" t="n"/>
+      <c r="M45" s="10" t="n"/>
+      <c r="N45" s="10" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O39" s="11" t="n"/>
-      <c r="P39" s="31" t="n"/>
-      <c r="Q39" s="11" t="n"/>
-      <c r="R39" s="11" t="inlineStr">
+      <c r="O45" s="10" t="n"/>
+      <c r="P45" s="30" t="n"/>
+      <c r="Q45" s="10" t="n"/>
+      <c r="R45" s="10" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S39" s="11" t="n"/>
-    </row>
-    <row r="40" ht="105" customHeight="1">
-      <c r="A40" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>FB-037</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="S45" s="10" t="n"/>
+    </row>
+    <row r="46" ht="105" customHeight="1">
+      <c r="A46" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>FB-044</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Save products and attach optional tags</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Managers/Super Admin can create; volunteers denied display/write. New stock is zero. Shared tags can be none/multiple. Validate errors, retained input, processing state and successful persisted record.</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>FB-036</t>
-        </is>
-      </c>
-      <c r="G40" s="4">
-        <f>IF(H40="Complete","Complete",IF(I40="Blocked","Blocked",IF(I40="In progress","Ready",IF(F40="","Ready",IF(COUNTIFS($B$4:$B$73,F40,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H40" s="4">
-        <f>IF(I40="Not started","Not started",IF(I40="Blocked","Blocked",IF(I40="In progress","In progress",IF(J40&lt;&gt;"Passed","Awaiting code review",IF(OR(K40="",NOT(ISNUMBER(L40))),"Awaiting review evidence",IF(N40&lt;&gt;"Passed","Awaiting test",IF(OR(M40="",O40="",NOT(ISNUMBER(P40))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I40" s="10" t="inlineStr">
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Add the tag filter</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Show products with the selected shared tag; combine with prior filters and search. Untagged products remain visible when tag filter is cleared.</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>FB-043</t>
+        </is>
+      </c>
+      <c r="G46" s="9">
+        <f>IF(H46="Complete","Complete",IF(I46="Blocked","Blocked",IF(I46="In progress","Ready",IF(F46="","Ready",IF(COUNTIFS($B$4:$B$73,F46,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H46" s="9">
+        <f>IF(I46="Not started","Not started",IF(I46="Blocked","Blocked",IF(I46="In progress","In progress",IF(J46&lt;&gt;"Passed","Awaiting code review",IF(OR(K46="",NOT(ISNUMBER(L46))),"Awaiting review evidence",IF(N46&lt;&gt;"Passed","Awaiting test",IF(OR(M46="",O46="",NOT(ISNUMBER(P46))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J40" s="10" t="inlineStr">
+      <c r="J46" s="11" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K40" s="10" t="n"/>
-      <c r="L40" s="30" t="n"/>
-      <c r="M40" s="10" t="n"/>
-      <c r="N40" s="10" t="inlineStr">
+      <c r="K46" s="11" t="n"/>
+      <c r="L46" s="31" t="n"/>
+      <c r="M46" s="11" t="n"/>
+      <c r="N46" s="11" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O40" s="10" t="n"/>
-      <c r="P40" s="30" t="n"/>
-      <c r="Q40" s="10" t="n"/>
-      <c r="R40" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Introduce the Product–Tag relationship through saving an optional tag selection. Enforce create policy on form and submission before enabling saving. Connect one save, then field errors, retained input and processing feedback separately. Verify the complete create action before list filters.</t>
-        </is>
-      </c>
-      <c r="S40" s="10" t="n"/>
-    </row>
-    <row r="41" ht="105" customHeight="1">
-      <c r="A41" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>FB-038</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Display the unfiltered product list</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="inlineStr">
-        <is>
-          <t>All roles see code, name, category path, package contents in saved units, available stock and status. Use visible baseline before filters; verify list access server-side.</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>FB-037</t>
-        </is>
-      </c>
-      <c r="G41" s="9">
-        <f>IF(H41="Complete","Complete",IF(I41="Blocked","Blocked",IF(I41="In progress","Ready",IF(F41="","Ready",IF(COUNTIFS($B$4:$B$73,F41,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H41" s="9">
-        <f>IF(I41="Not started","Not started",IF(I41="Blocked","Blocked",IF(I41="In progress","In progress",IF(J41&lt;&gt;"Passed","Awaiting code review",IF(OR(K41="",NOT(ISNUMBER(L41))),"Awaiting review evidence",IF(N41&lt;&gt;"Passed","Awaiting test",IF(OR(M41="",O41="",NOT(ISNUMBER(P41))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I41" s="11" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J41" s="11" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K41" s="11" t="n"/>
-      <c r="L41" s="31" t="n"/>
-      <c r="M41" s="11" t="n"/>
-      <c r="N41" s="11" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O41" s="11" t="n"/>
-      <c r="P41" s="31" t="n"/>
-      <c r="Q41" s="11" t="n"/>
-      <c r="R41" s="11" t="inlineStr">
+      <c r="O46" s="11" t="n"/>
+      <c r="P46" s="31" t="n"/>
+      <c r="Q46" s="11" t="n"/>
+      <c r="R46" s="11" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S41" s="11" t="n"/>
-    </row>
-    <row r="42" ht="105" customHeight="1">
-      <c r="A42" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>FB-039</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="S46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="105" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>FB-045</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Arrange product rows and the filter toolbar</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Teach readable widths, wrapping, table overflow and stacked toolbar on small screens. Keep code and available stock understandable without typography/colour lessons.</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>FB-038</t>
-        </is>
-      </c>
-      <c r="G42" s="4">
-        <f>IF(H42="Complete","Complete",IF(I42="Blocked","Blocked",IF(I42="In progress","Ready",IF(F42="","Ready",IF(COUNTIFS($B$4:$B$73,F42,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H42" s="4">
-        <f>IF(I42="Not started","Not started",IF(I42="Blocked","Blocked",IF(I42="In progress","In progress",IF(J42&lt;&gt;"Passed","Awaiting code review",IF(OR(K42="",NOT(ISNUMBER(L42))),"Awaiting review evidence",IF(N42&lt;&gt;"Passed","Awaiting test",IF(OR(M42="",O42="",NOT(ISNUMBER(P42))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I42" s="10" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Add the product status filter</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>All/Active/Inactive works with existing filters. General product list may show inactive/zero-stock products; distribution picker later has stricter rules.</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>FB-044</t>
+        </is>
+      </c>
+      <c r="G47" s="4">
+        <f>IF(H47="Complete","Complete",IF(I47="Blocked","Blocked",IF(I47="In progress","Ready",IF(F47="","Ready",IF(COUNTIFS($B$4:$B$73,F47,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H47" s="4">
+        <f>IF(I47="Not started","Not started",IF(I47="Blocked","Blocked",IF(I47="In progress","In progress",IF(J47&lt;&gt;"Passed","Awaiting code review",IF(OR(K47="",NOT(ISNUMBER(L47))),"Awaiting review evidence",IF(N47&lt;&gt;"Passed","Awaiting test",IF(OR(M47="",O47="",NOT(ISNUMBER(P47))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J42" s="10" t="inlineStr">
+      <c r="J47" s="10" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K42" s="10" t="n"/>
-      <c r="L42" s="30" t="n"/>
-      <c r="M42" s="10" t="n"/>
-      <c r="N42" s="10" t="inlineStr">
+      <c r="K47" s="10" t="n"/>
+      <c r="L47" s="30" t="n"/>
+      <c r="M47" s="10" t="n"/>
+      <c r="N47" s="10" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O42" s="10" t="n"/>
-      <c r="P42" s="30" t="n"/>
-      <c r="Q42" s="10" t="n"/>
-      <c r="R42" s="10" t="inlineStr">
+      <c r="O47" s="10" t="n"/>
+      <c r="P47" s="30" t="n"/>
+      <c r="Q47" s="10" t="n"/>
+      <c r="R47" s="10" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S42" s="10" t="n"/>
-    </row>
-    <row r="43" ht="105" customHeight="1">
-      <c r="A43" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>FB-040</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="S47" s="10" t="n"/>
+    </row>
+    <row r="48" ht="105" customHeight="1">
+      <c r="A48" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>FB-046</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
-        <is>
-          <t>Add search by product code or name</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>Search the full catalogue before pagination. Verify both code and name, clear search and no results.</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>FB-039</t>
-        </is>
-      </c>
-      <c r="G43" s="9">
-        <f>IF(H43="Complete","Complete",IF(I43="Blocked","Blocked",IF(I43="In progress","Ready",IF(F43="","Ready",IF(COUNTIFS($B$4:$B$73,F43,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H43" s="9">
-        <f>IF(I43="Not started","Not started",IF(I43="Blocked","Blocked",IF(I43="In progress","In progress",IF(J43&lt;&gt;"Passed","Awaiting code review",IF(OR(K43="",NOT(ISNUMBER(L43))),"Awaiting review evidence",IF(N43&lt;&gt;"Passed","Awaiting test",IF(OR(M43="",O43="",NOT(ISNUMBER(P43))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I43" s="11" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Paginate and verify the full product list</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>10 products per page after all search/filters. Preserve selections across pages; all roles may list/search/filter. Verify combinations and boundary/empty pages.</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>FB-045</t>
+        </is>
+      </c>
+      <c r="G48" s="9">
+        <f>IF(H48="Complete","Complete",IF(I48="Blocked","Blocked",IF(I48="In progress","Ready",IF(F48="","Ready",IF(COUNTIFS($B$4:$B$73,F48,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H48" s="9">
+        <f>IF(I48="Not started","Not started",IF(I48="Blocked","Blocked",IF(I48="In progress","In progress",IF(J48&lt;&gt;"Passed","Awaiting code review",IF(OR(K48="",NOT(ISNUMBER(L48))),"Awaiting review evidence",IF(N48&lt;&gt;"Passed","Awaiting test",IF(OR(M48="",O48="",NOT(ISNUMBER(P48))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J43" s="11" t="inlineStr">
+      <c r="J48" s="11" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K43" s="11" t="n"/>
-      <c r="L43" s="31" t="n"/>
-      <c r="M43" s="11" t="n"/>
-      <c r="N43" s="11" t="inlineStr">
+      <c r="K48" s="11" t="n"/>
+      <c r="L48" s="31" t="n"/>
+      <c r="M48" s="11" t="n"/>
+      <c r="N48" s="11" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O43" s="11" t="n"/>
-      <c r="P43" s="31" t="n"/>
-      <c r="Q43" s="11" t="n"/>
-      <c r="R43" s="11" t="inlineStr">
+      <c r="O48" s="11" t="n"/>
+      <c r="P48" s="31" t="n"/>
+      <c r="Q48" s="11" t="n"/>
+      <c r="R48" s="11" t="inlineStr">
         <is>
           <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Start this item after the previous item is complete.</t>
         </is>
       </c>
-      <c r="S43" s="11" t="n"/>
-    </row>
-    <row r="44" ht="105" customHeight="1">
-      <c r="A44" s="4" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>FB-041</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="S48" s="11" t="n"/>
+    </row>
+    <row r="49" ht="105" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>FB-047</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Add the department filter</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Filter by department alone and with search. Explain selected state and request values; do not introduce remaining filters yet.</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>FB-040</t>
-        </is>
-      </c>
-      <c r="G44" s="4">
-        <f>IF(H44="Complete","Complete",IF(I44="Blocked","Blocked",IF(I44="In progress","Ready",IF(F44="","Ready",IF(COUNTIFS($B$4:$B$73,F44,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H44" s="4">
-        <f>IF(I44="Not started","Not started",IF(I44="Blocked","Blocked",IF(I44="In progress","In progress",IF(J44&lt;&gt;"Passed","Awaiting code review",IF(OR(K44="",NOT(ISNUMBER(L44))),"Awaiting review evidence",IF(N44&lt;&gt;"Passed","Awaiting test",IF(OR(M44="",O44="",NOT(ISNUMBER(P44))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I44" s="10" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Edit catalogue product details</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Managers/Super Admin edit catalogue fields with duplicate checks and permanent code. No packaging/stock fields. Stock-related classification constraints must be decided at stock design checkpoint.</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>FB-046</t>
+        </is>
+      </c>
+      <c r="G49" s="4">
+        <f>IF(H49="Complete","Complete",IF(I49="Blocked","Blocked",IF(I49="In progress","Ready",IF(F49="","Ready",IF(COUNTIFS($B$4:$B$73,F49,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H49" s="4">
+        <f>IF(I49="Not started","Not started",IF(I49="Blocked","Blocked",IF(I49="In progress","In progress",IF(J49&lt;&gt;"Passed","Awaiting code review",IF(OR(K49="",NOT(ISNUMBER(L49))),"Awaiting review evidence",IF(N49&lt;&gt;"Passed","Awaiting test",IF(OR(M49="",O49="",NOT(ISNUMBER(P49))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J44" s="10" t="inlineStr">
+      <c r="J49" s="10" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K44" s="10" t="n"/>
-      <c r="L44" s="30" t="n"/>
-      <c r="M44" s="10" t="n"/>
-      <c r="N44" s="10" t="inlineStr">
+      <c r="K49" s="10" t="n"/>
+      <c r="L49" s="30" t="n"/>
+      <c r="M49" s="10" t="n"/>
+      <c r="N49" s="10" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O44" s="10" t="n"/>
-      <c r="P44" s="30" t="n"/>
-      <c r="Q44" s="10" t="n"/>
-      <c r="R44" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S44" s="10" t="n"/>
-    </row>
-    <row r="45" ht="105" customHeight="1">
-      <c r="A45" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>FB-042</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="O49" s="10" t="n"/>
+      <c r="P49" s="30" t="n"/>
+      <c r="Q49" s="10" t="n"/>
+      <c r="R49" s="10" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S49" s="10" t="n"/>
+    </row>
+    <row r="50" ht="105" customHeight="1">
+      <c r="A50" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>FB-048</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>Products</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
-        <is>
-          <t>Add the category filter</t>
-        </is>
-      </c>
-      <c r="E45" s="9" t="inlineStr">
-        <is>
-          <t>Filter by category and combine with department/search; changing parent must not leave incompatible selections.</t>
-        </is>
-      </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>FB-041</t>
-        </is>
-      </c>
-      <c r="G45" s="9">
-        <f>IF(H45="Complete","Complete",IF(I45="Blocked","Blocked",IF(I45="In progress","Ready",IF(F45="","Ready",IF(COUNTIFS($B$4:$B$73,F45,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H45" s="9">
-        <f>IF(I45="Not started","Not started",IF(I45="Blocked","Blocked",IF(I45="In progress","In progress",IF(J45&lt;&gt;"Passed","Awaiting code review",IF(OR(K45="",NOT(ISNUMBER(L45))),"Awaiting review evidence",IF(N45&lt;&gt;"Passed","Awaiting test",IF(OR(M45="",O45="",NOT(ISNUMBER(P45))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I45" s="11" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Activate/deactivate products and manage tag removal</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Deactivate only when Stock Management reports no remaining stock across product records. Server checks, generic blocked message without numbers/sizes. Reactivation and optional tag removal; shared tag deletion only if unused including inactive products. Verify nonzero check after stock setup at FB-053.</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>FB-047</t>
+        </is>
+      </c>
+      <c r="G50" s="9">
+        <f>IF(H50="Complete","Complete",IF(I50="Blocked","Blocked",IF(I50="In progress","Ready",IF(F50="","Ready",IF(COUNTIFS($B$4:$B$73,F50,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H50" s="9">
+        <f>IF(I50="Not started","Not started",IF(I50="Blocked","Blocked",IF(I50="In progress","In progress",IF(J50&lt;&gt;"Passed","Awaiting code review",IF(OR(K50="",NOT(ISNUMBER(L50))),"Awaiting review evidence",IF(N50&lt;&gt;"Passed","Awaiting test",IF(OR(M50="",O50="",NOT(ISNUMBER(P50))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J45" s="11" t="inlineStr">
+      <c r="J50" s="11" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K45" s="11" t="n"/>
-      <c r="L45" s="31" t="n"/>
-      <c r="M45" s="11" t="n"/>
-      <c r="N45" s="11" t="inlineStr">
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="31" t="n"/>
+      <c r="M50" s="11" t="n"/>
+      <c r="N50" s="11" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O45" s="11" t="n"/>
-      <c r="P45" s="31" t="n"/>
-      <c r="Q45" s="11" t="n"/>
-      <c r="R45" s="11" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S45" s="11" t="n"/>
-    </row>
-    <row r="46" ht="105" customHeight="1">
-      <c r="A46" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>FB-043</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Add the subcategory filter</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>Filter by subcategory alongside existing selections; verify full path and no skipped/contradictory parent selection.</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>FB-042</t>
-        </is>
-      </c>
-      <c r="G46" s="4">
-        <f>IF(H46="Complete","Complete",IF(I46="Blocked","Blocked",IF(I46="In progress","Ready",IF(F46="","Ready",IF(COUNTIFS($B$4:$B$73,F46,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H46" s="4">
-        <f>IF(I46="Not started","Not started",IF(I46="Blocked","Blocked",IF(I46="In progress","In progress",IF(J46&lt;&gt;"Passed","Awaiting code review",IF(OR(K46="",NOT(ISNUMBER(L46))),"Awaiting review evidence",IF(N46&lt;&gt;"Passed","Awaiting test",IF(OR(M46="",O46="",NOT(ISNUMBER(P46))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I46" s="10" t="inlineStr">
+      <c r="O50" s="11" t="n"/>
+      <c r="P50" s="31" t="n"/>
+      <c r="Q50" s="11" t="n"/>
+      <c r="R50" s="11" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S50" s="11" t="n"/>
+    </row>
+    <row r="51" ht="105" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>FB-067</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Verify completed Product Catalogue before Stock Management</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Review/test hierarchy/tags/product identity, codes, duplicate/required fields, filters/pagination, responsive views and permissions. Explicitly verify no sizes/units/quantities/history/totals appear in catalogue. Stock integration/deactivation checks at FB-053; packaging setup now FB-034 before Receive.</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>FB-048</t>
+        </is>
+      </c>
+      <c r="G51" s="4">
+        <f>IF(H51="Complete","Complete",IF(I51="Blocked","Blocked",IF(I51="In progress","Ready",IF(F51="","Ready",IF(COUNTIFS($B$4:$B$73,F51,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H51" s="4">
+        <f>IF(I51="Not started","Not started",IF(I51="Blocked","Blocked",IF(I51="In progress","In progress",IF(J51&lt;&gt;"Passed","Awaiting code review",IF(OR(K51="",NOT(ISNUMBER(L51))),"Awaiting review evidence",IF(N51&lt;&gt;"Passed","Awaiting test",IF(OR(M51="",O51="",NOT(ISNUMBER(P51))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I51" s="10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J46" s="10" t="inlineStr">
+      <c r="J51" s="10" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K46" s="10" t="n"/>
-      <c r="L46" s="30" t="n"/>
-      <c r="M46" s="10" t="n"/>
-      <c r="N46" s="10" t="inlineStr">
+      <c r="K51" s="10" t="n"/>
+      <c r="L51" s="30" t="n"/>
+      <c r="M51" s="10" t="n"/>
+      <c r="N51" s="10" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O46" s="10" t="n"/>
-      <c r="P46" s="30" t="n"/>
-      <c r="Q46" s="10" t="n"/>
-      <c r="R46" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S46" s="10" t="n"/>
-    </row>
-    <row r="47" ht="105" customHeight="1">
-      <c r="A47" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>FB-044</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="inlineStr">
-        <is>
-          <t>Add the tag filter</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="inlineStr">
-        <is>
-          <t>Show products with the selected shared tag; combine with prior filters and search. Untagged products remain visible when tag filter is cleared.</t>
-        </is>
-      </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>FB-043</t>
-        </is>
-      </c>
-      <c r="G47" s="9">
-        <f>IF(H47="Complete","Complete",IF(I47="Blocked","Blocked",IF(I47="In progress","Ready",IF(F47="","Ready",IF(COUNTIFS($B$4:$B$73,F47,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H47" s="9">
-        <f>IF(I47="Not started","Not started",IF(I47="Blocked","Blocked",IF(I47="In progress","In progress",IF(J47&lt;&gt;"Passed","Awaiting code review",IF(OR(K47="",NOT(ISNUMBER(L47))),"Awaiting review evidence",IF(N47&lt;&gt;"Passed","Awaiting test",IF(OR(M47="",O47="",NOT(ISNUMBER(P47))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I47" s="11" t="inlineStr">
+      <c r="O51" s="10" t="n"/>
+      <c r="P51" s="30" t="n"/>
+      <c r="Q51" s="10" t="n"/>
+      <c r="R51" s="10" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</t>
+        </is>
+      </c>
+      <c r="S51" s="10" t="n"/>
+    </row>
+    <row r="52" ht="105" customHeight="1">
+      <c r="A52" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>FB-034</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Stock Management</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>Build reusable package sizes and product stock items</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29 approved shared package design: Stock Management has package_sizes(id, package_type, contents, contents_unit), reusable across products; stock_items(id, product_id, package_size_id) links each catalogue product to a package definition. One unique product/package_size pair. stock_movements belongs to stock_item_id, so balances/history are separate even when package definitions are shared. Product catalogue has no size/unit/quantity fields or displays. Examples: Rice and Lentils share Bag5kg; Milk and Juice share Carton2litres; Eggs uses Carton12items (12 eggs/carton). Keep positive whole package movement quantities and whole-number individual-item contents. Reject duplicate package definitions, comparing equivalent kg/g and litres/ml contents within the same package type; a bottle differs from a carton. Once referenced by a stock item, package type/contents/unit are immutable; create another definition instead. This stronger shared-definition lock supersedes the earlier first-movement-only package lock. Shared package-size management permissions/UI, summary-configuration ownership and classification-lock details still need focused decisions before implementation. No loose-egg repacking workflow approved. Build and verify package definitions first, then stock_items connected to existing catalogue Products before Receive; preserve module order and review/testing evidence.</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>FB-067</t>
+        </is>
+      </c>
+      <c r="G52" s="9">
+        <f>IF(H52="Complete","Complete",IF(I52="Blocked","Blocked",IF(I52="In progress","Ready",IF(F52="","Ready",IF(COUNTIFS($B$4:$B$73,F52,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
+        <v/>
+      </c>
+      <c r="H52" s="9">
+        <f>IF(I52="Not started","Not started",IF(I52="Blocked","Blocked",IF(I52="In progress","In progress",IF(J52&lt;&gt;"Passed","Awaiting code review",IF(OR(K52="",NOT(ISNUMBER(L52))),"Awaiting review evidence",IF(N52&lt;&gt;"Passed","Awaiting test",IF(OR(M52="",O52="",NOT(ISNUMBER(P52))),"Awaiting test evidence","Complete")))))))</f>
+        <v/>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="J47" s="11" t="inlineStr">
+      <c r="J52" s="11" t="inlineStr">
         <is>
           <t>Not reviewed</t>
         </is>
       </c>
-      <c r="K47" s="11" t="n"/>
-      <c r="L47" s="31" t="n"/>
-      <c r="M47" s="11" t="n"/>
-      <c r="N47" s="11" t="inlineStr">
+      <c r="K52" s="11" t="n"/>
+      <c r="L52" s="31" t="n"/>
+      <c r="M52" s="11" t="n"/>
+      <c r="N52" s="11" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
-      <c r="O47" s="11" t="n"/>
-      <c r="P47" s="31" t="n"/>
-      <c r="Q47" s="11" t="n"/>
-      <c r="R47" s="11" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S47" s="11" t="n"/>
-    </row>
-    <row r="48" ht="105" customHeight="1">
-      <c r="A48" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>FB-045</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Add the product status filter</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>All/Active/Inactive works with existing filters. General product list may show inactive/zero-stock products; distribution picker later has stricter rules.</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>FB-044</t>
-        </is>
-      </c>
-      <c r="G48" s="4">
-        <f>IF(H48="Complete","Complete",IF(I48="Blocked","Blocked",IF(I48="In progress","Ready",IF(F48="","Ready",IF(COUNTIFS($B$4:$B$73,F48,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H48" s="4">
-        <f>IF(I48="Not started","Not started",IF(I48="Blocked","Blocked",IF(I48="In progress","In progress",IF(J48&lt;&gt;"Passed","Awaiting code review",IF(OR(K48="",NOT(ISNUMBER(L48))),"Awaiting review evidence",IF(N48&lt;&gt;"Passed","Awaiting test",IF(OR(M48="",O48="",NOT(ISNUMBER(P48))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I48" s="10" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J48" s="10" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K48" s="10" t="n"/>
-      <c r="L48" s="30" t="n"/>
-      <c r="M48" s="10" t="n"/>
-      <c r="N48" s="10" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O48" s="10" t="n"/>
-      <c r="P48" s="30" t="n"/>
-      <c r="Q48" s="10" t="n"/>
-      <c r="R48" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S48" s="10" t="n"/>
-    </row>
-    <row r="49" ht="105" customHeight="1">
-      <c r="A49" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>FB-046</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>Paginate and verify the full product list</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="inlineStr">
-        <is>
-          <t>10 products per page after all search/filters. Preserve selections across pages; all roles may list/search/filter. Verify combinations and boundary/empty pages.</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>FB-045</t>
-        </is>
-      </c>
-      <c r="G49" s="9">
-        <f>IF(H49="Complete","Complete",IF(I49="Blocked","Blocked",IF(I49="In progress","Ready",IF(F49="","Ready",IF(COUNTIFS($B$4:$B$73,F49,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H49" s="9">
-        <f>IF(I49="Not started","Not started",IF(I49="Blocked","Blocked",IF(I49="In progress","In progress",IF(J49&lt;&gt;"Passed","Awaiting code review",IF(OR(K49="",NOT(ISNUMBER(L49))),"Awaiting review evidence",IF(N49&lt;&gt;"Passed","Awaiting test",IF(OR(M49="",O49="",NOT(ISNUMBER(P49))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I49" s="11" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J49" s="11" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K49" s="11" t="n"/>
-      <c r="L49" s="31" t="n"/>
-      <c r="M49" s="11" t="n"/>
-      <c r="N49" s="11" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O49" s="11" t="n"/>
-      <c r="P49" s="31" t="n"/>
-      <c r="Q49" s="11" t="n"/>
-      <c r="R49" s="11" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S49" s="11" t="n"/>
-    </row>
-    <row r="50" ht="105" customHeight="1">
-      <c r="A50" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>FB-047</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Edit product details before movements</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>Managers/Super Admin may edit catalogue fields subject to validation and duplicates; codes permanent. Explain changes with local zero-stock products. Post-movement locks are added and verified with Receive.</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>FB-046</t>
-        </is>
-      </c>
-      <c r="G50" s="4">
-        <f>IF(H50="Complete","Complete",IF(I50="Blocked","Blocked",IF(I50="In progress","Ready",IF(F50="","Ready",IF(COUNTIFS($B$4:$B$73,F50,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H50" s="4">
-        <f>IF(I50="Not started","Not started",IF(I50="Blocked","Blocked",IF(I50="In progress","In progress",IF(J50&lt;&gt;"Passed","Awaiting code review",IF(OR(K50="",NOT(ISNUMBER(L50))),"Awaiting review evidence",IF(N50&lt;&gt;"Passed","Awaiting test",IF(OR(M50="",O50="",NOT(ISNUMBER(P50))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I50" s="10" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J50" s="10" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K50" s="10" t="n"/>
-      <c r="L50" s="30" t="n"/>
-      <c r="M50" s="10" t="n"/>
-      <c r="N50" s="10" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O50" s="10" t="n"/>
-      <c r="P50" s="30" t="n"/>
-      <c r="Q50" s="10" t="n"/>
-      <c r="R50" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
-        </is>
-      </c>
-      <c r="S50" s="10" t="n"/>
-    </row>
-    <row r="51" ht="105" customHeight="1">
-      <c r="A51" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>FB-048</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>Activate/deactivate products and manage tag removal</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>Deactivate only at zero stock, retain records instead of deleting. Reactivate later. Remove tags from a product without deleting shared tag; delete shared tag only if unused by active AND inactive products.</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="inlineStr">
-        <is>
-          <t>FB-047</t>
-        </is>
-      </c>
-      <c r="G51" s="9">
-        <f>IF(H51="Complete","Complete",IF(I51="Blocked","Blocked",IF(I51="In progress","Ready",IF(F51="","Ready",IF(COUNTIFS($B$4:$B$73,F51,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H51" s="9">
-        <f>IF(I51="Not started","Not started",IF(I51="Blocked","Blocked",IF(I51="In progress","In progress",IF(J51&lt;&gt;"Passed","Awaiting code review",IF(OR(K51="",NOT(ISNUMBER(L51))),"Awaiting review evidence",IF(N51&lt;&gt;"Passed","Awaiting test",IF(OR(M51="",O51="",NOT(ISNUMBER(P51))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I51" s="11" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J51" s="11" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K51" s="11" t="n"/>
-      <c r="L51" s="31" t="n"/>
-      <c r="M51" s="11" t="n"/>
-      <c r="N51" s="11" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O51" s="11" t="n"/>
-      <c r="P51" s="31" t="n"/>
-      <c r="Q51" s="11" t="n"/>
-      <c r="R51" s="11" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Verify zero-stock deactivation and reactivation first. Then teach removing a product tag and deleting only unused shared tags separately, after the relationship exists. Include inactive products in usage checks. Nonzero-stock rejection and movement locks are verified later in FB-053.</t>
-        </is>
-      </c>
-      <c r="S51" s="11" t="n"/>
-    </row>
-    <row r="52" ht="105" customHeight="1">
-      <c r="A52" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>FB-067</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Verify the completed catalogue before stock movements</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>Review and ask the developer to test completed Department, Category, Subcategory, Tag and Product actions, codes/duplicates/required fields, compatible units/precision, responsive layouts, individual filters and pagination, and permitted/denied direct requests. Stock-dependent locks and nonzero deactivation remain FB-053; totals are FB-065/FB-066; movement-wide checks are FB-068/FB-069. Record actual evidence before starting Receive.</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>FB-048</t>
-        </is>
-      </c>
-      <c r="G52" s="4">
-        <f>IF(H52="Complete","Complete",IF(I52="Blocked","Blocked",IF(I52="In progress","Ready",IF(F52="","Ready",IF(COUNTIFS($B$4:$B$73,F52,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</f>
-        <v/>
-      </c>
-      <c r="H52" s="4">
-        <f>IF(I52="Not started","Not started",IF(I52="Blocked","Blocked",IF(I52="In progress","In progress",IF(J52&lt;&gt;"Passed","Awaiting code review",IF(OR(K52="",NOT(ISNUMBER(L52))),"Awaiting review evidence",IF(N52&lt;&gt;"Passed","Awaiting test",IF(OR(M52="",O52="",NOT(ISNUMBER(P52))),"Awaiting test evidence","Complete")))))))</f>
-        <v/>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>Not reviewed</t>
-        </is>
-      </c>
-      <c r="K52" s="10" t="n"/>
-      <c r="L52" s="30" t="n"/>
-      <c r="M52" s="10" t="n"/>
-      <c r="N52" s="10" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-      <c r="O52" s="10" t="n"/>
-      <c r="P52" s="30" t="n"/>
-      <c r="Q52" s="10" t="n"/>
-      <c r="R52" s="10" t="inlineStr">
-        <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Run the catalogue checkpoint before Receive, with developer-first tests. Verify each completed module and combined list filters. Explicitly record stock-dependent checks as later FB-053/FB-065/FB-066/FB-068 checkpoints, not passed checks here.</t>
-        </is>
-      </c>
-      <c r="S52" s="10" t="n"/>
+      <c r="O52" s="11" t="n"/>
+      <c r="P52" s="31" t="n"/>
+      <c r="Q52" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+2026-10-29 approved shared package design: Stock Management has package_sizes(id, package_type, contents, contents_unit), reusable across products; stock_items(id, product_id, package_size_id) links each catalogue product to a package definition. One unique product/package_size pair. stock_movements belongs to stock_item_id, so balances/history are separate even when package definitions are shared. Product catalogue has no size/unit/quantity fields or displays. Examples: Rice and Lentils share Bag5kg; Milk and Juice share Carton2litres; Eggs uses Carton12items (12 eggs/carton). Keep positive whole package movement quantities and whole-number individual-item contents. Reject duplicate package definitions, comparing equivalent kg/g and litres/ml contents within the same package type; a bottle differs from a carton. Once referenced by a stock item, package type/contents/unit are immutable; create another definition instead. This stronger shared-definition lock supersedes the earlier first-movement-only package lock. Shared package-size management permissions/UI, summary-configuration ownership and classification-lock details still need focused decisions before implementation. No loose-egg repacking workflow approved.</t>
+        </is>
+      </c>
+      <c r="R52" s="11" t="inlineStr">
+        <is>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read shared package-size requirement; first settle package-management permissions and remaining summary/classification details, then teach package definitions and product/package stock_items in dependency order after FB-067. Approval is planning only; no implementation or completion evidence.</t>
+        </is>
+      </c>
+      <c r="S52" s="11" t="n"/>
     </row>
     <row r="53" ht="105" customHeight="1">
       <c r="A53" s="9" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B53" s="9" t="inlineStr">
         <is>
@@ -5537,12 +5546,12 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>All three roles may receive active products, including zero-stock products. Show saved package size; quantities are whole packages; one optional note for whole entry. Teach one row before multiple rows.</t>
+          <t>All three roles may receive active products, including zero-stock products. Show saved package size; quantities are whole packages; one optional note for whole entry. Teach one row before multiple rows. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>FB-067</t>
+          <t>FB-034</t>
         </is>
       </c>
       <c r="G53" s="9">
@@ -5576,15 +5585,14 @@
       <c r="Q53" s="11" t="n"/>
       <c r="R53" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Identify movement permissions and consistency rules first. Introduce receipt/movement storage and Product/recorder relationships only as needed for Receive. A local fictional one-row form may precede persistence. Teach package display and layout before multiple rows; do not enable submission without server checks.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S53" s="11" t="n"/>
     </row>
     <row r="54" ht="105" customHeight="1">
       <c r="A54" s="4" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
@@ -5603,7 +5611,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Each product appears once; update its quantity instead of duplicate rows. Multiple different products allowed. Reject zero/negative/fractional quantities; unit choice is on product creation, not movements.</t>
+          <t>Each product appears once; update its quantity instead of duplicate rows. Multiple different products allowed. Reject zero/negative/fractional quantities; unit choice is on product creation, not movements. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -5642,15 +5650,14 @@
       <c r="Q54" s="10" t="n"/>
       <c r="R54" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S54" s="10" t="n"/>
     </row>
     <row r="55" ht="105" customHeight="1">
       <c r="A55" s="9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
@@ -5669,7 +5676,7 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>All movements save or none. Increase counts, auto-capture recorder/save timestamp and resulting balances. Stock only changes via movements. No backdating or movement editing/deletion. Test rollback and inactive-product rejection. Attach movement permissions and active-account checks before enabling submission, not for the first time in FB-052. Teach the all-or-none transaction and required relationships before saving. Keep this local and fictional until FB-053 locks are verified.</t>
+          <t>All movements save or none. Increase counts, auto-capture recorder/save timestamp and resulting balances. Stock only changes via movements. No backdating or movement editing/deletion. Test rollback and inactive-product rejection. Attach movement permissions and active-account checks before enabling submission, not for the first time in FB-052. Teach the all-or-none transaction and required relationships before saving. Keep this local and fictional until FB-053 locks are verified. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
@@ -5708,15 +5715,14 @@
       <c r="Q55" s="11" t="n"/>
       <c r="R55" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Explain receipt, movement, Product and recorder links, validation and the transaction before enabling Save. Enforce server permissions and active status now. Verify saved balances and rollback with fictional data. FB-052 adds submission feedback; FB-053 completes post-movement locks before operational use.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S55" s="11" t="n"/>
     </row>
     <row r="56" ht="105" customHeight="1">
       <c r="A56" s="4" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
@@ -5735,7 +5741,7 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Show processing/errors/success; prevent repeated clicks while processing. Enforce active-account and movement permissions on server; opening stock uses Receive. Test a multiple-product receipt against actual balances.</t>
+          <t>Show processing/errors/success; prevent repeated clicks while processing. Enforce active-account and movement permissions on server; opening stock uses Receive. Test a multiple-product receipt against actual balances. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -5774,15 +5780,14 @@
       <c r="Q56" s="10" t="n"/>
       <c r="R56" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Add processing, retained errors and success feedback to the already authorized save operation. Recheck the server safeguards from FB-051; do not postpone them until this lesson. Verify a multi-product receipt, then finish required locks in FB-053.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S56" s="10" t="n"/>
     </row>
     <row r="57" ht="105" customHeight="1">
       <c r="A57" s="9" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
@@ -5796,12 +5801,12 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Lock product and summary units after first movement</t>
+          <t>Verify stock measurement locks and catalogue deactivation guard</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>After first movement lock product counting unit, contents/value/unit and subcategory. Lock subcategory summary unit once any child moved. Names/tags remain editable; nonzero products cannot deactivate. Direct writes cannot bypass locks.</t>
+          <t>Enforce immutable stock package measurement after movements; summary-configuration locks within Stock Management. Catalogue deactivation blocked if any stock remains, without exposing size/quantity. Confirm classification constraints at stock design checkpoint before implementing. Verify direct-write safeguards. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr">
@@ -5840,15 +5845,14 @@
       <c r="Q57" s="11" t="n"/>
       <c r="R57" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Use a real fictional Receive movement to observe why units/subcategory must now lock. Enforce each lock separately and verify direct-write rejection and nonzero deactivation. Retest earlier catalogue edit actions before calling Receive ready for operational use.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S57" s="11" t="n"/>
     </row>
     <row r="58" ht="105" customHeight="1">
       <c r="A58" s="4" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
@@ -5862,12 +5866,12 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Show product stock history to permitted roles</t>
+          <t>Show stock movement history within Stock Management</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>On product details, show type, +/- quantity, timestamp, resulting balance, recorder and receipt/household/reason details. History comes automatically from movements. Managers/Super Admin only; volunteers denied even direct requests.</t>
+          <t>Managers/Super Admin only; type/quantity/time/result/recorder/receipt/household/reason. History absent from catalogue product detail. Volunteer direct history access denied. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
@@ -5906,15 +5910,14 @@
       <c r="Q58" s="10" t="n"/>
       <c r="R58" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Build the permitted product details/history view using Receive records now available. Verify manager/Super Admin access and volunteer denial. Add adjustment reasons in FB-056 and household details in FB-063 when those movements exist, then recheck all history types in FB-068.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S58" s="10" t="n"/>
     </row>
     <row r="59" ht="105" customHeight="1">
       <c r="A59" s="9" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
@@ -5928,12 +5931,12 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Calculate subcategory totals accurately</t>
+          <t>Calculate stock summaries within Stock Management</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Multiply stock by contents, converting g to kg and ml to litres before summing; count eggs as individual items. Example 4x500g+3x1kg+2x5kg=15kg. Keep exact values until display; never replace product counts.</t>
+          <t>Use stock package balances/contents and kg/g, litres/ml conversions. Exact calculation then formatted display. Do not add quantities or measurement configuration to catalogue. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
@@ -5972,15 +5975,14 @@
       <c r="Q59" s="11" t="n"/>
       <c r="R59" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Use completed Receive balances to introduce one subcategory calculation. Verify the agreed rice example and unit conversion before adding display. Do not build later movement modules early; recheck totals after Adjust in FB-056 and Distribute in FB-063/FB-064.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S59" s="11" t="n"/>
     </row>
     <row r="60" ht="105" customHeight="1">
       <c r="A60" s="4" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
@@ -5994,12 +5996,12 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Display combined totals on subcategory management</t>
+          <t>Display combined totals within Stock Management</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Managers/Super Admin see totals in kg/litres/items with up to 3 decimals, fewer allowed; round display only. Individual product sizes keep saved units. Volunteer cannot access management/history screens.</t>
+          <t>Managers/Super Admin see stock summaries in kg/litres/items with at most3 displayed decimals. Product Catalogue/Subcategory screens show no units/sizes/quantities/totals. Verify later Adjust/Distribute update stock summaries. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -6038,15 +6040,14 @@
       <c r="Q60" s="10" t="n"/>
       <c r="R60" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Display the calculated total on the existing protected Subcategory screen and teach formatting separately. Verify manager/Super Admin access and volunteer denial using received stock. Later movement lessons must verify their changes update these totals.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S60" s="10" t="n"/>
     </row>
     <row r="61" ht="105" customHeight="1">
       <c r="A61" s="9" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B61" s="9" t="inlineStr">
         <is>
@@ -6065,7 +6066,7 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>All roles choose one active product, Add/Remove, positive whole quantity and mandatory reason. Show saved package size and current balance. Teach state and layout before save.</t>
+          <t>All roles choose one active product, Add/Remove, positive whole quantity and mandatory reason. Show saved package size and current balance. Teach state and layout before save. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr">
@@ -6104,15 +6105,14 @@
       <c r="Q61" s="11" t="n"/>
       <c r="R61" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: After Receive, history and totals are verified, identify Adjust permissions and stock rules. Reuse existing movement storage and introduce the required reason through this concrete action. Teach one product and Add/Remove state, then layout; attach checks before enabling save.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S61" s="11" t="n"/>
     </row>
     <row r="62" ht="105" customHeight="1">
       <c r="A62" s="4" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
@@ -6131,7 +6131,7 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>Add increases and Remove decreases stock. Reject removal above availability and missing reason. Record immutable movement with recorder/time/result; preserve original movements. Verify simultaneous stock updates and permission enforcement. Verify the new adjustment appears in product history and changes the already completed subcategory total correctly.</t>
+          <t>Add increases and Remove decreases stock. Reject removal above availability and missing reason. Record immutable movement with recorder/time/result; preserve original movements. Verify simultaneous stock updates and permission enforcement. Verify the new adjustment appears in product history and changes the already completed subcategory total correctly. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -6170,15 +6170,14 @@
       <c r="Q62" s="10" t="n"/>
       <c r="R62" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S62" s="10" t="n"/>
     </row>
     <row r="63" ht="105" customHeight="1">
       <c r="A63" s="9" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B63" s="9" t="inlineStr">
         <is>
@@ -6244,7 +6243,7 @@
     </row>
     <row r="64" ht="105" customHeight="1">
       <c r="A64" s="4" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
@@ -6310,7 +6309,7 @@
     </row>
     <row r="65" ht="105" customHeight="1">
       <c r="A65" s="9" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B65" s="9" t="inlineStr">
         <is>
@@ -6329,7 +6328,7 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Selecting Rice shows active products with positive stock: name, brand, code, saved size and available package count. Exclude inactive/zero-stock entries; distinguish equal sizes from different brands.</t>
+          <t>Selecting Rice shows active products with positive stock: name, brand, code, saved size and available package count. Exclude inactive/zero-stock entries; distinguish equal sizes from different brands. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
@@ -6368,15 +6367,14 @@
       <c r="Q65" s="11" t="n"/>
       <c r="R65" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S65" s="11" t="n"/>
     </row>
     <row r="66" ht="105" customHeight="1">
       <c r="A66" s="4" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
@@ -6395,7 +6393,7 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Search selectable products by code or name, preserving subcategory/availability restrictions. Verify clear/no-result cases.</t>
+          <t>Search selectable products by code or name, preserving subcategory/availability restrictions. Verify clear/no-result cases. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -6434,15 +6432,14 @@
       <c r="Q66" s="10" t="n"/>
       <c r="R66" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S66" s="10" t="n"/>
     </row>
     <row r="67" ht="105" customHeight="1">
       <c r="A67" s="9" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B67" s="9" t="inlineStr">
         <is>
@@ -6461,7 +6458,7 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Choose whole package quantities across products/sizes; each product appears once. Cannot split a 1kg bag to distribute 500g. Teach each row/quantity interaction separately and responsive layout.</t>
+          <t>Choose whole package quantities across products/sizes; each product appears once. Cannot split a 1kg bag to distribute 500g. Teach each row/quantity interaction separately and responsive layout. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
@@ -6500,15 +6497,14 @@
       <c r="Q67" s="11" t="n"/>
       <c r="R67" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S67" s="11" t="n"/>
     </row>
     <row r="68" ht="105" customHeight="1">
       <c r="A68" s="4" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
@@ -6527,7 +6523,7 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>Review one household plus all products/sizes/quantities before saving. Staff can correct the selection. Explain temporary selection state versus saved stock.</t>
+          <t>Review one household plus all products/sizes/quantities before saving. Staff can correct the selection. Explain temporary selection state versus saved stock. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -6566,15 +6562,14 @@
       <c r="Q68" s="10" t="n"/>
       <c r="R68" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S68" s="10" t="n"/>
     </row>
     <row r="69" ht="105" customHeight="1">
       <c r="A69" s="9" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
@@ -6593,7 +6588,7 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>One household per distribution; all stock changes succeed or none. Recheck availability and active status at save, prevent negative balances even under concurrent saves, record recorder/time/result. All three roles permitted. Explain and implement Distribution–Household and movement/Product/recorder links, authorization and transaction safeguards before enabling submission. Verify household details in history and the changed subcategory total.</t>
+          <t>One household per distribution; all stock changes succeed or none. Recheck availability and active status at save, prevent negative balances even under concurrent saves, record recorder/time/result. All three roles permitted. Explain and implement Distribution–Household and movement/Product/recorder links, authorization and transaction safeguards before enabling submission. Verify household details in history and the changed subcategory total. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
@@ -6632,15 +6627,14 @@
       <c r="Q69" s="11" t="n"/>
       <c r="R69" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S69" s="11" t="n"/>
     </row>
     <row r="70" ht="105" customHeight="1">
       <c r="A70" s="4" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
@@ -6659,7 +6653,7 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>Success message and read-only summary; failure retains entered data for correction. Prevent duplicate-click submission. Volunteer may see this result but not historical stock browsing; protect unrelated users’ accounts. Verify the already completed totals and product history reflect distribution, while volunteers see only their permitted result view.</t>
+          <t>Success message and read-only summary; failure retains entered data for correction. Prevent duplicate-click submission. Volunteer may see this result but not historical stock browsing; protect unrelated users’ accounts. Verify the already completed totals and product history reflect distribution, while volunteers see only their permitted result view. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -6698,15 +6692,14 @@
       <c r="Q70" s="10" t="n"/>
       <c r="R70" s="10" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S70" s="10" t="n"/>
     </row>
     <row r="71" ht="105" customHeight="1">
       <c r="A71" s="9" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B71" s="9" t="inlineStr">
         <is>
@@ -6725,7 +6718,7 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Review and test Receive/Adjust/Distribute totals/history, atomic rollback, concurrency/no negative stock, inactive/lock rules, one row/product, household selection, timestamps, immutable history and all-role permissions. Developer tests first; record automated evidence when delegated.</t>
+          <t>Review and test Receive/Adjust/Distribute totals/history, atomic rollback, concurrency/no negative stock, inactive/lock rules, one row/product, household selection, timestamps, immutable history and all-role permissions. Developer tests first; record automated evidence when delegated. 2026-10-29 module separation: sizes/units/balances/movements belong only to Stock Management; stock row identity is stock_items(product_id,package_size_id), referencing shared package_sizes. Preserve existing integrity/permission rules; do not create packaging fields on catalogue Product. Shared-package design: movement rows target stock_item_id; balances/history are per stock item, not per package definition; duplicate entry rows checked by stock_item_id. Package definition immutable as soon as referenced. Preserve approved movement safeguards.</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
@@ -6764,8 +6757,7 @@
       <c r="Q71" s="11" t="n"/>
       <c r="R71" s="11" t="inlineStr">
         <is>
-          <t>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Review and test completed Receive, Adjust and Distribute journeys together, including history and totals. Repeat affected catalogue-lock and permission checks after movement integration. This complements earlier module checks; it is not the first testing of those features.</t>
+          <t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</t>
         </is>
       </c>
       <c r="S71" s="11" t="n"/>
@@ -6953,7 +6945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7747,7 +7739,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Stories!B14</t>
+          <t>Stories!B7</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7938,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Stories!B12</t>
+          <t>Stories!B13</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8639,7 @@
       </c>
       <c r="F53" s="28" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8671,7 @@
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -8940,7 +8932,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -9166,7 +9158,7 @@
       </c>
       <c r="F69" s="28" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -9198,7 +9190,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -9230,7 +9222,7 @@
       </c>
       <c r="F71" s="28" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B9</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9287,7 @@
       </c>
       <c r="F73" s="28" t="inlineStr">
         <is>
-          <t>Stories!B16</t>
+          <t>Stories!B24</t>
         </is>
       </c>
     </row>
@@ -9327,7 +9319,7 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Stories!B23</t>
+          <t>Stories!B24</t>
         </is>
       </c>
     </row>
@@ -9359,7 +9351,7 @@
       </c>
       <c r="F75" s="28" t="inlineStr">
         <is>
-          <t>Stories!B23</t>
+          <t>Stories!B24</t>
         </is>
       </c>
     </row>
@@ -10163,7 +10155,7 @@
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>Every product has a unique, permanent, automatically generated code using the format PRD-000001, independent of its name and category. Use sequential numbers starting at 1, padded to at least six digits; allow longer numbers after PRD-999999. Users cannot edit product codes, and codes are never reused. Each separate product record, including brand and package-size variants, receives its own code.</t>
+          <t>Every product has a unique, permanent, automatically generated code using the format PRD-000001, independent of its name and category. Use sequential numbers starting at 1, padded to at least six digits; allow longer numbers after PRD-999999. Users cannot edit product codes, and codes are never reused. Each separate catalogue product record, including brand variants, receives its own code. Under the approved module separation, package sizes are reusable Stock Management definitions linked through stock_items; different package sizes of the same catalogue product share that product code. Neither a stock_items ID nor a package_sizes ID replaces the permanent catalogue product code.</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
@@ -10173,7 +10165,7 @@
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Stories!B38</t>
+          <t>Stories!B37</t>
         </is>
       </c>
     </row>
@@ -10451,7 +10443,7 @@
       </c>
       <c r="D109" s="28" t="inlineStr">
         <is>
-          <t>Different brands and package sizes are separate product records with their own stock counts, even when they share the same subcategory.</t>
+          <t>2026-10-29 approved module separation: Different brands remain distinguishable catalogue products. Package sizes and their separate stock balances belong exclusively to Stock Management; package size does not create a separate catalogue product. Exact stock-record structure will be settled before implementation. Shared package structure is now approved: products -&gt; stock_items &lt;- package_sizes; movements reference stock_items. See REQ-185.</t>
         </is>
       </c>
       <c r="E109" s="28" t="inlineStr">
@@ -10515,7 +10507,7 @@
       </c>
       <c r="D111" s="28" t="inlineStr">
         <is>
-          <t>Product form fields: required product name, full department/category/ subcategory selection, counting unit, positive contents per package/item, and status. Status defaults to Active. Brand and tags are optional. Choose a contents unit compatible with the selected subcategory's measure (weight, volume, or individual items). Product codes are generated automatically and stock starts at zero, not entered in this form.</t>
+          <t>2026-10-29 approved module separation: Product Catalogue form fields: required product name, full Department/Category/Subcategory selection and status (default Active); optional brand and tags. Product code generated automatically. No package size, counting/contents/summary unit, stock quantity, balance or calculated stock total in catalogue storage/forms/screens. Packaging and stock records belong to Stock Management.</t>
         </is>
       </c>
       <c r="E111" s="28" t="inlineStr">
@@ -10547,7 +10539,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Prevent duplicate products when name, brand, subcategory, counting unit, and package contents all match an existing product. Different brands or package sizes remain separate products. Ignore capitalization and surrounding spaces in product names and brands. Compare equivalent contents across units (500 g equals 0.5 kg; 500 ml equals 0.5 litres). Include inactive products in duplicate checks; reactivate the existing record instead of duplicating it.</t>
+          <t>2026-10-29 approved module separation: Prevent duplicate catalogue products by name, brand and Subcategory, ignoring capitalization and outer spaces in name/brand and including inactive products. Size/unit/quantity are excluded from catalogue identity and validation. Stock item product/package_size pairs are unique; reusable package definitions are unique by package type and equivalent contents.</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -10557,7 +10549,7 @@
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>Stories!B39</t>
+          <t>Stories!B38</t>
         </is>
       </c>
     </row>
@@ -10579,7 +10571,7 @@
       </c>
       <c r="D113" s="28" t="inlineStr">
         <is>
-          <t>First-version stock quantities are whole-number counts of packages or individual items. Each product has one counting unit, such as can, bag, or box. Package size describes the product; stock counts packages/items.</t>
+          <t>2026-10-29 approved module separation: Stock Management owns whole-number package/item quantities and counting units. Product Catalogue owns no counting units or quantity fields. Each stock package choice describes what is counted; exact stock-record design pending discussion. Shared package structure is now approved: products -&gt; stock_items &lt;- package_sizes; movements reference stock_items. See REQ-185.</t>
         </is>
       </c>
       <c r="E113" s="28" t="inlineStr">
@@ -10611,7 +10603,7 @@
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>Package contents measured in individual items must be a positive whole number (for example, 6 or 12 eggs per carton, never 6.5). Weight and volume contents may use up to three decimal places. Movement quantities remain whole packages/items regardless of how package contents are measured.</t>
+          <t>2026-10-29 approved module separation: Within Stock Management, package contents measured in individual items are positive whole numbers; weight/volume contents allow up to three decimal places. Movements remain whole packages/items. These fields do not belong to Product Catalogue.</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
@@ -10643,7 +10635,7 @@
       </c>
       <c r="D115" s="28" t="inlineStr">
         <is>
-          <t>Use fixed dropdown choices for counting units: bag, box, can, bottle, carton, jar, packet, and individual item.</t>
+          <t>2026-10-29 approved module separation: Stock Management counting-unit choices: bag, box, can, bottle, carton, jar, packet and individual item. No counting-unit field in catalogue.</t>
         </is>
       </c>
       <c r="E115" s="28" t="inlineStr">
@@ -10675,7 +10667,7 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>Subcategory summary unit choices remain kilograms, litres, and individual items. Product package sizes use their saved unit (kg/g or litres/ml). Automatically convert grams to kilograms and millilitres to litres when calculating subcategory totals, then multiply package contents by available whole-package counts and add the results. For example, four 500 g bags, three 1 kg bags, and two 5 kg bags total 15 kg. Product package sizes retain their saved units; conversion does not allow partial-package movements. Display combined weight/volume totals in kg or litres with at most three decimal places, allowing fewer digits (for example, 1 kg, 0.25 kg, 0.125 kg). Keep calculation values exact and round only the displayed total when needed. Individual product sizes display in their saved units. Existing unit-locking rules after stock movements still apply, including the saved package contents unit.</t>
+          <t>2026-10-29 approved module separation: Stock Management owns package sizes, contents units, summary units and calculated totals. Retain kg/g and litres/ml conversions and individual-item totals; exact values until display, at most three displayed decimals. Catalogue Subcategories have no summary-unit field. Placement/ownership of summary configuration within Stock Management must be agreed before implementation.</t>
         </is>
       </c>
       <c r="E116" s="4" t="inlineStr">
@@ -10803,7 +10795,7 @@
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>Each subcategory has one summary unit, such as kilograms or individual items. Every product specifies how much one package/item contains in a compatible unit; reconcile that unit with the summary unit for totals.</t>
+          <t>2026-10-29 approved module separation: Summary measurement configuration belongs exclusively to Stock Management. No summary-unit field on catalogue Subcategories. Stock product/package measurements must be compatible with stock summary configuration; exact configuration structure pending discussion.</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
@@ -10835,7 +10827,7 @@
       </c>
       <c r="D121" s="28" t="inlineStr">
         <is>
-          <t>Calculate subcategory totals by multiplying each product's whole-number stock count by its package contents and summing the results. For example, rice bags contribute kilograms and egg cartons contribute eggs.</t>
+          <t>2026-10-29 approved module separation: In Stock Management, multiply each stock package count by its contents and sum compatible measurements; for example rice bags contribute kilograms and cartons contribute eggs. These totals are absent from catalogue screens.</t>
         </is>
       </c>
       <c r="E121" s="28" t="inlineStr">
@@ -10867,7 +10859,7 @@
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>These calculated summaries do not replace individual product balances.</t>
+          <t>2026-10-29 approved module separation: Stock summaries do not replace individual stock package balances. All balances/totals are owned and displayed by Stock Management only.</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
@@ -11059,7 +11051,7 @@
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>Distribution flow: search/select one household by reference, contact name, or phone; select a subcategory such as Rice, then choose from its active products with stock greater than zero. Show available package sizes, product name, brand, product code, and available package counts so equal sizes from different products remain distinguishable. Retain product search by code or name within this selection flow. Users can select multiple products/sizes and enter positive whole-number quantities; review the household and product quantities before confirming. Recheck stock when saving. On success, show a success message and read-only distribution summary. On failure, retain entered information so staff can correct it.</t>
+          <t>Distribution flow: search/select one household by reference, contact name, or phone; select a subcategory such as Rice, then choose from its active products with stock greater than zero. Show available package sizes, product name, brand, product code, and available package counts so equal sizes from different products remain distinguishable. Retain product search by code or name within this selection flow. Users can select multiple products/sizes and enter positive whole-number quantities; review the household and product quantities before confirming. Recheck stock when saving. On success, show a success message and read-only distribution summary. On failure, retain entered information so staff can correct it. 2026-10-29 clarification: package choices and quantities are selected in Stock Management only; catalogue contains no such fields. Selectable stock rows are stock_items, each connecting an active product and package_sizes definition.</t>
         </is>
       </c>
       <c r="E128" s="4" t="inlineStr">
@@ -11123,7 +11115,7 @@
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>Each product may appear only once per Receive or Distribute entry. To change the amount, update its existing row's quantity rather than adding another row. Different products or package sizes may have separate rows.</t>
+          <t>Each stock_item may appear once per Receive or Distribute entry. Update its existing quantity instead of duplicate rows. The same catalogue product can appear on separate rows with different package_sizes. Quantities/packages belong exclusively to Stock Management.</t>
         </is>
       </c>
       <c r="E130" s="4" t="inlineStr">
@@ -11251,7 +11243,7 @@
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>Each Adjust entry handles one product. The user selects Add or Remove, enters a positive whole-number quantity, and provides a required reason. Removing stock must still respect the non-negative balance rule.</t>
+          <t>Each Adjust entry handles one stock_item (a product/package-size combination), Add or Remove, positive whole-number quantity and mandatory reason. Prevent negative balance. All packaging/quantities stay in Stock Management.</t>
         </is>
       </c>
       <c r="E134" s="4" t="inlineStr">
@@ -11283,7 +11275,7 @@
       </c>
       <c r="D135" s="28" t="inlineStr">
         <is>
-          <t>Managers and the Super Admin can view each product's stock-movement history in version one. Show movement type, quantity added or removed, date/time, resulting balance, who recorded it, and relevant details such as the receipt, distribution household, or adjustment reason.</t>
+          <t>2026-10-29 approved module separation: Within Stock Management, Managers/Super Admin can view movement history with movement type, quantity added/removed, save time, resulting balance, recorder and receipt/household/reason details. No stock history on catalogue product details.</t>
         </is>
       </c>
       <c r="E135" s="28" t="inlineStr">
@@ -11315,7 +11307,7 @@
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>Show product stock-movement history on the product details page and combined subcategory totals on the subcategory management screen, for managers and the Super Admin. Volunteers cannot view stock history.</t>
+          <t>2026-10-29 approved module separation: Show balances, movement history and combined summaries exclusively in Stock Management. No quantities, sizes, units or totals in Product Catalogue, including catalogue Subcategory screens. Existing history permission restriction remains: Volunteers cannot browse stock history.</t>
         </is>
       </c>
       <c r="E136" s="4" t="inlineStr">
@@ -11411,7 +11403,7 @@
       </c>
       <c r="D139" s="28" t="inlineStr">
         <is>
-          <t>New products start with zero stock. Add any existing stock through a Receive entry so every opening quantity has a recorded origin.</t>
+          <t>2026-10-29 approved module separation: Creating a catalogue product creates no stock quantity. Stock Management starts its stock records at zero and records opening stock through Receive so each quantity has an origin.</t>
         </is>
       </c>
       <c r="E139" s="28" t="inlineStr">
@@ -11443,7 +11435,7 @@
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>Products use Active/Inactive status instead of deletion in version one. A product can only be deactivated when its stock is zero. Inactive products cannot receive any stock movements until reactivated, but their records and stock-movement history remain available.</t>
+          <t>2026-10-29 approved module separation: Products use Active/Inactive instead of deletion. Product deactivation is blocked if ANY stock remains for that product across Stock Management records. Catalogue performs a server-side availability check without displaying sizes/quantities. A generic explanation may say stock remains. Inactive products cannot receive movements until reactivated; records/history retained.</t>
         </is>
       </c>
       <c r="E140" s="4" t="inlineStr">
@@ -11453,7 +11445,7 @@
       </c>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>Stories!B51</t>
+          <t>Stories!B50</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11467,7 @@
       </c>
       <c r="D141" s="28" t="inlineStr">
         <is>
-          <t>After a product's first stock movement, lock its counting unit, package contents, and subcategory. Names and tags remain editable. Different package sizes require separate product records.</t>
+          <t>Shared package_sizes package type/contents/unit become immutable once ANY stock_item references the definition, protecting every linked product. stock_items product/package_size identity must preserve movement history. No packaging fields on catalogue products. Catalogue classification/history constraints still require a focused decision before stock implementation.</t>
         </is>
       </c>
       <c r="E141" s="28" t="inlineStr">
@@ -11507,7 +11499,7 @@
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>Lock a subcategory's summary unit once any product beneath it has a stock movement, preserving the meaning of product contents and totals. Receiving and issuing stock still uses whole packages/items of a specific product; partial-package movements are outside current scope.</t>
+          <t>2026-10-29 approved module separation: Lock Stock Management summary measurement configuration after affected stock movements, preserving meaning of package contents and totals. Catalogue Subcategories have no summary-unit field. Exact summary configuration owner pending design discussion.</t>
         </is>
       </c>
       <c r="E142" s="4" t="inlineStr">
@@ -11539,7 +11531,7 @@
       </c>
       <c r="D143" s="28" t="inlineStr">
         <is>
-          <t>Consistent units within a subcategory and readable summary formatting are in scope; general unit conversions and loose-weight movements remain future work.</t>
+          <t>2026-10-29 approved module separation: Consistent stock measurement and readable summary formatting belong exclusively to Stock Management. General unit conversion/loose-weight movements remain future scope.</t>
         </is>
       </c>
       <c r="E143" s="28" t="inlineStr">
@@ -11603,7 +11595,7 @@
       </c>
       <c r="D145" s="28" t="inlineStr">
         <is>
-          <t>Include a product list showing product code, product name, category path, package contents, available stock, and status. Managers, the Super Admin, and volunteers can search by product code or product name and filter by department, category, subcategory, tag, and Active/Inactive status.</t>
+          <t>2026-10-29 approved module separation: Catalogue list shows product code, product name, category path, optional brand/tags and status; NO sizes, units, quantities, available stock or totals. Retain all-role search by code/name and filters for Department, Category, Subcategory, tag and status. Stock Management supplies its separate quantity/size views.</t>
         </is>
       </c>
       <c r="E145" s="28" t="inlineStr">
@@ -11613,7 +11605,7 @@
       </c>
       <c r="F145" s="28" t="inlineStr">
         <is>
-          <t>Stories!B40</t>
+          <t>Stories!B39</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11637,7 @@
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>Stories!B40</t>
+          <t>Stories!B39</t>
         </is>
       </c>
     </row>
@@ -11677,7 +11669,7 @@
       </c>
       <c r="F147" s="28" t="inlineStr">
         <is>
-          <t>Stories!B52</t>
+          <t>Stories!B51</t>
         </is>
       </c>
     </row>
@@ -11709,7 +11701,7 @@
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>Stories!B52</t>
+          <t>Stories!B51</t>
         </is>
       </c>
     </row>
@@ -11837,7 +11829,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>Stories!B51</t>
+          <t>Stories!B50</t>
         </is>
       </c>
     </row>
@@ -11869,7 +11861,7 @@
       </c>
       <c r="F153" s="28" t="inlineStr">
         <is>
-          <t>Stories!B52</t>
+          <t>Stories!B51</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11893,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>Stories!B52</t>
+          <t>Stories!B51</t>
         </is>
       </c>
     </row>
@@ -12941,6 +12933,102 @@
       <c r="F186" t="inlineStr">
         <is>
           <t>Stories!B31</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>REQ-184</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Module separation</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Current scope</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>2026-10-29 approved: Product Catalogue manages classification, product identity/description, optional brand/tags and status only. Stock Management owns all package sizes/types, counting/contents/summary units, quantities, receiving, distributing, adjustments, balances, totals and history. Catalogue must show no sizes or quantities. Block deactivation while any related stock remains through a server-side stock check. This supersedes prior package-on-product and Subcategory-summary-unit rules. Modules share product identity within one application; reusable package_sizes + product/package stock_items + stock_movements structure is now approved (see shared-package requirement). Summary configuration, package-management permissions and classification-lock details remain to be settled before implementation. Subcategory creation now requires only Category and name.</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>FB-029–FB-068</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Stories!B32</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>REQ-185</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Stock Management — shared package definitions</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Current scope</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>2026-10-29 approved shared package design: Stock Management has package_sizes(id, package_type, contents, contents_unit), reusable across products; stock_items(id, product_id, package_size_id) links each catalogue product to a package definition. One unique product/package_size pair. stock_movements belongs to stock_item_id, so balances/history are separate even when package definitions are shared. Product catalogue has no size/unit/quantity fields or displays. Examples: Rice and Lentils share Bag5kg; Milk and Juice share Carton2litres; Eggs uses Carton12items (12 eggs/carton). Keep positive whole package movement quantities and whole-number individual-item contents. Reject duplicate package definitions, comparing equivalent kg/g and litres/ml contents within the same package type; a bottle differs from a carton. Once referenced by a stock item, package type/contents/unit are immutable; create another definition instead. This stronger shared-definition lock supersedes the earlier first-movement-only package lock. Shared package-size management permissions/UI, summary-configuration ownership and classification-lock details still need focused decisions before implementation. No loose-egg repacking workflow approved.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>FB-034, FB-049–FB-056, FB-059–FB-068</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Stories!B52</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>REQ-186</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Product Catalogue — Subcategory creation</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Current scope</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>2026-10-29 approved Subcategory creation UI: Department dropdown, Category dropdown and required Subcategory name only. Category choices belong to selected Department; changing Department clears Category. Server validates existing Department/Category and their matching relationship. Persist Category link (category_id); Department is derived through Category rather than duplicated on Subcategory. No units, sizes, package or quantity fields. Inventory/catalogue completion remains the focus; stock design and size-specific code discussion are deferred, not new approved implementation. Original Subcategory scaffold/migration remain reverted/unstarted.</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>FB-029</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Stories!B32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add product creation with shared tags and validation
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rb829a08804ff497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R9f92529da0b1469f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rf034994724984047"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5072960b892545b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R729ccbd23610418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R415a6c94041e4a77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -637,7 +637,7 @@
       </x:c>
       <x:c r="B6" s="15" t="n">
         <x:f>COUNTIF(Stories!H4:H73,"Complete")</x:f>
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C6" s="15" t="n"/>
       <x:c r="D6" s="18" t="inlineStr">
@@ -694,7 +694,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>FB-032</x:v>
+        <x:v>FB-038</x:v>
       </x:c>
       <x:c r="C10" s="15" t="n"/>
       <x:c r="D10" s="18" t="inlineStr">
@@ -710,14 +710,14 @@
         </x:is>
       </x:c>
       <x:c r="B11" s="29" t="str">
-        <x:v>2026-10-30 Department, Category, Subcategory and Tags modules verified. Tags create/list/search/rename reviewed and tested; Product connections remain future checkpoints. Account deferrals preserved.</x:v>
+        <x:v>2026-10-30 hierarchy/Tags modules and Product creation verified. Product form saves catalogue fields and shared tags in both directions, with permissions/duplicate safeguards. Product list not started; account deferrals and baseline test failures preserved.</x:v>
       </x:c>
       <x:c r="C11" s="15" t="n"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="15" t="n"/>
       <x:c r="B12" s="15" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read FB-032 and related Requirements before beginning Products. Tags FB-031 verified; product-tag attachment and deletion stay at FB-037/048. User delegated Tags only. Explain Product storage/form progression in small lessons; do not write Product code without explicit authorization.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read full FB-038 and related Requirements before starting list. Product creation FB-032/033/036/037 verified with scoped checks; baseline global failures remain recorded. Next preview basic unfiltered Product list showing name/path/brand/tags/status, all-role server viewAny permission, no codes/stock fields. Complete basic list before filters; main name-or-tag search later FB-040 and tag filterFB-044. Preserve show-before-apply preference; current Product save/testing delegation does not automatically authorize unrelated list implementation. Product code decision stays after catalogue verification at FB-035; Stock Management not started.</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n"/>
       <x:c r="D12" s="15" t="n"/>
@@ -733,7 +733,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>FB-032</x:v>
+        <x:v>FB-038</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="100" customHeight="1">
@@ -743,7 +743,8 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>Tags FB-031 verified. Product storage/form FB-032 ready for its first small lesson; not started.</x:v>
+        <x:v>Product creation checkpoint complete after source review,157-test catalogue pass, MySQL concurrency and browser checks. Basic Product list is next; not started.
+Separate completed repair: 2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -753,7 +754,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read FB-032 and related Requirements before beginning Products. Tags FB-031 verified; product-tag attachment and deletion stay at FB-037/048. User delegated Tags only. Explain Product storage/form progression in small lessons; do not write Product code without explicit authorization.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read full FB-038 and related Requirements before starting list. Product creation FB-032/033/036/037 verified with scoped checks; baseline global failures remain recorded. Next preview basic unfiltered Product list showing name/path/brand/tags/status, all-role server viewAny permission, no codes/stock fields. Complete basic list before filters; main name-or-tag search later FB-040 and tag filterFB-044. Preserve show-before-apply preference; current Product save/testing delegation does not automatically authorize unrelated list implementation. Product code decision stays after catalogue verification at FB-035; Stock Management not started.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -763,7 +764,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Developer request to begin the Product module.</x:v>
+        <x:v>Developer readiness to begin basic Product list; show changes first.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -773,7 +774,7 @@
         </x:is>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>eabb3204ee4e2f9dbea824ef3b5939230e379d20 + uncommitted Tag files; completed-feature source review 2026-10-30.</x:v>
+        <x:v>HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -927,15 +928,14 @@
           <x:t xml:space="preserve">Reference format</x:t>
         </x:is>
       </x:c>
-      <x:c r="B30" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Order: FB-016/017/018, prepare FB-020, FB-019, FB-006/007, FB-024, FB-009–015, FB-008, remaining accounts. Catalogue modules create before list; Product already does. Super Admin recovery stays last.
+      <x:c r="B30" s="18" t="str">
+        <x:v>2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Order: FB-016/017/018, prepare FB-020, FB-019, FB-006/007, FB-024, FB-009–015, FB-008, remaining accounts. Catalogue modules create before list; Product already does. Super Admin recovery stays last.
 2026-10-27 sequence decision: place the bcrypt 72-byte repair and repeat test within FB-069, immediately before final FB-070. Existing first-login review/test failures remain recorded; this timing change does not verify them.
 2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
 2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.
 2026-10-29 approved Product Catalogue/Stock Management separation recorded in revised Requirements. Catalogue excludes all size/unit/quantity/history data, including Subcategory summary units; deactivation server-checks Stock Management and blocks while ANY stock remains without displaying counts. Stable FB-034 repurposed/moved after catalogue checkpoint FB-067 and before FB-049 Receive; Product code FB-035 now depends on FB-033. Stock package-record structure/summary owner/classification locks remain open before stock implementation. Subcategory creation revert preserved; no code changes in design discussion.
-2026-10-29 planning approval: reusable package_sizes in Stock Management; stock_items connects product_id/package_size_id and owns separate movement/balance identity. See shared-package Requirement/FB-034. Current Subcategory still Category+name only and unstarted after revert. No application code/migrations or feature tests run for this planning change.</x:t>
-        </x:is>
+2026-10-29 planning approval: reusable package_sizes in Stock Management; stock_items connects product_id/package_size_id and owns separate movement/balance identity. See shared-package Requirement/FB-034. Current Subcategory still Category+name only and unstarted after revert. No application code/migrations or feature tests run for this planning change.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="44" customHeight="1">
@@ -992,11 +992,11 @@
           <x:t xml:space="preserve">Application test status</x:t>
         </x:is>
       </x:c>
-      <x:c r="B35" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-26: assistant-delegated php artisan test PASS, 35 tests, 115 assertions; git diff --check passed. Developer-reported browser PASS: full name/initials, Settings Security/Appearance, /settings/profile 404. Account-creation journey remains incomplete. Earlier login test results retained as historical evidence.
-2026-10-26 developer-reported PASS: after explicit fictional-account browser save and database inspection instructions, developer confirmed everything worked, account created, and invalid-input checks behaved as expected. This confirms the requested dashboard/success and stored-field checks, including role/status/setup flag/password hash, as developer reports only. Additional invalid-input cases were not enumerated; do not claim exhaustive validation, denied-access, concurrency or first-login testing.</x:t>
-        </x:is>
+      <x:c r="B35" s="18" t="str">
+        <x:v>2026-10-26: assistant-delegated php artisan test PASS, 35 tests, 115 assertions; git diff --check passed. Developer-reported browser PASS: full name/initials, Settings Security/Appearance, /settings/profile 404. Account-creation journey remains incomplete. Earlier login test results retained as historical evidence.
+2026-10-26 developer-reported PASS: after explicit fictional-account browser save and database inspection instructions, developer confirmed everything worked, account created, and invalid-input checks behaved as expected. This confirms the requested dashboard/success and stored-field checks, including role/status/setup flag/password hash, as developer reports only. Additional invalid-input cases were not enumerated; do not claim exhaustive validation, denied-access, concurrency or first-login testing.
+2026-10-30 user delegated full tests for Product save. Full suite192/174 pass/17 failed/1 error; isolated HEAD snapshot150/132 pass/17 failed/1 error has identical failing/error test names. Auth/logout/email verification/password confirmation/verification notifications/dashboard/example/settings/security fixtures and UserSeeding assumptions are existing baseline failures. Source inspection: factory does not explicitly set active/setup-complete flags for in-memory auth tests; seeding tests expect one user while DatabaseSeeder includes DemoUserSeeder. No account/source fixes made; earlier project-end deferrals preserved. Full PHPStan7 existing unrelated catalogue annotation/empty-controller-stub issues unchanged; new Product scope PHPStan0 errors.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -3760,12 +3760,12 @@
           <x:t xml:space="preserve">Changes needed</x:t>
         </x:is>
       </x:c>
-      <x:c r="K28" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">
+      <x:c r="K28" s="10" t="str">
+        <x:v>
 2026-10-29 developer explicitly delegated completed user-module code review and own-browser testing, excluding every project-end deferral. Review snapshot HEAD91e157fb6d367016ef7181ce50ad81115e9648da plus existing working-tree Index.vue Edit-click and web.php root-route edits. Read UserController, UserPolicy, ListUsers, GetAssignableRoles, GenerateUsername, Store/Update/IndexUsersRequest, User/Role/RoleCode, active/setup guards and registration, Inertia shared data, protected user routes, users Create/Show/Edit/Index, sidebar/My details/account menu, user schema/factory and relevant existing tests. Password workflows/FB-024 review, FB-008/023, bcrypt, phone cleanup, username simultaneous-save fix and mobile directory are excluded. Findings: (1) REPRODUCED browser/MySQL PATCH500: first_name and last_name each100 Æ pass agreed100-character validation and generator rules, transliterate to401-character username, but users.username is varchar255; SQLSTATE22001/1406 at UserController update161. Applies to create/edit generation. No source fix applied. (2) repository DashboardTest authenticated test and ProfileUpdateTest settings redirect test fail: factory-created in-memory users omit explicit active/setup-complete values needed by current middleware; fixtures/assertions need correction. (3) PHPStan512M reports9 errors:6 missing array/generic/callback type descriptions in ListUsers;3 mutable-Carbon vs CarbonImmutable annotation mismatches in UserController68, DemoUserSeeder68, SuperAdminSeeder35 against User model email_verified_at annotation. Review remains Changes needed; do not start inventory on a claimed clean pass.
-2026-10-29 developer explicitly authorized resolving the nine PHP type-description errors only. Assistant changed ListUsers method PHPDoc to describe optional search string/null, Builder&lt;User&gt;, paginator integer keys/prepared row values, and prepared row key/value types; User date import/properties now CarbonImmutable, matching AppServiceProvider Date::use and actual model datetime casts. No runtime behavior changes. Scoped diff/source review PASS. app/Actions/Users/ListUsers.php SHA256 2d6479cf5525d05cd23f6620749486a1ff479d242bb59c285800713e968c0d07; app/Models/User.php SHA256 6200c8c7f6c76054dd5a8e046d639d1a11a893d73360404f568946da383892e6. PHPStan512M PASS zero errors; targeted Pint PASS; whitespace PASS; external isolated SQLite ListEditPermissionTest21tests288assertions PASS. Read-only unsaved model check confirms email_verified_at/created_at/updated_at resolve CarbonImmutable; initial check incorrectly passed these guarded date fields to constructor, corrected harness to direct assignments, no source defect. No live DB writes/users created, no browser checks or unrelated/password tests. Earlier long-name MySQL500 and two existing test failures remain unresolved; all project-end deferrals retained. This supersedes only the nine-error finding, not full user-module review/test status.</x:t>
-        </x:is>
+2026-10-29 developer explicitly authorized resolving the nine PHP type-description errors only. Assistant changed ListUsers method PHPDoc to describe optional search string/null, Builder&lt;User&gt;, paginator integer keys/prepared row values, and prepared row key/value types; User date import/properties now CarbonImmutable, matching AppServiceProvider Date::use and actual model datetime casts. No runtime behavior changes. Scoped diff/source review PASS. app/Actions/Users/ListUsers.php SHA256 2d6479cf5525d05cd23f6620749486a1ff479d242bb59c285800713e968c0d07; app/Models/User.php SHA256 6200c8c7f6c76054dd5a8e046d639d1a11a893d73360404f568946da383892e6. PHPStan512M PASS zero errors; targeted Pint PASS; whitespace PASS; external isolated SQLite ListEditPermissionTest21tests288assertions PASS. Read-only unsaved model check confirms email_verified_at/created_at/updated_at resolve CarbonImmutable; initial check incorrectly passed these guarded date fields to constructor, corrected harness to direct assignments, no source defect. No live DB writes/users created, no browser checks or unrelated/password tests. Earlier long-name MySQL500 and two existing test failures remain unresolved; all project-end deferrals retained. This supersedes only the nine-error finding, not full user-module review/test status.
+2026-10-30 user delegated full tests for Product save. Full suite192/174 pass/17 failed/1 error; isolated HEAD snapshot150/132 pass/17 failed/1 error has identical failing/error test names. Auth/logout/email verification/password confirmation/verification notifications/dashboard/example/settings/security fixtures and UserSeeding assumptions are existing baseline failures. Source inspection: factory does not explicitly set active/setup-complete flags for in-memory auth tests; seeding tests expect one user while DatabaseSeeder includes DemoUserSeeder. No account/source fixes made; earlier project-end deferrals preserved. Full PHPStan7 existing unrelated catalogue annotation/empty-controller-stub issues unchanged; new Product scope PHPStan0 errors.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L28" s="30" t="n">
         <x:v>46324</x:v>
@@ -3851,11 +3851,10 @@
           <x:t xml:space="preserve">Passed</x:t>
         </x:is>
       </x:c>
-      <x:c r="K29" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29 requested intermediate scaffold review: Department model empty; migration id/timestamps only; seeder empty; controller methods empty; Store/Update requests authorize=false with empty rules; policy denies all. Namespaces/imports correctly placed. No Department routes or Vue UI. Not feature completion; no application tests run or edits made. Poker reference inspected: Models/Player.php protected $fillable; Requests/Players/StorePlayerRequest.php validation; Policies/PlayerPolicy.php abilities; PlayerController.php validated simple saves/Inertia feedback; routes/web.php -&gt;can on display/write. HEAD befad9c75df55a0608a1ee45f68792d80996232a Snapshot SHA256: app/Models/Department.php c0e27aa79fab4cc4c6f1fa3dc0d39bb7a0bebaaa92edd06185e2c65fa492f3e8; database/migrations/2026_10_29_121954_create_departments_table.php ca713f8069394dcd2bc21d6c8e9e1eaebb6eb9c6e76cb69766fc8530a181e28e; database/seeders/DepartmentSeeder.php af1151523a40742dfdb1bbd8008fe92d60d2634e241e71427843fd68da4b5eb4; app/Http/Controllers/DepartmentController.php 1156ecf4b4f75bb6ed06a8185e36256a313e75acd41d4ef3f0aeada1706c552b; app/Http/Requests/Departments/StoreDepartmentRequest.php f22e783ca2e5201002eef108468ebf022050c06301ed355fb280f7585f6202d5; app/Http/Requests/Departments/UpdateDepartmentRequest.php 3150a0f8c9bafb83180818233de0d9a6f000eebfba65f44a70bf5e3a80a95b6c; app/Policies/DepartmentPolicy.php 1cc1c746232f3149db409af77393d9f3e600de0e7748f5d341d867ff0815ba6e; routes/web.php 93ccbe0e562268518969445fb2e3f0906a8294a95e7ff37300c9fb891f3079c2
-2026-10-29 completed creation source review at HEAD befad9c75df55a0608a1ee45f68792d80996232a plus current working files: Passed, no blocking functional findings. GET/POST auth+create policy Manager/Super Admin; FormRequest validated required string max255 unique; Laravel standard trimming retained; migration unique name and model fillable; controller validated save/flash/back; Vue reactive binding, error display, processing disabled, success reset, responsive field/button; repeatable seeder. Unused policy Response import/import order/whitespace are cosmetic cleanup only. Index/edit/update remain unused scaffold and outside creation verification. No assistant application tests/browser checks. Snapshot SHA256: app/Models/Department.php 137bfc6b754c5fe00eb129777ea2a900242c495684a9225c1699ea9888118a7c; database/migrations/2026_10_29_121954_create_departments_table.php 8734f6600b1ec7fa25ff9cf1bf994f2ea23d58a1c72404cdfd1b0ac385d7eb70; database/seeders/DepartmentSeeder.php f41eb90ea8bd6350fc0dc6c61b2aff8b990f4e67bd4387efb57981beb64acdf9; app/Policies/DepartmentPolicy.php f2daa67a85b43b239152639f654d91171ed7dbf687f279fea36fc5fd3680db86; app/Http/Requests/Departments/StoreDepartmentRequest.php 6ce5d49bf67923ef0fbf45bef51c9473bf67ae456a453dfb32778bc263528aa8; app/Http/Controllers/DepartmentController.php 3ca3024e3b534ad236999bf1a2d6c63dd9990f92871f8d50c51cafebd8502381; resources/js/pages/departments/Create.vue 3718a428704dd69322e36f0146be784dbdaaca4be9a55a8c9aac52183f608b1e; routes/web.php 08b9ccec98fe21124a6f7fd98fc20a4a23d8519d2c34a9538693c7e971440f64</x:t>
-        </x:is>
+      <x:c r="K29" s="11" t="str">
+        <x:v>2026-10-29 requested intermediate scaffold review: Department model empty; migration id/timestamps only; seeder empty; controller methods empty; Store/Update requests authorize=false with empty rules; policy denies all. Namespaces/imports correctly placed. No Department routes or Vue UI. Not feature completion; no application tests run or edits made. Poker reference inspected: Models/Player.php protected $fillable; Requests/Players/StorePlayerRequest.php validation; Policies/PlayerPolicy.php abilities; PlayerController.php validated simple saves/Inertia feedback; routes/web.php -&gt;can on display/write. HEAD befad9c75df55a0608a1ee45f68792d80996232a Snapshot SHA256: app/Models/Department.php c0e27aa79fab4cc4c6f1fa3dc0d39bb7a0bebaaa92edd06185e2c65fa492f3e8; database/migrations/2026_10_29_121954_create_departments_table.php ca713f8069394dcd2bc21d6c8e9e1eaebb6eb9c6e76cb69766fc8530a181e28e; database/seeders/DepartmentSeeder.php af1151523a40742dfdb1bbd8008fe92d60d2634e241e71427843fd68da4b5eb4; app/Http/Controllers/DepartmentController.php 1156ecf4b4f75bb6ed06a8185e36256a313e75acd41d4ef3f0aeada1706c552b; app/Http/Requests/Departments/StoreDepartmentRequest.php f22e783ca2e5201002eef108468ebf022050c06301ed355fb280f7585f6202d5; app/Http/Requests/Departments/UpdateDepartmentRequest.php 3150a0f8c9bafb83180818233de0d9a6f000eebfba65f44a70bf5e3a80a95b6c; app/Policies/DepartmentPolicy.php 1cc1c746232f3149db409af77393d9f3e600de0e7748f5d341d867ff0815ba6e; routes/web.php 93ccbe0e562268518969445fb2e3f0906a8294a95e7ff37300c9fb891f3079c2
+2026-10-29 completed creation source review at HEAD befad9c75df55a0608a1ee45f68792d80996232a plus current working files: Passed, no blocking functional findings. GET/POST auth+create policy Manager/Super Admin; FormRequest validated required string max255 unique; Laravel standard trimming retained; migration unique name and model fillable; controller validated save/flash/back; Vue reactive binding, error display, processing disabled, success reset, responsive field/button; repeatable seeder. Unused policy Response import/import order/whitespace are cosmetic cleanup only. Index/edit/update remain unused scaffold and outside creation verification. No assistant application tests/browser checks. Snapshot SHA256: app/Models/Department.php 137bfc6b754c5fe00eb129777ea2a900242c495684a9225c1699ea9888118a7c; database/migrations/2026_10_29_121954_create_departments_table.php 8734f6600b1ec7fa25ff9cf1bf994f2ea23d58a1c72404cdfd1b0ac385d7eb70; database/seeders/DepartmentSeeder.php f41eb90ea8bd6350fc0dc6c61b2aff8b990f4e67bd4387efb57981beb64acdf9; app/Policies/DepartmentPolicy.php f2daa67a85b43b239152639f654d91171ed7dbf687f279fea36fc5fd3680db86; app/Http/Requests/Departments/StoreDepartmentRequest.php 6ce5d49bf67923ef0fbf45bef51c9473bf67ae456a453dfb32778bc263528aa8; app/Http/Controllers/DepartmentController.php 3ca3024e3b534ad236999bf1a2d6c63dd9990f92871f8d50c51cafebd8502381; resources/js/pages/departments/Create.vue 3718a428704dd69322e36f0146be784dbdaaca4be9a55a8c9aac52183f608b1e; routes/web.php 08b9ccec98fe21124a6f7fd98fc20a4a23d8519d2c34a9538693c7e971440f64
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L29" s="31" t="n">
         <x:v>46324</x:v>
@@ -3939,10 +3938,9 @@
           <x:t xml:space="preserve">Passed</x:t>
         </x:is>
       </x:c>
-      <x:c r="K30" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29: User explicitly authorized full assistant implementation of Department edit following Edit User coding/layout. Reviewed Department controller, update/store/index requests, policy, model, migration, ListDepartments, Index/Create/Edit Vue pages, routes and new DepartmentEditTest. Edit/update routes enforce update policy; request repeats authorization and unique-name validation ignoring bound record; Laravel trims outer spaces, configured MySQL utf8mb4_unicode_ci ignores case. Update changes validated name only and preserves ID; success flash and redirect to list; prefill/errors/processing/Cancel match users/Edit. PHP syntax, targeted Pint and Vue type checks passed. Application tests/browser checks NOT run: developer-first verification pending. Child-link behavior must be repeated after Category exists. Reference inspected: skander/app/Http/Controllers/PlayerController.php and app/Http/Requests/Players/UpdatePlayerRequest.php; route policy + request authorization, simple controller update, Inertia flash. Snapshot base c1c0a96 + working changes: app/Http/Controllers/DepartmentController.php sha256:19d121961aa2; app/Http/Requests/Departments/UpdateDepartmentRequest.php sha256:ef403a4eef70; routes/web.php sha256:0fb8147a54fa; resources/js/pages/departments/Edit.vue sha256:6e67b2b73176; tests/Feature/DepartmentEditTest.php sha256:1322bfe93bfa</x:t>
-        </x:is>
+      <x:c r="K30" s="10" t="str">
+        <x:v>2026-10-29: User explicitly authorized full assistant implementation of Department edit following Edit User coding/layout. Reviewed Department controller, update/store/index requests, policy, model, migration, ListDepartments, Index/Create/Edit Vue pages, routes and new DepartmentEditTest. Edit/update routes enforce update policy; request repeats authorization and unique-name validation ignoring bound record; Laravel trims outer spaces, configured MySQL utf8mb4_unicode_ci ignores case. Update changes validated name only and preserves ID; success flash and redirect to list; prefill/errors/processing/Cancel match users/Edit. PHP syntax, targeted Pint and Vue type checks passed. Application tests/browser checks NOT run: developer-first verification pending. Child-link behavior must be repeated after Category exists. Reference inspected: skander/app/Http/Controllers/PlayerController.php and app/Http/Requests/Players/UpdatePlayerRequest.php; route policy + request authorization, simple controller update, Inertia flash. Snapshot base c1c0a96 + working changes: app/Http/Controllers/DepartmentController.php sha256:19d121961aa2; app/Http/Requests/Departments/UpdateDepartmentRequest.php sha256:ef403a4eef70; routes/web.php sha256:0fb8147a54fa; resources/js/pages/departments/Edit.vue sha256:6e67b2b73176; tests/Feature/DepartmentEditTest.php sha256:1322bfe93bfa
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L30" s="30" t="n">
         <x:v>46324</x:v>
@@ -4040,11 +4038,10 @@
           <x:t xml:space="preserve">Passed</x:t>
         </x:is>
       </x:c>
-      <x:c r="K31" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29 completed Category module source review passed: reviewed app/Http/Controllers/CategoryController.php, app/Policies/CategoryPolicy.php, app/Http/Requests/Categories/StoreCategoryRequest.php, app/Http/Requests/Categories/UpdateCategoryRequest.php, app/Http/Requests/Categories/IndexCategoriesRequest.php, app/Actions/Categories/ListCategories.php, app/Models/Category.php, app/Models/Department.php, database/migrations/2026_10_29_210437_create_categories_table.php, routes/web.php, resources/js/pages/categories/Create.vue, resources/js/pages/categories/Index.vue, resources/js/pages/categories/Edit.vue, tests/Feature/CategoryEditTest.php. Protected create/viewAny/update routes; repeated create/update request authorization; scoped name uniqueness; update ignores submitted parent/ID and validates only name against SAVED department; existing ID and parent retained. Eager-loaded parent on list/edit; stable pagination, OR name search, Vue form error/processing/cancel and success feedback. Following inspected Poker controller/request/route patterns and current Department edit. No blocking findings. Snapshots: app/Http/Controllers/CategoryController.php 8bd02ab4a46c; app/Policies/CategoryPolicy.php 727780b74cc6; app/Http/Requests/Categories/StoreCategoryRequest.php 5819301d79ab; app/Http/Requests/Categories/UpdateCategoryRequest.php fa34e0cb7cab; app/Http/Requests/Categories/IndexCategoriesRequest.php 6167bfe92ae6; app/Actions/Categories/ListCategories.php 0b8499c42ea0; app/Models/Category.php 714239df06eb; app/Models/Department.php 77c81e2ce045; database/migrations/2026_10_29_210437_create_categories_table.php 50ae1cd2d815; routes/web.php dab57df7c166; resources/js/pages/categories/Create.vue b47f65a7e2b2; resources/js/pages/categories/Index.vue ca004b43eb2e; resources/js/pages/categories/Edit.vue a4ee52f1f872; tests/Feature/CategoryEditTest.php b87e2c7bcb0a
-2026-10-29 user approved/authorized Category department moves, superseding fixed-parent rule for Category only. Controller supplies alphabetical departments; Edit uses shared Select preselected via String(saved ID), and Edit User window.confirm pattern on Save only when parent changes (old/new names). Cancel returns before PATCH. Request requires existing integer department and scopes unique name to selected department; controller persists validated name+department_id, preserving ID. Reviewed all changed source and tests; no findings. PASS delegated php artisan test tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php:29 tests183 assertions (SQLite). Updated old fixed-parent tests; covers permitted moves, destination duplicates, source-only duplicates allowed after move, malformed/missing/nonexistent destinations, identity retention and prior role/rename regressions. Vue types/format/Pint/whitespace pass. Browser Super Admin: saved department initially Baby Care; selected Bakery; Save displayed exact old/new confirmation; Cancel kept form open; repeat+OK saved Bakery in list and reopening preselected Bakery; restored Baby Care through same confirmation and verified list. Original Category ID23/name Baby Wipes retained. Browser dropdown/confirmation tested; prior unrelated source review and developer create/list evidence preserved. No new future-module scope approved. Snapshots: app/Http/Controllers/CategoryController.php b1d4de4fe8d0; app/Http/Requests/Categories/UpdateCategoryRequest.php 9aa09e5b6eec; resources/js/pages/categories/Edit.vue 517fbb111d42; tests/Feature/CategoryEditTest.php 5ff867bf7040</x:t>
-        </x:is>
+      <x:c r="K31" s="11" t="str">
+        <x:v>2026-10-29 completed Category module source review passed: reviewed app/Http/Controllers/CategoryController.php, app/Policies/CategoryPolicy.php, app/Http/Requests/Categories/StoreCategoryRequest.php, app/Http/Requests/Categories/UpdateCategoryRequest.php, app/Http/Requests/Categories/IndexCategoriesRequest.php, app/Actions/Categories/ListCategories.php, app/Models/Category.php, app/Models/Department.php, database/migrations/2026_10_29_210437_create_categories_table.php, routes/web.php, resources/js/pages/categories/Create.vue, resources/js/pages/categories/Index.vue, resources/js/pages/categories/Edit.vue, tests/Feature/CategoryEditTest.php. Protected create/viewAny/update routes; repeated create/update request authorization; scoped name uniqueness; update ignores submitted parent/ID and validates only name against SAVED department; existing ID and parent retained. Eager-loaded parent on list/edit; stable pagination, OR name search, Vue form error/processing/cancel and success feedback. Following inspected Poker controller/request/route patterns and current Department edit. No blocking findings. Snapshots: app/Http/Controllers/CategoryController.php 8bd02ab4a46c; app/Policies/CategoryPolicy.php 727780b74cc6; app/Http/Requests/Categories/StoreCategoryRequest.php 5819301d79ab; app/Http/Requests/Categories/UpdateCategoryRequest.php fa34e0cb7cab; app/Http/Requests/Categories/IndexCategoriesRequest.php 6167bfe92ae6; app/Actions/Categories/ListCategories.php 0b8499c42ea0; app/Models/Category.php 714239df06eb; app/Models/Department.php 77c81e2ce045; database/migrations/2026_10_29_210437_create_categories_table.php 50ae1cd2d815; routes/web.php dab57df7c166; resources/js/pages/categories/Create.vue b47f65a7e2b2; resources/js/pages/categories/Index.vue ca004b43eb2e; resources/js/pages/categories/Edit.vue a4ee52f1f872; tests/Feature/CategoryEditTest.php b87e2c7bcb0a
+2026-10-29 user approved/authorized Category department moves, superseding fixed-parent rule for Category only. Controller supplies alphabetical departments; Edit uses shared Select preselected via String(saved ID), and Edit User window.confirm pattern on Save only when parent changes (old/new names). Cancel returns before PATCH. Request requires existing integer department and scopes unique name to selected department; controller persists validated name+department_id, preserving ID. Reviewed all changed source and tests; no findings. PASS delegated php artisan test tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php:29 tests183 assertions (SQLite). Updated old fixed-parent tests; covers permitted moves, destination duplicates, source-only duplicates allowed after move, malformed/missing/nonexistent destinations, identity retention and prior role/rename regressions. Vue types/format/Pint/whitespace pass. Browser Super Admin: saved department initially Baby Care; selected Bakery; Save displayed exact old/new confirmation; Cancel kept form open; repeat+OK saved Bakery in list and reopening preselected Bakery; restored Baby Care through same confirmation and verified list. Original Category ID23/name Baby Wipes retained. Browser dropdown/confirmation tested; prior unrelated source review and developer create/list evidence preserved. No new future-module scope approved. Snapshots: app/Http/Controllers/CategoryController.php b1d4de4fe8d0; app/Http/Requests/Categories/UpdateCategoryRequest.php 9aa09e5b6eec; resources/js/pages/categories/Edit.vue 517fbb111d42; tests/Feature/CategoryEditTest.php 5ff867bf7040
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L31" s="31" t="n">
         <x:v>46324</x:v>
@@ -4153,7 +4150,9 @@
       </x:c>
       <x:c r="K32" s="10" t="str">
         <x:v>2026-10-29 explicit user authorization: implement Subcategory creation with Department/dependent Category/name and run all necessary tests. Creation-only source review PASS for app/Models/Subcategory.php, app/Models/Category.php, app/Http/Controllers/SubcategoryController.php, app/Http/Requests/Subcategories/StoreSubcategoryRequest.php, app/Policies/SubcategoryPolicy.php, database/migrations/2026_10_29_214439_create_subcategories_table.php, resources/js/pages/subcategories/Create.vue, routes/web.php, tests/Feature/SubcategoryCreateTest.php. Implemented Category hasMany Subcategory / Subcategory belongsTo Category; fillable only category_id/name. Migration FK restrict/composite category-name uniqueness, no department duplicate/stock fields. Controller alphabetical minimal dropdown data; Vue computed filters Categories by department, watch clears selected Category on department change; category disabled until usable choices, no-category placeholder; keyed Select clears display; Inertia useForm success reset/errors/processing. Server create policy at auth GET+POST and request recheck for Manager/Super Admin; validates existing Department and Category scoped to Department, required name max255 unique within category. Store safe only category_id/name; flash/back follows current Category/Poker pattern. Read all relevant files together; no blocking findings. Snapshot: app/Models/Subcategory.php 77fcceb49da0; app/Models/Category.php cd7247b2dfd2; app/Http/Controllers/SubcategoryController.php 6a2c07b38475; app/Http/Requests/Subcategories/StoreSubcategoryRequest.php f0e9809b77cd; app/Policies/SubcategoryPolicy.php b15f69c79371; database/migrations/2026_10_29_214439_create_subcategories_table.php 8ed44d2b7e96; resources/js/pages/subcategories/Create.vue 6dfc2aa48f55; routes/web.php 38c6bea83c4e; tests/Feature/SubcategoryCreateTest.php 6dcf08a984f1
-2026-10-30 completed-feature source review PASS at clean application HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20. Read SubcategoryController, all three Subcategories requests, SubcategoryPolicy, ListSubcategories, Subcategory and Category models, subcategory migration and seeder, routes/web.php, all three subcategories Vue pages and SubcategoryCreate/List/Edit tests together. Creation, scoped uniqueness, matched parent validation, safe saved fields, derived Department, parent links, filtered/paginated list, edit/move confirmation, preserved identity, error/processing/reset state and GET/write policy checks match current scope. No blocking findings. Recorded delegated 96-test/681-assertion pass and 2026-10-30 browser passes retained; no tests or browser checks rerun this chat.</x:v>
+2026-10-30 completed-feature source review PASS at clean application HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20. Read SubcategoryController, all three Subcategories requests, SubcategoryPolicy, ListSubcategories, Subcategory and Category models, subcategory migration and seeder, routes/web.php, all three subcategories Vue pages and SubcategoryCreate/List/Edit tests together. Creation, scoped uniqueness, matched parent validation, safe saved fields, derived Department, parent links, filtered/paginated list, edit/move confirmation, preserved identity, error/processing/reset state and GET/write policy checks match current scope. No blocking findings. Recorded delegated 96-test/681-assertion pass and 2026-10-30 browser passes retained; no tests or browser checks rerun this chat.
+2026-10-30 developer explicitly requested removing assistant-added defineOptions({ inheritAttrs:false }) from Product Create, Tag Create/Index/Edit and Subcategory Create/Index/Edit; follow Poker pages and avoid unnecessary code. Removed only those declarations, associated explanatory comments and blank separators in all7 pages. Shared components unchanged. Poker page scan confirmed no inheritAttrs declarations. Scoped source diff/absence/whitespace check, Vue typecheck and asset build PASS. No browser/feature acceptance tests rerun; prior behaviour evidence remains historical. Earlier page-scaffold instructions including inheritAttrs are superseded by this explicit correction. No other Product implementation authorization.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L32" s="30" t="n">
         <x:v>46325</x:v>
@@ -4169,7 +4168,8 @@
 2026-10-29 delegated tests: initial targeted suite failed7 page requests due stale Vite manifest (Subcategory and existing edit pages absent); npm run build PASS regenerated assets. Rerun php artisan test tests/Feature/SubcategoryCreateTest.php tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php PASS53 tests324 assertions (SQLite in-memory), covering both permitted roles, invalid fields, required name/parents, scoped duplicates, mismatched parent pair, stale Category moved after form load, guest redirects, Volunteer403 GET/POST, ignored stock/forged fields, relationship retention across Category rename/move; no full unrelated account suite run. npm run types:check PASS, targeted Pint/Vue formatter PASS, syntax and diff whitespace PASS. Applied only Subcategory migration successfully to local MySQL. Browser existing Super Admin /subcategories/create PASS: Category initially disabled; blank errors for all3 fields; Baby Care shows Baby Wipes/Diapers/Infant Formula only; selected Baby Wipes then switching to Bakery clears category; Bakery shows Bread/Pastries/Rolls and Buns. Created temporary QA Dropdown Creation 20261029 under Bakery/Bread, success toast and Department/Category/name reset with Category disabled. Database row relationship verified; MySQL case-insensitive duplicate validator PASS. Removed only that self-created fixture. Wide and390px screenshots passed; phone stacked controls/full-width button. DevTools/device preview restored/closed. No sizes/units/quantities anywhere in creation UI/model/table. List/edit not implemented or verified.
 2026-10-29 user explicitly requested assistant run database seeding for five realistic Subcategories per Category. Inspected local database:30 categories under10 named departments, zero existing Subcategories. Implemented database/seeders/SubcategorySeeder.php mapping five name-only examples under each exact Department/Category pair, DB transaction and relationship firstOrCreate. Source review/Pint/PHP syntax/whitespace PASS. Executed php artisan db:seed --class=SubcategorySeeder successfully. Repeated via Artisan and compared ordered id/category_id/name snapshots: unchanged. Verified all30 categories have exactly5 Subcategories,150 total, no duplicates on rerun. No sizes/units/quantity fields or new scope. SHA256:23edc5ca69b9. Creation remains verified; list/rename and full module review pending.
 2026-10-29 assistant-run delegated catalogue tests PASS: php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryCreateTest.php tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php,70 tests509 assertions. List tests cover permitted roles/full parent path, partial matches on all3 names incl trimmed search, clear/no-match, search-before-pagination and retained link filter, multi-level match without duplicated row, empty catalogue, invalid filter/page, Volunteer403 including search and guest login redirect. npm run build PASS; npm run types:check PASS; targeted PHP Pint/Vue formatter, PHP syntax and whitespace PASS. Native Brave UI attempts interrupted repeatedly with user-changed-application responses; no new list browser/UI behavior or mobile verification performed. Preserve prior creation/browser and seed evidence; do not claim list browser pass or module completion.
-2026-10-30 assistant-run browser checks explicitly delegated by developer, ChatGPT in-app browser, developer signed-in session, source HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 (clean worktree before tracker update). PASS: automatic Fresh search without Enter returned only matching Department paths, page1 ten rows/page2 five rows with search retained; Enter zzqNoMatch reset page1 and displayed No subcategories found; clearing restored unfiltered page1 of15. Edit Apples ID2 initially Fresh Produce/Fruit/Apples. Blank name showed required error; spaced uppercase BANANAS rejected as duplicate with input/parents retained and Save reenabled. Cancel returned list with original Apples. At390x844 phone width, stacked edit controls/buttons/error fit; changing Department to Bakery cleared Category, Save showed required Category error and retained Bakery/name. Cancel and reopen restored saved Fresh Produce/Fruit/Apples. Phone list document width390 with table horizontally contained (table446, container306); no page overflow. Viewport reset. Only invalid submissions/Cancel performed; no saved record changes. No new automated suite run; prior96 catalogue tests681 assertions retained. Remaining requested browser checks passed. Consolidate completed-feature code-review evidence before closing FB-029/030.</x:v>
+2026-10-30 assistant-run browser checks explicitly delegated by developer, ChatGPT in-app browser, developer signed-in session, source HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 (clean worktree before tracker update). PASS: automatic Fresh search without Enter returned only matching Department paths, page1 ten rows/page2 five rows with search retained; Enter zzqNoMatch reset page1 and displayed No subcategories found; clearing restored unfiltered page1 of15. Edit Apples ID2 initially Fresh Produce/Fruit/Apples. Blank name showed required error; spaced uppercase BANANAS rejected as duplicate with input/parents retained and Save reenabled. Cancel returned list with original Apples. At390x844 phone width, stacked edit controls/buttons/error fit; changing Department to Bakery cleared Category, Save showed required Category error and retained Bakery/name. Cancel and reopen restored saved Fresh Produce/Fruit/Apples. Phone list document width390 with table horizontally contained (table446, container306); no page overflow. Viewport reset. Only invalid submissions/Cancel performed; no saved record changes. No new automated suite run; prior96 catalogue tests681 assertions retained. Remaining requested browser checks passed. Consolidate completed-feature code-review evidence before closing FB-029/030.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="P32" s="30" t="n">
         <x:v>46325</x:v>
@@ -4228,7 +4228,9 @@
       <x:c r="K33" s="11" t="str">
         <x:v>2026-10-29 user explicitly authorized Subcategory edit, authorized list buttons, all necessary tests. Read full AGENTS.md and full FB-030/related REQ-100/101/102/141. Followed Department Edit/Update request and ListUsers row-canEdit preparation. Read-only Department/Category context, prefilled editable name only; useForm PATCH/error/processing/Cancel; server update policy at GET/PATCH and request; name uniqueness scoped to SAVED category ignoring bound record; validated name only so forged id/category/department/stock fields cannot change identity or links. ListSubcategories now receives actor and returns prepared arrays with nested parents/canEdit from policy; Vue v-if canEdit Edit button and four-column empty state. Source review passed, no blocking findings. Snapshots: app/Http/Controllers/SubcategoryController.php 5578c0981f7c; app/Http/Requests/Subcategories/UpdateSubcategoryRequest.php eebe7e5599cf; app/Policies/SubcategoryPolicy.php 6d7c31bf3b34; app/Actions/Subcategories/ListSubcategories.php 36b8a8835b06; routes/web.php c7a64ff3ab36; resources/js/pages/subcategories/Index.vue 2066c12b396d; resources/js/pages/subcategories/Edit.vue fdaba55ae3ce; tests/Feature/SubcategoryEditTest.php cb49ff90bf11
 2026-10-29 authorized revision implemented. Source review PASS: dropdown data matches Create, initial form values use saved Department/Category IDs as strings, watch is NOT immediate so initial Category remains selected; computed filters choices; keyed Category Select resets stale display. Confirmation on Save compares saved Category ID and includes old/new paths; selected Category lookup uses filtered choices; missing choice goes to server validation. Request validates Category within Department and destination-scoped name uniqueness; controller safe only name/category_id; existing policy/button checks unchanged. No migrations. Tests updated from fixed-parent to allowed move behavior, no speculative Product connections. PASS96 tests681 assertions across SubcategoryEdit/List/Create and CategoryEdit/DepartmentEdit. Covers cross-department/same-department moves, unchanged parent/name, destination duplicates/source-only duplicate allowed, invalid destinations, parent mismatch, no partial writes, permissions and list/search regressions. Vue typecheck/build/Pint/formatter/syntax/diff whitespace PASS. Browser Super Admin opened existing ID90 Canned Fish with Pantry Staples/Canned Goods preselected; switched Meat and Seafood cleared Category; filtered Category choices selected Fish and Seafood; Save confirmation showed both paths, Cancel left form unsaved. Repeat/OK saved and reopening showed NEW Meat and Seafood/Fish and Seafood selected. Restored original Pantry Staples/Canned Goods through same confirmed UI and verified DB ID/name/path restored. Same-department moves automated-tested; latest mobile layout not browser-verified. Prior outstanding full-module/list UI checks remain pending. Snapshots:app/Http/Controllers/SubcategoryController.php 395e1fe9fe48; app/Http/Requests/Subcategories/UpdateSubcategoryRequest.php d6fc5d714b63; resources/js/pages/subcategories/Edit.vue cf9bc227539f; tests/Feature/SubcategoryEditTest.php 9e3f4112abdc
-2026-10-30 completed-feature source review PASS at clean application HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20. Read SubcategoryController, all three Subcategories requests, SubcategoryPolicy, ListSubcategories, Subcategory and Category models, subcategory migration and seeder, routes/web.php, all three subcategories Vue pages and SubcategoryCreate/List/Edit tests together. Creation, scoped uniqueness, matched parent validation, safe saved fields, derived Department, parent links, filtered/paginated list, edit/move confirmation, preserved identity, error/processing/reset state and GET/write policy checks match current scope. No blocking findings. Recorded delegated 96-test/681-assertion pass and 2026-10-30 browser passes retained; no tests or browser checks rerun this chat.</x:v>
+2026-10-30 completed-feature source review PASS at clean application HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20. Read SubcategoryController, all three Subcategories requests, SubcategoryPolicy, ListSubcategories, Subcategory and Category models, subcategory migration and seeder, routes/web.php, all three subcategories Vue pages and SubcategoryCreate/List/Edit tests together. Creation, scoped uniqueness, matched parent validation, safe saved fields, derived Department, parent links, filtered/paginated list, edit/move confirmation, preserved identity, error/processing/reset state and GET/write policy checks match current scope. No blocking findings. Recorded delegated 96-test/681-assertion pass and 2026-10-30 browser passes retained; no tests or browser checks rerun this chat.
+2026-10-30 developer explicitly requested removing assistant-added defineOptions({ inheritAttrs:false }) from Product Create, Tag Create/Index/Edit and Subcategory Create/Index/Edit; follow Poker pages and avoid unnecessary code. Removed only those declarations, associated explanatory comments and blank separators in all7 pages. Shared components unchanged. Poker page scan confirmed no inheritAttrs declarations. Scoped source diff/absence/whitespace check, Vue typecheck and asset build PASS. No browser/feature acceptance tests rerun; prior behaviour evidence remains historical. Earlier page-scaffold instructions including inheritAttrs are superseded by this explicit correction. No other Product implementation authorization.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="L33" s="31" t="n">
         <x:v>46325</x:v>
@@ -4242,7 +4244,8 @@
       <x:c r="O33" s="11" t="str">
         <x:v>2026-10-29 delegated tests: first85-test catalogue run84 pass, one synthetic-denial test failed because separately defined Gate update ability does not override registered model policy. Corrected ONLY test to register ReadOnlySubcategoryTestPolicy; rerun PASS85 tests617 assertions. Command: php artisan test tests/Feature/SubcategoryEditTest.php tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryCreateTest.php tests/Feature/CategoryEditTest.php tests/Feature/DepartmentEditTest.php. Covers both allowed roles, canEdit true/false, independent list/edit permissions and forbidden routes, prefill parents, successful trimmed rename preserving ID/category despite forged fields, same name/current record and across categories,255-char success, blank/null/array/256-char/duplicate rejection, forged category duplicate bypass rejected, guest redirects/missing records404, full create/list/search regressions. Actual UpdateSubcategoryRequest rules checked read-only on local MySQL Body Lotion versus body wash under same category: case-insensitive duplicate rejected/current name accepted; no DB writes. npm run build PASS, npm run types:check PASS, Pint/Vue formatter/PHP syntax/whitespace PASS. Browser observed list page2 with Edit links (including Body Lotion135); attempted click was interrupted by user-changed-application response. No browser edit save/Cancel/error/mobile checks performed; no successful browser form claim. Previous list typing/layout verification remains pending. No full unrelated application suite run.
 2026-10-29 authorized revision implemented. Source review PASS: dropdown data matches Create, initial form values use saved Department/Category IDs as strings, watch is NOT immediate so initial Category remains selected; computed filters choices; keyed Category Select resets stale display. Confirmation on Save compares saved Category ID and includes old/new paths; selected Category lookup uses filtered choices; missing choice goes to server validation. Request validates Category within Department and destination-scoped name uniqueness; controller safe only name/category_id; existing policy/button checks unchanged. No migrations. Tests updated from fixed-parent to allowed move behavior, no speculative Product connections. PASS96 tests681 assertions across SubcategoryEdit/List/Create and CategoryEdit/DepartmentEdit. Covers cross-department/same-department moves, unchanged parent/name, destination duplicates/source-only duplicate allowed, invalid destinations, parent mismatch, no partial writes, permissions and list/search regressions. Vue typecheck/build/Pint/formatter/syntax/diff whitespace PASS. Browser Super Admin opened existing ID90 Canned Fish with Pantry Staples/Canned Goods preselected; switched Meat and Seafood cleared Category; filtered Category choices selected Fish and Seafood; Save confirmation showed both paths, Cancel left form unsaved. Repeat/OK saved and reopening showed NEW Meat and Seafood/Fish and Seafood selected. Restored original Pantry Staples/Canned Goods through same confirmed UI and verified DB ID/name/path restored. Same-department moves automated-tested; latest mobile layout not browser-verified. Prior outstanding full-module/list UI checks remain pending. Snapshots:app/Http/Controllers/SubcategoryController.php 395e1fe9fe48; app/Http/Requests/Subcategories/UpdateSubcategoryRequest.php d6fc5d714b63; resources/js/pages/subcategories/Edit.vue cf9bc227539f; tests/Feature/SubcategoryEditTest.php 9e3f4112abdc
-2026-10-30 assistant-run browser checks explicitly delegated by developer, ChatGPT in-app browser, developer signed-in session, source HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 (clean worktree before tracker update). PASS: automatic Fresh search without Enter returned only matching Department paths, page1 ten rows/page2 five rows with search retained; Enter zzqNoMatch reset page1 and displayed No subcategories found; clearing restored unfiltered page1 of15. Edit Apples ID2 initially Fresh Produce/Fruit/Apples. Blank name showed required error; spaced uppercase BANANAS rejected as duplicate with input/parents retained and Save reenabled. Cancel returned list with original Apples. At390x844 phone width, stacked edit controls/buttons/error fit; changing Department to Bakery cleared Category, Save showed required Category error and retained Bakery/name. Cancel and reopen restored saved Fresh Produce/Fruit/Apples. Phone list document width390 with table horizontally contained (table446, container306); no page overflow. Viewport reset. Only invalid submissions/Cancel performed; no saved record changes. No new automated suite run; prior96 catalogue tests681 assertions retained. Remaining requested browser checks passed. Consolidate completed-feature code-review evidence before closing FB-029/030.</x:v>
+2026-10-30 assistant-run browser checks explicitly delegated by developer, ChatGPT in-app browser, developer signed-in session, source HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 (clean worktree before tracker update). PASS: automatic Fresh search without Enter returned only matching Department paths, page1 ten rows/page2 five rows with search retained; Enter zzqNoMatch reset page1 and displayed No subcategories found; clearing restored unfiltered page1 of15. Edit Apples ID2 initially Fresh Produce/Fruit/Apples. Blank name showed required error; spaced uppercase BANANAS rejected as duplicate with input/parents retained and Save reenabled. Cancel returned list with original Apples. At390x844 phone width, stacked edit controls/buttons/error fit; changing Department to Bakery cleared Category, Save showed required Category error and retained Bakery/name. Cancel and reopen restored saved Fresh Produce/Fruit/Apples. Phone list document width390 with table horizontally contained (table446, container306); no page overflow. Viewport reset. Only invalid submissions/Cancel performed; no saved record changes. No new automated suite run; prior96 catalogue tests681 assertions retained. Remaining requested browser checks passed. Consolidate completed-feature code-review evidence before closing FB-029/030.
+2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
       </x:c>
       <x:c r="P33" s="31" t="n">
         <x:v>46325</x:v>
@@ -4302,7 +4305,10 @@
       <x:c r="K34" s="10" t="str">
         <x:v>2026-10-30 reference inspection for upcoming Tags: skander app/Models/Player.php protected $fillable; PlayerController create/store/edit/update uses Inertia pages, simple direct model persistence, flash toast/back; routes/web.php checks create on GET/POST and update on GET/PATCH; PlayerPolicy defines abilities. StorePlayerRequest holds validation. Follow these responsibilities with FoodBank roles. No Tag code reviewed or implemented.
 2026-10-30 developer-requested intermediate scaffold check: read Tag model, TagController, StoreTagRequest, UpdateTagRequest, TagPolicy, create_tags_table migration and TagSeeder. All are generated scaffolds; migration currently id/timestamps only, requests/policy deny by default, no tag routes or Vue page. No implemented behaviour or passed feature test claimed. Requests currently at root Http/Requests; organize under Tags with matching namespaces/imports in a later small lesson. No application changes made.
-2026-10-30 developer explicitly delegated all current Tag work and testing, following this project catalogue UI/coding/workflows. Completed-feature source review PASS at HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 plus uncommitted Tag implementation: app/Models/Tag.php, app/Http/Controllers/TagController.php, app/Http/Requests/Tags/{IndexTagsRequest,StoreTagRequest,UpdateTagRequest}.php, app/Actions/Tags/ListTags.php, app/Policies/TagPolicy.php, routes/web.php, database/migrations/2026_10_30_061953_create_tags_table.php, resources/js/pages/tags/{Create,Index,Edit}.vue, tests/Feature/TagTest.php. Department screen/controller/request conventions and Subcategory per-row canEdit preparation reused. Protected GET list/create/edit and POST/PATCH; Manager/Super Admin allowed, Volunteer denied. Required unique max255 name; Laravel trims, local MySQL collation ignores case. Rename preserves ID, ignores self in uniqueness. Protected fillable/validated fields. Search before alphabetical paginate(10), links retain search; 300ms typing/Enter/empty states. Forms errors, processing, success reset/toast, Cancel/list redirect, accessible labels/error links and phone layout. No blocking findings. No Product/pivot/stock work or deletion endpoint; Product tag attachment FB-037 and deletion rule FB-048 remain open. TagSeeder remains original empty scaffold; no production seed data requested.</x:v>
+2026-10-30 developer explicitly delegated all current Tag work and testing, following this project catalogue UI/coding/workflows. Completed-feature source review PASS at HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 plus uncommitted Tag implementation: app/Models/Tag.php, app/Http/Controllers/TagController.php, app/Http/Requests/Tags/{IndexTagsRequest,StoreTagRequest,UpdateTagRequest}.php, app/Actions/Tags/ListTags.php, app/Policies/TagPolicy.php, routes/web.php, database/migrations/2026_10_30_061953_create_tags_table.php, resources/js/pages/tags/{Create,Index,Edit}.vue, tests/Feature/TagTest.php. Department screen/controller/request conventions and Subcategory per-row canEdit preparation reused. Protected GET list/create/edit and POST/PATCH; Manager/Super Admin allowed, Volunteer denied. Required unique max255 name; Laravel trims, local MySQL collation ignores case. Rename preserves ID, ignores self in uniqueness. Protected fillable/validated fields. Search before alphabetical paginate(10), links retain search; 300ms typing/Enter/empty states. Forms errors, processing, success reset/toast, Cancel/list redirect, accessible labels/error links and phone layout. No blocking findings. No Product/pivot/stock work or deletion endpoint; Product tag attachment FB-037 and deletion rule FB-048 remain open. TagSeeder remains original empty scaffold; no production seed data requested.
+2026-10-30 developer explicitly requested TagSeeder file with50 realistic tags so developer can run it. Updated database/seeders/TagSeeder.php only:50 distinct dietary/storage/preparation/meal/personal-care/household labels; Tag::firstOrCreate inside DB::transaction follows current catalogue seeder conventions and preserves existing names/records on reruns. Source review, PHP syntax, scoped Pint and static count/case-folded uniqueness checks PASS. Seeder NOT executed; no database changes or runtime/idempotence pass claimed. Supplied php artisan db:seed --class=TagSeeder for developer to run. Product lesson remains pending; no Product code read/changed.
+2026-10-30 developer explicitly requested removing assistant-added defineOptions({ inheritAttrs:false }) from Product Create, Tag Create/Index/Edit and Subcategory Create/Index/Edit; follow Poker pages and avoid unnecessary code. Removed only those declarations, associated explanatory comments and blank separators in all7 pages. Shared components unchanged. Poker page scan confirmed no inheritAttrs declarations. Scoped source diff/absence/whitespace check, Vue typecheck and asset build PASS. No browser/feature acceptance tests rerun; prior behaviour evidence remains historical. Earlier page-scaffold instructions including inheritAttrs are superseded by this explicit correction. No other Product implementation authorization.
+2026-10-30 Tag inverse products relationship reviewed and tested with Product creation; TagTest regressions included in157-test pass. Shared tag rename preserves product links.</x:v>
       </x:c>
       <x:c r="L34" s="30" t="n">
         <x:v>46325</x:v>
@@ -4346,10 +4352,8 @@
           <x:t xml:space="preserve">Introduce Product storage and its hierarchy form</x:t>
         </x:is>
       </x:c>
-      <x:c r="E35" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Product belongs to Subcategory. Required name/hierarchy/status; optional brand/tags; automatic code. No sizes, packaging, counting/contents units, balances or quantity fields. Introduce tag persistence at FB-037.</x:t>
-        </x:is>
+      <x:c r="E35" s="9" t="str">
+        <x:v>Product belongs to Subcategory. Required name/hierarchy/status; optional brand/tags. Build without product codes; retain internal database id. No sizes, packaging, counting/contents units, balances or quantities. Introduce tag persistence at FB-037. Reconsider codes after FB-067 at FB-035.</x:v>
       </x:c>
       <x:c r="F35" s="9" t="inlineStr">
         <x:is>
@@ -4358,39 +4362,47 @@
       </x:c>
       <x:c r="G35" s="9" t="str">
         <x:f>IF(H35="Complete","Complete",IF(I35="Blocked","Blocked",IF(I35="In progress","Ready",IF(F35="","Ready",IF(COUNTIFS($B$4:$B$73,F35,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Ready</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="H35" s="9" t="str">
         <x:f>IF(I35="Not started","Not started",IF(I35="Blocked","Blocked",IF(I35="In progress","In progress",IF(J35&lt;&gt;"Passed","Awaiting code review",IF(OR(K35="",NOT(ISNUMBER(L35))),"Awaiting review evidence",IF(N35&lt;&gt;"Passed","Awaiting test",IF(OR(M35="",O35="",NOT(ISNUMBER(P35))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I35" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J35" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not reviewed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K35" s="11" t="n"/>
-      <x:c r="L35" s="31" t="n"/>
-      <x:c r="M35" s="11" t="n"/>
-      <x:c r="N35" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O35" s="11" t="n"/>
-      <x:c r="P35" s="31" t="n"/>
-      <x:c r="Q35" s="11" t="n"/>
-      <x:c r="R35" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S35" s="11" t="n"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I35" s="11" t="str">
+        <x:v>Ready for review</x:v>
+      </x:c>
+      <x:c r="J35" s="11" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K35" s="11" t="str">
+        <x:v>
+2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.</x:v>
+      </x:c>
+      <x:c r="L35" s="31" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="M35" s="11" t="str">
+        <x:v>Assistant (explicitly delegated automated, MySQL and browser checks)</x:v>
+      </x:c>
+      <x:c r="N35" s="11" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="O35" s="11" t="str">
+        <x:v>
+2026-10-30 developer explicitly reported scoped Product migration ran successfully. Record as developer-reported migration check only; not source review or full Product feature behaviour verification.
+2026-10-30 developer replied done to explicit protected Create Product page check and stated page opens successfully. Developer-reported PASS for minimal page display only; role-specific denial, saving and full feature not verified.
+2026-10-30 Assistant (explicitly delegated) PASS creation-scoped catalogue regression: php artisan test ProductCreateTest,TagTest,SubcategoryCreateTest,SubcategoryListTest,SubcategoryEditTest,CategoryEditTest,DepartmentEditTest —157 tests1162 assertions; rerun after request normalization/controller cleanup same pass.42 new Product tests cover both permitted roles, page data, successful trimmed create, Active/Inactive casts, ignored forged fields, both tag relationships/shared rename, optional blank/null/omitted tags and brand,255-char fields, null/blank/array/long inputs, existing/matching parents, invalid/status/tag IDs, repeated tag IDs, duplicate identity incl inactive/unbranded/case/spaces, distinct brand/Subcategory acceptance, guest/Volunteer denied GET/POST, action authorization, stale parent/tag rechecks, forced real pivot-insert failure rolls product back, pivot uniqueness/used-tag FK. Vue typecheck, build, scoped Pint/PHPStan(0 errors)/PHP syntax/whitespace PASS. Applied only new product_tag migration to local MySQL. Browser in-app existing Super Admin PASS blank errors; Pantry Staples/Rice and Grains/White Rice choices; inactive QA product with trimmed name/brand saved; selected Halal then Vegan while Halal hidden, both persisted and Tag-&gt;products inverse verified in MySQL. Toast and complete form/search/tag reset/restored Active; Category/Subcategory disabled/reset. Uppercase/spaced duplicate of INACTIVE saved product rejected despite new Active status; hierarchy/text/selected Halal retained and button reenabled. Search300ms case-insensitive, Enter, no-match/clear; optional unbranded/untagged Active save passed on390x844 phone and DB null brand/zero links verified. Category change cleared Subcategory; Department change cleared both children. Phone document width390/no overflow, stacked controls/readable error; normal1280 viewport restored, Department and tag-search widths both289.328px. MySQL two simultaneous action processes on same Subcategory: one SAVED, second DUPLICATE_REJECTED; one row created. All3 exact QA products/pivot links removed, shared tags untouched. Full suite192 tests174 pass17 failed1 error; separate isolated clean HEAD baseline150 tests132 pass17 failed1 error, identical failing/error test names (account/auth/settings/seeding), no additional failures. Full PHPStan still7 pre-existing unrelated catalogue issues; no scope expansion to fix deferred accounts or other controllers. Product-list Halal search remains later FB-040/044.</x:v>
+      </x:c>
+      <x:c r="P35" s="31" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="Q35" s="11" t="str">
+        <x:v>2026-10-30 Product creation feature implemented/reviewed/tested; this item verified. Product list next; no product code/stock features implemented.</x:v>
+      </x:c>
+      <x:c r="R35" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Completed. Next ready item FB-038 Product list; show proposed changes before applying, preserve Poker coding/current catalogue UI and name-or-tag search checkpoints.</x:v>
+      </x:c>
+      <x:c r="S35" s="11" t="str"/>
     </x:row>
     <x:row r="36" ht="105" customHeight="1">
       <x:c r="A36" s="4" t="n">
@@ -4423,43 +4435,49 @@
       </x:c>
       <x:c r="G36" s="4" t="str">
         <x:f>IF(H36="Complete","Complete",IF(I36="Blocked","Blocked",IF(I36="In progress","Ready",IF(F36="","Ready",IF(COUNTIFS($B$4:$B$73,F36,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="H36" s="4" t="str">
         <x:f>IF(I36="Not started","Not started",IF(I36="Blocked","Blocked",IF(I36="In progress","In progress",IF(J36&lt;&gt;"Passed","Awaiting code review",IF(OR(K36="",NOT(ISNUMBER(L36))),"Awaiting review evidence",IF(N36&lt;&gt;"Passed","Awaiting test",IF(OR(M36="",O36="",NOT(ISNUMBER(P36))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I36" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J36" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not reviewed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K36" s="10" t="n"/>
-      <x:c r="L36" s="30" t="n"/>
-      <x:c r="M36" s="10" t="n"/>
-      <x:c r="N36" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O36" s="10" t="n"/>
-      <x:c r="P36" s="30" t="n"/>
-      <x:c r="Q36" s="10" t="n"/>
-      <x:c r="R36" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S36" s="10" t="n"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I36" s="10" t="str">
+        <x:v>Ready for review</x:v>
+      </x:c>
+      <x:c r="J36" s="10" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K36" s="10" t="str">
+        <x:v>
+2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.</x:v>
+      </x:c>
+      <x:c r="L36" s="30" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="M36" s="10" t="str">
+        <x:v>Assistant (explicitly delegated automated, MySQL and browser checks)</x:v>
+      </x:c>
+      <x:c r="N36" s="10" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="O36" s="10" t="str">
+        <x:v>
+2026-10-30 Assistant (explicitly delegated) PASS creation-scoped catalogue regression: php artisan test ProductCreateTest,TagTest,SubcategoryCreateTest,SubcategoryListTest,SubcategoryEditTest,CategoryEditTest,DepartmentEditTest —157 tests1162 assertions; rerun after request normalization/controller cleanup same pass.42 new Product tests cover both permitted roles, page data, successful trimmed create, Active/Inactive casts, ignored forged fields, both tag relationships/shared rename, optional blank/null/omitted tags and brand,255-char fields, null/blank/array/long inputs, existing/matching parents, invalid/status/tag IDs, repeated tag IDs, duplicate identity incl inactive/unbranded/case/spaces, distinct brand/Subcategory acceptance, guest/Volunteer denied GET/POST, action authorization, stale parent/tag rechecks, forced real pivot-insert failure rolls product back, pivot uniqueness/used-tag FK. Vue typecheck, build, scoped Pint/PHPStan(0 errors)/PHP syntax/whitespace PASS. Applied only new product_tag migration to local MySQL. Browser in-app existing Super Admin PASS blank errors; Pantry Staples/Rice and Grains/White Rice choices; inactive QA product with trimmed name/brand saved; selected Halal then Vegan while Halal hidden, both persisted and Tag-&gt;products inverse verified in MySQL. Toast and complete form/search/tag reset/restored Active; Category/Subcategory disabled/reset. Uppercase/spaced duplicate of INACTIVE saved product rejected despite new Active status; hierarchy/text/selected Halal retained and button reenabled. Search300ms case-insensitive, Enter, no-match/clear; optional unbranded/untagged Active save passed on390x844 phone and DB null brand/zero links verified. Category change cleared Subcategory; Department change cleared both children. Phone document width390/no overflow, stacked controls/readable error; normal1280 viewport restored, Department and tag-search widths both289.328px. MySQL two simultaneous action processes on same Subcategory: one SAVED, second DUPLICATE_REJECTED; one row created. All3 exact QA products/pivot links removed, shared tags untouched. Full suite192 tests174 pass17 failed1 error; separate isolated clean HEAD baseline150 tests132 pass17 failed1 error, identical failing/error test names (account/auth/settings/seeding), no additional failures. Full PHPStan still7 pre-existing unrelated catalogue issues; no scope expansion to fix deferred accounts or other controllers. Product-list Halal search remains later FB-040/044.</x:v>
+      </x:c>
+      <x:c r="P36" s="30" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="Q36" s="10" t="str">
+        <x:v>2026-10-30 Product creation feature implemented/reviewed/tested; this item verified. Product list next; no product code/stock features implemented.</x:v>
+      </x:c>
+      <x:c r="R36" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Completed. Next ready item FB-038 Product list; show proposed changes before applying, preserve Poker coding/current catalogue UI and name-or-tag search checkpoints.</x:v>
+      </x:c>
+      <x:c r="S36" s="10" t="str"/>
     </x:row>
     <x:row r="37" ht="105" customHeight="1">
       <x:c r="A37" s="4" t="n">
-        <x:v>34</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B37" s="4" t="inlineStr">
         <x:is>
@@ -4471,20 +4489,14 @@
           <x:t xml:space="preserve">Products</x:t>
         </x:is>
       </x:c>
-      <x:c r="D37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Generate permanent product codes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unique automatic PRD-000001 onward, at least six digits and growth beyond999999, never edited/reused or derived from categories. Codes identify catalogue products independently of package sizes.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F37" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-033</x:t>
-        </x:is>
+      <x:c r="D37" s="4" t="str">
+        <x:v>Reconsider product codes and stock connections after the catalogue works</x:v>
+      </x:c>
+      <x:c r="E37" s="4" t="str">
+        <x:v>After FB-067 verified functional catalogue, discuss whether human-readable codes are needed and revisit the connection to Stock Management. No mandatory code format/generation/backfill or replacement design approved. Record developer decision and affected requirements before any implementation. Preserve prior PRD design as history only.</x:v>
+      </x:c>
+      <x:c r="F37" s="4" t="str">
+        <x:v>FB-067</x:v>
       </x:c>
       <x:c r="G37" s="4" t="str">
         <x:f>IF(H37="Complete","Complete",IF(I37="Blocked","Blocked",IF(I37="In progress","Ready",IF(F37="","Ready",IF(COUNTIFS($B$4:$B$73,F37,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
@@ -4514,17 +4526,17 @@
       </x:c>
       <x:c r="O37" s="10" t="n"/>
       <x:c r="P37" s="30" t="n"/>
-      <x:c r="Q37" s="10" t="n"/>
-      <x:c r="R37" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="Q37" s="10" t="str">
+        <x:v>2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
+      </x:c>
+      <x:c r="R37" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Do not start before FB-067 verified. Brainstorm code need and stock connections with developer, record approved decisions, then decide whether any code implementation/backfill is needed before FB-034. No automatic implementation of old PRD proposal.</x:v>
       </x:c>
       <x:c r="S37" s="10" t="n"/>
     </x:row>
     <x:row r="38" ht="105" customHeight="1">
       <x:c r="A38" s="9" t="n">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B38" s="9" t="inlineStr">
         <x:is>
@@ -4546,50 +4558,54 @@
           <x:t xml:space="preserve">Compare name/brand/Subcategory, ignore case/outer spaces and include inactive products. No package contents, counting unit or size in catalogue duplicate identity.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F38" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-035</x:t>
-        </x:is>
+      <x:c r="F38" s="9" t="str">
+        <x:v>FB-033</x:v>
       </x:c>
       <x:c r="G38" s="9" t="str">
         <x:f>IF(H38="Complete","Complete",IF(I38="Blocked","Blocked",IF(I38="In progress","Ready",IF(F38="","Ready",IF(COUNTIFS($B$4:$B$73,F38,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="H38" s="9" t="str">
         <x:f>IF(I38="Not started","Not started",IF(I38="Blocked","Blocked",IF(I38="In progress","In progress",IF(J38&lt;&gt;"Passed","Awaiting code review",IF(OR(K38="",NOT(ISNUMBER(L38))),"Awaiting review evidence",IF(N38&lt;&gt;"Passed","Awaiting test",IF(OR(M38="",O38="",NOT(ISNUMBER(P38))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I38" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J38" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not reviewed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K38" s="11" t="n"/>
-      <x:c r="L38" s="31" t="n"/>
-      <x:c r="M38" s="11" t="n"/>
-      <x:c r="N38" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O38" s="11" t="n"/>
-      <x:c r="P38" s="31" t="n"/>
-      <x:c r="Q38" s="11" t="n"/>
-      <x:c r="R38" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S38" s="11" t="n"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="str">
+        <x:v>Ready for review</x:v>
+      </x:c>
+      <x:c r="J38" s="11" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K38" s="11" t="str">
+        <x:v>
+2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.</x:v>
+      </x:c>
+      <x:c r="L38" s="31" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="M38" s="11" t="str">
+        <x:v>Assistant (explicitly delegated automated, MySQL and browser checks)</x:v>
+      </x:c>
+      <x:c r="N38" s="11" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="O38" s="11" t="str">
+        <x:v>
+2026-10-30 Assistant (explicitly delegated) PASS creation-scoped catalogue regression: php artisan test ProductCreateTest,TagTest,SubcategoryCreateTest,SubcategoryListTest,SubcategoryEditTest,CategoryEditTest,DepartmentEditTest —157 tests1162 assertions; rerun after request normalization/controller cleanup same pass.42 new Product tests cover both permitted roles, page data, successful trimmed create, Active/Inactive casts, ignored forged fields, both tag relationships/shared rename, optional blank/null/omitted tags and brand,255-char fields, null/blank/array/long inputs, existing/matching parents, invalid/status/tag IDs, repeated tag IDs, duplicate identity incl inactive/unbranded/case/spaces, distinct brand/Subcategory acceptance, guest/Volunteer denied GET/POST, action authorization, stale parent/tag rechecks, forced real pivot-insert failure rolls product back, pivot uniqueness/used-tag FK. Vue typecheck, build, scoped Pint/PHPStan(0 errors)/PHP syntax/whitespace PASS. Applied only new product_tag migration to local MySQL. Browser in-app existing Super Admin PASS blank errors; Pantry Staples/Rice and Grains/White Rice choices; inactive QA product with trimmed name/brand saved; selected Halal then Vegan while Halal hidden, both persisted and Tag-&gt;products inverse verified in MySQL. Toast and complete form/search/tag reset/restored Active; Category/Subcategory disabled/reset. Uppercase/spaced duplicate of INACTIVE saved product rejected despite new Active status; hierarchy/text/selected Halal retained and button reenabled. Search300ms case-insensitive, Enter, no-match/clear; optional unbranded/untagged Active save passed on390x844 phone and DB null brand/zero links verified. Category change cleared Subcategory; Department change cleared both children. Phone document width390/no overflow, stacked controls/readable error; normal1280 viewport restored, Department and tag-search widths both289.328px. MySQL two simultaneous action processes on same Subcategory: one SAVED, second DUPLICATE_REJECTED; one row created. All3 exact QA products/pivot links removed, shared tags untouched. Full suite192 tests174 pass17 failed1 error; separate isolated clean HEAD baseline150 tests132 pass17 failed1 error, identical failing/error test names (account/auth/settings/seeding), no additional failures. Full PHPStan still7 pre-existing unrelated catalogue issues; no scope expansion to fix deferred accounts or other controllers. Product-list Halal search remains later FB-040/044.</x:v>
+      </x:c>
+      <x:c r="P38" s="31" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="Q38" s="11" t="str">
+        <x:v>2026-10-30 Product creation feature implemented/reviewed/tested; this item verified. Product list next; no product code/stock features implemented.</x:v>
+      </x:c>
+      <x:c r="R38" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Completed. Next ready item FB-038 Product list; show proposed changes before applying, preserve Poker coding/current catalogue UI and name-or-tag search checkpoints.</x:v>
+      </x:c>
+      <x:c r="S38" s="11" t="str"/>
     </x:row>
     <x:row r="39" ht="105" customHeight="1">
       <x:c r="A39" s="4" t="n">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B39" s="4" t="inlineStr">
         <x:is>
@@ -4606,10 +4622,8 @@
           <x:t xml:space="preserve">Save products and attach optional tags</x:t>
         </x:is>
       </x:c>
-      <x:c r="E39" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Managers/Super Admin create; Volunteers denied display/write. Save catalogue identity/classification/status only; no stock quantity/packaging. Optional shared tags; errors/retained input/processing and persisted fields.</x:t>
-        </x:is>
+      <x:c r="E39" s="4" t="str">
+        <x:v>Managers/Super Admin create; Volunteers denied display/write. Save catalogue identity/classification/status only; no stock quantity/packaging. Optional shared tags; errors/retained input/processing and persisted fields. Both Product::tags() and Tag::products() use same product_tag pivot; tag-based lookup is required, verified in list/search phase.</x:v>
       </x:c>
       <x:c r="F39" s="4" t="inlineStr">
         <x:is>
@@ -4618,43 +4632,49 @@
       </x:c>
       <x:c r="G39" s="4" t="str">
         <x:f>IF(H39="Complete","Complete",IF(I39="Blocked","Blocked",IF(I39="In progress","Ready",IF(F39="","Ready",IF(COUNTIFS($B$4:$B$73,F39,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="H39" s="4" t="str">
         <x:f>IF(I39="Not started","Not started",IF(I39="Blocked","Blocked",IF(I39="In progress","In progress",IF(J39&lt;&gt;"Passed","Awaiting code review",IF(OR(K39="",NOT(ISNUMBER(L39))),"Awaiting review evidence",IF(N39&lt;&gt;"Passed","Awaiting test",IF(OR(M39="",O39="",NOT(ISNUMBER(P39))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I39" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J39" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not reviewed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K39" s="10" t="n"/>
-      <x:c r="L39" s="30" t="n"/>
-      <x:c r="M39" s="10" t="n"/>
-      <x:c r="N39" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O39" s="10" t="n"/>
-      <x:c r="P39" s="30" t="n"/>
-      <x:c r="Q39" s="10" t="n"/>
-      <x:c r="R39" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S39" s="10" t="n"/>
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="I39" s="10" t="str">
+        <x:v>Ready for review</x:v>
+      </x:c>
+      <x:c r="J39" s="10" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K39" s="10" t="str">
+        <x:v>
+2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.</x:v>
+      </x:c>
+      <x:c r="L39" s="30" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="M39" s="10" t="str">
+        <x:v>Assistant (explicitly delegated automated, MySQL and browser checks)</x:v>
+      </x:c>
+      <x:c r="N39" s="10" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="O39" s="10" t="str">
+        <x:v>
+2026-10-30 Assistant (explicitly delegated) PASS creation-scoped catalogue regression: php artisan test ProductCreateTest,TagTest,SubcategoryCreateTest,SubcategoryListTest,SubcategoryEditTest,CategoryEditTest,DepartmentEditTest —157 tests1162 assertions; rerun after request normalization/controller cleanup same pass.42 new Product tests cover both permitted roles, page data, successful trimmed create, Active/Inactive casts, ignored forged fields, both tag relationships/shared rename, optional blank/null/omitted tags and brand,255-char fields, null/blank/array/long inputs, existing/matching parents, invalid/status/tag IDs, repeated tag IDs, duplicate identity incl inactive/unbranded/case/spaces, distinct brand/Subcategory acceptance, guest/Volunteer denied GET/POST, action authorization, stale parent/tag rechecks, forced real pivot-insert failure rolls product back, pivot uniqueness/used-tag FK. Vue typecheck, build, scoped Pint/PHPStan(0 errors)/PHP syntax/whitespace PASS. Applied only new product_tag migration to local MySQL. Browser in-app existing Super Admin PASS blank errors; Pantry Staples/Rice and Grains/White Rice choices; inactive QA product with trimmed name/brand saved; selected Halal then Vegan while Halal hidden, both persisted and Tag-&gt;products inverse verified in MySQL. Toast and complete form/search/tag reset/restored Active; Category/Subcategory disabled/reset. Uppercase/spaced duplicate of INACTIVE saved product rejected despite new Active status; hierarchy/text/selected Halal retained and button reenabled. Search300ms case-insensitive, Enter, no-match/clear; optional unbranded/untagged Active save passed on390x844 phone and DB null brand/zero links verified. Category change cleared Subcategory; Department change cleared both children. Phone document width390/no overflow, stacked controls/readable error; normal1280 viewport restored, Department and tag-search widths both289.328px. MySQL two simultaneous action processes on same Subcategory: one SAVED, second DUPLICATE_REJECTED; one row created. All3 exact QA products/pivot links removed, shared tags untouched. Full suite192 tests174 pass17 failed1 error; separate isolated clean HEAD baseline150 tests132 pass17 failed1 error, identical failing/error test names (account/auth/settings/seeding), no additional failures. Full PHPStan still7 pre-existing unrelated catalogue issues; no scope expansion to fix deferred accounts or other controllers. Product-list Halal search remains later FB-040/044.</x:v>
+      </x:c>
+      <x:c r="P39" s="30" t="n">
+        <x:v>46325</x:v>
+      </x:c>
+      <x:c r="Q39" s="10" t="str">
+        <x:v>2026-10-30 Product creation feature implemented/reviewed/tested; this item verified. Product list next; no product code/stock features implemented.</x:v>
+      </x:c>
+      <x:c r="R39" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Completed. Next ready item FB-038 Product list; show proposed changes before applying, preserve Poker coding/current catalogue UI and name-or-tag search checkpoints.</x:v>
+      </x:c>
+      <x:c r="S39" s="10" t="str"/>
     </x:row>
     <x:row r="40" ht="105" customHeight="1">
       <x:c r="A40" s="9" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B40" s="9" t="inlineStr">
         <x:is>
@@ -4671,10 +4691,8 @@
           <x:t xml:space="preserve">Display the unfiltered catalogue product list</x:t>
         </x:is>
       </x:c>
-      <x:c r="E40" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">All roles see product code/name/category path/brand/status. No size, measurement units, available quantity or totals. Verify server permissions.</x:t>
-        </x:is>
+      <x:c r="E40" s="9" t="str">
+        <x:v>All roles see product name/category path/brand/status; no user-facing code. No size, measurement units, available quantity or totals. Verify server permissions.</x:v>
       </x:c>
       <x:c r="F40" s="9" t="inlineStr">
         <x:is>
@@ -4683,7 +4701,7 @@
       </x:c>
       <x:c r="G40" s="9" t="str">
         <x:f>IF(H40="Complete","Complete",IF(I40="Blocked","Blocked",IF(I40="In progress","Ready",IF(F40="","Ready",IF(COUNTIFS($B$4:$B$73,F40,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H40" s="9" t="str">
         <x:f>IF(I40="Not started","Not started",IF(I40="Blocked","Blocked",IF(I40="In progress","In progress",IF(J40&lt;&gt;"Passed","Awaiting code review",IF(OR(K40="",NOT(ISNUMBER(L40))),"Awaiting review evidence",IF(N40&lt;&gt;"Passed","Awaiting test",IF(OR(M40="",O40="",NOT(ISNUMBER(P40))),"Awaiting test evidence","Complete")))))))</x:f>
@@ -4710,16 +4728,15 @@
       <x:c r="O40" s="11" t="n"/>
       <x:c r="P40" s="31" t="n"/>
       <x:c r="Q40" s="11" t="n"/>
-      <x:c r="R40" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="R40" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S40" s="11" t="n"/>
     </x:row>
     <x:row r="41" ht="105" customHeight="1">
       <x:c r="A41" s="4" t="n">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B41" s="4" t="inlineStr">
         <x:is>
@@ -4775,16 +4792,15 @@
       <x:c r="O41" s="10" t="n"/>
       <x:c r="P41" s="30" t="n"/>
       <x:c r="Q41" s="10" t="n"/>
-      <x:c r="R41" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="R41" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S41" s="10" t="n"/>
     </x:row>
     <x:row r="42" ht="105" customHeight="1">
       <x:c r="A42" s="9" t="n">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B42" s="9" t="inlineStr">
         <x:is>
@@ -4796,15 +4812,11 @@
           <x:t xml:space="preserve">Products</x:t>
         </x:is>
       </x:c>
-      <x:c r="D42" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Add search by product code or name</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E42" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Search the full catalogue before pagination. Verify both code and name, clear search and no results.</x:t>
-        </x:is>
+      <x:c r="D42" s="9" t="str">
+        <x:v>Add search by product name or tag name</x:v>
+      </x:c>
+      <x:c r="E42" s="9" t="str">
+        <x:v>Search product names OR attached tag names across full catalogue before pagination. Halal finds products attached to Halal tag. Case-insensitive partial matching; avoid duplicate product rows for multiple matching tags; clear/no-result checks and combine with separate filters. Product-code search remains deferred to post-catalogue decision FB-035.</x:v>
       </x:c>
       <x:c r="F42" s="9" t="inlineStr">
         <x:is>
@@ -4840,17 +4852,16 @@
       <x:c r="O42" s="11" t="n"/>
       <x:c r="P42" s="31" t="n"/>
       <x:c r="Q42" s="11" t="n"/>
-      <x:c r="R42" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R42" s="11" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S42" s="11" t="n"/>
     </x:row>
     <x:row r="43" ht="105" customHeight="1">
       <x:c r="A43" s="4" t="n">
-        <x:v>40</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B43" s="4" t="inlineStr">
         <x:is>
@@ -4906,17 +4917,16 @@
       <x:c r="O43" s="10" t="n"/>
       <x:c r="P43" s="30" t="n"/>
       <x:c r="Q43" s="10" t="n"/>
-      <x:c r="R43" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R43" s="10" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S43" s="10" t="n"/>
     </x:row>
     <x:row r="44" ht="105" customHeight="1">
       <x:c r="A44" s="9" t="n">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B44" s="9" t="inlineStr">
         <x:is>
@@ -4972,17 +4982,16 @@
       <x:c r="O44" s="11" t="n"/>
       <x:c r="P44" s="31" t="n"/>
       <x:c r="Q44" s="11" t="n"/>
-      <x:c r="R44" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R44" s="11" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S44" s="11" t="n"/>
     </x:row>
     <x:row r="45" ht="105" customHeight="1">
       <x:c r="A45" s="4" t="n">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B45" s="4" t="inlineStr">
         <x:is>
@@ -5038,17 +5047,16 @@
       <x:c r="O45" s="10" t="n"/>
       <x:c r="P45" s="30" t="n"/>
       <x:c r="Q45" s="10" t="n"/>
-      <x:c r="R45" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R45" s="10" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S45" s="10" t="n"/>
     </x:row>
     <x:row r="46" ht="105" customHeight="1">
       <x:c r="A46" s="9" t="n">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B46" s="9" t="inlineStr">
         <x:is>
@@ -5104,17 +5112,16 @@
       <x:c r="O46" s="11" t="n"/>
       <x:c r="P46" s="31" t="n"/>
       <x:c r="Q46" s="11" t="n"/>
-      <x:c r="R46" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R46" s="11" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S46" s="11" t="n"/>
     </x:row>
     <x:row r="47" ht="105" customHeight="1">
       <x:c r="A47" s="4" t="n">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B47" s="4" t="inlineStr">
         <x:is>
@@ -5170,17 +5177,16 @@
       <x:c r="O47" s="10" t="n"/>
       <x:c r="P47" s="30" t="n"/>
       <x:c r="Q47" s="10" t="n"/>
-      <x:c r="R47" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R47" s="10" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S47" s="10" t="n"/>
     </x:row>
     <x:row r="48" ht="105" customHeight="1">
       <x:c r="A48" s="9" t="n">
-        <x:v>45</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B48" s="9" t="inlineStr">
         <x:is>
@@ -5236,17 +5242,16 @@
       <x:c r="O48" s="11" t="n"/>
       <x:c r="P48" s="31" t="n"/>
       <x:c r="Q48" s="11" t="n"/>
-      <x:c r="R48" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Start this item after the previous item is complete.</x:t>
-        </x:is>
+      <x:c r="R48" s="11" t="str">
+        <x:v>Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+Next: Start this item after the previous item is complete.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S48" s="11" t="n"/>
     </x:row>
     <x:row r="49" ht="105" customHeight="1">
       <x:c r="A49" s="4" t="n">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B49" s="4" t="inlineStr">
         <x:is>
@@ -5263,10 +5268,8 @@
           <x:t xml:space="preserve">Edit catalogue product details</x:t>
         </x:is>
       </x:c>
-      <x:c r="E49" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Managers/Super Admin edit catalogue fields with duplicate checks and permanent code. No packaging/stock fields. Stock-related classification constraints must be decided at stock design checkpoint.</x:t>
-        </x:is>
+      <x:c r="E49" s="4" t="str">
+        <x:v>Managers/Super Admin edit catalogue fields with duplicate checks. No code, packaging or stock fields. Stock-related classification constraints remain for the post-catalogue design checkpoint.</x:v>
       </x:c>
       <x:c r="F49" s="4" t="inlineStr">
         <x:is>
@@ -5302,16 +5305,16 @@
       <x:c r="O49" s="10" t="n"/>
       <x:c r="P49" s="30" t="n"/>
       <x:c r="Q49" s="10" t="n"/>
-      <x:c r="R49" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="R49" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.
+When adding Product edits later, preserve same duplicate identity semantics and serialize conflicting creates/edits on affected Subcategory records; current CreateProduct action is verified for creation, not future concurrent edit workflows.</x:v>
       </x:c>
       <x:c r="S49" s="10" t="n"/>
     </x:row>
     <x:row r="50" ht="105" customHeight="1">
       <x:c r="A50" s="9" t="n">
-        <x:v>47</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B50" s="9" t="inlineStr">
         <x:is>
@@ -5367,16 +5370,15 @@
       <x:c r="O50" s="11" t="n"/>
       <x:c r="P50" s="31" t="n"/>
       <x:c r="Q50" s="11" t="n"/>
-      <x:c r="R50" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="R50" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S50" s="11" t="n"/>
     </x:row>
     <x:row r="51" ht="105" customHeight="1">
       <x:c r="A51" s="4" t="n">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B51" s="4" t="inlineStr">
         <x:is>
@@ -5393,10 +5395,8 @@
           <x:t xml:space="preserve">Verify completed Product Catalogue before Stock Management</x:t>
         </x:is>
       </x:c>
-      <x:c r="E51" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Review/test hierarchy/tags/product identity, codes, duplicate/required fields, filters/pagination, responsive views and permissions. Explicitly verify no sizes/units/quantities/history/totals appear in catalogue. Stock integration/deactivation checks at FB-053; packaging setup now FB-034 before Receive.</x:t>
-        </x:is>
+      <x:c r="E51" s="4" t="str">
+        <x:v>Review/test hierarchy/tags/product identity, duplicate/required fields, name search, filters/pagination, responsive views and permissions. No product-code requirement in this phase. Verify no sizes/units/quantities/history/totals appear. Stock integration/deactivation checks remain at FB-053. Next discuss whether codes are needed at FB-035 before Stock Management FB-034.</x:v>
       </x:c>
       <x:c r="F51" s="4" t="inlineStr">
         <x:is>
@@ -5432,10 +5432,9 @@
       <x:c r="O51" s="10" t="n"/>
       <x:c r="P51" s="30" t="n"/>
       <x:c r="Q51" s="10" t="n"/>
-      <x:c r="R51" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.</x:t>
-        </x:is>
+      <x:c r="R51" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S51" s="10" t="n"/>
     </x:row>
@@ -5463,10 +5462,8 @@
           <x:t xml:space="preserve">2026-10-29 approved shared package design: Stock Management has package_sizes(id, package_type, contents, contents_unit), reusable across products; stock_items(id, product_id, package_size_id) links each catalogue product to a package definition. One unique product/package_size pair. stock_movements belongs to stock_item_id, so balances/history are separate even when package definitions are shared. Product catalogue has no size/unit/quantity fields or displays. Examples: Rice and Lentils share Bag5kg; Milk and Juice share Carton2litres; Eggs uses Carton12items (12 eggs/carton). Keep positive whole package movement quantities and whole-number individual-item contents. Reject duplicate package definitions, comparing equivalent kg/g and litres/ml contents within the same package type; a bottle differs from a carton. Once referenced by a stock item, package type/contents/unit are immutable; create another definition instead. This stronger shared-definition lock supersedes the earlier first-movement-only package lock. Shared package-size management permissions/UI, summary-configuration ownership and classification-lock details still need focused decisions before implementation. No loose-egg repacking workflow approved. Build and verify package definitions first, then stock_items connected to existing catalogue Products before Receive; preserve module order and review/testing evidence.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F52" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-067</x:t>
-        </x:is>
+      <x:c r="F52" s="9" t="str">
+        <x:v>FB-035</x:v>
       </x:c>
       <x:c r="G52" s="9" t="str">
         <x:f>IF(H52="Complete","Complete",IF(I52="Blocked","Blocked",IF(I52="In progress","Ready",IF(F52="","Ready",IF(COUNTIFS($B$4:$B$73,F52,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
@@ -5502,10 +5499,9 @@
 2026-10-29 approved shared package design: Stock Management has package_sizes(id, package_type, contents, contents_unit), reusable across products; stock_items(id, product_id, package_size_id) links each catalogue product to a package definition. One unique product/package_size pair. stock_movements belongs to stock_item_id, so balances/history are separate even when package definitions are shared. Product catalogue has no size/unit/quantity fields or displays. Examples: Rice and Lentils share Bag5kg; Milk and Juice share Carton2litres; Eggs uses Carton12items (12 eggs/carton). Keep positive whole package movement quantities and whole-number individual-item contents. Reject duplicate package definitions, comparing equivalent kg/g and litres/ml contents within the same package type; a bottle differs from a carton. Once referenced by a stock item, package type/contents/unit are immutable; create another definition instead. This stronger shared-definition lock supersedes the earlier first-movement-only package lock. Shared package-size management permissions/UI, summary-configuration ownership and classification-lock details still need focused decisions before implementation. No loose-egg repacking workflow approved.</x:t>
         </x:is>
       </x:c>
-      <x:c r="R52" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read shared package-size requirement; first settle package-management permissions and remaining summary/classification details, then teach package definitions and product/package stock_items in dependency order after FB-067. Approval is planning only; no implementation or completion evidence.</x:t>
-        </x:is>
+      <x:c r="R52" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read shared package-size requirement; first settle package-management permissions and remaining summary/classification details, then teach package definitions and product/package stock_items in dependency order after FB-067. Approval is planning only; no implementation or completion evidence.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S52" s="11" t="n"/>
     </x:row>
@@ -6348,11 +6344,13 @@
       </x:c>
       <x:c r="O65" s="11" t="n"/>
       <x:c r="P65" s="31" t="n"/>
-      <x:c r="Q65" s="11" t="n"/>
-      <x:c r="R65" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</x:t>
-        </x:is>
+      <x:c r="Q65" s="11" t="str">
+        <x:v>
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
+      </x:c>
+      <x:c r="R65" s="11" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S65" s="11" t="n"/>
     </x:row>
@@ -6413,11 +6411,13 @@
       </x:c>
       <x:c r="O66" s="10" t="n"/>
       <x:c r="P66" s="30" t="n"/>
-      <x:c r="Q66" s="10" t="n"/>
-      <x:c r="R66" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.</x:t>
-        </x:is>
+      <x:c r="Q66" s="10" t="str">
+        <x:v>
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
+      </x:c>
+      <x:c r="R66" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Use stock_items linked to reusable package_sizes per revised FB-034. Preserve module prerequisites, integrity and role checks; no sizes/quantities in catalogue. Teach/test only the current item.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
       </x:c>
       <x:c r="S66" s="10" t="n"/>
     </x:row>
@@ -6917,7 +6917,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f52d7a4e7e04b94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R519ba3ef057c447b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10129,20 +10129,14 @@
           <x:t xml:space="preserve">Inventory management — first version, planning complete</x:t>
         </x:is>
       </x:c>
-      <x:c r="C100" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current scope</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D100" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Every product has a unique, permanent, automatically generated code using the format PRD-000001, independent of its name and category. Use sequential numbers starting at 1, padded to at least six digits; allow longer numbers after PRD-999999. Users cannot edit product codes, and codes are never reused. Each separate catalogue product record, including brand variants, receives its own code. Under the approved module separation, package sizes are reusable Stock Management definitions linked through stock_items; different package sizes of the same catalogue product share that product code. Neither a stock_items ID nor a package_sizes ID replaces the permanent catalogue product code.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E100" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-035</x:t>
-        </x:is>
+      <x:c r="C100" s="4" t="str">
+        <x:v>Deferred decision after catalogue</x:v>
+      </x:c>
+      <x:c r="D100" s="4" t="str">
+        <x:v>2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion. Previous agreed design retained for discussion only: unique permanent automatically generated PRD-000001 onward, sequential at least six digits/growing beyond999999, never edited/reused, independent of classification and package sizes. Do not implement automatically.</x:v>
+      </x:c>
+      <x:c r="E100" s="4" t="str">
+        <x:v>FB-035 (after FB-067, before FB-034)</x:v>
       </x:c>
       <x:c r="F100" s="4" t="inlineStr">
         <x:is>
@@ -10358,15 +10352,12 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D107" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tags are shared across the product catalogue: create a tag once and reuse it on multiple products. A product can have multiple tags or none.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E107" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FB-031, FB-037, FB-048</x:t>
-        </x:is>
+      <x:c r="D107" s="28" t="str">
+        <x:v>Tags are shared across the product catalogue: create a tag once and reuse it on multiple products. A product can have multiple tags or none.
+2026-10-30 developer explicitly requires the reverse Tag-&gt;products relationship so products can be looked up for a tag. Use Tag::products() and Product::tags(), both belongsToMany through the SAME product_tag linking table. Future product-list main search must match tag names as well as product names: searching Halal returns products attached to the Halal tag. Keep existing separate tag filter and other filters; filter before pagination and avoid duplicated product rows when several tags match. No product-code search. Relationship is part of pending save implementation; list-search behaviour belongs at FB-040/044 and is not implemented by merely declaring the relationship.</x:v>
+      </x:c>
+      <x:c r="E107" s="28" t="str">
+        <x:v>FB-031, FB-037, FB-040, FB-044, FB-048</x:v>
       </x:c>
       <x:c r="F107" s="28" t="inlineStr">
         <x:is>
@@ -10486,10 +10477,9 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D111" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29 approved module separation: Product Catalogue form fields: required product name, full Department/Category/Subcategory selection and status (default Active); optional brand and tags. Product code generated automatically. No package size, counting/contents/summary unit, stock quantity, balance or calculated stock total in catalogue storage/forms/screens. Packaging and stock records belong to Stock Management.</x:t>
-        </x:is>
+      <x:c r="D111" s="28" t="str">
+        <x:v>2026-10-30 revised: Product Catalogue form fields: required product name, full Department/Category/Subcategory selection and status (default Active); optional brand and tags. Build this phase without product codes or code generation. Keep internal database id. Reconsider user-facing codes after functional catalogue verification at FB-035. No package size, counting/contents/summary unit, stock quantity, balance or total in catalogue storage/forms/screens; these belong to Stock Management.
+2026-10-30 developer explicitly changed PRODUCT Status UI from radio buttons to paired Active/Inactive checkboxes. Follow existing FoodBank User Create pattern: both bind same boolean is_active, Active true-value=true/false-value=false, Inactive inverted values. Exactly one remains checked, Active default preserved. Supersedes Product-form radio UI only; no other account requirement changed.</x:v>
       </x:c>
       <x:c r="E111" s="28" t="inlineStr">
         <x:is>
@@ -11030,10 +11020,9 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D128" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Distribution flow: search/select one household by reference, contact name, or phone; select a subcategory such as Rice, then choose from its active products with stock greater than zero. Show available package sizes, product name, brand, product code, and available package counts so equal sizes from different products remain distinguishable. Retain product search by code or name within this selection flow. Users can select multiple products/sizes and enter positive whole-number quantities; review the household and product quantities before confirming. Recheck stock when saving. On success, show a success message and read-only distribution summary. On failure, retain entered information so staff can correct it. 2026-10-29 clarification: package choices and quantities are selected in Stock Management only; catalogue contains no such fields. Selectable stock rows are stock_items, each connecting an active product and package_sizes definition.</x:t>
-        </x:is>
+      <x:c r="D128" s="4" t="str">
+        <x:v>Distribution flow: search/select one household by reference, contact name, or phone; select a subcategory such as Rice, then choose from its active products with stock greater than zero. Show available package sizes, product name, brand, product code, and available package counts so equal sizes from different products remain distinguishable. Retain product search by code or name within this selection flow. Users can select multiple products/sizes and enter positive whole-number quantities; review the household and product quantities before confirming. Recheck stock when saving. On success, show a success message and read-only distribution summary. On failure, retain entered information so staff can correct it. 2026-10-29 clarification: package choices and quantities are selected in Stock Management only; catalogue contains no such fields. Selectable stock rows are stock_items, each connecting an active product and package_sizes definition.
+2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion. Code display/search in this later stock workflow must be reconciled with the post-catalogue decision before implementation; all other agreed workflow safeguards remain.</x:v>
       </x:c>
       <x:c r="E128" s="4" t="inlineStr">
         <x:is>
@@ -11574,10 +11563,9 @@
           <x:t xml:space="preserve">Current scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D145" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-29 approved module separation: Catalogue list shows product code, product name, category path, optional brand/tags and status; NO sizes, units, quantities, available stock or totals. Retain all-role search by code/name and filters for Department, Category, Subcategory, tag and status. Stock Management supplies its separate quantity/size views.</x:t>
-        </x:is>
+      <x:c r="D145" s="28" t="str">
+        <x:v>2026-10-30 revised: Catalogue list shows product name, category path, optional brand/tags and status; no user-facing product code. All roles can search by product name and filter by Department, Category, Subcategory, tag and status. No sizes, units, quantities, available stock or totals. Reconsider product codes only after catalogue verification at FB-035.
+2026-10-30 developer explicitly requires the reverse Tag-&gt;products relationship so products can be looked up for a tag. Use Tag::products() and Product::tags(), both belongsToMany through the SAME product_tag linking table. Future product-list main search must match tag names as well as product names: searching Halal returns products attached to the Halal tag. Keep existing separate tag filter and other filters; filter before pagination and avoid duplicated product rows when several tags match. No product-code search. Relationship is part of pending save implementation; list-search behaviour belongs at FB-040/044 and is not implemented by merely declaring the relationship.</x:v>
       </x:c>
       <x:c r="E145" s="28" t="inlineStr">
         <x:is>
@@ -13077,6 +13065,27 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="192">
+      <x:c r="A192" t="str">
+        <x:v>REQ-189</x:v>
+      </x:c>
+      <x:c r="B192" t="str">
+        <x:v>Product Catalogue — Create form tag search</x:v>
+      </x:c>
+      <x:c r="C192" t="str">
+        <x:v>Current scope</x:v>
+      </x:c>
+      <x:c r="D192" t="str">
+        <x:v>2026-10-30 developer approved Product creation tag search: labelled Search tags input filters the already-loaded tag list locally with case-insensitive partial name matching, ignoring outer search spaces. Apply300ms after typing stops or immediately on Enter; Enter must not submit Product form, and cancels pending timer. Clear search restores all tags. Hidden checked tags stay selected. Show No matching tags found for zero matches; distinguish No tags available when catalogue has none. Cancel timer on leaving page. No server requests or persistence added.
+2026-10-30 developer requested tag width same as Department; implemented as tag SEARCH field width. Added grid gap-4 lg:grid-cols-3 search row containing existing grid gap-2 label/input group, matching hierarchy parent columns/gap exactly on wide screens; full width on smaller screens. Tag checkbox list remains full-width. Changed only products/Create.vue layout. Formatter/build/whitespace PASS; no browser check performed. Await developer confirmation of intended width/search behaviour.</x:v>
+      </x:c>
+      <x:c r="E192" t="str">
+        <x:v>FB-032, FB-033, FB-037</x:v>
+      </x:c>
+      <x:c r="F192" t="str">
+        <x:v>Stories!B35</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:F2"/>
@@ -13087,7 +13096,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88c854d9e0594d9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f3392e708a64010"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Seed five branded products per subcategory with tags
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5072960b892545b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R729ccbd23610418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R415a6c94041e4a77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R736468c541374ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R7806b91ff2fa40be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rd966852c4b0e4580"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -717,7 +717,7 @@
     <x:row r="12">
       <x:c r="A12" s="15" t="n"/>
       <x:c r="B12" s="15" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read full FB-038 and related Requirements before starting list. Product creation FB-032/033/036/037 verified with scoped checks; baseline global failures remain recorded. Next preview basic unfiltered Product list showing name/path/brand/tags/status, all-role server viewAny permission, no codes/stock fields. Complete basic list before filters; main name-or-tag search later FB-040 and tag filterFB-044. Preserve show-before-apply preference; current Product save/testing delegation does not automatically authorize unrelated list implementation. Product code decision stays after catalogue verification at FB-035; Stock Management not started.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. ProductSeeder approved/installed/run and rerun verified;750 branded Active Products now ready for list development. Read FB-038 and related Requirements; preview basic unfiltered Product list with name/path/brand/tags/status and all-role viewAny permission before applying. Show changes first per developer preference. No Product list implementation authorized by the seeding request. Main product-or-tag search and filters remain later FB-040/044, no product codes/stock fields. Existing baseline account test failures remain separate; PHP analysis now0 errors.</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n"/>
       <x:c r="D12" s="15" t="n"/>
@@ -743,8 +743,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>Product creation checkpoint complete after source review,157-test catalogue pass, MySQL concurrency and browser checks. Basic Product list is next; not started.
-Separate completed repair: 2026-10-30 developer explicitly authorized fixing all7 PHP analysis issues only. Updated ListSubcategories precise paginator row-shape annotation and explicit scalar field mapping (same outgoing keys/values); added void return types to empty show/destroy methods in DepartmentController, CategoryController and SubcategoryController, matching inspected Poker empty destroy convention. No runtime features, account tests, suppression comments or config/baselines changed. Scoped source/diff review PASS; full vendor/bin/phpstan analyse --memory-limit=512M --no-progress PASS0 errors; scoped Pint and whitespace PASS. Delegated affected regression php artisan test tests/Feature/SubcategoryListTest.php tests/Feature/SubcategoryEditTest.php PASS43 tests357 assertions. This supersedes earlier notes that7 PHP analysis issues remain unresolved. Previously recorded18 baseline account/auth test failures remain separate and unfixed; no full-suite rerun for this typing-only fix.</x:v>
+        <x:v>2026-10-30 developer approved draft and explicitly requested creating/running ProductSeeder. Installed reviewed /tmp/foodbank-tags-tracker/ProductSeeder.preview.php into database/seeders/ProductSeeder.php (previously empty scaffold), then ran php artisan db:seed --class=ProductSeeder successfully against local MySQL. Actual database verification PASS:750 products across150 Subcategories, EXACTLY5 each, all Active/nonblank brand, each2–4 tags,1618 product_tag links,0 duplicate product identities. Shared tags now54 (original50 plus approved Baby Essentials/Personal Hygiene/Cleaning Supplies/Paper Goods). Ran seeder again successfully; SHA256 fingerprint of ALL ordered product records including timestamps, tag records and pivot links was identical before/after rerun: no added rows, changes or duplicates. Full PHPStan PASS0 errors, scoped Pint/whitespace PASS. Source review preserves exact-path lookup, Subcategory locking/transaction, firstOrCreate identity and syncWithoutDetaching manual-tag preservation; no code/stock fields and no default DatabaseSeeder registration added. No application test suite/browser checks needed/run for this data-only side task. Next Product list FB-038 remains NOT STARTED.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -754,7 +753,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Read full FB-038 and related Requirements before starting list. Product creation FB-032/033/036/037 verified with scoped checks; baseline global failures remain recorded. Next preview basic unfiltered Product list showing name/path/brand/tags/status, all-role server viewAny permission, no codes/stock fields. Complete basic list before filters; main name-or-tag search later FB-040 and tag filterFB-044. Preserve show-before-apply preference; current Product save/testing delegation does not automatically authorize unrelated list implementation. Product code decision stays after catalogue verification at FB-035; Stock Management not started.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. ProductSeeder approved/installed/run and rerun verified;750 branded Active Products now ready for list development. Read FB-038 and related Requirements; preview basic unfiltered Product list with name/path/brand/tags/status and all-role viewAny permission before applying. Show changes first per developer preference. No Product list implementation authorized by the seeding request. Main product-or-tag search and filters remain later FB-040/044, no product codes/stock fields. Existing baseline account test failures remain separate; PHP analysis now0 errors.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -764,7 +763,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Developer readiness to begin basic Product list; show changes first.</x:v>
+        <x:v>Developer readiness to begin Product list; seeding side task complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -4308,7 +4307,8 @@
 2026-10-30 developer explicitly delegated all current Tag work and testing, following this project catalogue UI/coding/workflows. Completed-feature source review PASS at HEAD eabb3204ee4e2f9dbea824ef3b5939230e379d20 plus uncommitted Tag implementation: app/Models/Tag.php, app/Http/Controllers/TagController.php, app/Http/Requests/Tags/{IndexTagsRequest,StoreTagRequest,UpdateTagRequest}.php, app/Actions/Tags/ListTags.php, app/Policies/TagPolicy.php, routes/web.php, database/migrations/2026_10_30_061953_create_tags_table.php, resources/js/pages/tags/{Create,Index,Edit}.vue, tests/Feature/TagTest.php. Department screen/controller/request conventions and Subcategory per-row canEdit preparation reused. Protected GET list/create/edit and POST/PATCH; Manager/Super Admin allowed, Volunteer denied. Required unique max255 name; Laravel trims, local MySQL collation ignores case. Rename preserves ID, ignores self in uniqueness. Protected fillable/validated fields. Search before alphabetical paginate(10), links retain search; 300ms typing/Enter/empty states. Forms errors, processing, success reset/toast, Cancel/list redirect, accessible labels/error links and phone layout. No blocking findings. No Product/pivot/stock work or deletion endpoint; Product tag attachment FB-037 and deletion rule FB-048 remain open. TagSeeder remains original empty scaffold; no production seed data requested.
 2026-10-30 developer explicitly requested TagSeeder file with50 realistic tags so developer can run it. Updated database/seeders/TagSeeder.php only:50 distinct dietary/storage/preparation/meal/personal-care/household labels; Tag::firstOrCreate inside DB::transaction follows current catalogue seeder conventions and preserves existing names/records on reruns. Source review, PHP syntax, scoped Pint and static count/case-folded uniqueness checks PASS. Seeder NOT executed; no database changes or runtime/idempotence pass claimed. Supplied php artisan db:seed --class=TagSeeder for developer to run. Product lesson remains pending; no Product code read/changed.
 2026-10-30 developer explicitly requested removing assistant-added defineOptions({ inheritAttrs:false }) from Product Create, Tag Create/Index/Edit and Subcategory Create/Index/Edit; follow Poker pages and avoid unnecessary code. Removed only those declarations, associated explanatory comments and blank separators in all7 pages. Shared components unchanged. Poker page scan confirmed no inheritAttrs declarations. Scoped source diff/absence/whitespace check, Vue typecheck and asset build PASS. No browser/feature acceptance tests rerun; prior behaviour evidence remains historical. Earlier page-scaffold instructions including inheritAttrs are superseded by this explicit correction. No other Product implementation authorization.
-2026-10-30 Tag inverse products relationship reviewed and tested with Product creation; TagTest regressions included in157-test pass. Shared tag rename preserves product links.</x:v>
+2026-10-30 Tag inverse products relationship reviewed and tested with Product creation; TagTest regressions included in157-test pass. Shared tag rename preserves product links.
+2026-10-30 developer approved draft and explicitly requested creating/running ProductSeeder. Installed reviewed /tmp/foodbank-tags-tracker/ProductSeeder.preview.php into database/seeders/ProductSeeder.php (previously empty scaffold), then ran php artisan db:seed --class=ProductSeeder successfully against local MySQL. Actual database verification PASS:750 products across150 Subcategories, EXACTLY5 each, all Active/nonblank brand, each2–4 tags,1618 product_tag links,0 duplicate product identities. Shared tags now54 (original50 plus approved Baby Essentials/Personal Hygiene/Cleaning Supplies/Paper Goods). Ran seeder again successfully; SHA256 fingerprint of ALL ordered product records including timestamps, tag records and pivot links was identical before/after rerun: no added rows, changes or duplicates. Full PHPStan PASS0 errors, scoped Pint/whitespace PASS. Source review preserves exact-path lookup, Subcategory locking/transaction, firstOrCreate identity and syncWithoutDetaching manual-tag preservation; no code/stock fields and no default DatabaseSeeder registration added. No application test suite/browser checks needed/run for this data-only side task. Next Product list FB-038 remains NOT STARTED.</x:v>
       </x:c>
       <x:c r="L34" s="30" t="n">
         <x:v>46325</x:v>
@@ -4646,7 +4646,8 @@
       </x:c>
       <x:c r="K39" s="10" t="str">
         <x:v>
-2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.</x:v>
+2026-10-30 completed Product CREATION feature source review PASS; no blocking findings. Developer explicitly approved save workflow including both relationship directions and delegated all tests. Read together ProductController, ProductPolicy, StoreProductRequest, CreateProduct action, Product/Subcategory/Tag models, Product and product_tag migrations, full products/Create.vue, protected GET/POST routes and ProductCreateTest. Follows inspected Poker Player request/controller/flash/back, Inertia Form+generated action/errors/processing/resetOnSuccess; CreatePlayerGame/CreateGameSession action Gate+transaction+row lock conventions. StoreProductRequest organized under Products; productData normalizes already-validated scalar/list values for typed action input. Duplicate business guard executes under Subcategory exclusive lock inside transaction after Category shared lock/current hierarchy recheck; ignores name/brand case/outer spaces, blank brands equivalent, includes inactive products. Selected tag existence rechecked/locked. Save only name/brand/subcategory_id/is_active; no forged IDs/code/quantity/parent duplication. Product::tags and Tag::products both belongsToMany through same unique-pair product_tag with restrictive FKs. Form transform sends all selected tag IDs even when search hides inputs; invalid submissions retain state; success clears controls/search/tags/restores Active and resets Select display. Existing layout/tag search/checkbox status preserved. Removed unused empty ProductController scaffold methods, leaving create/store only; unused UpdateProductRequest scaffold unchanged. No list/search-by-tag UI added early; FB-040/044 remain upcoming. HEAD 3c9d80b6e737c9c750d0eaadc5e9bec3b2f71123 plus current uncommitted Product creation implementation, reviewed2026-10-30. SHA256 prefixes: action3659726855ae; request3bfa3f723881; controllercad1463244ea; Product068970cd06b8; Tagd8f3fd7ceb8f; policy12099f89fdad; Vue8f12052c3721; Product migration3f2353b33f65; pivot migratione210a481a24a; testeeef404a32c0; routes900151e5ce7a.
+2026-10-30 developer approved draft and explicitly requested creating/running ProductSeeder. Installed reviewed /tmp/foodbank-tags-tracker/ProductSeeder.preview.php into database/seeders/ProductSeeder.php (previously empty scaffold), then ran php artisan db:seed --class=ProductSeeder successfully against local MySQL. Actual database verification PASS:750 products across150 Subcategories, EXACTLY5 each, all Active/nonblank brand, each2–4 tags,1618 product_tag links,0 duplicate product identities. Shared tags now54 (original50 plus approved Baby Essentials/Personal Hygiene/Cleaning Supplies/Paper Goods). Ran seeder again successfully; SHA256 fingerprint of ALL ordered product records including timestamps, tag records and pivot links was identical before/after rerun: no added rows, changes or duplicates. Full PHPStan PASS0 errors, scoped Pint/whitespace PASS. Source review preserves exact-path lookup, Subcategory locking/transaction, firstOrCreate identity and syncWithoutDetaching manual-tag preservation; no code/stock fields and no default DatabaseSeeder registration added. No application test suite/browser checks needed/run for this data-only side task. Next Product list FB-038 remains NOT STARTED.</x:v>
       </x:c>
       <x:c r="L39" s="30" t="n">
         <x:v>46325</x:v>
@@ -4727,10 +4728,11 @@
       </x:c>
       <x:c r="O40" s="11" t="n"/>
       <x:c r="P40" s="31" t="n"/>
-      <x:c r="Q40" s="11" t="n"/>
+      <x:c r="Q40" s="11" t="str">
+        <x:v>2026-10-30 developer approved draft and explicitly requested creating/running ProductSeeder. Installed reviewed /tmp/foodbank-tags-tracker/ProductSeeder.preview.php into database/seeders/ProductSeeder.php (previously empty scaffold), then ran php artisan db:seed --class=ProductSeeder successfully against local MySQL. Actual database verification PASS:750 products across150 Subcategories, EXACTLY5 each, all Active/nonblank brand, each2–4 tags,1618 product_tag links,0 duplicate product identities. Shared tags now54 (original50 plus approved Baby Essentials/Personal Hygiene/Cleaning Supplies/Paper Goods). Ran seeder again successfully; SHA256 fingerprint of ALL ordered product records including timestamps, tag records and pivot links was identical before/after rerun: no added rows, changes or duplicates. Full PHPStan PASS0 errors, scoped Pint/whitespace PASS. Source review preserves exact-path lookup, Subcategory locking/transaction, firstOrCreate identity and syncWithoutDetaching manual-tag preservation; no code/stock fields and no default DatabaseSeeder registration added. No application test suite/browser checks needed/run for this data-only side task. Next Product list FB-038 remains NOT STARTED.</x:v>
+      </x:c>
       <x:c r="R40" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
-2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. ProductSeeder approved/installed/run and rerun verified;750 branded Active Products now ready for list development. Read FB-038 and related Requirements; preview basic unfiltered Product list with name/path/brand/tags/status and all-role viewAny permission before applying. Show changes first per developer preference. No Product list implementation authorized by the seeding request. Main product-or-tag search and filters remain later FB-040/044, no product codes/stock fields. Existing baseline account test failures remain separate; PHP analysis now0 errors.</x:v>
       </x:c>
       <x:c r="S40" s="11" t="n"/>
     </x:row>
@@ -6917,7 +6919,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R519ba3ef057c447b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d9b8b46002643f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13096,7 +13098,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f3392e708a64010"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R040b1ade40b8441f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
User Module and Product Catalog Completed
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R785979c1128340a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R02a01c9269424ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R4718d7d39cbb4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R18fee2bffe2b41db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="Rd80bb63010684da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3bdfb2fe6a142c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -654,7 +654,7 @@
       </x:c>
       <x:c r="B7" s="15" t="n">
         <x:f>COUNTIF(Stories!H4:H73,"In progress")</x:f>
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C7" s="15" t="n"/>
     </x:row>
@@ -717,7 +717,7 @@
     <x:row r="12">
       <x:c r="A12" s="15" t="n"/>
       <x:c r="B12" s="15" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-047 verified. Commit checkpoint: Add protected product editing with validation and tag syncing. Next FB-048: teach existing Active/Inactive and tag removal behavior in small steps; inspect agreed tag deletion requirements/conventions before additional implementation. Stock-based deactivation integrity requires explicit later FB-053 checkpoint; do not mark FB-048 complete before required evidence. No new application changes authorized beyond Edit link.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Developer check sidebar links, list/create/edit highlights, collapsed/mobile layout and role visibility. Then return to FB-048/067 catalogue evidence reconciliation. Stock guard stays FB-053; remaining FB-008 landing-page work deferred.</x:v>
       </x:c>
       <x:c r="C12" s="15" t="n"/>
       <x:c r="D12" s="15" t="n"/>
@@ -733,7 +733,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="22" t="str">
-        <x:v>FB-048</x:v>
+        <x:v>FB-008</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="100" customHeight="1">
@@ -743,7 +743,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>2026-10-30 explicitly authorized list Edit link implemented: ListProducts::get accepts actor and evaluates can(update,product) per row; ProductController passes authenticated user; Index.vue typed canUpdate, policy-aware Actions/header/cells and dynamic empty colspan, accessible Edit product-name labels linking correct ID. Existing server GET/PATCH protections unchanged. Reviewed changes against prior completed-feature review at HEAD7c24b5cf9e6a50e730d746ad821ee76d9e26671d plus editing working tree. Missing-entry finding resolved; source review PASS for FB-047 catalogue editing scope. Delegated affected checks PASS48 tests515 assertions (temporary edit checks22 plus ProductListTest26), covering Manager/SuperAdmin permission true and GET allowed, Volunteer false/403; prior save/rollback/validation tests still pass. PHPStan0 errors, Vue types, scoped Pint/Vue formatting, build and whitespace PASS. Brave as SuperAdmin list showed Actions/Edit links, clicked Edit Acorn Squash and verified /products/41/edit with correct saved details; no record edits in this final check. No Volunteer browser sign-in performed; omission follows server flags and reviewed Vue condition. Previous browser save/required-error/restoration evidence retained. FB-047 verified; FB-048 remains separate, stock-dependent checks not claimed.</x:v>
+        <x:v>2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -753,7 +753,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. FB-047 verified. Commit checkpoint: Add protected product editing with validation and tag syncing. Next FB-048: teach existing Active/Inactive and tag removal behavior in small steps; inspect agreed tag deletion requirements/conventions before additional implementation. Stock-based deactivation integrity requires explicit later FB-053 checkpoint; do not mark FB-048 complete before required evidence. No new application changes authorized beyond Edit link.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Developer check sidebar links, list/create/edit highlights, collapsed/mobile layout and role visibility. Then return to FB-048/067 catalogue evidence reconciliation. Stock guard stays FB-053; remaining FB-008 landing-page work deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -763,7 +763,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Next small lesson: FB-048 status and tags; no new code authorized.</x:v>
+        <x:v>Developer-first sidebar behaviour checks pending; remaining FB-008 deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -773,7 +773,7 @@
         </x:is>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>7c24b5cf9e6a50e730d746ad821ee76d9e26671d plus uncommitted Product editing files; reviewed2026-10-30; Product editing including permission-aware list Edit link reviewed and verified2026-10-30.</x:v>
+        <x:v>f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus four sidebar-related files, source-reviewed2026-10-30.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -783,7 +783,7 @@
         </x:is>
       </x:c>
       <x:c r="B18" s="18" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Sidebar implemented; behaviour checks pending. Remaining FB-008 deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3390,20 +3390,21 @@
       </x:c>
       <x:c r="O24" s="10" t="n"/>
       <x:c r="P24" s="30" t="n"/>
-      <x:c r="Q24" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R24" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Deferred to project end by developer on 2026-10-29. Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
+      <x:c r="Q24" s="10" t="str">
+        <x:v>
+2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
+2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
+      </x:c>
+      <x:c r="R24" s="10" t="str">
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Deferred to project end by developer on 2026-10-29. Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
 Next: Connect login redirects to the already verified lists from FB-009–FB-015. Build the volunteer welcome page and connect the completed password-change action from FB-024 and logout. Verify each role and forced-setup priority; add inventory links only as those modules are completed.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S24" s="10" t="n"/>
+2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
+Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Developer check sidebar links, list/create/edit highlights, collapsed/mobile layout and role visibility. Then return to FB-048/067 catalogue evidence reconciliation. Stock guard stays FB-053; remaining FB-008 landing-page work deferred.</x:v>
+      </x:c>
+      <x:c r="S24" s="10" t="str">
+        <x:v>
+2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="105" customHeight="1">
       <x:c r="A25" s="9" t="n">
@@ -5500,12 +5501,10 @@
       </x:c>
       <x:c r="H50" s="9" t="str">
         <x:f>IF(I50="Not started","Not started",IF(I50="Blocked","Blocked",IF(I50="In progress","In progress",IF(J50&lt;&gt;"Passed","Awaiting code review",IF(OR(K50="",NOT(ISNUMBER(L50))),"Awaiting review evidence",IF(N50&lt;&gt;"Passed","Awaiting test",IF(OR(M50="",O50="",NOT(ISNUMBER(P50))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I50" s="11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J50" s="11" t="inlineStr">
         <x:is>
@@ -5522,12 +5521,22 @@
       </x:c>
       <x:c r="O50" s="11" t="n"/>
       <x:c r="P50" s="31" t="n"/>
-      <x:c r="Q50" s="11" t="n"/>
+      <x:c r="Q50" s="11" t="str">
+        <x:v>2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.</x:v>
+      </x:c>
       <x:c r="R50" s="11" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
-2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
-      </x:c>
-      <x:c r="S50" s="11" t="n"/>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Browser blocked-tag error and phone layout checks PASS2026-10-30 in in-app browser; preserve historical191 catalogue+24 editing passes. Reconcile catalogue checkpoint FB-067 evidence and deferred FB-053 stock guard before completion; do not claim successful-delete/toast interaction observed. Then approved next discussion FB-035: whether visible product codes are needed before Stock Management FB-034.</x:v>
+      </x:c>
+      <x:c r="S50" s="11" t="str">
+        <x:v>2026-10-30 developer explicitly delegated checking status changes/tag removal. Read AGENTS and FB-048/related requirements. Targeted isolated in-memory SQLite HTTP tests outside repo PASS2 tests86 assertions (Manager and SuperAdmin). Verified deactivate persists false, saved edit props false/tag IDs, inactive list inclusion, removal of one selected shared tag leaves shared tag record and other inactive product link unchanged, reactivation true, remove-all tags supported with both tag records retained, active list inclusion, reattach existing tags, products not deleted. Source review of current UpdateProduct sync/update implementation supports this subset. No application source or permanent test changes. Browser attempt interrupted by user browser activity before executing status/tag changes; no browser status/tag acceptance claimed and no browser record changes performed. Shared-tag deletion not implemented/verified in this check. Stock-based deactivation guard remains unimplemented/unverified until FB-053; full FB-048 not complete.
+2026-10-30 developer explicitly authorized unused shared tag deletion, blocking all product usage. Inspected Poker DeactivatePlayer action and FoodBank TagController/TagPolicy/ListTags/tags Index/product_tag RESTRICT foreign key. Implemented DeleteTag action: independent delete Gate, transaction and exclusive tag lock interoperating with Product save shared tag locks, products()-&gt;exists without active filter, ValidationException blocked message, delete only unused tag; no detach/cascade. TagPolicy delete Manager/SuperAdmin; protected numeric DELETE /tags/{tag} route and controller destroy success toast/back. ListTags canDelete per policy; Vue Delete confirmation, useForm deletion/errors, disabled concurrent deletion and Deleting label, accessible labels, flex-wrap/gap actions, alert on used-tag failure. Source review PASS for this change; PHPStan0 errors, Vue types, scoped Pint/Vue format, production build and whitespace PASS. No browser deletion or application behaviour tests executed: developer-first check pending. Prior delegated status/tag-removal evidence retained. No migrations or existing data changes. FB-048 remains in progress: shared deletion behaviour and later stock guard not verified.
+2026-10-30 developer explicitly delegated tag-deletion checks including active/inactive usage. Added temporary isolated checks outside repo /tmp/foodbank-lesson-tracker/TagDeleteCheckTest.php, in-memory SQLite. New11 checks PASS: Manager and SuperAdmin delete unused tag and keep unrelated tag; both roles blocked for active and inactive linked product preserving tag/pivot/status; independent action blocks mixed active+inactive usage and still blocks after active link removed, permits only after last inactive link removed without deleting products; guests/Volunteers denied; direct action denies Volunteer; missing/nonnumeric IDs404. Combined with existing TagTest:30 tests29 passed1 failed311 assertions. Sole failure existing tests/Feature/TagTest.php line118 expects405 deletion not exposed, now actual302 success redirect by approved feature; obsolete assertion, not a failed active/inactive guard. No permanent tests or application source modified in checking turn. Shared-tag deletion backend guards/source reviewed PASS; browser confirmation/cancel/loading/error display not exercised in this turn. No current catalogue records modified. Stock guard remains unverified at FB-053; FB-048 stays open pending obsolete regression-test repair and full remaining checks.
+2026-10-30 developer explicitly authorized updating outdated TagTest and rerunning tests. Changed only tests/Feature/TagTest.php: removed obsolete405 deletion-not-exposed expectation; retained missing-tag checks and added missing/nonnumeric DELETE404; added permanent Manager/SuperAdmin unused deletion, both roles active/inactive usage rejection preserving links/status, mixed-user last-link release action coverage and direct Volunteer action denial; existing guest/Volunteer write tests now include DELETE. Reviewed focused test diff PASS; Pint/whitespace PASS. Delegated run php artisan test tests/Feature/TagTest.php tests/Feature/ProductCreateTest.php tests/Feature/ProductListTest.php PASS95 tests898 assertions. This resolves prior obsolete regression failure; no application source changes. Previous temporary guard tests/status tests preserved. Browser confirmation/Cancel/loading/error flow still unverified; stock-dependent deactivation remains later FB-053. FB-048 not marked complete.
+2026-10-30 developer explicitly delegated browser tag-deletion screen then whole catalogue review. Read current AGENTS and related catalogue Requirements. Reviewed current hierarchy/tag/product models, migrations, protected routes, policies, controllers, form requests/actions and Vue state/layout/filter/error flows against current scope at HEADf26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus current Tag deletion/test working changes. No blocking finding in reviewed current-phase code; stock-dependent deactivation remains explicit later checkpoint, not passed. Automated catalogue suite PASS191 tests1579 assertions (DepartmentEdit,CategoryEdit,SubcategoryCreate/Edit/List,Tag,ProductCreate/List); focused outside-repo edit/status/list-permission checks PASS24 tests248 assertions. Full PHPStan0 errors, Vue types and whitespace PASS. Browser as SuperAdmin foodbank.test/tags: clicked Delete Cooking Required, confirmation named exact tag; Cancel returned with row preserved. Created unused disposable tag ZZ Browser Deletion Practice1030 via Create screen (actual exact name ZZ Browser Deletion Practice 1030, id69), search isolated it; Delete confirmation now open, not confirmed. Browser-use policy requires action-time confirmation before permanent deletion. Pending async question authorizes deleting ONLY this exact test tag; no response yet. No existing tag deleted. Browser successful deletion/blocked error and phone layout remain unverified in this review. No application source edits. Do not mark FB-048/067 complete pending browser evidence and scope-specific deferred guard accounting.
+2026-10-30 user approved permanent deletion of ONLY unused test tag ZZ Browser Deletion Practice 1030. On reacquiring FoodBank tab after approval, confirmation was no longer open and filtered list already showed No tags found. Reload confirmed absence; read-only live Tag query by exact name returned false. Assistant did not click OK or delete anything after approval, and did not observe success toast; cannot attribute deletion or claim full successful-deletion interaction observed. Disposable tag absent and no cleanup needed. Previous source/tests/Cancel confirmation evidence remains valid. Remaining browser blocked-error and narrow-screen verification still open; no whole-catalogue completion claimed.
+2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.
+2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="105" customHeight="1">
       <x:c r="A51" s="4" t="n">
@@ -5558,16 +5567,14 @@
       </x:c>
       <x:c r="G51" s="4" t="str">
         <x:f>IF(H51="Complete","Complete",IF(I51="Blocked","Blocked",IF(I51="In progress","Ready",IF(F51="","Ready",IF(COUNTIFS($B$4:$B$73,F51,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</x:f>
-        <x:v>Waiting</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="H51" s="4" t="str">
         <x:f>IF(I51="Not started","Not started",IF(I51="Blocked","Blocked",IF(I51="In progress","In progress",IF(J51&lt;&gt;"Passed","Awaiting code review",IF(OR(K51="",NOT(ISNUMBER(L51))),"Awaiting review evidence",IF(N51&lt;&gt;"Passed","Awaiting test",IF(OR(M51="",O51="",NOT(ISNUMBER(P51))),"Awaiting test evidence","Complete")))))))</x:f>
-        <x:v>Not started</x:v>
-      </x:c>
-      <x:c r="I51" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not started</x:t>
-        </x:is>
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I51" s="10" t="str">
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J51" s="10" t="inlineStr">
         <x:is>
@@ -5584,12 +5591,18 @@
       </x:c>
       <x:c r="O51" s="10" t="n"/>
       <x:c r="P51" s="30" t="n"/>
-      <x:c r="Q51" s="10" t="n"/>
+      <x:c r="Q51" s="10" t="str">
+        <x:v>2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.</x:v>
+      </x:c>
       <x:c r="R51" s="10" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Follow revised module separation and dependencies; implement only this item’s approved scope in small lessons. Record source review and developer-first/delegated test evidence.
-2026-10-30 developer-approved sequence/scope revision: build and verify functional Product Catalogue without human-readable product codes. Omit code column, generation, display, code search and code acceptance checks for this catalogue phase. Keep normal internal Product id and Subcategory relationship. After catalogue checkpoint FB-067, brainstorm again at preserved FB-035 whether a user-facing code is needed and revisit code/stock design before Stock Management FB-034. Earlier PRD format is historical proposal pending reconsideration, not a current implementation requirement; no replacement format/design approved and no application code edits authorized by this discussion.</x:v>
-      </x:c>
-      <x:c r="S51" s="10" t="n"/>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Browser blocked-tag error and phone layout checks PASS2026-10-30 in in-app browser; preserve historical191 catalogue+24 editing passes. Reconcile catalogue checkpoint FB-067 evidence and deferred FB-053 stock guard before completion; do not claim successful-delete/toast interaction observed. Then approved next discussion FB-035: whether visible product codes are needed before Stock Management FB-034.</x:v>
+      </x:c>
+      <x:c r="S51" s="10" t="str">
+        <x:v>2026-10-30 developer explicitly delegated browser tag-deletion screen then whole catalogue review. Read current AGENTS and related catalogue Requirements. Reviewed current hierarchy/tag/product models, migrations, protected routes, policies, controllers, form requests/actions and Vue state/layout/filter/error flows against current scope at HEADf26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus current Tag deletion/test working changes. No blocking finding in reviewed current-phase code; stock-dependent deactivation remains explicit later checkpoint, not passed. Automated catalogue suite PASS191 tests1579 assertions (DepartmentEdit,CategoryEdit,SubcategoryCreate/Edit/List,Tag,ProductCreate/List); focused outside-repo edit/status/list-permission checks PASS24 tests248 assertions. Full PHPStan0 errors, Vue types and whitespace PASS. Browser as SuperAdmin foodbank.test/tags: clicked Delete Cooking Required, confirmation named exact tag; Cancel returned with row preserved. Created unused disposable tag ZZ Browser Deletion Practice1030 via Create screen (actual exact name ZZ Browser Deletion Practice 1030, id69), search isolated it; Delete confirmation now open, not confirmed. Browser-use policy requires action-time confirmation before permanent deletion. Pending async question authorizes deleting ONLY this exact test tag; no response yet. No existing tag deleted. Browser successful deletion/blocked error and phone layout remain unverified in this review. No application source edits. Do not mark FB-048/067 complete pending browser evidence and scope-specific deferred guard accounting.
+2026-10-30 user approved permanent deletion of ONLY unused test tag ZZ Browser Deletion Practice 1030. On reacquiring FoodBank tab after approval, confirmation was no longer open and filtered list already showed No tags found. Reload confirmed absence; read-only live Tag query by exact name returned false. Assistant did not click OK or delete anything after approval, and did not observe success toast; cannot attribute deletion or claim full successful-deletion interaction observed. Disposable tag absent and no cleanup needed. Previous source/tests/Cancel confirmation evidence remains valid. Remaining browser blocked-error and narrow-screen verification still open; no whole-catalogue completion claimed.
+2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.
+2026-10-30 assistant, explicitly delegated remaining browser checks in own browser, NOT Brave: ChatGPT in-app browser signed in to local foodbank.test with configured SuperAdmin account. Read-only database query established Cooking Required id42 has180 product links. Delete confirmation cancelled once; developer then explicitly approved confirming this exact blocked-deletion test. Confirmed: request processing disabled Delete; response visibly displayed "This tag cannot be deleted because a product still uses it. Remove it from all products, including inactive products, first." Row preserved and Delete reenabled. At390x844 tag list/action buttons wrap, error text readable, document scrollWidth390 equals innerWidth390; no horizontal page overflow. Saved screenshot /tmp/foodbank-browser-checks/blocked-tag-phone.jpg. Viewport reset. No application source edits; no successful deletion/toast interaction claimed. Remaining blocked-error and narrow-screen checks PASS. Historical successful-deletion interaction remains unobserved; stock guard deferred FB-053. Broader catalogue checkpoint not newly marked complete by these narrow checks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="105" customHeight="1">
       <x:c r="A52" s="9" t="n">
@@ -7070,7 +7083,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra55f98d23a114912"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcbad10d03eb47a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12683,9 +12696,8 @@
           <x:t xml:space="preserve">Project context</x:t>
         </x:is>
       </x:c>
-      <x:c r="D175" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The current learning order is the # column on Stories in Docs/FoodBank_Developer_Story_Tracker.xlsx. FB-001 through FB-070 remain stable IDs, not sequence numbers. Revised 2026-10-25 against AGENTS.md: complete each module before dependants; introduce required storage/relationships before use; move catalogue verification before Receive and totals after Receive. Code review and passed behaviour testing are required for completion.
+      <x:c r="D175" s="28" t="str">
+        <x:v>The current learning order is the # column on Stories in Docs/FoodBank_Developer_Story_Tracker.xlsx. FB-001 through FB-070 remain stable IDs, not sequence numbers. Revised 2026-10-25 against AGENTS.md: complete each module before dependants; introduce required storage/relationships before use; move catalogue verification before Receive and totals after Receive. Code review and passed behaviour testing are required for completion.
 2026-10-26 approved sequence: complete creation of a record before teaching its list. User creation first, then first-login setup and review/testing of the connected creation journey, then user lists. Keep unverified evidence open. No new requirements or application-code changes. Account creation lessons FB-016–FB-020 precede FB-009–FB-015. FB-006/FB-007 connect after the first frontend-created user and before creation completion.
 2026-10-27 developer-directed late checkpoint: FB-069 now includes the bcrypt 72-byte long-password repair and repeat test before its combined verification. FB-070 remains the final implementation item. Earlier FB-007 failed evidence stays visible; rescheduling does not complete or validate it.
 2026-10-28 developer-directed timing change: defer final QA of the frontend-created QA Volunteer first-password setup, direct /users/create denial, logout, and personal-password re-login until final project verification after FB-070 implementation, review, and testing. These required checks remain open; this timing change does not verify FB-019 or FB-006/FB-007. Continue eligible work meanwhile and retain these checks as a final completion gate.
@@ -12694,8 +12706,8 @@
 2026-10-28 latest developer instruction: defer every password-related test in the CURRENT pending task list until project-end verification after FB-070 implementation, review and testing, and execute remaining non-password checks now. Includes pending first-login/setup, password changes and credential-related verification; no password checks run in this delegated session. Existing FB-069 bcrypt repair implementation stays there, but its pending password repeat verification is now part of the final password checkpoint. Does not defer all future features or non-password checks. Preserve original failed/unverified password evidence; no completion inferred.
 2026-10-28 developer explicitly deferred the reproduced phone-display cleanup issue (type 506 then x; +1 506x stays visible) and its repair/review/retest until project-end verification after FB-070 implementation/review/testing, and explicitly requested moving to user lists now. Keep failed evidence and affected FB-017/FB-019 items open. This is an approved sequencing exception; it does not fix or verify the issue and is not FUTURE scope.
 2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
-2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.</x:t>
-        </x:is>
+2026-10-29 developer explicitly said user module is done FOR NOW and inventory will be next. Approved sequencing exception: park remaining user-module findings and advance upcoming lesson to FB-026 Department storage/creation despite unfinished FB-025. This is not a passed review/test or verified completion: long-name username overflow/server500 and two existing test-fixture failures remain unresolved, with all previous project-end deferrals preserved. Nine PHP type-description errors have been fixed/verified separately. No inventory implementation or new lesson supplied in this handoff; await developer request to begin. No application edits authorized by this planning decision.
+2026-10-30 explicit developer-approved early sidebar integration of User Management and Product Catalogue only. Remaining FB-008 role landing pages and account/password deferrals unchanged; preserve existing policy permissions.</x:v>
       </x:c>
       <x:c r="E175" s="28" t="inlineStr">
         <x:is>
@@ -13256,7 +13268,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5846f4532ef404b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd7df31d5e044b43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add breadcrumbs to user and catalogue pages
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R18fee2bffe2b41db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="Rd80bb63010684da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="Rb3bdfb2fe6a142c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R5930e05db8ec4066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stories" sheetId="2" r:id="R8baec4b4e770449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="3" r:id="R002b1f12d5564771"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -743,7 +743,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="22" t="str">
-        <x:v>2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
+        <x:v>2026-10-30 developer replied done, breadcrumbs work after explicit refresh/create-or-edit/parent-link check: developer-reported breadcrumb display and return-to-list navigation PASS. No assistant browser check. Does not verify all sidebar roles/mobile behaviour or complete full FB-008. Developer requests continued Stock Management planning; no stock implementation authorized. Next planning topic: propose Manager/Super Admin management of shared package definitions, Volunteers selection of existing definitions; decision pending. Catalogue FB-067 evidence reconciliation and product-code reconsideration remain before stock implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="100" customHeight="1">
@@ -753,7 +753,7 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="22" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Developer check sidebar links, list/create/edit highlights, collapsed/mobile layout and role visibility. Then return to FB-048/067 catalogue evidence reconciliation. Stock guard stays FB-053; remaining FB-008 landing-page work deferred.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Continue Stock Management planning one decision at a time: package-management permissions first, then summary ownership and classification locks. Reconcile catalogue FB-048/067 evidence and discuss visible product codes at FB-035 before stock implementation FB-034. Preserve pending sidebar checks and project-end deferrals.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65" customHeight="1">
@@ -763,7 +763,7 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="22" t="str">
-        <x:v>Developer-first sidebar behaviour checks pending; remaining FB-008 deferred.</x:v>
+        <x:v>Awaiting package-management permissions decision; planning only.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65" customHeight="1">
@@ -773,7 +773,7 @@
         </x:is>
       </x:c>
       <x:c r="B17" s="22" t="str">
-        <x:v>f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus four sidebar-related files, source-reviewed2026-10-30.</x:v>
+        <x:v>39a201c76a8e7421894db1b7d9da24fec1c14569 plus 19 breadcrumb page additions; source-reviewed 2026-10-30.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -783,7 +783,7 @@
         </x:is>
       </x:c>
       <x:c r="B18" s="18" t="str">
-        <x:v>Sidebar implemented; behaviour checks pending. Remaining FB-008 deferred.</x:v>
+        <x:v>Breadcrumb checks developer-reported PASS; full FB-008 remains deferred/open. Stock planning resumed.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3388,22 +3388,25 @@
           <x:t xml:space="preserve">Not tested</x:t>
         </x:is>
       </x:c>
-      <x:c r="O24" s="10" t="n"/>
+      <x:c r="O24" s="10" t="str">
+        <x:v>
+2026-10-30 developer replied done, breadcrumbs work after explicit refresh/create-or-edit/parent-link check: developer-reported breadcrumb display and return-to-list navigation PASS. No assistant browser check. Does not verify all sidebar roles/mobile behaviour or complete full FB-008. Developer requests continued Stock Management planning; no stock implementation authorized. Next planning topic: propose Manager/Super Admin management of shared package definitions, Volunteers selection of existing definitions; decision pending. Catalogue FB-067 evidence reconciliation and product-code reconsideration remain before stock implementation.</x:v>
+      </x:c>
       <x:c r="P24" s="30" t="n"/>
       <x:c r="Q24" s="10" t="str">
         <x:v>
 2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
-2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
+2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.
+2026-10-30 developer explicitly requested breadcrumbs everywhere. Added static defineOptions layout.breadcrumbs to all 19 users/departments/categories/subcategories/tags/products Index/Create/Edit and User Show pages. List crumb links to resource index; current action is non-clickable through existing Breadcrumbs component. Existing Dashboard/settings trails retained; auth/public pages use separate layouts. Followed inspected Skander game-settings/Edit.vue layout props pattern. Source review at HEAD 39a201c76a8e7421894db1b7d9da24fec1c14569 plus breadcrumb-only working changes PASS. Vue types, production build, scoped formatting and diff whitespace PASS. No application/browser behaviour tests run. Developer-first breadcrumb/navigation checks pending; full FB-008 remains open. Stock planning overview supplied; no stock implementation begun.
+2026-10-30 developer replied done, breadcrumbs work after explicit refresh/create-or-edit/parent-link check: developer-reported breadcrumb display and return-to-list navigation PASS. No assistant browser check. Does not verify all sidebar roles/mobile behaviour or complete full FB-008. Developer requests continued Stock Management planning; no stock implementation authorized. Next planning topic: propose Manager/Super Admin management of shared package definitions, Volunteers selection of existing definitions; decision pending. Catalogue FB-067 evidence reconciliation and product-code reconsideration remain before stock implementation.</x:v>
       </x:c>
       <x:c r="R24" s="10" t="str">
-        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Deferred to project end by developer on 2026-10-29. Before starting this item or feature: reread AGENTS.md from disk; apply its teaching and testing rules.
-Next: Connect login redirects to the already verified lists from FB-009–FB-015. Build the volunteer welcome page and connect the completed password-change action from FB-024 and logout. Verify each role and forced-setup priority; add inventory links only as those modules are completed.
-2026-10-29 developer explicitly deferred FB-008 (role landing pages/navigation) and FB-023 (administrative manager/volunteer password reset), including implementation, review and testing, to project end. Both remain required current scope, unstarted and unverified; not FUTURE. Eligible inventory lessons may proceed after non-deferred account work/checks. Schedule FB-008 then FB-023 after FB-068 and before FB-069 combined verification; FB-070 remains final implementation. Existing post-FB-070 password verification and other deferred repairs/checks remain unchanged. FB-025 can review/test implemented non-deferred account behaviour now but full completion awaits these deferred features and required final checks. At FB-008 reconcile legacy manager volunteer-list landing text with newer shared-directory requirement before teaching; no new destination approved by this deferral.
-Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Developer check sidebar links, list/create/edit highlights, collapsed/mobile layout and role visibility. Then return to FB-048/067 catalogue evidence reconciliation. Stock guard stays FB-053; remaining FB-008 landing-page work deferred.</x:v>
+        <x:v>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Continue Stock Management planning one decision at a time: package-management permissions first, then summary ownership and classification locks. Reconcile catalogue FB-048/067 evidence and discuss visible product codes at FB-035 before stock implementation FB-034. Preserve pending sidebar checks and project-end deferrals.</x:v>
       </x:c>
       <x:c r="S24" s="10" t="str">
         <x:v>
-2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.</x:v>
+2026-10-30 user explicitly requested assistant sidebar integration, confirmed User Management and Product Catalogue. Narrow early-navigation exception to FB-008; landing pages/password work remain deferred. Added Overview, User Management (Users/Create user), Product Catalogue (Products first then Departments/Categories/Subcategories/Tags), My Account. Kept Create user because user list lacks create button; removed starter-kit footer links. Shared auth.navigation uses existing resource viewAny and User create policies; routes unchanged. Reviewed AppSidebar.vue/NavMain.vue/types/auth.ts/HandleInertiaRequests.php at HEAD f26f5989a4ba56a2d76c2381f3d8690caeec8e36 plus working changes. Reactive links/empty groups/child-page highlighting. Poker AppSidebar inspected: same NavMain/NavUser/generated-route conventions. Vue types, production build, full PHPStan0 errors, scoped formatting/Pint, whitespace PASS. Developer-first sidebar behaviour checks pending; no application behaviour tests/browser acceptance performed for this new change. Full FB-008 not complete.
+2026-10-30 developer explicitly requested breadcrumbs everywhere. Added static defineOptions layout.breadcrumbs to all 19 users/departments/categories/subcategories/tags/products Index/Create/Edit and User Show pages. List crumb links to resource index; current action is non-clickable through existing Breadcrumbs component. Existing Dashboard/settings trails retained; auth/public pages use separate layouts. Followed inspected Skander game-settings/Edit.vue layout props pattern. Source review at HEAD 39a201c76a8e7421894db1b7d9da24fec1c14569 plus breadcrumb-only working changes PASS. Vue types, production build, scoped formatting and diff whitespace PASS. No application/browser behaviour tests run. Developer-first breadcrumb/navigation checks pending; full FB-008 remains open. Stock planning overview supplied; no stock implementation begun.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="105" customHeight="1">
@@ -7083,7 +7086,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcbad10d03eb47a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01e1bb276d1a4615"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13268,7 +13271,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd7df31d5e044b43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefa3dac671b440e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add package size management with searchable list and editing
</commit_message>
<xml_diff>
--- a/Docs/FoodBank_Developer_Story_Tracker.xlsx
+++ b/Docs/FoodBank_Developer_Story_Tracker.xlsx
@@ -637,7 +637,7 @@
       </ns0:c>
       <ns0:c r="B6" s="15" t="n">
         <ns0:f>COUNTIF(Stories!H4:H73,"Complete")</ns0:f>
-        <ns0:v>21</ns0:v>
+        <ns0:v>22</ns0:v>
       </ns0:c>
       <ns0:c r="C6" s="15" t="n"/>
       <ns0:c r="D6" s="18" t="inlineStr">
@@ -695,7 +695,7 @@
       </ns0:c>
       <ns0:c r="B10" s="15" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">FB-067</ns0:t>
+          <ns0:t xml:space="preserve">FB-034</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C10" s="15" t="n"/>
@@ -713,7 +713,7 @@
       </ns0:c>
       <ns0:c r="B11" s="29" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">FB-048 verified: status controls removed, database field/default retained; stock implementation not started.</ns0:t>
+          <ns0:t xml:space="preserve">Catalogue verified including REQ-197 Product status change. Stock implementation begins with Package sizes; no stock code generated by assistant.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C11" s="15" t="n"/>
@@ -722,7 +722,7 @@
       <ns0:c r="A12" s="15" t="n"/>
       <ns0:c r="B12" s="15" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer Volunteer Product-list and direct /products/create403 check. Then finish FB-067 scoped completed-feature review using prior review plus current source as needed and record exact evidence, advance to Package sizes FB-034. Do not rerun passed checks without new concerns; preserve account deferrals.</ns0:t>
+          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Scoped Package sizes create/list/edit/search milestone has passed delegated browser and30 focused tests; title review finding corrected by explicit authorization with exact before/after shown. TypeScript/whitespace checks pass after2 literal-title changes; no browser rerun claimed. Suitable scoped commit checkpoint, then continue Stock items prerequisites within FB-034. Actual package deletion stays disabled until stock_items dependencies and restrictive FK/reference/concurrency safeguards can be implemented and verified. Full FB-034 remains In progress; preserve18 identical baseline account/auth failures.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="C12" s="15" t="n"/>
@@ -740,7 +740,7 @@
       </ns0:c>
       <ns0:c r="B13" s="22" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">FB-067</ns0:t>
+          <ns0:t xml:space="preserve">FB-034</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -752,7 +752,7 @@
       </ns0:c>
       <ns0:c r="B14" s="22" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-10-31 FB-048 verified using completed-feature source review and developer-reported automated/browser PASS. FB-067 resumes with current REQ-197 retained-status-storage scope. Automated Product tests cover duplicates, role checks and list behaviour; previously reviewed unchanged catalogue evidence retained. Next small browser check: signed-in Volunteer can view Products without management buttons and direct /products/create is403. This additional direct-request browser check has not been reported passed for this revision.</ns0:t>
+          <ns0:t xml:space="preserve">2026-10-31 browser-title finding fixed by explicit request: Create/Edit Head titles now correct. Exact2 source changes, Vue type/whitespace checks PASS. Earlier30 focused tests/browser checks and original-data checksum verification preserved. Scoped package milestone ready for commit; full FB-034 still open for Stock items and deletion dependencies.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -764,7 +764,7 @@
       </ns0:c>
       <ns0:c r="B15" s="22" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer Volunteer Product-list and direct /products/create403 check. Then finish FB-067 scoped completed-feature review using prior review plus current source as needed and record exact evidence, advance to Package sizes FB-034. Do not rerun passed checks without new concerns; preserve account deferrals.</ns0:t>
+          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Scoped Package sizes create/list/edit/search milestone has passed delegated browser and30 focused tests; title review finding corrected by explicit authorization with exact before/after shown. TypeScript/whitespace checks pass after2 literal-title changes; no browser rerun claimed. Suitable scoped commit checkpoint, then continue Stock items prerequisites within FB-034. Actual package deletion stays disabled until stock_items dependencies and restrictive FK/reference/concurrency safeguards can be implemented and verified. Full FB-034 remains In progress; preserve18 identical baseline account/auth failures.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -776,7 +776,7 @@
       </ns0:c>
       <ns0:c r="B16" s="22" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Waiting for developer Volunteer catalogue/direct-create permission check.</ns0:t>
+          <ns0:t xml:space="preserve">No title blocker; developer controls commit and next implementation lesson. Stock-dependent deletion remains disabled.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -788,7 +788,7 @@
       </ns0:c>
       <ns0:c r="B17" s="22" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">HEAD 8e02225c01342cc598712b990636f057b15f4951 plus existing working changes and delegated Product status changes; source review 2026-10-31.</ns0:t>
+          <ns0:t xml:space="preserve">Scoped package source review2026-10-31, HEAD e08b6b6d5652909ad14cad745425e16c0ac8f9d6 plus package working snapshot: title finding open; prior catalogue verification unchanged.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -800,7 +800,7 @@
       </ns0:c>
       <ns0:c r="B18" s="18" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">FB-048 complete; FB-067 scoped catalogue recheck in progress.</ns0:t>
+          <ns0:t xml:space="preserve">FB-034 In progress; package-screen milestone verified with title fix; Stock items and delete integration pending.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -969,7 +969,7 @@
       </ns0:c>
       <ns0:c r="B31" s="18" t="inlineStr">
         <ns0:is>
-          <ns0:t>Resume: reread AGENTS.md, Start Here, current FB-048 full Stories row and related Requirements. Plan is finalized; do not restart questionnaires. Wait for permission if not given. Developer writes code; review at feature checkpoint,developer-first behaviour checks. Preserve all account deferrals and final FB-070.</ns0:t>
+          <ns0:t xml:space="preserve">Resume: reread AGENTS.md, Start Here, FB-034 full Stories row and related Requirements. Preserve deferred tests; do not mark complete or advance to Stock items before coherent Package sizes review/testing. Developer writes code unless an explicit scoped exception is given.</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -5756,63 +5756,67 @@
       </ns0:c>
       <ns0:c r="G51" s="4" t="str">
         <ns0:f>IF(H51="Complete","Complete",IF(I51="Blocked","Blocked",IF(I51="In progress","Ready",IF(F51="","Ready",IF(COUNTIFS($B$4:$B$73,F51,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</ns0:f>
-        <ns0:v>Ready</ns0:v>
+        <ns0:v>Complete</ns0:v>
       </ns0:c>
       <ns0:c r="H51" s="4" t="str">
         <ns0:f>IF(I51="Not started","Not started",IF(I51="Blocked","Blocked",IF(I51="In progress","In progress",IF(J51&lt;&gt;"Passed","Awaiting code review",IF(OR(K51="",NOT(ISNUMBER(L51))),"Awaiting review evidence",IF(N51&lt;&gt;"Passed","Awaiting test",IF(OR(M51="",O51="",NOT(ISNUMBER(P51))),"Awaiting test evidence","Complete")))))))</ns0:f>
-        <ns0:v>In progress</ns0:v>
+        <ns0:v>Complete</ns0:v>
       </ns0:c>
       <ns0:c r="I51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t>In progress</ns0:t>
+          <ns0:t xml:space="preserve">Ready for review</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="J51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t>Not reviewed</ns0:t>
+          <ns0:t xml:space="preserve">Passed</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t>
+          <ns0:t xml:space="preserve">
 2026-10-30 source review PASS at HEAD 39a201c76a8e7421894db1b7d9da24fec1c14569 plus current three-level working changes: app Models/Actions/Products/Requests/Products/ProductController/HandleInertiaRequests, protected routes, ProductPolicy, ProductForm/products pages/sidebar/types, original products migration, CatalogueData and seeders/tests. Inspected Poker PlayerController/DeactivatePlayer and prior game-settings layout pattern. No blocking source finding. Server permissions on GET Create/Edit and POST/PATCH via policy plus request/action Gate; same-category normalized duplicate always blocked; cross-category confirmation before write; no catalogue stock fields. Types/build/PHPStan0 errors/Pint/frontend checks/whitespace PASS. Browser and local MySQL rebuild pending.
 Browser usability findings: Browser review findings2026-10-30: Department and Category list pages have no Create button and sidebar offers only their list links, so creation requires direct URL; confirmed sources resources/js/pages/departments/Index.vue and categories/Index.vue. Mobile sidebar also remains open after selecting Products; Escape closes it. These usability issues are not fixed or newly approved scope. Full catalogue checkpoint remains open pending decision/fix/recheck. No data-integrity or permission failure observed in exercised catalogue checks.
 2026-10-30 developer explicitly authorized fixing both browser usability findings and verifying in assistant browser NOT Brave. Added policy-derived canCreate props in DepartmentController/CategoryController index; conditional Create department/Create category links in list Card headers. NavMain uses existing useSidebar context and setOpenMobile(false) on Link click, leaving desktop open state unchanged. Scoped source review PASS. ChatGPT in-app browser SuperAdmin: both links visible and open correct Create forms;390x844 drawer closes after Departments navigation and when selecting same Departments link via Enter; page and Create button immediately usable.1280x900 desktop sidebar remains visible after Categories navigation and Create category link visible. Final browser warnings/errors empty. Vue types, production build, PHPStan0 errors, scoped formatting/Pint and whitespace PASS. Prior57 automated catalogue tests434 assertions and broader browser evidence retained; no redundant suite run for these UI fixes. No new database records or source changes beyond the5 scoped files. Screenshots /tmp/foodbank-catalogue-browser/fixed-mobile-sidebar.png and fixed-create-buttons.png. Both prior usability findings RESOLVED. Existing inactive browser test Product111 unchanged. Stock zero-balance deactivation guard remains later FB-053; remaining FB-008 role landing work deferred.
-2026-10-31 scope revision: prior evidence applies to historical status-bearing snapshot. Product-status removal and affected behaviour require fresh review/developer tests; no regression/failure of unrelated prior behaviour claimed.</ns0:t>
+2026-10-31 scope revision: prior evidence applies to historical status-bearing snapshot. Product-status removal and affected behaviour require fresh review/developer tests; no regression/failure of unrelated prior behaviour claimed.
+2026-10-31 FB-067 scoped completed-feature source review PASS on HEAD 8e02225c01342cc598712b990636f057b15f4951 plus existing three-level catalogue and delegated Product status working changes. Rechecked ProductPolicy, Product routes GET/POST/PATCH abilities, Product model/migration (category FK, retained default true, name_key uniqueness), StoreProductRequest editable allowlist, CreateProduct/UpdateProduct Gates and transactions, CheckProductName including stored-inactive duplicate checks. Reused same-chat completed-feature review of ListProducts, ProductController, ProductForm and products Edit/Index, updated tests; no changes since reported checks. No blocking finding. Earlier Department/Category baseline review retained; this is scoped re-verification of REQ-197, not new stock or account verification.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="L51" s="30" t="n">
-        <ns0:v>46325</ns0:v>
-      </ns0:c>
-      <ns0:c r="M51" s="10" t="str">
-        <ns0:v>Assistant (delegated automated + in-app browser verification)</ns0:v>
+        <ns0:v>46326</ns0:v>
+      </ns0:c>
+      <ns0:c r="M51" s="10" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">Developer (reported automated and browser checks)</ns0:t>
+        </ns0:is>
       </ns0:c>
       <ns0:c r="N51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t>Not tested</ns0:t>
+          <ns0:t xml:space="preserve">Passed</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="O51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t>
+          <ns0:t xml:space="preserve">
 2026-10-30 assistant explicitly delegated temporary in-memory catalogue tests: PASS56 tests429 assertions, ProductCreateTest/ProductListTest/CatalogueSeederTest/DepartmentEditTest/CategoryEditTest. Includes direct action Volunteer denial, form/save route permissions, invalid fields/parent mismatch, inactive/case/space duplicate block and database uniqueness, cross-category warning/confirmation at create/rename/move, status-only edit, pagination/search/filter/no results, retired routes404, new schema and idempotent realistic seeds. No browser acceptance or MySQL migration executed. Full unrelated account suite not rerun; prior baseline account failures remain separately recorded.
 Final 2026-10-30 delegated catalogue suite PASS57 tests434 assertions after adding default DatabaseSeeder integration coverage. All migrations created in temporary SQLite, default seeder creates configured accounts plus exactly4 Departments/25 Categories/110 Products. Earlier commentary count115 corrected by direct seed-data count:110. No local MySQL reset or browser acceptance performed. Current source review remains PASS; browser checks pending.
 2026-10-30 developer explicitly delegated full catalogue verification in assistant browser, NOT Brave. Used ChatGPT in-app browser foodbank.test only. Signed in as seeded SuperAdmin then developer-supplied setup-complete Manager amina.rahman and Volunteer farah.khan (do not record passwords). Live UI PASS: Product→Category→Department→Status column order, Rice search, no matches, clear search, next-page10 rows, Department+Category filters/reset to page1; required Create errors; normalized same-category rICE duplicate blocked; cross-category warning shows Food→Grains→Rice; acknowledgement cleared after name edit; explicit confirmation creates and resets form with success; Edit rename warning/Cancel preserves saved name; move into duplicate category blocked; cross-category confirmed move persists same Product111 ID; confirmed rename persists; status-only edit no repeated warning; deactivate/reactivate; Inactive list; cross-Department move clears stale Category and persists selected valid Category. Phone390x844: page scrollWidth390, form fits, table scrolls in306px container rather than page overflow. Desktop1280x900 visually checked; viewport reset. Department search/duplicate errors/rename, Category search/rename and current Department labels checked; original Food and Grains names restored. Manager Create/Edit and no-op Product save successful; Department/Category Create forms accessible and duplicate input rejected. Volunteer Product list has no Create/Edit/actions, only Product catalogue sidebar link; direct Product Create/Edit and Department/Category URLs return403; guest Products redirects login. Removed Tags/Subcategories URLs404. Browser console warn/error log empty at final check. No browser POST/PATCH forgery attempted; prior57 automated tests434 assertions cover those server rules. No account/password changes, local DB reset or source edits in this turn.
 2026-10-30 developer explicitly authorized fixing both browser usability findings and verifying in assistant browser NOT Brave. Added policy-derived canCreate props in DepartmentController/CategoryController index; conditional Create department/Create category links in list Card headers. NavMain uses existing useSidebar context and setOpenMobile(false) on Link click, leaving desktop open state unchanged. Scoped source review PASS. ChatGPT in-app browser SuperAdmin: both links visible and open correct Create forms;390x844 drawer closes after Departments navigation and when selecting same Departments link via Enter; page and Create button immediately usable.1280x900 desktop sidebar remains visible after Categories navigation and Create category link visible. Final browser warnings/errors empty. Vue types, production build, PHPStan0 errors, scoped formatting/Pint and whitespace PASS. Prior57 automated catalogue tests434 assertions and broader browser evidence retained; no redundant suite run for these UI fixes. No new database records or source changes beyond the5 scoped files. Screenshots /tmp/foodbank-catalogue-browser/fixed-mobile-sidebar.png and fixed-create-buttons.png. Both prior usability findings RESOLVED. Existing inactive browser test Product111 unchanged. Stock zero-balance deactivation guard remains later FB-053; remaining FB-008 role landing work deferred.
-2026-10-31 scope revision: prior evidence applies to historical status-bearing snapshot. Product-status removal and affected behaviour require fresh review/developer tests; no regression/failure of unrelated prior behaviour claimed.</ns0:t>
+2026-10-31 scope revision: prior evidence applies to historical status-bearing snapshot. Product-status removal and affected behaviour require fresh review/developer tests; no regression/failure of unrelated prior behaviour claimed.
+2026-10-31 developer-reported PASS: all requested ProductCreateTest/ProductListTest/CatalogueSeederTest automated checks and browser Create/Edit/List/status absence/save/search/hierarchy/pagination (previous all passed), plus explicit Volunteer list visible with no Create/Edit buttons and direct /products/create403 (done,both work). Product suite covers missing/forged status, action status protection, legacy inactive values, duplicates/confirmation and role denied requests. No assistant application/browser tests executed and no counts invented. Preserves historical catalogue evidence and unrelated account deferrals.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="P51" s="30" t="n">
-        <ns0:v>46325</ns0:v>
+        <ns0:v>46326</ns0:v>
       </ns0:c>
       <ns0:c r="Q51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">2026-10-31 FB-048 verified using completed-feature source review and developer-reported automated/browser PASS. FB-067 resumes with current REQ-197 retained-status-storage scope. Automated Product tests cover duplicates, role checks and list behaviour; previously reviewed unchanged catalogue evidence retained. Next small browser check: signed-in Volunteer can view Products without management buttons and direct /products/create is403. This additional direct-request browser check has not been reported passed for this revision.</ns0:t>
+          <ns0:t xml:space="preserve">2026-10-31 FB-067 complete after scoped source review and developer-reported passing checks. Proceed to Package sizes FB-034.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="R51" s="10" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer Volunteer Product-list and direct /products/create403 check. Then finish FB-067 scoped completed-feature review using prior review plus current source as needed and record exact evidence, advance to Package sizes FB-034. Do not rerun passed checks without new concerns; preserve account deferrals.</ns0:t>
+          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Catalogue checkpoint verified. Continue Package sizes FB-034; preserve account deferrals and final FB-070.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="S51" s="10" t="str">
@@ -5850,15 +5854,15 @@
       </ns0:c>
       <ns0:c r="G52" s="9" t="str">
         <ns0:f>IF(H52="Complete","Complete",IF(I52="Blocked","Blocked",IF(I52="In progress","Ready",IF(F52="","Ready",IF(COUNTIFS($B$4:$B$73,F52,$H$4:$H$73,"Complete")=1,"Ready","Waiting")))))</ns0:f>
-        <ns0:v>Waiting</ns0:v>
+        <ns0:v>Ready</ns0:v>
       </ns0:c>
       <ns0:c r="H52" s="9" t="str">
         <ns0:f>IF(I52="Not started","Not started",IF(I52="Blocked","Blocked",IF(I52="In progress","In progress",IF(J52&lt;&gt;"Passed","Awaiting code review",IF(OR(K52="",NOT(ISNUMBER(L52))),"Awaiting review evidence",IF(N52&lt;&gt;"Passed","Awaiting test",IF(OR(M52="",O52="",NOT(ISNUMBER(P52))),"Awaiting test evidence","Complete")))))))</ns0:f>
-        <ns0:v>Not started</ns0:v>
+        <ns0:v>In progress</ns0:v>
       </ns0:c>
       <ns0:c r="I52" s="11" t="inlineStr">
         <ns0:is>
-          <ns0:t xml:space="preserve">Not started</ns0:t>
+          <ns0:t xml:space="preserve">In progress</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="J52" s="11" t="inlineStr">
@@ -5866,7 +5870,12 @@
           <ns0:t xml:space="preserve">Not reviewed</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="K52" s="11" t="n"/>
+      <ns0:c r="K52" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-10-31 scoped source review over HEAD e08b6b6d5652909ad14cad745425e16c0ac8f9d6 + package working tree: app/Actions/PackageSizes/*, PackageSize model/policy, PackageSize requests/controller, routes/web.php, HandleInertiaRequests, AppSidebar/auth types, PackageSizeForm, package-sizes/Create/Edit/Index, shared choices, PackageSizeSeeder/DatabaseSeeder and migration. Finding: Create.vue18 and Edit.vue26 Head title is literal +title+, reproduced in browser. No application source fixes authorized/performed during test run. Create/edit/search/permissions behaviour verified as described in test evidence. Delete logic explicitly deferred to actual Stock items dependency; button disabled. Keep full FB-034 open (includes Stock items), no module-wide Passed review/test claim.
+2026-10-31 follow-up: title finding corrected by explicit authorization;2 literal Head titles source-reviewed PASS, Vue type and whitespace checks PASS. Scoped source review has no remaining finding; overall stock setup/deletion integration remains pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="L52" s="31" t="n"/>
       <ns0:c r="M52" s="11" t="n"/>
       <ns0:c r="N52" s="11" t="inlineStr">
@@ -5874,11 +5883,15 @@
           <ns0:t xml:space="preserve">Not tested</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="O52" s="11" t="n"/>
+      <ns0:c r="O52" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">2026-10-31 assistant-delegated checks: dedicated IAB browser only, Brave untouched. Existing PackageSizeManagementTest PASS12 tests129 assertions (list, edit, validation, roles, guest, simulated reference fixture). Additional temporary isolated SQLite CreateAndSearchTest PASS18 tests89 assertions (create roles/validation, g-kg/ml-L/item equivalence, protected submissions, search-before-pagination, repeat seeder without changes). Initial extra test count assumption36 corrected to37 after inspecting developer-added Can1kg seed; application source unchanged. Total focused30 tests218 assertions pass. Full current suite105 tests87 pass17 failures1 error; clean HEAD temporary copy93 tests75 pass has identical18 failing/error names, no new failures. PHPStan0 errors, Vue type check, scoped Pint and whitespace PASS. Browser PASS Manager create/reset/toast, exact kg/g and L/ml duplicates+retained input, distinct package types, fractional items/zero/negative/excess precision/missing input browser validity, whole items, edit/self-equivalent/no duplicate/redirect/cancel, live/case/space/empty search, ten-row pages/query persistence/reset, sidebar permissions, Volunteer403 list/create/edit, guest login redirects, SuperAdmin edit, simultaneous two-tab creation gives one success/one duplicate with DB count1, disabled Delete, 1440px desktop and390px phone stacked fields/table overflow contained (page width390/table463/container306). Real stock_items table absent: reference fixture does not prove later real concurrent integration. Browser title review finding remains. Five tracked browser test definitions and three temporary accounts removed; baseline SHA256 comparisons confirmed EVERY row unchanged in categories25,departments4,products110,package_sizes37,users14,roles3,migrations8 and other business tables; runtime sessions/cache excluded. Original data never edited; no stock schema created on live DB. All browser tabs closed and viewport restored.</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="P52" s="31" t="n"/>
       <ns0:c r="Q52" s="11" t="inlineStr">
         <ns0:is>
-          <ns0:t>2026-10-31: visible Product codes excluded from version one. Latest approved Stock Management design in REQ-185 supersedes historical Subcategory/classification-lock proposals. Continue planning only; ask developer before first implementation lesson.
+          <ns0:t xml:space="preserve">2026-10-31: visible Product codes excluded from version one. Latest approved Stock Management design in REQ-185 supersedes historical Subcategory/classification-lock proposals. Continue planning only; ask developer before first implementation lesson.
 2026-10-31 developer-approved brand decision: brand is an optional text field stored on each stock choice, not a shared brand list or separate Brand resource. Empty means unbranded. Ignore extra spaces and letter case when checking duplicate Product/brand/package combinations. Manager/Super Admin enter brand during stock-choice setup; Volunteers select existing choices only. Preserve approved brand spelling corrections subject to duplicate checks.
 2026-10-31 developer-approved scope change: leave stock tags out of version one. No stock tag fields, tables, management screens, selection, filters or tag editing required. This supersedes earlier optional shared stock-tag requirements. Reconsider tags only through a later scope decision.
 2026-10-31 developer-approved inactive-choice rule: block inactive stock choices from all three movement types: Receive, Distribute and Adjust. Manager/Super Admin must reactivate before further movements. Preserve history. Enforce on server at submission, including stale forms; hiding choices alone is insufficient. Existing zero-balance deactivation rule remains.
@@ -5908,15 +5921,24 @@
 2026-10-31 developer approved permanently fixing Product total unit after first saved movement on ANY linked stock item (Receive/Distribute/Adjust), superseding first-receipt-only summary lock. Remains locked at zero stock. Same-family alternative package stock items remain allowed; cross-family setup correction after history remains version-two ##FUTURE. No stock implementation started; ask before first implementation lesson.
 2026-10-31 developer approved Volunteers viewing Product totals, alongside Managers/Super Admin. Supersedes earlier manager-only summary permission. All three roles may view Stock items and combined Product totals. This is read access only: stock/package setup and permitted unused deletion remain Manager/Super Admin; movement history remains Manager/Super Admin only. Enforce permissions on routes and requests, not only links. Planning only; ask before first implementation lesson.
 2026-10-31 developer approved one searchable stock-item picker for Receive, Distribute and Adjust, as demoed. Search Product name/optional brand, results identify Product+brand+package and current whole-package availability. Receive/Adjust include zero-stock items; Distribute only positive balances. Replaces prior Product-first then stock-choice distribution selection. Retain household selection before distribution, multiple stock items for Receive/Distribute, one row per stock_item_id, single-item Adjust with Add/Remove and required reason, whole-package validation and final server stock recheck. Picker demo is selection-only, not full form implementation. No stock code authorization; ask before first implementation lesson.
-2026-10-31 developer explicitly confirmed Receive, Distribute and Adjust are separate screens, sharing searchable stock-item picker behaviour only; demo mode buttons are not proposed application tabs. Receive supports multiple items/optional whole-entry note; Distribute one household/multiple items/review before save; Adjust one item/Add-or-Remove/required reason. Developer approved stock-item history newest first, 10 movements per page. Retain Manager/Super Admin history permissions and all movement safeguards. Stock planning continues; ask before first implementation lesson.</ns0:t>
+2026-10-31 developer explicitly confirmed Receive, Distribute and Adjust are separate screens, sharing searchable stock-item picker behaviour only; demo mode buttons are not proposed application tabs. Receive supports multiple items/optional whole-entry note; Distribute one household/multiple items/review before save; Adjust one item/Add-or-Remove/required reason. Developer approved stock-item history newest first, 10 movements per page. Retain Manager/Super Admin history permissions and all movement safeguards. Stock planning continues; ask before first implementation lesson.
+2026-10-31 FB-034 first small lesson assigned after verified catalogue: developer runs php artisan make:model PackageSize -m. Explain model as Laravel representation of one reusable package definition and migration as table blueprint. This command only generates two files; no table creation or data mutation until a later explained migrate step. Await developer confirmation without reviewing generated code after ordinary done. Do not add speculative stock relationships. Prior all-status-code authorization was scoped to Product status; no stock source edits delegated.
+2026-10-31 progress: developer generated PackageSize/model/migration, policy/controller/requests and CreatePackageSize. Assistant moved requests into PackageSizes with namespaces/imports by explicit authorization. Developer reported migration runs and empty-table rollback/recreation; definition_key folded into original create migration and extra pending migration deleted by explicit instruction. Create form/action implemented incrementally on request; definition_key uses exact thousandths for weight/volume and unscaled whole counts for items (box:item:12). Server rejects fractional item contents; duplicate precheck + unique constraint + readable race error. User requested short references for previously taught FoodBank patterns; explain new concepts, restart explanations in any new project. Developer reported minimal page and button layout looked correct, but explicitly postponed creation behaviour checks (save/reset, equivalent duplicates, fractional items). Latest explicit instruction: implement full list/edit/sidebar despite deferred tests. Added ListPackageSizes, UpdatePackageSize (transaction/row lock, policy recheck, equivalent duplicate exclusion of self), Index request, shared inherited Store/Update validation, decimal:3 model cast, typed validated packageData, shared GetPackageSizeDefinitionKey and PackageSizeForm, Index/Edit pages, route permissions, sidebar permission/type. Manager/Super Admin only; viewAny on list, update on GET/PATCH and action. Sidebar Stock Management &gt; Package sizes. Ten-row deterministic pagination, no extra filters. isReferenced uses existing stock_items table only if present; no stock schema/models created. Actual FK and concurrent reference-writer lock integration must be verified at stock-item checkpoint. Added tests/Feature/PackageSizeManagementTest.php but did not run it: developer-first testing not delegated. Scoped syntax/format and full PHPStan/Vue type checks PASS. No DB mutation or acceptance checks by assistant this request. Package deletion and stock-item setup remain unimplemented; FB-034 stays In progress, Not reviewed, Not tested. Upcoming module-wide review remains pending; current implementation inspection is not final-feature signoff. Working snapshot over HEAD e08b6b6d5652909ad14cad745425e16c0ac8f9d6. Inspected reference: Poker routes/web.php policy middleware; PlayerController list/Inertia flow; Actions/Games/CorrectCashout.php transaction/lock/recheck convention.
+2026-10-31 developer explicitly requested package-type search on Package sizes list. Implemented validated search (100 characters), case-insensitive partial type match with individual_item treated as individual item, filtering before pagination, retained search in page links and 300ms Vue debounce/reset to page one. Scoped format, full PHPStan and Vue type checks PASS; behaviour checks remain deferred/not run. PackageSizeSeeder was also explicitly authorized, written with36 reusable definitions, registered in DatabaseSeeder and later run alone on explicit user request; database total37 afterward, box:item:12 confirmed present. No creation/edit/list acceptance tests implied by seeding.
+2026-10-31 superseding testing state: developer explicitly delegated all tests in assistant browser (not Brave), cleanup only new test data and preserve existing records. See review/test evidence K/O. Browser+focused tests passed apart from title presentation finding; full-suite18 failures reproduced exactly on committed baseline. Deleted all5 owned test packages and3 owned test users, complete original business-row checksum verification PASS. User also explicitly deferred delete implementation until dependencies are ready; Delete button is disabled in every row, no DELETE route/action added. Later real stock-item FK/lock/reference verification remains required.
+2026-10-31 developer explicitly authorized necessary title fixes and requested exact changes. Assistant changed ONLY Head title literals: resources/js/pages/package-sizes/Create.vue18 +title+ -&gt; Create Package Size; Edit.vue26 +title+ -&gt; Edit Package Size. Source review confirms correct literals; npm run types:check and git diff --check PASS. No DB mutations, browser rerun, unrelated application edits or baseline test repairs. Previous30 focused tests218 assertions/browser/data-preservation evidence remains valid; title fix verified statically only. Title review finding resolved; package delete and actual stock-item integration remain explicit later checkpoints, so whole FB-034 not complete.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="R52" s="11" t="inlineStr">
         <ns0:is>
-          <ns0:t>Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Await developer confirmation before first lesson. Catalogue no-status alignment and FB-067 recheck precede stock setup. Then begin Package sizes storage in small steps; finish create before list, full feature review/testing before stock-item module.</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="S52" s="11" t="n"/>
+          <ns0:t xml:space="preserve">Before starting/resuming this item or feature: reread AGENTS.md from disk; apply teaching/testing rules. Scoped Package sizes create/list/edit/search milestone has passed delegated browser and30 focused tests; title review finding corrected by explicit authorization with exact before/after shown. TypeScript/whitespace checks pass after2 literal-title changes; no browser rerun claimed. Suitable scoped commit checkpoint, then continue Stock items prerequisites within FB-034. Actual package deletion stays disabled until stock_items dependencies and restrictive FK/reference/concurrency safeguards can be implemented and verified. Full FB-034 remains In progress; preserve18 identical baseline account/auth failures.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="S52" s="11" t="inlineStr">
+        <ns0:is>
+          <ns0:t xml:space="preserve">No current package-screen blocker. Actual Stock items dependencies and delete/reference/concurrency integration remain pending.</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="53" ht="100" customHeight="1">
       <ns0:c r="A53" s="9" t="n">
@@ -13571,7 +13593,8 @@
       </ns0:c>
       <ns0:c r="D194" t="inlineStr">
         <ns0:is>
-          <ns0:t>2026-10-31 finalized: Separate Package sizes screen for Manager/Super Admin. Define package type (bag, box, can, bottle, carton, jar, packet, individual item), positive contents and contents unit. Reuse across Products. Reject equivalent definitions in same package type after g/kg or ml/litre normalization; different package types remain distinct. Definition fields editable only before reference.</ns0:t>
+          <ns0:t xml:space="preserve">2026-10-31 finalized: Separate Package sizes screen for Manager/Super Admin. Define package type (bag, box, can, bottle, carton, jar, packet, individual item), positive contents and contents unit. Reuse across Products. Reject equivalent definitions in same package type after g/kg or ml/litre normalization; different package types remain distinct. Definition fields editable only before reference.
+2026-10-31 approved addition: Package sizes list includes one text search for package type. Search all matching definitions before pagination and retain search while changing pages.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E194" t="inlineStr">
@@ -13635,7 +13658,8 @@
       </ns0:c>
       <ns0:c r="D196" t="inlineStr">
         <ns0:is>
-          <ns0:t>2026-10-31 finalized: Manager/Super Admin may delete package definition only if no stock_item references package_size_id, including zero-balance items. Enforce policy and restrictive foreign key. No cascading deletion.</ns0:t>
+          <ns0:t xml:space="preserve">2026-10-31 finalized: Manager/Super Admin may delete package definition only if no stock_item references package_size_id, including zero-balance items. Enforce policy and restrictive foreign key. No cascading deletion.
+2026-10-31 implementation timing explicitly revised by developer: show disabled Delete button now; defer actual delete action/route/guards until Stock items table and dependencies exist. Unused-only policy and restrictive FK requirements remain current scope.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E196" t="inlineStr">

</xml_diff>